<commit_message>
Logs: auto summary & updates (2025-10-03 05:24:01)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -1733,10 +1733,12 @@
       <c r="F37" t="n">
         <v>0.2150537634408602</v>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="n">
+        <v>0.1666666666666667</v>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>0.2067 (0.0118)</t>
+          <t>0.1934 (0.0246)</t>
         </is>
       </c>
     </row>
@@ -1839,10 +1841,12 @@
       <c r="F40" t="n">
         <v>0.25</v>
       </c>
-      <c r="G40" t="inlineStr"/>
+      <c r="G40" t="n">
+        <v>0.2127659574468085</v>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>0.2687 (0.0265)</t>
+          <t>0.2501 (0.0374)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 07:24:37)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -2552,11 +2552,13 @@
       <c r="E60" t="n">
         <v>0.1212121212121212</v>
       </c>
-      <c r="F60" t="inlineStr"/>
+      <c r="F60" t="n">
+        <v>0.2133333333333333</v>
+      </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
-          <t>0.1212 (0.0000)</t>
+          <t>0.1673 (0.0651)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 08:24:56)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -2727,10 +2727,12 @@
       <c r="F65" t="n">
         <v>0.2380952380952381</v>
       </c>
-      <c r="G65" t="inlineStr"/>
+      <c r="G65" t="n">
+        <v>0.2278481012658228</v>
+      </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>0.1770 (0.0864)</t>
+          <t>0.1940 (0.0678)</t>
         </is>
       </c>
     </row>
@@ -2761,10 +2763,12 @@
       <c r="F66" t="n">
         <v>0.1041666666666667</v>
       </c>
-      <c r="G66" t="inlineStr"/>
+      <c r="G66" t="n">
+        <v>0.1020408163265306</v>
+      </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>0.1262 (0.0311)</t>
+          <t>0.1181 (0.0260)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 10:25:33)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -2448,11 +2448,13 @@
       <c r="E57" t="n">
         <v>0.1408450704225352</v>
       </c>
-      <c r="F57" t="inlineStr"/>
+      <c r="F57" t="n">
+        <v>0.24</v>
+      </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>0.1408 (0.0000)</t>
+          <t>0.1904 (0.0701)</t>
         </is>
       </c>
     </row>
@@ -2586,11 +2588,13 @@
       <c r="E61" t="n">
         <v>0.1052631578947368</v>
       </c>
-      <c r="F61" t="inlineStr"/>
+      <c r="F61" t="n">
+        <v>0.05555555555555555</v>
+      </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>0.1053 (0.0000)</t>
+          <t>0.0804 (0.0351)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 11:25:50)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -2625,10 +2625,12 @@
       <c r="F62" t="n">
         <v>0.2388059701492537</v>
       </c>
-      <c r="G62" t="inlineStr"/>
+      <c r="G62" t="n">
+        <v>0.1891891891891892</v>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>0.1682 (0.0999)</t>
+          <t>0.1752 (0.0717)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 12:26:09)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -2557,10 +2557,12 @@
       <c r="F60" t="n">
         <v>0.2133333333333333</v>
       </c>
-      <c r="G60" t="inlineStr"/>
+      <c r="G60" t="n">
+        <v>0.2340425531914894</v>
+      </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>0.1673 (0.0651)</t>
+          <t>0.1895 (0.0601)</t>
         </is>
       </c>
     </row>
@@ -3653,10 +3655,12 @@
       <c r="F91" t="n">
         <v>0.3120567375886525</v>
       </c>
-      <c r="G91" t="inlineStr"/>
+      <c r="G91" t="n">
+        <v>0.3289473684210527</v>
+      </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>0.3656 (0.0757)</t>
+          <t>0.3534 (0.0576)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 13:26:27)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -3344,11 +3344,13 @@
       <c r="E82" t="n">
         <v>0.4931506849315068</v>
       </c>
-      <c r="F82" t="inlineStr"/>
+      <c r="F82" t="n">
+        <v>0.4148148148148148</v>
+      </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>0.4932 (0.0000)</t>
+          <t>0.4540 (0.0554)</t>
         </is>
       </c>
     </row>
@@ -3448,11 +3450,13 @@
       <c r="E85" t="n">
         <v>0.5176470588235295</v>
       </c>
-      <c r="F85" t="inlineStr"/>
+      <c r="F85" t="n">
+        <v>0.373134328358209</v>
+      </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>0.5176 (0.0000)</t>
+          <t>0.4454 (0.1022)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 14:26:46)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -3625,10 +3625,12 @@
       <c r="F90" t="n">
         <v>0.358974358974359</v>
       </c>
-      <c r="G90" t="inlineStr"/>
+      <c r="G90" t="n">
+        <v>0.4260355029585799</v>
+      </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>0.4483 (0.1263)</t>
+          <t>0.4409 (0.0903)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 15:27:06)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -3484,11 +3484,13 @@
       <c r="E86" t="n">
         <v>0.4888888888888889</v>
       </c>
-      <c r="F86" t="inlineStr"/>
+      <c r="F86" t="n">
+        <v>0.2769230769230769</v>
+      </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>0.4889 (0.0000)</t>
+          <t>0.3829 (0.1499)</t>
         </is>
       </c>
     </row>
@@ -3519,10 +3521,12 @@
       <c r="F87" t="n">
         <v>0.3529411764705883</v>
       </c>
-      <c r="G87" t="inlineStr"/>
+      <c r="G87" t="n">
+        <v>0.3878787878787879</v>
+      </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>0.4281 (0.1063)</t>
+          <t>0.4147 (0.0786)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 16:27:26)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -2451,10 +2451,12 @@
       <c r="F57" t="n">
         <v>0.24</v>
       </c>
-      <c r="G57" t="inlineStr"/>
+      <c r="G57" t="n">
+        <v>0.1739130434782609</v>
+      </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>0.1904 (0.0701)</t>
+          <t>0.1849 (0.0505)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 17:27:44)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -3455,10 +3455,12 @@
       <c r="F85" t="n">
         <v>0.373134328358209</v>
       </c>
-      <c r="G85" t="inlineStr"/>
+      <c r="G85" t="n">
+        <v>0.3880597014925373</v>
+      </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>0.4454 (0.1022)</t>
+          <t>0.4263 (0.0795)</t>
         </is>
       </c>
     </row>
@@ -4551,10 +4553,12 @@
       <c r="F116" t="n">
         <v>0.1747572815533981</v>
       </c>
-      <c r="G116" t="inlineStr"/>
+      <c r="G116" t="n">
+        <v>0.1505376344086022</v>
+      </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>0.1516 (0.0328)</t>
+          <t>0.1512 (0.0232)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 18:28:02)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -2595,10 +2595,12 @@
       <c r="F61" t="n">
         <v>0.05555555555555555</v>
       </c>
-      <c r="G61" t="inlineStr"/>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>0.0804 (0.0351)</t>
+          <t>0.0536 (0.0527)</t>
         </is>
       </c>
     </row>
@@ -3349,10 +3351,12 @@
       <c r="F82" t="n">
         <v>0.4148148148148148</v>
       </c>
-      <c r="G82" t="inlineStr"/>
+      <c r="G82" t="n">
+        <v>0.3305785123966942</v>
+      </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>0.4540 (0.0554)</t>
+          <t>0.4128 (0.0813)</t>
         </is>
       </c>
     </row>
@@ -4519,10 +4523,12 @@
       <c r="F115" t="n">
         <v>0.2083333333333333</v>
       </c>
-      <c r="G115" t="inlineStr"/>
+      <c r="G115" t="n">
+        <v>0.1372549019607843</v>
+      </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>0.1929 (0.0219)</t>
+          <t>0.1743 (0.0356)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 19:28:20)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -4246,11 +4246,13 @@
       <c r="E107" t="n">
         <v>0.2368421052631579</v>
       </c>
-      <c r="F107" t="inlineStr"/>
+      <c r="F107" t="n">
+        <v>0.2376237623762376</v>
+      </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
-          <t>0.2368 (0.0000)</t>
+          <t>0.2372 (0.0006)</t>
         </is>
       </c>
     </row>
@@ -4350,11 +4352,13 @@
       <c r="E110" t="n">
         <v>0.2909090909090909</v>
       </c>
-      <c r="F110" t="inlineStr"/>
+      <c r="F110" t="n">
+        <v>0.3285714285714286</v>
+      </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
-          <t>0.2909 (0.0000)</t>
+          <t>0.3097 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -4417,10 +4421,12 @@
       <c r="F112" t="n">
         <v>0.2276422764227642</v>
       </c>
-      <c r="G112" t="inlineStr"/>
+      <c r="G112" t="n">
+        <v>0.158273381294964</v>
+      </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>0.2625 (0.0493)</t>
+          <t>0.2277 (0.0695)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 20:28:38)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -4386,11 +4386,13 @@
       <c r="E111" t="n">
         <v>0.3043478260869565</v>
       </c>
-      <c r="F111" t="inlineStr"/>
+      <c r="F111" t="n">
+        <v>0.1772151898734177</v>
+      </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr">
         <is>
-          <t>0.3043 (0.0000)</t>
+          <t>0.2408 (0.0899)</t>
         </is>
       </c>
     </row>
@@ -5285,10 +5287,12 @@
       <c r="F136" t="n">
         <v>0.3225806451612903</v>
       </c>
-      <c r="G136" t="inlineStr"/>
+      <c r="G136" t="n">
+        <v>0.2954545454545455</v>
+      </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>0.3125 (0.0143)</t>
+          <t>0.3068 (0.0141)</t>
         </is>
       </c>
     </row>
@@ -6183,10 +6187,12 @@
       <c r="F161" t="n">
         <v>0.3428571428571429</v>
       </c>
-      <c r="G161" t="inlineStr"/>
+      <c r="G161" t="n">
+        <v>0.3783783783783784</v>
+      </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>0.2854 (0.0813)</t>
+          <t>0.3164 (0.0787)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 21:28:57)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -7087,10 +7087,12 @@
       <c r="F186" t="n">
         <v>0.2711864406779661</v>
       </c>
-      <c r="G186" t="inlineStr"/>
+      <c r="G186" t="n">
+        <v>0.2608695652173913</v>
+      </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>0.2810 (0.0139)</t>
+          <t>0.2743 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -7985,10 +7987,12 @@
       <c r="F211" t="n">
         <v>0.2051282051282051</v>
       </c>
-      <c r="G211" t="inlineStr"/>
+      <c r="G211" t="n">
+        <v>0.1363636363636364</v>
+      </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>0.1836 (0.0304)</t>
+          <t>0.1679 (0.0347)</t>
         </is>
       </c>
     </row>
@@ -8883,10 +8887,12 @@
       <c r="F236" t="n">
         <v>0.3235294117647059</v>
       </c>
-      <c r="G236" t="inlineStr"/>
+      <c r="G236" t="n">
+        <v>0.48</v>
+      </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>0.3137 (0.0140)</t>
+          <t>0.3691 (0.0965)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 22:29:15)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H287"/>
+  <dimension ref="A1:H288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3495,10 +3495,12 @@
       <c r="F86" t="n">
         <v>0.2769230769230769</v>
       </c>
-      <c r="G86" t="inlineStr"/>
+      <c r="G86" t="n">
+        <v>0.2962962962962963</v>
+      </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>0.3829 (0.1499)</t>
+          <t>0.3540 (0.1172)</t>
         </is>
       </c>
     </row>
@@ -9747,10 +9749,12 @@
       <c r="F260" t="n">
         <v>0.3448275862068966</v>
       </c>
-      <c r="G260" t="inlineStr"/>
+      <c r="G260" t="n">
+        <v>0.2181818181818182</v>
+      </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>0.3130 (0.0450)</t>
+          <t>0.2814 (0.0633)</t>
         </is>
       </c>
     </row>
@@ -9919,10 +9923,12 @@
       <c r="F265" t="n">
         <v>0.4307692307692308</v>
       </c>
-      <c r="G265" t="inlineStr"/>
+      <c r="G265" t="n">
+        <v>0.3076923076923077</v>
+      </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>0.3475 (0.1178)</t>
+          <t>0.3342 (0.0864)</t>
         </is>
       </c>
     </row>
@@ -9953,10 +9959,12 @@
       <c r="F266" t="n">
         <v>0.2962962962962963</v>
       </c>
-      <c r="G266" t="inlineStr"/>
+      <c r="G266" t="n">
+        <v>0.2295081967213115</v>
+      </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>0.2301 (0.0936)</t>
+          <t>0.2299 (0.0662)</t>
         </is>
       </c>
     </row>
@@ -10713,6 +10721,40 @@
       <c r="H287" t="inlineStr">
         <is>
           <t>0.4102 (0.0788)</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>0.3294117647058823</v>
+      </c>
+      <c r="F288" t="n">
+        <v>0.3544303797468354</v>
+      </c>
+      <c r="G288" t="inlineStr"/>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>0.3419 (0.0177)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-03 23:29:33)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H288"/>
+  <dimension ref="A1:H293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9642,11 +9642,13 @@
       <c r="E257" t="n">
         <v>0.2325581395348837</v>
       </c>
-      <c r="F257" t="inlineStr"/>
+      <c r="F257" t="n">
+        <v>0.2857142857142857</v>
+      </c>
       <c r="G257" t="inlineStr"/>
       <c r="H257" t="inlineStr">
         <is>
-          <t>0.2326 (0.0000)</t>
+          <t>0.2591 (0.0376)</t>
         </is>
       </c>
     </row>
@@ -9782,11 +9784,13 @@
       <c r="E261" t="n">
         <v>0.1081081081081081</v>
       </c>
-      <c r="F261" t="inlineStr"/>
+      <c r="F261" t="n">
+        <v>0.1621621621621622</v>
+      </c>
       <c r="G261" t="inlineStr"/>
       <c r="H261" t="inlineStr">
         <is>
-          <t>0.1081 (0.0000)</t>
+          <t>0.1351 (0.0382)</t>
         </is>
       </c>
     </row>
@@ -9817,10 +9821,12 @@
       <c r="F262" t="n">
         <v>0.34375</v>
       </c>
-      <c r="G262" t="inlineStr"/>
+      <c r="G262" t="n">
+        <v>0.3508771929824561</v>
+      </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>0.2596 (0.1190)</t>
+          <t>0.2900 (0.0993)</t>
         </is>
       </c>
     </row>
@@ -10516,31 +10522,31 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>0.1724137931034483</v>
+        <v>0.3023255813953488</v>
       </c>
       <c r="F282" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G282" t="n">
-        <v>0.3384615384615385</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>0.2572 (0.0831)</t>
+          <t>0.3677 (0.0598)</t>
         </is>
       </c>
     </row>
@@ -10552,31 +10558,27 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>0.3037974683544304</v>
-      </c>
-      <c r="F283" t="n">
         <v>0.4096385542168675</v>
       </c>
-      <c r="G283" t="n">
-        <v>0.3611111111111111</v>
-      </c>
+      <c r="F283" t="inlineStr"/>
+      <c r="G283" t="inlineStr"/>
       <c r="H283" t="inlineStr">
         <is>
-          <t>0.3582 (0.0530)</t>
+          <t>0.4096 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -10593,7 +10595,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -10602,17 +10604,17 @@
         </is>
       </c>
       <c r="E284" t="n">
-        <v>0.2</v>
+        <v>0.1724137931034483</v>
       </c>
       <c r="F284" t="n">
-        <v>0.2571428571428571</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="G284" t="n">
-        <v>0.253968253968254</v>
+        <v>0.3384615384615385</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>0.2370 (0.0321)</t>
+          <t>0.2572 (0.0831)</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10631,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -10638,17 +10640,17 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F285" t="n">
-        <v>0.4395604395604396</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="G285" t="n">
-        <v>0.4594594594594595</v>
+        <v>0.3611111111111111</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>0.4493 (0.0100)</t>
+          <t>0.3582 (0.0530)</t>
         </is>
       </c>
     </row>
@@ -10665,7 +10667,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -10674,17 +10676,17 @@
         </is>
       </c>
       <c r="E286" t="n">
-        <v>0.1153846153846154</v>
+        <v>0.2</v>
       </c>
       <c r="F286" t="n">
-        <v>0.125</v>
+        <v>0.2571428571428571</v>
       </c>
       <c r="G286" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.253968253968254</v>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>0.1771 (0.0987)</t>
+          <t>0.2370 (0.0321)</t>
         </is>
       </c>
     </row>
@@ -10696,31 +10698,31 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>0.3296703296703297</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F287" t="n">
-        <v>0.4871794871794872</v>
+        <v>0.4395604395604396</v>
       </c>
       <c r="G287" t="n">
-        <v>0.4137931034482759</v>
+        <v>0.4594594594594595</v>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>0.4102 (0.0788)</t>
+          <t>0.4493 (0.0100)</t>
         </is>
       </c>
     </row>
@@ -10732,29 +10734,203 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>0.1153846153846154</v>
+      </c>
+      <c r="F288" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="G288" t="n">
+        <v>0.2909090909090909</v>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>0.1771 (0.0987)</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
           <t>xgb</t>
         </is>
       </c>
-      <c r="C288" t="inlineStr">
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>0.2253521126760563</v>
+      </c>
+      <c r="F289" t="inlineStr"/>
+      <c r="G289" t="inlineStr"/>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>0.2254 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>0.3296703296703297</v>
+      </c>
+      <c r="F290" t="n">
+        <v>0.4871794871794872</v>
+      </c>
+      <c r="G290" t="n">
+        <v>0.4137931034482759</v>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>0.4102 (0.0788)</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
         <is>
           <t>Morgan</t>
         </is>
       </c>
-      <c r="D288" t="inlineStr">
+      <c r="D291" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E288" t="n">
+      <c r="E291" t="n">
         <v>0.3294117647058823</v>
       </c>
-      <c r="F288" t="n">
+      <c r="F291" t="n">
         <v>0.3544303797468354</v>
       </c>
-      <c r="G288" t="inlineStr"/>
-      <c r="H288" t="inlineStr">
-        <is>
-          <t>0.3419 (0.0177)</t>
+      <c r="G291" t="n">
+        <v>0.3188405797101449</v>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>0.3342 (0.0183)</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="F292" t="n">
+        <v>0.358974358974359</v>
+      </c>
+      <c r="G292" t="inlineStr"/>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>0.3519 (0.0100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>0.2777777777777778</v>
+      </c>
+      <c r="F293" t="n">
+        <v>0.360655737704918</v>
+      </c>
+      <c r="G293" t="inlineStr"/>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>0.3192 (0.0586)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 00:29:51)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H293"/>
+  <dimension ref="A1:H295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4357,10 +4357,12 @@
       <c r="F110" t="n">
         <v>0.3285714285714286</v>
       </c>
-      <c r="G110" t="inlineStr"/>
+      <c r="G110" t="n">
+        <v>0.18</v>
+      </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>0.3097 (0.0266)</t>
+          <t>0.2665 (0.0772)</t>
         </is>
       </c>
     </row>
@@ -10574,11 +10576,13 @@
       <c r="E283" t="n">
         <v>0.4096385542168675</v>
       </c>
-      <c r="F283" t="inlineStr"/>
+      <c r="F283" t="n">
+        <v>0.2597402597402597</v>
+      </c>
       <c r="G283" t="inlineStr"/>
       <c r="H283" t="inlineStr">
         <is>
-          <t>0.4096 (0.0000)</t>
+          <t>0.3347 (0.1060)</t>
         </is>
       </c>
     </row>
@@ -10590,31 +10594,31 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>0.1724137931034483</v>
+        <v>0.3760683760683761</v>
       </c>
       <c r="F284" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.46</v>
       </c>
       <c r="G284" t="n">
-        <v>0.3384615384615385</v>
+        <v>0.4081632653061225</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>0.2572 (0.0831)</t>
+          <t>0.4147 (0.0424)</t>
         </is>
       </c>
     </row>
@@ -10626,31 +10630,27 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>0.3037974683544304</v>
-      </c>
-      <c r="F285" t="n">
-        <v>0.4096385542168675</v>
-      </c>
-      <c r="G285" t="n">
-        <v>0.3611111111111111</v>
-      </c>
+        <v>0.2574257425742574</v>
+      </c>
+      <c r="F285" t="inlineStr"/>
+      <c r="G285" t="inlineStr"/>
       <c r="H285" t="inlineStr">
         <is>
-          <t>0.3582 (0.0530)</t>
+          <t>0.2574 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -10667,7 +10667,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -10676,17 +10676,17 @@
         </is>
       </c>
       <c r="E286" t="n">
-        <v>0.2</v>
+        <v>0.1724137931034483</v>
       </c>
       <c r="F286" t="n">
-        <v>0.2571428571428571</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="G286" t="n">
-        <v>0.253968253968254</v>
+        <v>0.3384615384615385</v>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>0.2370 (0.0321)</t>
+          <t>0.2572 (0.0831)</t>
         </is>
       </c>
     </row>
@@ -10703,7 +10703,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -10712,17 +10712,17 @@
         </is>
       </c>
       <c r="E287" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F287" t="n">
-        <v>0.4395604395604396</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="G287" t="n">
-        <v>0.4594594594594595</v>
+        <v>0.3611111111111111</v>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>0.4493 (0.0100)</t>
+          <t>0.3582 (0.0530)</t>
         </is>
       </c>
     </row>
@@ -10739,7 +10739,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -10748,17 +10748,17 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>0.1153846153846154</v>
+        <v>0.2</v>
       </c>
       <c r="F288" t="n">
-        <v>0.125</v>
+        <v>0.2571428571428571</v>
       </c>
       <c r="G288" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.253968253968254</v>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>0.1771 (0.0987)</t>
+          <t>0.2370 (0.0321)</t>
         </is>
       </c>
     </row>
@@ -10770,27 +10770,31 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>0.2253521126760563</v>
-      </c>
-      <c r="F289" t="inlineStr"/>
-      <c r="G289" t="inlineStr"/>
+        <v>0.4489795918367347</v>
+      </c>
+      <c r="F289" t="n">
+        <v>0.4395604395604396</v>
+      </c>
+      <c r="G289" t="n">
+        <v>0.4594594594594595</v>
+      </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>0.2254 (0.0000)</t>
+          <t>0.4493 (0.0100)</t>
         </is>
       </c>
     </row>
@@ -10802,31 +10806,31 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>0.3296703296703297</v>
+        <v>0.1153846153846154</v>
       </c>
       <c r="F290" t="n">
-        <v>0.4871794871794872</v>
+        <v>0.125</v>
       </c>
       <c r="G290" t="n">
-        <v>0.4137931034482759</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>0.4102 (0.0788)</t>
+          <t>0.1771 (0.0987)</t>
         </is>
       </c>
     </row>
@@ -10843,7 +10847,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -10852,17 +10856,17 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.2253521126760563</v>
       </c>
       <c r="F291" t="n">
-        <v>0.3544303797468354</v>
+        <v>0.3188405797101449</v>
       </c>
       <c r="G291" t="n">
-        <v>0.3188405797101449</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>0.3342 (0.0183)</t>
+          <t>0.3203 (0.0957)</t>
         </is>
       </c>
     </row>
@@ -10879,7 +10883,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
@@ -10888,15 +10892,17 @@
         </is>
       </c>
       <c r="E292" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.3296703296703297</v>
       </c>
       <c r="F292" t="n">
-        <v>0.358974358974359</v>
-      </c>
-      <c r="G292" t="inlineStr"/>
+        <v>0.4871794871794872</v>
+      </c>
+      <c r="G292" t="n">
+        <v>0.4137931034482759</v>
+      </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>0.3519 (0.0100)</t>
+          <t>0.4102 (0.0788)</t>
         </is>
       </c>
     </row>
@@ -10913,24 +10919,98 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>0.3294117647058823</v>
+      </c>
+      <c r="F293" t="n">
+        <v>0.3544303797468354</v>
+      </c>
+      <c r="G293" t="n">
+        <v>0.3188405797101449</v>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>0.3342 (0.0183)</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="F294" t="n">
+        <v>0.358974358974359</v>
+      </c>
+      <c r="G294" t="n">
+        <v>0.4810126582278481</v>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>0.3949 (0.0749)</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D293" t="inlineStr">
+      <c r="D295" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E293" t="n">
+      <c r="E295" t="n">
         <v>0.2777777777777778</v>
       </c>
-      <c r="F293" t="n">
+      <c r="F295" t="n">
         <v>0.360655737704918</v>
       </c>
-      <c r="G293" t="inlineStr"/>
-      <c r="H293" t="inlineStr">
-        <is>
-          <t>0.3192 (0.0586)</t>
+      <c r="G295" t="n">
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>0.3278 (0.0440)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 01:30:09)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H295"/>
+  <dimension ref="A1:H301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4251,10 +4251,12 @@
       <c r="F107" t="n">
         <v>0.2376237623762376</v>
       </c>
-      <c r="G107" t="inlineStr"/>
+      <c r="G107" t="n">
+        <v>0.07142857142857142</v>
+      </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>0.2372 (0.0006)</t>
+          <t>0.1820 (0.0957)</t>
         </is>
       </c>
     </row>
@@ -8543,7 +8545,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -8553,7 +8555,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
@@ -8562,24 +8564,24 @@
         </is>
       </c>
       <c r="E227" t="n">
-        <v>0.3106796116504854</v>
+        <v>0.2888888888888889</v>
       </c>
       <c r="F227" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.4047619047619048</v>
       </c>
       <c r="G227" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.4158415841584158</v>
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>0.3618 (0.0444)</t>
+          <t>0.3698 (0.0703)</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -8589,7 +8591,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -8598,24 +8600,24 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.2702702702702703</v>
       </c>
       <c r="F228" t="n">
-        <v>0.3863636363636364</v>
+        <v>0.3555555555555556</v>
       </c>
       <c r="G228" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.32</v>
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>0.3811 (0.0259)</t>
+          <t>0.3153 (0.0428)</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -8625,7 +8627,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -8634,24 +8636,24 @@
         </is>
       </c>
       <c r="E229" t="n">
-        <v>0.2365591397849462</v>
+        <v>0.3908045977011494</v>
       </c>
       <c r="F229" t="n">
-        <v>0.275</v>
+        <v>0.4791666666666667</v>
       </c>
       <c r="G229" t="n">
-        <v>0.3595505617977528</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>0.2904 (0.0629)</t>
+          <t>0.3852 (0.0968)</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -8661,7 +8663,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -8670,17 +8672,17 @@
         </is>
       </c>
       <c r="E230" t="n">
-        <v>0.4912280701754386</v>
+        <v>0.25</v>
       </c>
       <c r="F230" t="n">
-        <v>0.345679012345679</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G230" t="n">
-        <v>0.459016393442623</v>
+        <v>0.2432432432432433</v>
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>0.4320 (0.0764)</t>
+          <t>0.2250 (0.0376)</t>
         </is>
       </c>
     </row>
@@ -8697,7 +8699,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -8706,17 +8708,17 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>0.24</v>
+        <v>0.3106796116504854</v>
       </c>
       <c r="F231" t="n">
-        <v>0.25</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G231" t="n">
-        <v>0.4466019417475728</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>0.3122 (0.1165)</t>
+          <t>0.3618 (0.0444)</t>
         </is>
       </c>
     </row>
@@ -8728,31 +8730,31 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E232" t="n">
-        <v>0.367816091954023</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F232" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.3863636363636364</v>
       </c>
       <c r="G232" t="n">
-        <v>0.3953488372093023</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>0.3826 (0.0139)</t>
+          <t>0.3811 (0.0259)</t>
         </is>
       </c>
     </row>
@@ -8764,31 +8766,31 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E233" t="n">
-        <v>0.3260869565217391</v>
+        <v>0.2365591397849462</v>
       </c>
       <c r="F233" t="n">
-        <v>0.4086021505376344</v>
+        <v>0.275</v>
       </c>
       <c r="G233" t="n">
-        <v>0.449438202247191</v>
+        <v>0.3595505617977528</v>
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>0.3947 (0.0628)</t>
+          <t>0.2904 (0.0629)</t>
         </is>
       </c>
     </row>
@@ -8800,31 +8802,31 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E234" t="n">
-        <v>0.247191011235955</v>
+        <v>0.4912280701754386</v>
       </c>
       <c r="F234" t="n">
-        <v>0.3376623376623377</v>
+        <v>0.345679012345679</v>
       </c>
       <c r="G234" t="n">
-        <v>0.2716049382716049</v>
+        <v>0.459016393442623</v>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>0.2855 (0.0468)</t>
+          <t>0.4320 (0.0764)</t>
         </is>
       </c>
     </row>
@@ -8836,31 +8838,31 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E235" t="n">
-        <v>0.5045045045045045</v>
+        <v>0.24</v>
       </c>
       <c r="F235" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.25</v>
       </c>
       <c r="G235" t="n">
-        <v>0.4554455445544555</v>
+        <v>0.4466019417475728</v>
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>0.4599 (0.0426)</t>
+          <t>0.3122 (0.1165)</t>
         </is>
       </c>
     </row>
@@ -8877,7 +8879,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -8886,17 +8888,17 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.367816091954023</v>
       </c>
       <c r="F236" t="n">
-        <v>0.3235294117647059</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G236" t="n">
-        <v>0.48</v>
+        <v>0.3953488372093023</v>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>0.3691 (0.0965)</t>
+          <t>0.3826 (0.0139)</t>
         </is>
       </c>
     </row>
@@ -8908,31 +8910,31 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E237" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3260869565217391</v>
       </c>
       <c r="F237" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.4086021505376344</v>
       </c>
       <c r="G237" t="n">
-        <v>0.3655913978494624</v>
+        <v>0.449438202247191</v>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>0.3654 (0.0124)</t>
+          <t>0.3947 (0.0628)</t>
         </is>
       </c>
     </row>
@@ -8944,31 +8946,31 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E238" t="n">
-        <v>0.4</v>
+        <v>0.247191011235955</v>
       </c>
       <c r="F238" t="n">
-        <v>0.4885496183206107</v>
+        <v>0.3376623376623377</v>
       </c>
       <c r="G238" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.2716049382716049</v>
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>0.4443 (0.0443)</t>
+          <t>0.2855 (0.0468)</t>
         </is>
       </c>
     </row>
@@ -8980,31 +8982,31 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>0.3963963963963964</v>
+        <v>0.5045045045045045</v>
       </c>
       <c r="F239" t="n">
-        <v>0.2823529411764706</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G239" t="n">
-        <v>0.3505154639175257</v>
+        <v>0.4554455445544555</v>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>0.3431 (0.0574)</t>
+          <t>0.4599 (0.0426)</t>
         </is>
       </c>
     </row>
@@ -9016,31 +9018,31 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E240" t="n">
-        <v>0.4905660377358491</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F240" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.3235294117647059</v>
       </c>
       <c r="G240" t="n">
-        <v>0.4888888888888889</v>
+        <v>0.48</v>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>0.4524 (0.0646)</t>
+          <t>0.3691 (0.0965)</t>
         </is>
       </c>
     </row>
@@ -9057,7 +9059,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -9066,17 +9068,17 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>0.3423423423423423</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F241" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G241" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.3655913978494624</v>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>0.3306 (0.0403)</t>
+          <t>0.3654 (0.0124)</t>
         </is>
       </c>
     </row>
@@ -9088,31 +9090,31 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E242" t="n">
-        <v>0.4369747899159664</v>
+        <v>0.4</v>
       </c>
       <c r="F242" t="n">
-        <v>0.3013698630136986</v>
+        <v>0.4885496183206107</v>
       </c>
       <c r="G242" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>0.3850 (0.0731)</t>
+          <t>0.4443 (0.0443)</t>
         </is>
       </c>
     </row>
@@ -9124,31 +9126,31 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E243" t="n">
+        <v>0.3963963963963964</v>
+      </c>
+      <c r="F243" t="n">
+        <v>0.2823529411764706</v>
+      </c>
+      <c r="G243" t="n">
         <v>0.3505154639175257</v>
       </c>
-      <c r="F243" t="n">
-        <v>0.3902439024390244</v>
-      </c>
-      <c r="G243" t="n">
-        <v>0.4050632911392405</v>
-      </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>0.3819 (0.0282)</t>
+          <t>0.3431 (0.0574)</t>
         </is>
       </c>
     </row>
@@ -9160,31 +9162,31 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E244" t="n">
-        <v>0.2619047619047619</v>
+        <v>0.4905660377358491</v>
       </c>
       <c r="F244" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G244" t="n">
-        <v>0.2318840579710145</v>
+        <v>0.4888888888888889</v>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>0.2501 (0.0160)</t>
+          <t>0.4524 (0.0646)</t>
         </is>
       </c>
     </row>
@@ -9196,31 +9198,31 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E245" t="n">
-        <v>0.5546218487394958</v>
+        <v>0.3423423423423423</v>
       </c>
       <c r="F245" t="n">
-        <v>0.5217391304347826</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G245" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>0.5084 (0.0541)</t>
+          <t>0.3306 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -9237,7 +9239,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -9246,17 +9248,17 @@
         </is>
       </c>
       <c r="E246" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.4369747899159664</v>
       </c>
       <c r="F246" t="n">
-        <v>0.1875</v>
+        <v>0.3013698630136986</v>
       </c>
       <c r="G246" t="n">
-        <v>0.32</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>0.2136 (0.0960)</t>
+          <t>0.3850 (0.0731)</t>
         </is>
       </c>
     </row>
@@ -9268,31 +9270,31 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E247" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="F247" t="n">
-        <v>0.4155844155844156</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="G247" t="n">
-        <v>0.4470588235294118</v>
+        <v>0.4050632911392405</v>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>0.4372 (0.0188)</t>
+          <t>0.3819 (0.0282)</t>
         </is>
       </c>
     </row>
@@ -9304,31 +9306,31 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E248" t="n">
-        <v>0.4117647058823529</v>
+        <v>0.2619047619047619</v>
       </c>
       <c r="F248" t="n">
-        <v>0.3958333333333333</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="G248" t="n">
-        <v>0.4044943820224719</v>
+        <v>0.2318840579710145</v>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>0.4040 (0.0080)</t>
+          <t>0.2501 (0.0160)</t>
         </is>
       </c>
     </row>
@@ -9340,31 +9342,31 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E249" t="n">
-        <v>0.2888888888888889</v>
+        <v>0.5546218487394958</v>
       </c>
       <c r="F249" t="n">
-        <v>0.2077922077922078</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="G249" t="n">
-        <v>0.3908045977011494</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>0.2958 (0.0917)</t>
+          <t>0.5084 (0.0541)</t>
         </is>
       </c>
     </row>
@@ -9376,31 +9378,31 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E250" t="n">
-        <v>0.4835164835164835</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="F250" t="n">
-        <v>0.3950617283950617</v>
+        <v>0.1875</v>
       </c>
       <c r="G250" t="n">
-        <v>0.4946236559139785</v>
+        <v>0.32</v>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>0.4577 (0.0546)</t>
+          <t>0.2136 (0.0960)</t>
         </is>
       </c>
     </row>
@@ -9417,7 +9419,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -9426,161 +9428,161 @@
         </is>
       </c>
       <c r="E251" t="n">
-        <v>0.1578947368421053</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F251" t="n">
-        <v>0.2121212121212121</v>
+        <v>0.4155844155844156</v>
       </c>
       <c r="G251" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.4470588235294118</v>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>0.2706 (0.1508)</t>
+          <t>0.4372 (0.0188)</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>0.1558441558441558</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="F252" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.3958333333333333</v>
       </c>
       <c r="G252" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.4044943820224719</v>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>0.2654 (0.1127)</t>
+          <t>0.4040 (0.0080)</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E253" t="n">
-        <v>0.2037037037037037</v>
+        <v>0.2888888888888889</v>
       </c>
       <c r="F253" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.2077922077922078</v>
       </c>
       <c r="G253" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.3908045977011494</v>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>0.2974 (0.0906)</t>
+          <t>0.2958 (0.0917)</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>0.0625</v>
+        <v>0.4835164835164835</v>
       </c>
       <c r="F254" t="n">
-        <v>0.2898550724637681</v>
+        <v>0.3950617283950617</v>
       </c>
       <c r="G254" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.4946236559139785</v>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>0.2110 (0.1287)</t>
+          <t>0.4577 (0.0546)</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E255" t="n">
-        <v>0.2769230769230769</v>
+        <v>0.1578947368421053</v>
       </c>
       <c r="F255" t="n">
-        <v>0.3661971830985916</v>
+        <v>0.2121212121212121</v>
       </c>
       <c r="G255" t="n">
-        <v>0.208955223880597</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>0.2840 (0.0789)</t>
+          <t>0.2706 (0.1508)</t>
         </is>
       </c>
     </row>
@@ -9597,7 +9599,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -9606,17 +9608,17 @@
         </is>
       </c>
       <c r="E256" t="n">
-        <v>0.1212121212121212</v>
+        <v>0.1558441558441558</v>
       </c>
       <c r="F256" t="n">
-        <v>0.2424242424242424</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="G256" t="n">
-        <v>0.2432432432432433</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>0.2023 (0.0702)</t>
+          <t>0.2654 (0.1127)</t>
         </is>
       </c>
     </row>
@@ -9628,29 +9630,31 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E257" t="n">
-        <v>0.2325581395348837</v>
+        <v>0.2037037037037037</v>
       </c>
       <c r="F257" t="n">
-        <v>0.2857142857142857</v>
-      </c>
-      <c r="G257" t="inlineStr"/>
+        <v>0.3846153846153846</v>
+      </c>
+      <c r="G257" t="n">
+        <v>0.3037974683544304</v>
+      </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>0.2591 (0.0376)</t>
+          <t>0.2974 (0.0906)</t>
         </is>
       </c>
     </row>
@@ -9662,31 +9666,31 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E258" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.0625</v>
       </c>
       <c r="F258" t="n">
+        <v>0.2898550724637681</v>
+      </c>
+      <c r="G258" t="n">
         <v>0.2807017543859649</v>
       </c>
-      <c r="G258" t="n">
-        <v>0.3137254901960784</v>
-      </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>0.2751 (0.0418)</t>
+          <t>0.2110 (0.1287)</t>
         </is>
       </c>
     </row>
@@ -9698,31 +9702,31 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>0.08</v>
+        <v>0.2769230769230769</v>
       </c>
       <c r="F259" t="n">
-        <v>0.1176470588235294</v>
+        <v>0.3661971830985916</v>
       </c>
       <c r="G259" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>0.1528 (0.0954)</t>
+          <t>0.2840 (0.0789)</t>
         </is>
       </c>
     </row>
@@ -9734,31 +9738,31 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E260" t="n">
-        <v>0.28125</v>
+        <v>0.1212121212121212</v>
       </c>
       <c r="F260" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.2424242424242424</v>
       </c>
       <c r="G260" t="n">
-        <v>0.2181818181818182</v>
+        <v>0.2432432432432433</v>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>0.2814 (0.0633)</t>
+          <t>0.2023 (0.0702)</t>
         </is>
       </c>
     </row>
@@ -9775,7 +9779,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -9784,15 +9788,17 @@
         </is>
       </c>
       <c r="E261" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.2325581395348837</v>
       </c>
       <c r="F261" t="n">
-        <v>0.1621621621621622</v>
-      </c>
-      <c r="G261" t="inlineStr"/>
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="G261" t="n">
+        <v>0.2553191489361702</v>
+      </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>0.1351 (0.0382)</t>
+          <t>0.2579 (0.0267)</t>
         </is>
       </c>
     </row>
@@ -9804,31 +9810,31 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E262" t="n">
-        <v>0.1754385964912281</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="F262" t="n">
-        <v>0.34375</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="G262" t="n">
-        <v>0.3508771929824561</v>
+        <v>0.3137254901960784</v>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>0.2900 (0.0993)</t>
+          <t>0.2751 (0.0418)</t>
         </is>
       </c>
     </row>
@@ -9840,31 +9846,31 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E263" t="n">
-        <v>0.1839080459770115</v>
+        <v>0.08</v>
       </c>
       <c r="F263" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.1176470588235294</v>
       </c>
       <c r="G263" t="n">
-        <v>0.2702702702702703</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>0.2690 (0.0845)</t>
+          <t>0.1528 (0.0954)</t>
         </is>
       </c>
     </row>
@@ -9876,31 +9882,31 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E264" t="n">
-        <v>0.09230769230769231</v>
+        <v>0.28125</v>
       </c>
       <c r="F264" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="G264" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.2181818181818182</v>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>0.1654 (0.0725)</t>
+          <t>0.2814 (0.0633)</t>
         </is>
       </c>
     </row>
@@ -9912,31 +9918,29 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E265" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="F265" t="n">
-        <v>0.4307692307692308</v>
-      </c>
-      <c r="G265" t="n">
-        <v>0.3076923076923077</v>
-      </c>
+        <v>0.1621621621621622</v>
+      </c>
+      <c r="G265" t="inlineStr"/>
       <c r="H265" t="inlineStr">
         <is>
-          <t>0.3342 (0.0864)</t>
+          <t>0.1351 (0.0382)</t>
         </is>
       </c>
     </row>
@@ -9953,7 +9957,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -9962,17 +9966,17 @@
         </is>
       </c>
       <c r="E266" t="n">
-        <v>0.1639344262295082</v>
+        <v>0.1754385964912281</v>
       </c>
       <c r="F266" t="n">
-        <v>0.2962962962962963</v>
+        <v>0.34375</v>
       </c>
       <c r="G266" t="n">
-        <v>0.2295081967213115</v>
+        <v>0.3508771929824561</v>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>0.2299 (0.0662)</t>
+          <t>0.2900 (0.0993)</t>
         </is>
       </c>
     </row>
@@ -9984,31 +9988,31 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>0.1777777777777778</v>
+        <v>0.1839080459770115</v>
       </c>
       <c r="F267" t="n">
-        <v>0.2272727272727273</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="G267" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.2702702702702703</v>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>0.2205 (0.0398)</t>
+          <t>0.2690 (0.0845)</t>
         </is>
       </c>
     </row>
@@ -10020,31 +10024,31 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>0.2790697674418605</v>
+        <v>0.09230769230769231</v>
       </c>
       <c r="F268" t="n">
-        <v>0.3859649122807017</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="G268" t="n">
-        <v>0.3673469387755102</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>0.3441 (0.0571)</t>
+          <t>0.1654 (0.0725)</t>
         </is>
       </c>
     </row>
@@ -10056,31 +10060,31 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F269" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.4307692307692308</v>
       </c>
       <c r="G269" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>0.1530 (0.0500)</t>
+          <t>0.3342 (0.0864)</t>
         </is>
       </c>
     </row>
@@ -10092,31 +10096,31 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.1639344262295082</v>
       </c>
       <c r="F270" t="n">
-        <v>0.4</v>
+        <v>0.2962962962962963</v>
       </c>
       <c r="G270" t="n">
-        <v>0.3571428571428572</v>
+        <v>0.2295081967213115</v>
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>0.3226 (0.0994)</t>
+          <t>0.2299 (0.0662)</t>
         </is>
       </c>
     </row>
@@ -10133,7 +10137,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -10142,17 +10146,17 @@
         </is>
       </c>
       <c r="E271" t="n">
-        <v>0.0975609756097561</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="F271" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2272727272727273</v>
       </c>
       <c r="G271" t="n">
-        <v>0.25</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>0.1462 (0.0900)</t>
+          <t>0.2205 (0.0398)</t>
         </is>
       </c>
     </row>
@@ -10164,31 +10168,31 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>0.2380952380952381</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="F272" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.3859649122807017</v>
       </c>
       <c r="G272" t="n">
-        <v>0.3478260869565217</v>
+        <v>0.3673469387755102</v>
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>0.2429 (0.1026)</t>
+          <t>0.3441 (0.0571)</t>
         </is>
       </c>
     </row>
@@ -10200,31 +10204,31 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>0.24</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="F273" t="n">
-        <v>0.303030303030303</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G273" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>0.2708 (0.0315)</t>
+          <t>0.1530 (0.0500)</t>
         </is>
       </c>
     </row>
@@ -10236,31 +10240,31 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="F274" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.4</v>
       </c>
       <c r="G274" t="n">
-        <v>0.2173913043478261</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>0.1515 (0.0671)</t>
+          <t>0.3226 (0.0994)</t>
         </is>
       </c>
     </row>
@@ -10272,31 +10276,31 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E275" t="n">
+        <v>0.0975609756097561</v>
+      </c>
+      <c r="F275" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="G275" t="n">
         <v>0.25</v>
       </c>
-      <c r="F275" t="n">
-        <v>0.3636363636363636</v>
-      </c>
-      <c r="G275" t="n">
-        <v>0.2857142857142857</v>
-      </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>0.2998 (0.0581)</t>
+          <t>0.1462 (0.0900)</t>
         </is>
       </c>
     </row>
@@ -10313,7 +10317,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -10322,161 +10326,161 @@
         </is>
       </c>
       <c r="E276" t="n">
-        <v>0.25</v>
+        <v>0.2380952380952381</v>
       </c>
       <c r="F276" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="G276" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3478260869565217</v>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>0.2146 (0.0939)</t>
+          <t>0.2429 (0.1026)</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>0.2391304347826087</v>
+        <v>0.24</v>
       </c>
       <c r="F277" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G277" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>0.3070 (0.0589)</t>
+          <t>0.2708 (0.0315)</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>0.3168316831683168</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F278" t="n">
-        <v>0.3454545454545455</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="G278" t="n">
-        <v>0.3793103448275862</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>0.3472 (0.0313)</t>
+          <t>0.1515 (0.0671)</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.25</v>
       </c>
       <c r="F279" t="n">
-        <v>0.4303797468354431</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="G279" t="n">
-        <v>0.3820224719101123</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>0.4054 (0.0242)</t>
+          <t>0.2998 (0.0581)</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>0.4036697247706422</v>
+        <v>0.25</v>
       </c>
       <c r="F280" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="G280" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>0.4326 (0.0256)</t>
+          <t>0.2146 (0.0939)</t>
         </is>
       </c>
     </row>
@@ -10493,7 +10497,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -10502,17 +10506,17 @@
         </is>
       </c>
       <c r="E281" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.2391304347826087</v>
       </c>
       <c r="F281" t="n">
-        <v>0.2117647058823529</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="G281" t="n">
-        <v>0.2921348314606741</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>0.2538 (0.0403)</t>
+          <t>0.3070 (0.0589)</t>
         </is>
       </c>
     </row>
@@ -10524,7 +10528,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10534,21 +10538,21 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>0.3023255813953488</v>
+        <v>0.3168316831683168</v>
       </c>
       <c r="F282" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.3454545454545455</v>
       </c>
       <c r="G282" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.3793103448275862</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>0.3677 (0.0598)</t>
+          <t>0.3472 (0.0313)</t>
         </is>
       </c>
     </row>
@@ -10560,7 +10564,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -10570,19 +10574,21 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="F283" t="n">
-        <v>0.2597402597402597</v>
-      </c>
-      <c r="G283" t="inlineStr"/>
+        <v>0.4303797468354431</v>
+      </c>
+      <c r="G283" t="n">
+        <v>0.3820224719101123</v>
+      </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>0.3347 (0.1060)</t>
+          <t>0.4054 (0.0242)</t>
         </is>
       </c>
     </row>
@@ -10594,31 +10600,31 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>0.3760683760683761</v>
+        <v>0.4036697247706422</v>
       </c>
       <c r="F284" t="n">
-        <v>0.46</v>
+        <v>0.4523809523809524</v>
       </c>
       <c r="G284" t="n">
-        <v>0.4081632653061225</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>0.4147 (0.0424)</t>
+          <t>0.4326 (0.0256)</t>
         </is>
       </c>
     </row>
@@ -10630,27 +10636,31 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E285" t="n">
         <v>0.2574257425742574</v>
       </c>
-      <c r="F285" t="inlineStr"/>
-      <c r="G285" t="inlineStr"/>
+      <c r="F285" t="n">
+        <v>0.2117647058823529</v>
+      </c>
+      <c r="G285" t="n">
+        <v>0.2921348314606741</v>
+      </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>0.2574 (0.0000)</t>
+          <t>0.2538 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -10662,31 +10672,31 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E286" t="n">
-        <v>0.1724137931034483</v>
+        <v>0.3023255813953488</v>
       </c>
       <c r="F286" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G286" t="n">
-        <v>0.3384615384615385</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>0.2572 (0.0831)</t>
+          <t>0.3677 (0.0598)</t>
         </is>
       </c>
     </row>
@@ -10698,31 +10708,31 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="F287" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.2597402597402597</v>
       </c>
       <c r="G287" t="n">
-        <v>0.3611111111111111</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>0.3582 (0.0530)</t>
+          <t>0.3101 (0.0862)</t>
         </is>
       </c>
     </row>
@@ -10734,31 +10744,27 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F288" t="n">
-        <v>0.2571428571428571</v>
-      </c>
-      <c r="G288" t="n">
-        <v>0.253968253968254</v>
-      </c>
+        <v>0.4356435643564356</v>
+      </c>
+      <c r="F288" t="inlineStr"/>
+      <c r="G288" t="inlineStr"/>
       <c r="H288" t="inlineStr">
         <is>
-          <t>0.2370 (0.0321)</t>
+          <t>0.4356 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -10770,31 +10776,31 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.3760683760683761</v>
       </c>
       <c r="F289" t="n">
-        <v>0.4395604395604396</v>
+        <v>0.46</v>
       </c>
       <c r="G289" t="n">
-        <v>0.4594594594594595</v>
+        <v>0.4081632653061225</v>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>0.4493 (0.0100)</t>
+          <t>0.4147 (0.0424)</t>
         </is>
       </c>
     </row>
@@ -10806,31 +10812,31 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>0.1153846153846154</v>
+        <v>0.2574257425742574</v>
       </c>
       <c r="F290" t="n">
-        <v>0.125</v>
+        <v>0.3294117647058823</v>
       </c>
       <c r="G290" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.3838383838383838</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>0.1771 (0.0987)</t>
+          <t>0.3236 (0.0634)</t>
         </is>
       </c>
     </row>
@@ -10842,31 +10848,27 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>0.2253521126760563</v>
-      </c>
-      <c r="F291" t="n">
-        <v>0.3188405797101449</v>
-      </c>
-      <c r="G291" t="n">
-        <v>0.4166666666666667</v>
-      </c>
+        <v>0.3125</v>
+      </c>
+      <c r="F291" t="inlineStr"/>
+      <c r="G291" t="inlineStr"/>
       <c r="H291" t="inlineStr">
         <is>
-          <t>0.3203 (0.0957)</t>
+          <t>0.3125 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -10878,31 +10880,31 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>0.3296703296703297</v>
+        <v>0.1724137931034483</v>
       </c>
       <c r="F292" t="n">
-        <v>0.4871794871794872</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="G292" t="n">
-        <v>0.4137931034482759</v>
+        <v>0.3384615384615385</v>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>0.4102 (0.0788)</t>
+          <t>0.2572 (0.0831)</t>
         </is>
       </c>
     </row>
@@ -10914,31 +10916,31 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F293" t="n">
-        <v>0.3544303797468354</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="G293" t="n">
-        <v>0.3188405797101449</v>
+        <v>0.3611111111111111</v>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>0.3342 (0.0183)</t>
+          <t>0.3582 (0.0530)</t>
         </is>
       </c>
     </row>
@@ -10950,31 +10952,31 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.2</v>
       </c>
       <c r="F294" t="n">
-        <v>0.358974358974359</v>
+        <v>0.2571428571428571</v>
       </c>
       <c r="G294" t="n">
-        <v>0.4810126582278481</v>
+        <v>0.253968253968254</v>
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>0.3949 (0.0749)</t>
+          <t>0.2370 (0.0321)</t>
         </is>
       </c>
     </row>
@@ -10986,29 +10988,245 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>0.4489795918367347</v>
+      </c>
+      <c r="F295" t="n">
+        <v>0.4395604395604396</v>
+      </c>
+      <c r="G295" t="n">
+        <v>0.4594594594594595</v>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>0.4493 (0.0100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>0.1153846153846154</v>
+      </c>
+      <c r="F296" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="G296" t="n">
+        <v>0.2909090909090909</v>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>0.1771 (0.0987)</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
           <t>xgb</t>
         </is>
       </c>
-      <c r="C295" t="inlineStr">
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>0.2253521126760563</v>
+      </c>
+      <c r="F297" t="n">
+        <v>0.3188405797101449</v>
+      </c>
+      <c r="G297" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>0.3203 (0.0957)</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>0.3296703296703297</v>
+      </c>
+      <c r="F298" t="n">
+        <v>0.4871794871794872</v>
+      </c>
+      <c r="G298" t="n">
+        <v>0.4137931034482759</v>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>0.4102 (0.0788)</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E299" t="n">
+        <v>0.3294117647058823</v>
+      </c>
+      <c r="F299" t="n">
+        <v>0.3544303797468354</v>
+      </c>
+      <c r="G299" t="n">
+        <v>0.3188405797101449</v>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>0.3342 (0.0183)</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="F300" t="n">
+        <v>0.358974358974359</v>
+      </c>
+      <c r="G300" t="n">
+        <v>0.4810126582278481</v>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>0.3949 (0.0749)</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
         <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D295" t="inlineStr">
+      <c r="D301" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E295" t="n">
+      <c r="E301" t="n">
         <v>0.2777777777777778</v>
       </c>
-      <c r="F295" t="n">
+      <c r="F301" t="n">
         <v>0.360655737704918</v>
       </c>
-      <c r="G295" t="n">
+      <c r="G301" t="n">
         <v>0.3448275862068966</v>
       </c>
-      <c r="H295" t="inlineStr">
+      <c r="H301" t="inlineStr">
         <is>
           <t>0.3278 (0.0440)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 02:30:27)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H301"/>
+  <dimension ref="A1:H313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8555,7 +8555,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
@@ -8564,17 +8564,17 @@
         </is>
       </c>
       <c r="E227" t="n">
-        <v>0.2888888888888889</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F227" t="n">
-        <v>0.4047619047619048</v>
+        <v>0.4044943820224719</v>
       </c>
       <c r="G227" t="n">
-        <v>0.4158415841584158</v>
+        <v>0.5</v>
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>0.3698 (0.0703)</t>
+          <t>0.3904 (0.1173)</t>
         </is>
       </c>
     </row>
@@ -8591,7 +8591,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -8600,17 +8600,17 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>0.2702702702702703</v>
+        <v>0.2888888888888889</v>
       </c>
       <c r="F228" t="n">
-        <v>0.3555555555555556</v>
+        <v>0.4047619047619048</v>
       </c>
       <c r="G228" t="n">
-        <v>0.32</v>
+        <v>0.4158415841584158</v>
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>0.3153 (0.0428)</t>
+          <t>0.3698 (0.0703)</t>
         </is>
       </c>
     </row>
@@ -8627,7 +8627,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -8636,17 +8636,17 @@
         </is>
       </c>
       <c r="E229" t="n">
-        <v>0.3908045977011494</v>
+        <v>0.2702702702702703</v>
       </c>
       <c r="F229" t="n">
-        <v>0.4791666666666667</v>
+        <v>0.3555555555555556</v>
       </c>
       <c r="G229" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.32</v>
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>0.3852 (0.0968)</t>
+          <t>0.3153 (0.0428)</t>
         </is>
       </c>
     </row>
@@ -8663,7 +8663,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -8672,24 +8672,24 @@
         </is>
       </c>
       <c r="E230" t="n">
-        <v>0.25</v>
+        <v>0.3908045977011494</v>
       </c>
       <c r="F230" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.4791666666666667</v>
       </c>
       <c r="G230" t="n">
-        <v>0.2432432432432433</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>0.2250 (0.0376)</t>
+          <t>0.3852 (0.0968)</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -8699,7 +8699,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -8708,209 +8708,209 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>0.3106796116504854</v>
+        <v>0.25</v>
       </c>
       <c r="F231" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G231" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.2432432432432433</v>
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>0.3618 (0.0444)</t>
+          <t>0.2250 (0.0376)</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E232" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F232" t="n">
-        <v>0.3863636363636364</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G232" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>0.3811 (0.0259)</t>
+          <t>0.2337 (0.1519)</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E233" t="n">
-        <v>0.2365591397849462</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="F233" t="n">
-        <v>0.275</v>
+        <v>0.48</v>
       </c>
       <c r="G233" t="n">
-        <v>0.3595505617977528</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>0.2904 (0.0629)</t>
+          <t>0.3681 (0.1225)</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E234" t="n">
-        <v>0.4912280701754386</v>
+        <v>0.3</v>
       </c>
       <c r="F234" t="n">
-        <v>0.345679012345679</v>
+        <v>0.3714285714285714</v>
       </c>
       <c r="G234" t="n">
-        <v>0.459016393442623</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>0.4320 (0.0764)</t>
+          <t>0.3029 (0.0671)</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E235" t="n">
-        <v>0.24</v>
+        <v>0.4848484848484849</v>
       </c>
       <c r="F235" t="n">
-        <v>0.25</v>
+        <v>0.5151515151515151</v>
       </c>
       <c r="G235" t="n">
-        <v>0.4466019417475728</v>
+        <v>0.4</v>
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>0.3122 (0.1165)</t>
+          <t>0.4667 (0.0597)</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E236" t="n">
-        <v>0.367816091954023</v>
+        <v>0.0975609756097561</v>
       </c>
       <c r="F236" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G236" t="n">
-        <v>0.3953488372093023</v>
+        <v>0.3214285714285715</v>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>0.3826 (0.0139)</t>
+          <t>0.2166 (0.1126)</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -8920,33 +8920,33 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E237" t="n">
-        <v>0.3260869565217391</v>
+        <v>0.3116883116883117</v>
       </c>
       <c r="F237" t="n">
-        <v>0.4086021505376344</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="G237" t="n">
-        <v>0.449438202247191</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>0.3947 (0.0628)</t>
+          <t>0.3581 (0.0492)</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -8956,21 +8956,19 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E238" t="n">
-        <v>0.247191011235955</v>
+        <v>0.3050847457627119</v>
       </c>
       <c r="F238" t="n">
-        <v>0.3376623376623377</v>
-      </c>
-      <c r="G238" t="n">
-        <v>0.2716049382716049</v>
-      </c>
+        <v>0.3278688524590164</v>
+      </c>
+      <c r="G238" t="inlineStr"/>
       <c r="H238" t="inlineStr">
         <is>
-          <t>0.2855 (0.0468)</t>
+          <t>0.3165 (0.0161)</t>
         </is>
       </c>
     </row>
@@ -8982,31 +8980,31 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>0.5045045045045045</v>
+        <v>0.3106796116504854</v>
       </c>
       <c r="F239" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G239" t="n">
-        <v>0.4554455445544555</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>0.4599 (0.0426)</t>
+          <t>0.3618 (0.0444)</t>
         </is>
       </c>
     </row>
@@ -9018,31 +9016,31 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E240" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F240" t="n">
-        <v>0.3235294117647059</v>
+        <v>0.3863636363636364</v>
       </c>
       <c r="G240" t="n">
-        <v>0.48</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>0.3691 (0.0965)</t>
+          <t>0.3811 (0.0259)</t>
         </is>
       </c>
     </row>
@@ -9054,31 +9052,31 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E241" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.2365591397849462</v>
       </c>
       <c r="F241" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.275</v>
       </c>
       <c r="G241" t="n">
-        <v>0.3655913978494624</v>
+        <v>0.3595505617977528</v>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>0.3654 (0.0124)</t>
+          <t>0.2904 (0.0629)</t>
         </is>
       </c>
     </row>
@@ -9090,31 +9088,31 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E242" t="n">
-        <v>0.4</v>
+        <v>0.4912280701754386</v>
       </c>
       <c r="F242" t="n">
-        <v>0.4885496183206107</v>
+        <v>0.345679012345679</v>
       </c>
       <c r="G242" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.459016393442623</v>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>0.4443 (0.0443)</t>
+          <t>0.4320 (0.0764)</t>
         </is>
       </c>
     </row>
@@ -9126,31 +9124,31 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E243" t="n">
-        <v>0.3963963963963964</v>
+        <v>0.24</v>
       </c>
       <c r="F243" t="n">
-        <v>0.2823529411764706</v>
+        <v>0.25</v>
       </c>
       <c r="G243" t="n">
-        <v>0.3505154639175257</v>
+        <v>0.4466019417475728</v>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>0.3431 (0.0574)</t>
+          <t>0.3122 (0.1165)</t>
         </is>
       </c>
     </row>
@@ -9162,31 +9160,31 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E244" t="n">
-        <v>0.4905660377358491</v>
+        <v>0.367816091954023</v>
       </c>
       <c r="F244" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G244" t="n">
-        <v>0.4888888888888889</v>
+        <v>0.3953488372093023</v>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>0.4524 (0.0646)</t>
+          <t>0.3826 (0.0139)</t>
         </is>
       </c>
     </row>
@@ -9198,31 +9196,31 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E245" t="n">
-        <v>0.3423423423423423</v>
+        <v>0.3260869565217391</v>
       </c>
       <c r="F245" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.4086021505376344</v>
       </c>
       <c r="G245" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.449438202247191</v>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>0.3306 (0.0403)</t>
+          <t>0.3947 (0.0628)</t>
         </is>
       </c>
     </row>
@@ -9234,31 +9232,31 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E246" t="n">
-        <v>0.4369747899159664</v>
+        <v>0.247191011235955</v>
       </c>
       <c r="F246" t="n">
-        <v>0.3013698630136986</v>
+        <v>0.3376623376623377</v>
       </c>
       <c r="G246" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.2716049382716049</v>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>0.3850 (0.0731)</t>
+          <t>0.2855 (0.0468)</t>
         </is>
       </c>
     </row>
@@ -9270,31 +9268,31 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E247" t="n">
-        <v>0.3505154639175257</v>
+        <v>0.5045045045045045</v>
       </c>
       <c r="F247" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G247" t="n">
-        <v>0.4050632911392405</v>
+        <v>0.4554455445544555</v>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>0.3819 (0.0282)</t>
+          <t>0.4599 (0.0426)</t>
         </is>
       </c>
     </row>
@@ -9306,31 +9304,31 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E248" t="n">
-        <v>0.2619047619047619</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F248" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.3235294117647059</v>
       </c>
       <c r="G248" t="n">
-        <v>0.2318840579710145</v>
+        <v>0.48</v>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>0.2501 (0.0160)</t>
+          <t>0.3691 (0.0965)</t>
         </is>
       </c>
     </row>
@@ -9342,31 +9340,31 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E249" t="n">
-        <v>0.5546218487394958</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F249" t="n">
-        <v>0.5217391304347826</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G249" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.3655913978494624</v>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>0.5084 (0.0541)</t>
+          <t>0.3654 (0.0124)</t>
         </is>
       </c>
     </row>
@@ -9378,31 +9376,31 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E250" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="F250" t="n">
-        <v>0.1875</v>
+        <v>0.4885496183206107</v>
       </c>
       <c r="G250" t="n">
-        <v>0.32</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>0.2136 (0.0960)</t>
+          <t>0.4443 (0.0443)</t>
         </is>
       </c>
     </row>
@@ -9414,31 +9412,31 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E251" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.3963963963963964</v>
       </c>
       <c r="F251" t="n">
-        <v>0.4155844155844156</v>
+        <v>0.2823529411764706</v>
       </c>
       <c r="G251" t="n">
-        <v>0.4470588235294118</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>0.4372 (0.0188)</t>
+          <t>0.3431 (0.0574)</t>
         </is>
       </c>
     </row>
@@ -9450,31 +9448,31 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>0.4117647058823529</v>
+        <v>0.4905660377358491</v>
       </c>
       <c r="F252" t="n">
-        <v>0.3958333333333333</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G252" t="n">
-        <v>0.4044943820224719</v>
+        <v>0.4888888888888889</v>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>0.4040 (0.0080)</t>
+          <t>0.4524 (0.0646)</t>
         </is>
       </c>
     </row>
@@ -9486,31 +9484,31 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E253" t="n">
-        <v>0.2888888888888889</v>
+        <v>0.3423423423423423</v>
       </c>
       <c r="F253" t="n">
-        <v>0.2077922077922078</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G253" t="n">
-        <v>0.3908045977011494</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>0.2958 (0.0917)</t>
+          <t>0.3306 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -9522,31 +9520,31 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>0.4835164835164835</v>
+        <v>0.4369747899159664</v>
       </c>
       <c r="F254" t="n">
-        <v>0.3950617283950617</v>
+        <v>0.3013698630136986</v>
       </c>
       <c r="G254" t="n">
-        <v>0.4946236559139785</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>0.4577 (0.0546)</t>
+          <t>0.3850 (0.0731)</t>
         </is>
       </c>
     </row>
@@ -9558,319 +9556,319 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E255" t="n">
-        <v>0.1578947368421053</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="F255" t="n">
-        <v>0.2121212121212121</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="G255" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.4050632911392405</v>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>0.2706 (0.1508)</t>
+          <t>0.3819 (0.0282)</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>0.1558441558441558</v>
+        <v>0.2619047619047619</v>
       </c>
       <c r="F256" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="G256" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2318840579710145</v>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>0.2654 (0.1127)</t>
+          <t>0.2501 (0.0160)</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E257" t="n">
-        <v>0.2037037037037037</v>
+        <v>0.5546218487394958</v>
       </c>
       <c r="F257" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="G257" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>0.2974 (0.0906)</t>
+          <t>0.5084 (0.0541)</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E258" t="n">
-        <v>0.0625</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="F258" t="n">
-        <v>0.2898550724637681</v>
+        <v>0.1875</v>
       </c>
       <c r="G258" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.32</v>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>0.2110 (0.1287)</t>
+          <t>0.2136 (0.0960)</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>0.2769230769230769</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F259" t="n">
-        <v>0.3661971830985916</v>
+        <v>0.4155844155844156</v>
       </c>
       <c r="G259" t="n">
-        <v>0.208955223880597</v>
+        <v>0.4470588235294118</v>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>0.2840 (0.0789)</t>
+          <t>0.4372 (0.0188)</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E260" t="n">
-        <v>0.1212121212121212</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="F260" t="n">
-        <v>0.2424242424242424</v>
+        <v>0.3958333333333333</v>
       </c>
       <c r="G260" t="n">
-        <v>0.2432432432432433</v>
+        <v>0.4044943820224719</v>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>0.2023 (0.0702)</t>
+          <t>0.4040 (0.0080)</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E261" t="n">
-        <v>0.2325581395348837</v>
+        <v>0.2888888888888889</v>
       </c>
       <c r="F261" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2077922077922078</v>
       </c>
       <c r="G261" t="n">
-        <v>0.2553191489361702</v>
+        <v>0.3908045977011494</v>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>0.2579 (0.0267)</t>
+          <t>0.2958 (0.0917)</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E262" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.4835164835164835</v>
       </c>
       <c r="F262" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.3950617283950617</v>
       </c>
       <c r="G262" t="n">
-        <v>0.3137254901960784</v>
+        <v>0.4946236559139785</v>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>0.2751 (0.0418)</t>
+          <t>0.4577 (0.0546)</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E263" t="n">
-        <v>0.08</v>
+        <v>0.1578947368421053</v>
       </c>
       <c r="F263" t="n">
-        <v>0.1176470588235294</v>
+        <v>0.2121212121212121</v>
       </c>
       <c r="G263" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>0.1528 (0.0954)</t>
+          <t>0.2706 (0.1508)</t>
         </is>
       </c>
     </row>
@@ -9882,31 +9880,31 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E264" t="n">
-        <v>0.28125</v>
+        <v>0.1558441558441558</v>
       </c>
       <c r="F264" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="G264" t="n">
-        <v>0.2181818181818182</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>0.2814 (0.0633)</t>
+          <t>0.2654 (0.1127)</t>
         </is>
       </c>
     </row>
@@ -9918,29 +9916,31 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E265" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.2037037037037037</v>
       </c>
       <c r="F265" t="n">
-        <v>0.1621621621621622</v>
-      </c>
-      <c r="G265" t="inlineStr"/>
+        <v>0.3846153846153846</v>
+      </c>
+      <c r="G265" t="n">
+        <v>0.3037974683544304</v>
+      </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>0.1351 (0.0382)</t>
+          <t>0.2974 (0.0906)</t>
         </is>
       </c>
     </row>
@@ -9952,31 +9952,31 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E266" t="n">
-        <v>0.1754385964912281</v>
+        <v>0.0625</v>
       </c>
       <c r="F266" t="n">
-        <v>0.34375</v>
+        <v>0.2898550724637681</v>
       </c>
       <c r="G266" t="n">
-        <v>0.3508771929824561</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>0.2900 (0.0993)</t>
+          <t>0.2110 (0.1287)</t>
         </is>
       </c>
     </row>
@@ -9988,31 +9988,31 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>0.1839080459770115</v>
+        <v>0.2769230769230769</v>
       </c>
       <c r="F267" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3661971830985916</v>
       </c>
       <c r="G267" t="n">
-        <v>0.2702702702702703</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>0.2690 (0.0845)</t>
+          <t>0.2840 (0.0789)</t>
         </is>
       </c>
     </row>
@@ -10024,31 +10024,31 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>0.09230769230769231</v>
+        <v>0.1212121212121212</v>
       </c>
       <c r="F268" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.2424242424242424</v>
       </c>
       <c r="G268" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.2432432432432433</v>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>0.1654 (0.0725)</t>
+          <t>0.2023 (0.0702)</t>
         </is>
       </c>
     </row>
@@ -10060,31 +10060,31 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2325581395348837</v>
       </c>
       <c r="F269" t="n">
-        <v>0.4307692307692308</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G269" t="n">
-        <v>0.3076923076923077</v>
+        <v>0.2553191489361702</v>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>0.3342 (0.0864)</t>
+          <t>0.2579 (0.0267)</t>
         </is>
       </c>
     </row>
@@ -10096,31 +10096,31 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>0.1639344262295082</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="F270" t="n">
-        <v>0.2962962962962963</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="G270" t="n">
-        <v>0.2295081967213115</v>
+        <v>0.3137254901960784</v>
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>0.2299 (0.0662)</t>
+          <t>0.2751 (0.0418)</t>
         </is>
       </c>
     </row>
@@ -10132,31 +10132,31 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E271" t="n">
-        <v>0.1777777777777778</v>
+        <v>0.08</v>
       </c>
       <c r="F271" t="n">
-        <v>0.2272727272727273</v>
+        <v>0.1176470588235294</v>
       </c>
       <c r="G271" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>0.2205 (0.0398)</t>
+          <t>0.1528 (0.0954)</t>
         </is>
       </c>
     </row>
@@ -10168,31 +10168,31 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>0.2790697674418605</v>
+        <v>0.28125</v>
       </c>
       <c r="F272" t="n">
-        <v>0.3859649122807017</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="G272" t="n">
-        <v>0.3673469387755102</v>
+        <v>0.2181818181818182</v>
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>0.3441 (0.0571)</t>
+          <t>0.2814 (0.0633)</t>
         </is>
       </c>
     </row>
@@ -10204,31 +10204,31 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="F273" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.1621621621621622</v>
       </c>
       <c r="G273" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>0.1530 (0.0500)</t>
+          <t>0.1831 (0.0874)</t>
         </is>
       </c>
     </row>
@@ -10240,31 +10240,31 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.1754385964912281</v>
       </c>
       <c r="F274" t="n">
-        <v>0.4</v>
+        <v>0.34375</v>
       </c>
       <c r="G274" t="n">
-        <v>0.3571428571428572</v>
+        <v>0.3508771929824561</v>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>0.3226 (0.0994)</t>
+          <t>0.2900 (0.0993)</t>
         </is>
       </c>
     </row>
@@ -10276,31 +10276,31 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>0.0975609756097561</v>
+        <v>0.1839080459770115</v>
       </c>
       <c r="F275" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="G275" t="n">
-        <v>0.25</v>
+        <v>0.2702702702702703</v>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>0.1462 (0.0900)</t>
+          <t>0.2690 (0.0845)</t>
         </is>
       </c>
     </row>
@@ -10312,31 +10312,31 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>0.2380952380952381</v>
+        <v>0.09230769230769231</v>
       </c>
       <c r="F276" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="G276" t="n">
-        <v>0.3478260869565217</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>0.2429 (0.1026)</t>
+          <t>0.1654 (0.0725)</t>
         </is>
       </c>
     </row>
@@ -10348,31 +10348,31 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>0.24</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F277" t="n">
-        <v>0.303030303030303</v>
+        <v>0.4307692307692308</v>
       </c>
       <c r="G277" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>0.2708 (0.0315)</t>
+          <t>0.3342 (0.0864)</t>
         </is>
       </c>
     </row>
@@ -10384,31 +10384,31 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.1639344262295082</v>
       </c>
       <c r="F278" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2962962962962963</v>
       </c>
       <c r="G278" t="n">
-        <v>0.2173913043478261</v>
+        <v>0.2295081967213115</v>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>0.1515 (0.0671)</t>
+          <t>0.2299 (0.0662)</t>
         </is>
       </c>
     </row>
@@ -10420,31 +10420,31 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>0.25</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="F279" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2272727272727273</v>
       </c>
       <c r="G279" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>0.2998 (0.0581)</t>
+          <t>0.2205 (0.0398)</t>
         </is>
       </c>
     </row>
@@ -10456,315 +10456,319 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>0.25</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="F280" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.3859649122807017</v>
       </c>
       <c r="G280" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3673469387755102</v>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>0.2146 (0.0939)</t>
+          <t>0.3441 (0.0571)</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>0.2391304347826087</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="F281" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G281" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>0.3070 (0.0589)</t>
+          <t>0.1530 (0.0500)</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>0.3168316831683168</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="F282" t="n">
-        <v>0.3454545454545455</v>
+        <v>0.4</v>
       </c>
       <c r="G282" t="n">
-        <v>0.3793103448275862</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>0.3472 (0.0313)</t>
+          <t>0.3226 (0.0994)</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.0975609756097561</v>
       </c>
       <c r="F283" t="n">
-        <v>0.4303797468354431</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="G283" t="n">
-        <v>0.3820224719101123</v>
+        <v>0.25</v>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>0.4054 (0.0242)</t>
+          <t>0.1462 (0.0900)</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>0.4036697247706422</v>
+        <v>0.2380952380952381</v>
       </c>
       <c r="F284" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="G284" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.3478260869565217</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>0.4326 (0.0256)</t>
+          <t>0.2429 (0.1026)</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.24</v>
       </c>
       <c r="F285" t="n">
-        <v>0.2117647058823529</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G285" t="n">
-        <v>0.2921348314606741</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>0.2538 (0.0403)</t>
+          <t>0.2708 (0.0315)</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E286" t="n">
-        <v>0.3023255813953488</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F286" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="G286" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>0.3677 (0.0598)</t>
+          <t>0.1515 (0.0671)</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.25</v>
       </c>
       <c r="F287" t="n">
-        <v>0.2597402597402597</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="G287" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>0.3101 (0.0862)</t>
+          <t>0.2998 (0.0581)</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>0.4356435643564356</v>
-      </c>
-      <c r="F288" t="inlineStr"/>
-      <c r="G288" t="inlineStr"/>
+        <v>0.25</v>
+      </c>
+      <c r="F288" t="n">
+        <v>0.1081081081081081</v>
+      </c>
+      <c r="G288" t="n">
+        <v>0.2857142857142857</v>
+      </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>0.4356 (0.0000)</t>
+          <t>0.2146 (0.0939)</t>
         </is>
       </c>
     </row>
@@ -10776,31 +10780,31 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>0.3760683760683761</v>
+        <v>0.2391304347826087</v>
       </c>
       <c r="F289" t="n">
-        <v>0.46</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="G289" t="n">
-        <v>0.4081632653061225</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>0.4147 (0.0424)</t>
+          <t>0.3070 (0.0589)</t>
         </is>
       </c>
     </row>
@@ -10812,31 +10816,31 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.3168316831683168</v>
       </c>
       <c r="F290" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.3454545454545455</v>
       </c>
       <c r="G290" t="n">
-        <v>0.3838383838383838</v>
+        <v>0.3793103448275862</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>0.3236 (0.0634)</t>
+          <t>0.3472 (0.0313)</t>
         </is>
       </c>
     </row>
@@ -10848,27 +10852,31 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F291" t="inlineStr"/>
-      <c r="G291" t="inlineStr"/>
+        <v>0.4038461538461539</v>
+      </c>
+      <c r="F291" t="n">
+        <v>0.4303797468354431</v>
+      </c>
+      <c r="G291" t="n">
+        <v>0.3820224719101123</v>
+      </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>0.3125 (0.0000)</t>
+          <t>0.4054 (0.0242)</t>
         </is>
       </c>
     </row>
@@ -10880,31 +10888,31 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>0.1724137931034483</v>
+        <v>0.4036697247706422</v>
       </c>
       <c r="F292" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.4523809523809524</v>
       </c>
       <c r="G292" t="n">
-        <v>0.3384615384615385</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>0.2572 (0.0831)</t>
+          <t>0.4326 (0.0256)</t>
         </is>
       </c>
     </row>
@@ -10916,31 +10924,31 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.2574257425742574</v>
       </c>
       <c r="F293" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.2117647058823529</v>
       </c>
       <c r="G293" t="n">
-        <v>0.3611111111111111</v>
+        <v>0.2921348314606741</v>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>0.3582 (0.0530)</t>
+          <t>0.2538 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -10952,31 +10960,27 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F294" t="n">
-        <v>0.2571428571428571</v>
-      </c>
-      <c r="G294" t="n">
-        <v>0.253968253968254</v>
-      </c>
+        <v>0.2285714285714286</v>
+      </c>
+      <c r="F294" t="inlineStr"/>
+      <c r="G294" t="inlineStr"/>
       <c r="H294" t="inlineStr">
         <is>
-          <t>0.2370 (0.0321)</t>
+          <t>0.2286 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -10988,31 +10992,31 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.3023255813953488</v>
       </c>
       <c r="F295" t="n">
-        <v>0.4395604395604396</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G295" t="n">
-        <v>0.4594594594594595</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>0.4493 (0.0100)</t>
+          <t>0.3677 (0.0598)</t>
         </is>
       </c>
     </row>
@@ -11024,31 +11028,31 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>0.1153846153846154</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="F296" t="n">
-        <v>0.125</v>
+        <v>0.2597402597402597</v>
       </c>
       <c r="G296" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>0.1771 (0.0987)</t>
+          <t>0.3101 (0.0862)</t>
         </is>
       </c>
     </row>
@@ -11060,31 +11064,27 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>0.2253521126760563</v>
-      </c>
-      <c r="F297" t="n">
-        <v>0.3188405797101449</v>
-      </c>
-      <c r="G297" t="n">
-        <v>0.4166666666666667</v>
-      </c>
+        <v>0.4356435643564356</v>
+      </c>
+      <c r="F297" t="inlineStr"/>
+      <c r="G297" t="inlineStr"/>
       <c r="H297" t="inlineStr">
         <is>
-          <t>0.3203 (0.0957)</t>
+          <t>0.4356 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -11096,31 +11096,27 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>0.3296703296703297</v>
-      </c>
-      <c r="F298" t="n">
-        <v>0.4871794871794872</v>
-      </c>
-      <c r="G298" t="n">
-        <v>0.4137931034482759</v>
-      </c>
+        <v>0.3235294117647059</v>
+      </c>
+      <c r="F298" t="inlineStr"/>
+      <c r="G298" t="inlineStr"/>
       <c r="H298" t="inlineStr">
         <is>
-          <t>0.4102 (0.0788)</t>
+          <t>0.3235 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -11132,31 +11128,27 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>0.3294117647058823</v>
-      </c>
-      <c r="F299" t="n">
-        <v>0.3544303797468354</v>
-      </c>
-      <c r="G299" t="n">
-        <v>0.3188405797101449</v>
-      </c>
+        <v>0.2736842105263158</v>
+      </c>
+      <c r="F299" t="inlineStr"/>
+      <c r="G299" t="inlineStr"/>
       <c r="H299" t="inlineStr">
         <is>
-          <t>0.3342 (0.0183)</t>
+          <t>0.2737 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -11168,31 +11160,31 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.3760683760683761</v>
       </c>
       <c r="F300" t="n">
-        <v>0.358974358974359</v>
+        <v>0.46</v>
       </c>
       <c r="G300" t="n">
-        <v>0.4810126582278481</v>
+        <v>0.4081632653061225</v>
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>0.3949 (0.0749)</t>
+          <t>0.4147 (0.0424)</t>
         </is>
       </c>
     </row>
@@ -11204,29 +11196,455 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>0.2574257425742574</v>
+      </c>
+      <c r="F301" t="n">
+        <v>0.3294117647058823</v>
+      </c>
+      <c r="G301" t="n">
+        <v>0.3838383838383838</v>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>0.3236 (0.0634)</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>0.4791666666666667</v>
+      </c>
+      <c r="F302" t="inlineStr"/>
+      <c r="G302" t="inlineStr"/>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>0.4792 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F303" t="n">
+        <v>0.4337349397590362</v>
+      </c>
+      <c r="G303" t="inlineStr"/>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>0.3731 (0.0857)</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>0.1724137931034483</v>
+      </c>
+      <c r="F304" t="n">
+        <v>0.2608695652173913</v>
+      </c>
+      <c r="G304" t="n">
+        <v>0.3384615384615385</v>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>0.2572 (0.0831)</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>0.3037974683544304</v>
+      </c>
+      <c r="F305" t="n">
+        <v>0.4096385542168675</v>
+      </c>
+      <c r="G305" t="n">
+        <v>0.3611111111111111</v>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>0.3582 (0.0530)</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F306" t="n">
+        <v>0.2571428571428571</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0.253968253968254</v>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>0.2370 (0.0321)</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>0.4489795918367347</v>
+      </c>
+      <c r="F307" t="n">
+        <v>0.4395604395604396</v>
+      </c>
+      <c r="G307" t="n">
+        <v>0.4594594594594595</v>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>0.4493 (0.0100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>0.1153846153846154</v>
+      </c>
+      <c r="F308" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="G308" t="n">
+        <v>0.2909090909090909</v>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>0.1771 (0.0987)</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
           <t>xgb</t>
         </is>
       </c>
-      <c r="C301" t="inlineStr">
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E309" t="n">
+        <v>0.2253521126760563</v>
+      </c>
+      <c r="F309" t="n">
+        <v>0.3188405797101449</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>0.3203 (0.0957)</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>0.3296703296703297</v>
+      </c>
+      <c r="F310" t="n">
+        <v>0.4871794871794872</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0.4137931034482759</v>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>0.4102 (0.0788)</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>0.3294117647058823</v>
+      </c>
+      <c r="F311" t="n">
+        <v>0.3544303797468354</v>
+      </c>
+      <c r="G311" t="n">
+        <v>0.3188405797101449</v>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>0.3342 (0.0183)</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E312" t="n">
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="F312" t="n">
+        <v>0.358974358974359</v>
+      </c>
+      <c r="G312" t="n">
+        <v>0.4810126582278481</v>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>0.3949 (0.0749)</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
         <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D301" t="inlineStr">
+      <c r="D313" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E301" t="n">
+      <c r="E313" t="n">
         <v>0.2777777777777778</v>
       </c>
-      <c r="F301" t="n">
+      <c r="F313" t="n">
         <v>0.360655737704918</v>
       </c>
-      <c r="G301" t="n">
+      <c r="G313" t="n">
         <v>0.3448275862068966</v>
       </c>
-      <c r="H301" t="inlineStr">
+      <c r="H313" t="inlineStr">
         <is>
           <t>0.3278 (0.0440)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 03:30:46)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H313"/>
+  <dimension ref="A1:H317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4395,10 +4395,12 @@
       <c r="F111" t="n">
         <v>0.1772151898734177</v>
       </c>
-      <c r="G111" t="inlineStr"/>
+      <c r="G111" t="n">
+        <v>0.08571428571428572</v>
+      </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>0.2408 (0.0899)</t>
+          <t>0.1891 (0.1098)</t>
         </is>
       </c>
     </row>
@@ -8730,31 +8732,27 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E232" t="n">
-        <v>0.08333333333333333</v>
-      </c>
-      <c r="F232" t="n">
-        <v>0.2307692307692308</v>
-      </c>
-      <c r="G232" t="n">
-        <v>0.3870967741935484</v>
-      </c>
+        <v>0.2133333333333333</v>
+      </c>
+      <c r="F232" t="inlineStr"/>
+      <c r="G232" t="inlineStr"/>
       <c r="H232" t="inlineStr">
         <is>
-          <t>0.2337 (0.1519)</t>
+          <t>0.2133 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -8771,7 +8769,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -8780,17 +8778,17 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F233" t="n">
-        <v>0.48</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G233" t="n">
         <v>0.3870967741935484</v>
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>0.3681 (0.1225)</t>
+          <t>0.2337 (0.1519)</t>
         </is>
       </c>
     </row>
@@ -8807,7 +8805,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -8816,17 +8814,17 @@
         </is>
       </c>
       <c r="E234" t="n">
-        <v>0.3</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="F234" t="n">
-        <v>0.3714285714285714</v>
+        <v>0.48</v>
       </c>
       <c r="G234" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>0.3029 (0.0671)</t>
+          <t>0.3681 (0.1225)</t>
         </is>
       </c>
     </row>
@@ -8843,7 +8841,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -8852,17 +8850,17 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>0.4848484848484849</v>
+        <v>0.3</v>
       </c>
       <c r="F235" t="n">
-        <v>0.5151515151515151</v>
+        <v>0.3714285714285714</v>
       </c>
       <c r="G235" t="n">
-        <v>0.4</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>0.4667 (0.0597)</t>
+          <t>0.3029 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -8879,7 +8877,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -8888,17 +8886,17 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>0.0975609756097561</v>
+        <v>0.4848484848484849</v>
       </c>
       <c r="F236" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.5151515151515151</v>
       </c>
       <c r="G236" t="n">
-        <v>0.3214285714285715</v>
+        <v>0.4</v>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>0.2166 (0.1126)</t>
+          <t>0.4667 (0.0597)</t>
         </is>
       </c>
     </row>
@@ -8910,31 +8908,31 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E237" t="n">
-        <v>0.3116883116883117</v>
+        <v>0.0975609756097561</v>
       </c>
       <c r="F237" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G237" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3214285714285715</v>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>0.3581 (0.0492)</t>
+          <t>0.2166 (0.1126)</t>
         </is>
       </c>
     </row>
@@ -8951,7 +8949,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -8960,159 +8958,153 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>0.3050847457627119</v>
-      </c>
-      <c r="F238" t="n">
-        <v>0.3278688524590164</v>
-      </c>
+        <v>0.2307692307692308</v>
+      </c>
+      <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr"/>
       <c r="H238" t="inlineStr">
         <is>
-          <t>0.3165 (0.0161)</t>
+          <t>0.2308 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>0.3106796116504854</v>
+        <v>0.3116883116883117</v>
       </c>
       <c r="F239" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="G239" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>0.3618 (0.0444)</t>
+          <t>0.3581 (0.0492)</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E240" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3050847457627119</v>
       </c>
       <c r="F240" t="n">
-        <v>0.3863636363636364</v>
+        <v>0.3278688524590164</v>
       </c>
       <c r="G240" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.3050847457627119</v>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>0.3811 (0.0259)</t>
+          <t>0.3127 (0.0132)</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E241" t="n">
-        <v>0.2365591397849462</v>
+        <v>0.3666666666666666</v>
       </c>
       <c r="F241" t="n">
-        <v>0.275</v>
-      </c>
-      <c r="G241" t="n">
-        <v>0.3595505617977528</v>
-      </c>
+        <v>0.5161290322580645</v>
+      </c>
+      <c r="G241" t="inlineStr"/>
       <c r="H241" t="inlineStr">
         <is>
-          <t>0.2904 (0.0629)</t>
+          <t>0.4414 (0.1057)</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E242" t="n">
-        <v>0.4912280701754386</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="F242" t="n">
-        <v>0.345679012345679</v>
-      </c>
-      <c r="G242" t="n">
-        <v>0.459016393442623</v>
-      </c>
+        <v>0.2692307692307692</v>
+      </c>
+      <c r="G242" t="inlineStr"/>
       <c r="H242" t="inlineStr">
         <is>
-          <t>0.4320 (0.0764)</t>
+          <t>0.1801 (0.1261)</t>
         </is>
       </c>
     </row>
@@ -9129,7 +9121,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -9138,17 +9130,17 @@
         </is>
       </c>
       <c r="E243" t="n">
-        <v>0.24</v>
+        <v>0.3106796116504854</v>
       </c>
       <c r="F243" t="n">
-        <v>0.25</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G243" t="n">
-        <v>0.4466019417475728</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>0.3122 (0.1165)</t>
+          <t>0.3618 (0.0444)</t>
         </is>
       </c>
     </row>
@@ -9160,31 +9152,31 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E244" t="n">
-        <v>0.367816091954023</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F244" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.3863636363636364</v>
       </c>
       <c r="G244" t="n">
-        <v>0.3953488372093023</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>0.3826 (0.0139)</t>
+          <t>0.3811 (0.0259)</t>
         </is>
       </c>
     </row>
@@ -9196,31 +9188,31 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E245" t="n">
-        <v>0.3260869565217391</v>
+        <v>0.2365591397849462</v>
       </c>
       <c r="F245" t="n">
-        <v>0.4086021505376344</v>
+        <v>0.275</v>
       </c>
       <c r="G245" t="n">
-        <v>0.449438202247191</v>
+        <v>0.3595505617977528</v>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>0.3947 (0.0628)</t>
+          <t>0.2904 (0.0629)</t>
         </is>
       </c>
     </row>
@@ -9232,31 +9224,31 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E246" t="n">
-        <v>0.247191011235955</v>
+        <v>0.4912280701754386</v>
       </c>
       <c r="F246" t="n">
-        <v>0.3376623376623377</v>
+        <v>0.345679012345679</v>
       </c>
       <c r="G246" t="n">
-        <v>0.2716049382716049</v>
+        <v>0.459016393442623</v>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>0.2855 (0.0468)</t>
+          <t>0.4320 (0.0764)</t>
         </is>
       </c>
     </row>
@@ -9268,31 +9260,31 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E247" t="n">
-        <v>0.5045045045045045</v>
+        <v>0.24</v>
       </c>
       <c r="F247" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.25</v>
       </c>
       <c r="G247" t="n">
-        <v>0.4554455445544555</v>
+        <v>0.4466019417475728</v>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>0.4599 (0.0426)</t>
+          <t>0.3122 (0.1165)</t>
         </is>
       </c>
     </row>
@@ -9309,7 +9301,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -9318,17 +9310,17 @@
         </is>
       </c>
       <c r="E248" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.367816091954023</v>
       </c>
       <c r="F248" t="n">
-        <v>0.3235294117647059</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G248" t="n">
-        <v>0.48</v>
+        <v>0.3953488372093023</v>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>0.3691 (0.0965)</t>
+          <t>0.3826 (0.0139)</t>
         </is>
       </c>
     </row>
@@ -9340,31 +9332,31 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E249" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3260869565217391</v>
       </c>
       <c r="F249" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.4086021505376344</v>
       </c>
       <c r="G249" t="n">
-        <v>0.3655913978494624</v>
+        <v>0.449438202247191</v>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>0.3654 (0.0124)</t>
+          <t>0.3947 (0.0628)</t>
         </is>
       </c>
     </row>
@@ -9376,31 +9368,31 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E250" t="n">
-        <v>0.4</v>
+        <v>0.247191011235955</v>
       </c>
       <c r="F250" t="n">
-        <v>0.4885496183206107</v>
+        <v>0.3376623376623377</v>
       </c>
       <c r="G250" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.2716049382716049</v>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>0.4443 (0.0443)</t>
+          <t>0.2855 (0.0468)</t>
         </is>
       </c>
     </row>
@@ -9412,31 +9404,31 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E251" t="n">
-        <v>0.3963963963963964</v>
+        <v>0.5045045045045045</v>
       </c>
       <c r="F251" t="n">
-        <v>0.2823529411764706</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G251" t="n">
-        <v>0.3505154639175257</v>
+        <v>0.4554455445544555</v>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>0.3431 (0.0574)</t>
+          <t>0.4599 (0.0426)</t>
         </is>
       </c>
     </row>
@@ -9448,31 +9440,31 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>0.4905660377358491</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F252" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.3235294117647059</v>
       </c>
       <c r="G252" t="n">
-        <v>0.4888888888888889</v>
+        <v>0.48</v>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>0.4524 (0.0646)</t>
+          <t>0.3691 (0.0965)</t>
         </is>
       </c>
     </row>
@@ -9489,7 +9481,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -9498,17 +9490,17 @@
         </is>
       </c>
       <c r="E253" t="n">
-        <v>0.3423423423423423</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F253" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G253" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.3655913978494624</v>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>0.3306 (0.0403)</t>
+          <t>0.3654 (0.0124)</t>
         </is>
       </c>
     </row>
@@ -9520,31 +9512,31 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>0.4369747899159664</v>
+        <v>0.4</v>
       </c>
       <c r="F254" t="n">
-        <v>0.3013698630136986</v>
+        <v>0.4885496183206107</v>
       </c>
       <c r="G254" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>0.3850 (0.0731)</t>
+          <t>0.4443 (0.0443)</t>
         </is>
       </c>
     </row>
@@ -9556,31 +9548,31 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E255" t="n">
+        <v>0.3963963963963964</v>
+      </c>
+      <c r="F255" t="n">
+        <v>0.2823529411764706</v>
+      </c>
+      <c r="G255" t="n">
         <v>0.3505154639175257</v>
       </c>
-      <c r="F255" t="n">
-        <v>0.3902439024390244</v>
-      </c>
-      <c r="G255" t="n">
-        <v>0.4050632911392405</v>
-      </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>0.3819 (0.0282)</t>
+          <t>0.3431 (0.0574)</t>
         </is>
       </c>
     </row>
@@ -9592,31 +9584,31 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>0.2619047619047619</v>
+        <v>0.4905660377358491</v>
       </c>
       <c r="F256" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G256" t="n">
-        <v>0.2318840579710145</v>
+        <v>0.4888888888888889</v>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>0.2501 (0.0160)</t>
+          <t>0.4524 (0.0646)</t>
         </is>
       </c>
     </row>
@@ -9628,31 +9620,31 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E257" t="n">
-        <v>0.5546218487394958</v>
+        <v>0.3423423423423423</v>
       </c>
       <c r="F257" t="n">
-        <v>0.5217391304347826</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G257" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>0.5084 (0.0541)</t>
+          <t>0.3306 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -9669,7 +9661,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -9678,17 +9670,17 @@
         </is>
       </c>
       <c r="E258" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.4369747899159664</v>
       </c>
       <c r="F258" t="n">
-        <v>0.1875</v>
+        <v>0.3013698630136986</v>
       </c>
       <c r="G258" t="n">
-        <v>0.32</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>0.2136 (0.0960)</t>
+          <t>0.3850 (0.0731)</t>
         </is>
       </c>
     </row>
@@ -9700,31 +9692,31 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="F259" t="n">
-        <v>0.4155844155844156</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="G259" t="n">
-        <v>0.4470588235294118</v>
+        <v>0.4050632911392405</v>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>0.4372 (0.0188)</t>
+          <t>0.3819 (0.0282)</t>
         </is>
       </c>
     </row>
@@ -9736,31 +9728,31 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E260" t="n">
-        <v>0.4117647058823529</v>
+        <v>0.2619047619047619</v>
       </c>
       <c r="F260" t="n">
-        <v>0.3958333333333333</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="G260" t="n">
-        <v>0.4044943820224719</v>
+        <v>0.2318840579710145</v>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>0.4040 (0.0080)</t>
+          <t>0.2501 (0.0160)</t>
         </is>
       </c>
     </row>
@@ -9772,31 +9764,31 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E261" t="n">
-        <v>0.2888888888888889</v>
+        <v>0.5546218487394958</v>
       </c>
       <c r="F261" t="n">
-        <v>0.2077922077922078</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="G261" t="n">
-        <v>0.3908045977011494</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>0.2958 (0.0917)</t>
+          <t>0.5084 (0.0541)</t>
         </is>
       </c>
     </row>
@@ -9808,31 +9800,31 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E262" t="n">
-        <v>0.4835164835164835</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="F262" t="n">
-        <v>0.3950617283950617</v>
+        <v>0.1875</v>
       </c>
       <c r="G262" t="n">
-        <v>0.4946236559139785</v>
+        <v>0.32</v>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>0.4577 (0.0546)</t>
+          <t>0.2136 (0.0960)</t>
         </is>
       </c>
     </row>
@@ -9849,7 +9841,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -9858,161 +9850,161 @@
         </is>
       </c>
       <c r="E263" t="n">
-        <v>0.1578947368421053</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F263" t="n">
-        <v>0.2121212121212121</v>
+        <v>0.4155844155844156</v>
       </c>
       <c r="G263" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.4470588235294118</v>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>0.2706 (0.1508)</t>
+          <t>0.4372 (0.0188)</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E264" t="n">
-        <v>0.1558441558441558</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="F264" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.3958333333333333</v>
       </c>
       <c r="G264" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.4044943820224719</v>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>0.2654 (0.1127)</t>
+          <t>0.4040 (0.0080)</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E265" t="n">
-        <v>0.2037037037037037</v>
+        <v>0.2888888888888889</v>
       </c>
       <c r="F265" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.2077922077922078</v>
       </c>
       <c r="G265" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.3908045977011494</v>
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>0.2974 (0.0906)</t>
+          <t>0.2958 (0.0917)</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E266" t="n">
-        <v>0.0625</v>
+        <v>0.4835164835164835</v>
       </c>
       <c r="F266" t="n">
-        <v>0.2898550724637681</v>
+        <v>0.3950617283950617</v>
       </c>
       <c r="G266" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.4946236559139785</v>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>0.2110 (0.1287)</t>
+          <t>0.4577 (0.0546)</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>0.2769230769230769</v>
+        <v>0.1578947368421053</v>
       </c>
       <c r="F267" t="n">
-        <v>0.3661971830985916</v>
+        <v>0.2121212121212121</v>
       </c>
       <c r="G267" t="n">
-        <v>0.208955223880597</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>0.2840 (0.0789)</t>
+          <t>0.2706 (0.1508)</t>
         </is>
       </c>
     </row>
@@ -10029,7 +10021,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -10038,17 +10030,17 @@
         </is>
       </c>
       <c r="E268" t="n">
-        <v>0.1212121212121212</v>
+        <v>0.1558441558441558</v>
       </c>
       <c r="F268" t="n">
-        <v>0.2424242424242424</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="G268" t="n">
-        <v>0.2432432432432433</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>0.2023 (0.0702)</t>
+          <t>0.2654 (0.1127)</t>
         </is>
       </c>
     </row>
@@ -10060,31 +10052,31 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>0.2325581395348837</v>
+        <v>0.2037037037037037</v>
       </c>
       <c r="F269" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G269" t="n">
-        <v>0.2553191489361702</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>0.2579 (0.0267)</t>
+          <t>0.2974 (0.0906)</t>
         </is>
       </c>
     </row>
@@ -10096,31 +10088,31 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.0625</v>
       </c>
       <c r="F270" t="n">
+        <v>0.2898550724637681</v>
+      </c>
+      <c r="G270" t="n">
         <v>0.2807017543859649</v>
       </c>
-      <c r="G270" t="n">
-        <v>0.3137254901960784</v>
-      </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>0.2751 (0.0418)</t>
+          <t>0.2110 (0.1287)</t>
         </is>
       </c>
     </row>
@@ -10132,31 +10124,31 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E271" t="n">
-        <v>0.08</v>
+        <v>0.2769230769230769</v>
       </c>
       <c r="F271" t="n">
-        <v>0.1176470588235294</v>
+        <v>0.3661971830985916</v>
       </c>
       <c r="G271" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>0.1528 (0.0954)</t>
+          <t>0.2840 (0.0789)</t>
         </is>
       </c>
     </row>
@@ -10168,31 +10160,31 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>0.28125</v>
+        <v>0.1212121212121212</v>
       </c>
       <c r="F272" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.2424242424242424</v>
       </c>
       <c r="G272" t="n">
-        <v>0.2181818181818182</v>
+        <v>0.2432432432432433</v>
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>0.2814 (0.0633)</t>
+          <t>0.2023 (0.0702)</t>
         </is>
       </c>
     </row>
@@ -10209,7 +10201,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -10218,17 +10210,17 @@
         </is>
       </c>
       <c r="E273" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.2325581395348837</v>
       </c>
       <c r="F273" t="n">
-        <v>0.1621621621621622</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G273" t="n">
-        <v>0.2790697674418605</v>
+        <v>0.2553191489361702</v>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>0.1831 (0.0874)</t>
+          <t>0.2579 (0.0267)</t>
         </is>
       </c>
     </row>
@@ -10240,31 +10232,31 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>0.1754385964912281</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="F274" t="n">
-        <v>0.34375</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="G274" t="n">
-        <v>0.3508771929824561</v>
+        <v>0.3137254901960784</v>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>0.2900 (0.0993)</t>
+          <t>0.2751 (0.0418)</t>
         </is>
       </c>
     </row>
@@ -10276,31 +10268,31 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>0.1839080459770115</v>
+        <v>0.08</v>
       </c>
       <c r="F275" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.1176470588235294</v>
       </c>
       <c r="G275" t="n">
-        <v>0.2702702702702703</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>0.2690 (0.0845)</t>
+          <t>0.1528 (0.0954)</t>
         </is>
       </c>
     </row>
@@ -10312,31 +10304,31 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>0.09230769230769231</v>
+        <v>0.28125</v>
       </c>
       <c r="F276" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="G276" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.2181818181818182</v>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>0.1654 (0.0725)</t>
+          <t>0.2814 (0.0633)</t>
         </is>
       </c>
     </row>
@@ -10348,31 +10340,31 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="F277" t="n">
-        <v>0.4307692307692308</v>
+        <v>0.1621621621621622</v>
       </c>
       <c r="G277" t="n">
-        <v>0.3076923076923077</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>0.3342 (0.0864)</t>
+          <t>0.1831 (0.0874)</t>
         </is>
       </c>
     </row>
@@ -10389,7 +10381,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -10398,17 +10390,17 @@
         </is>
       </c>
       <c r="E278" t="n">
-        <v>0.1639344262295082</v>
+        <v>0.1754385964912281</v>
       </c>
       <c r="F278" t="n">
-        <v>0.2962962962962963</v>
+        <v>0.34375</v>
       </c>
       <c r="G278" t="n">
-        <v>0.2295081967213115</v>
+        <v>0.3508771929824561</v>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>0.2299 (0.0662)</t>
+          <t>0.2900 (0.0993)</t>
         </is>
       </c>
     </row>
@@ -10420,31 +10412,31 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>0.1777777777777778</v>
+        <v>0.1839080459770115</v>
       </c>
       <c r="F279" t="n">
-        <v>0.2272727272727273</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="G279" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.2702702702702703</v>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>0.2205 (0.0398)</t>
+          <t>0.2690 (0.0845)</t>
         </is>
       </c>
     </row>
@@ -10456,31 +10448,31 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>0.2790697674418605</v>
+        <v>0.09230769230769231</v>
       </c>
       <c r="F280" t="n">
-        <v>0.3859649122807017</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="G280" t="n">
-        <v>0.3673469387755102</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>0.3441 (0.0571)</t>
+          <t>0.1654 (0.0725)</t>
         </is>
       </c>
     </row>
@@ -10492,31 +10484,31 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F281" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.4307692307692308</v>
       </c>
       <c r="G281" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>0.1530 (0.0500)</t>
+          <t>0.3342 (0.0864)</t>
         </is>
       </c>
     </row>
@@ -10528,31 +10520,31 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.1639344262295082</v>
       </c>
       <c r="F282" t="n">
-        <v>0.4</v>
+        <v>0.2962962962962963</v>
       </c>
       <c r="G282" t="n">
-        <v>0.3571428571428572</v>
+        <v>0.2295081967213115</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>0.3226 (0.0994)</t>
+          <t>0.2299 (0.0662)</t>
         </is>
       </c>
     </row>
@@ -10569,7 +10561,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -10578,17 +10570,17 @@
         </is>
       </c>
       <c r="E283" t="n">
-        <v>0.0975609756097561</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="F283" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2272727272727273</v>
       </c>
       <c r="G283" t="n">
-        <v>0.25</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>0.1462 (0.0900)</t>
+          <t>0.2205 (0.0398)</t>
         </is>
       </c>
     </row>
@@ -10600,31 +10592,31 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>0.2380952380952381</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="F284" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.3859649122807017</v>
       </c>
       <c r="G284" t="n">
-        <v>0.3478260869565217</v>
+        <v>0.3673469387755102</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>0.2429 (0.1026)</t>
+          <t>0.3441 (0.0571)</t>
         </is>
       </c>
     </row>
@@ -10636,31 +10628,31 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>0.24</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="F285" t="n">
-        <v>0.303030303030303</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G285" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>0.2708 (0.0315)</t>
+          <t>0.1530 (0.0500)</t>
         </is>
       </c>
     </row>
@@ -10672,31 +10664,31 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E286" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="F286" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.4</v>
       </c>
       <c r="G286" t="n">
-        <v>0.2173913043478261</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>0.1515 (0.0671)</t>
+          <t>0.3226 (0.0994)</t>
         </is>
       </c>
     </row>
@@ -10708,31 +10700,31 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E287" t="n">
+        <v>0.0975609756097561</v>
+      </c>
+      <c r="F287" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="G287" t="n">
         <v>0.25</v>
       </c>
-      <c r="F287" t="n">
-        <v>0.3636363636363636</v>
-      </c>
-      <c r="G287" t="n">
-        <v>0.2857142857142857</v>
-      </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>0.2998 (0.0581)</t>
+          <t>0.1462 (0.0900)</t>
         </is>
       </c>
     </row>
@@ -10749,7 +10741,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -10758,161 +10750,161 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>0.25</v>
+        <v>0.2380952380952381</v>
       </c>
       <c r="F288" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="G288" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3478260869565217</v>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>0.2146 (0.0939)</t>
+          <t>0.2429 (0.1026)</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>0.2391304347826087</v>
+        <v>0.24</v>
       </c>
       <c r="F289" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G289" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>0.3070 (0.0589)</t>
+          <t>0.2708 (0.0315)</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>0.3168316831683168</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F290" t="n">
-        <v>0.3454545454545455</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="G290" t="n">
-        <v>0.3793103448275862</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>0.3472 (0.0313)</t>
+          <t>0.1515 (0.0671)</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.25</v>
       </c>
       <c r="F291" t="n">
-        <v>0.4303797468354431</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="G291" t="n">
-        <v>0.3820224719101123</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>0.4054 (0.0242)</t>
+          <t>0.2998 (0.0581)</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>0.4036697247706422</v>
+        <v>0.25</v>
       </c>
       <c r="F292" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="G292" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>0.4326 (0.0256)</t>
+          <t>0.2146 (0.0939)</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10921,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
@@ -10938,17 +10930,17 @@
         </is>
       </c>
       <c r="E293" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.2391304347826087</v>
       </c>
       <c r="F293" t="n">
-        <v>0.2117647058823529</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="G293" t="n">
-        <v>0.2921348314606741</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>0.2538 (0.0403)</t>
+          <t>0.3070 (0.0589)</t>
         </is>
       </c>
     </row>
@@ -10960,27 +10952,31 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>0.2285714285714286</v>
-      </c>
-      <c r="F294" t="inlineStr"/>
-      <c r="G294" t="inlineStr"/>
+        <v>0.3168316831683168</v>
+      </c>
+      <c r="F294" t="n">
+        <v>0.3454545454545455</v>
+      </c>
+      <c r="G294" t="n">
+        <v>0.3793103448275862</v>
+      </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>0.2286 (0.0000)</t>
+          <t>0.3472 (0.0313)</t>
         </is>
       </c>
     </row>
@@ -10992,31 +10988,31 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>0.3023255813953488</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="F295" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.4303797468354431</v>
       </c>
       <c r="G295" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.3820224719101123</v>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>0.3677 (0.0598)</t>
+          <t>0.4054 (0.0242)</t>
         </is>
       </c>
     </row>
@@ -11028,31 +11024,31 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.4036697247706422</v>
       </c>
       <c r="F296" t="n">
-        <v>0.2597402597402597</v>
+        <v>0.4523809523809524</v>
       </c>
       <c r="G296" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>0.3101 (0.0862)</t>
+          <t>0.4326 (0.0256)</t>
         </is>
       </c>
     </row>
@@ -11064,27 +11060,31 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>0.4356435643564356</v>
-      </c>
-      <c r="F297" t="inlineStr"/>
-      <c r="G297" t="inlineStr"/>
+        <v>0.2574257425742574</v>
+      </c>
+      <c r="F297" t="n">
+        <v>0.2117647058823529</v>
+      </c>
+      <c r="G297" t="n">
+        <v>0.2921348314606741</v>
+      </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>0.4356 (0.0000)</t>
+          <t>0.2538 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -11101,7 +11101,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
@@ -11110,13 +11110,13 @@
         </is>
       </c>
       <c r="E298" t="n">
-        <v>0.3235294117647059</v>
+        <v>0.2285714285714286</v>
       </c>
       <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr"/>
       <c r="H298" t="inlineStr">
         <is>
-          <t>0.3235 (0.0000)</t>
+          <t>0.2286 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -11128,27 +11128,31 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>0.2736842105263158</v>
-      </c>
-      <c r="F299" t="inlineStr"/>
-      <c r="G299" t="inlineStr"/>
+        <v>0.3023255813953488</v>
+      </c>
+      <c r="F299" t="n">
+        <v>0.4197530864197531</v>
+      </c>
+      <c r="G299" t="n">
+        <v>0.3809523809523809</v>
+      </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>0.2737 (0.0000)</t>
+          <t>0.3677 (0.0598)</t>
         </is>
       </c>
     </row>
@@ -11160,31 +11164,31 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>0.3760683760683761</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="F300" t="n">
-        <v>0.46</v>
+        <v>0.2597402597402597</v>
       </c>
       <c r="G300" t="n">
-        <v>0.4081632653061225</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>0.4147 (0.0424)</t>
+          <t>0.3101 (0.0862)</t>
         </is>
       </c>
     </row>
@@ -11196,31 +11200,29 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.4356435643564356</v>
       </c>
       <c r="F301" t="n">
-        <v>0.3294117647058823</v>
-      </c>
-      <c r="G301" t="n">
-        <v>0.3838383838383838</v>
-      </c>
+        <v>0.4878048780487805</v>
+      </c>
+      <c r="G301" t="inlineStr"/>
       <c r="H301" t="inlineStr">
         <is>
-          <t>0.3236 (0.0634)</t>
+          <t>0.4617 (0.0369)</t>
         </is>
       </c>
     </row>
@@ -11232,27 +11234,27 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E302" t="n">
-        <v>0.4791666666666667</v>
+        <v>0.3235294117647059</v>
       </c>
       <c r="F302" t="inlineStr"/>
       <c r="G302" t="inlineStr"/>
       <c r="H302" t="inlineStr">
         <is>
-          <t>0.4792 (0.0000)</t>
+          <t>0.3235 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -11269,7 +11271,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
@@ -11278,15 +11280,15 @@
         </is>
       </c>
       <c r="E303" t="n">
-        <v>0.3125</v>
+        <v>0.2736842105263158</v>
       </c>
       <c r="F303" t="n">
-        <v>0.4337349397590362</v>
+        <v>0.3736263736263736</v>
       </c>
       <c r="G303" t="inlineStr"/>
       <c r="H303" t="inlineStr">
         <is>
-          <t>0.3731 (0.0857)</t>
+          <t>0.3237 (0.0707)</t>
         </is>
       </c>
     </row>
@@ -11298,31 +11300,31 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>0.1724137931034483</v>
+        <v>0.3760683760683761</v>
       </c>
       <c r="F304" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.46</v>
       </c>
       <c r="G304" t="n">
-        <v>0.3384615384615385</v>
+        <v>0.4081632653061225</v>
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>0.2572 (0.0831)</t>
+          <t>0.4147 (0.0424)</t>
         </is>
       </c>
     </row>
@@ -11334,31 +11336,31 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.2574257425742574</v>
       </c>
       <c r="F305" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.3294117647058823</v>
       </c>
       <c r="G305" t="n">
-        <v>0.3611111111111111</v>
+        <v>0.3838383838383838</v>
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>0.3582 (0.0530)</t>
+          <t>0.3236 (0.0634)</t>
         </is>
       </c>
     </row>
@@ -11370,31 +11372,29 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E306" t="n">
-        <v>0.2</v>
+        <v>0.4791666666666667</v>
       </c>
       <c r="F306" t="n">
-        <v>0.2571428571428571</v>
-      </c>
-      <c r="G306" t="n">
-        <v>0.253968253968254</v>
-      </c>
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="G306" t="inlineStr"/>
       <c r="H306" t="inlineStr">
         <is>
-          <t>0.2370 (0.0321)</t>
+          <t>0.4539 (0.0358)</t>
         </is>
       </c>
     </row>
@@ -11406,31 +11406,29 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E307" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.3125</v>
       </c>
       <c r="F307" t="n">
-        <v>0.4395604395604396</v>
-      </c>
-      <c r="G307" t="n">
-        <v>0.4594594594594595</v>
-      </c>
+        <v>0.4337349397590362</v>
+      </c>
+      <c r="G307" t="inlineStr"/>
       <c r="H307" t="inlineStr">
         <is>
-          <t>0.4493 (0.0100)</t>
+          <t>0.3731 (0.0857)</t>
         </is>
       </c>
     </row>
@@ -11447,7 +11445,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
@@ -11456,17 +11454,17 @@
         </is>
       </c>
       <c r="E308" t="n">
-        <v>0.1153846153846154</v>
+        <v>0.1724137931034483</v>
       </c>
       <c r="F308" t="n">
-        <v>0.125</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="G308" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.3384615384615385</v>
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>0.1771 (0.0987)</t>
+          <t>0.2572 (0.0831)</t>
         </is>
       </c>
     </row>
@@ -11478,31 +11476,31 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E309" t="n">
-        <v>0.2253521126760563</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F309" t="n">
-        <v>0.3188405797101449</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="G309" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.3611111111111111</v>
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>0.3203 (0.0957)</t>
+          <t>0.3582 (0.0530)</t>
         </is>
       </c>
     </row>
@@ -11514,31 +11512,31 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E310" t="n">
-        <v>0.3296703296703297</v>
+        <v>0.2</v>
       </c>
       <c r="F310" t="n">
-        <v>0.4871794871794872</v>
+        <v>0.2571428571428571</v>
       </c>
       <c r="G310" t="n">
-        <v>0.4137931034482759</v>
+        <v>0.253968253968254</v>
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>0.4102 (0.0788)</t>
+          <t>0.2370 (0.0321)</t>
         </is>
       </c>
     </row>
@@ -11550,31 +11548,31 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E311" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F311" t="n">
-        <v>0.3544303797468354</v>
+        <v>0.4395604395604396</v>
       </c>
       <c r="G311" t="n">
-        <v>0.3188405797101449</v>
+        <v>0.4594594594594595</v>
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>0.3342 (0.0183)</t>
+          <t>0.4493 (0.0100)</t>
         </is>
       </c>
     </row>
@@ -11586,31 +11584,31 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E312" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.1153846153846154</v>
       </c>
       <c r="F312" t="n">
-        <v>0.358974358974359</v>
+        <v>0.125</v>
       </c>
       <c r="G312" t="n">
-        <v>0.4810126582278481</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>0.3949 (0.0749)</t>
+          <t>0.1771 (0.0987)</t>
         </is>
       </c>
     </row>
@@ -11627,24 +11625,168 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E313" t="n">
+        <v>0.2253521126760563</v>
+      </c>
+      <c r="F313" t="n">
+        <v>0.3188405797101449</v>
+      </c>
+      <c r="G313" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>0.3203 (0.0957)</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E314" t="n">
+        <v>0.3296703296703297</v>
+      </c>
+      <c r="F314" t="n">
+        <v>0.4871794871794872</v>
+      </c>
+      <c r="G314" t="n">
+        <v>0.4137931034482759</v>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>0.4102 (0.0788)</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E315" t="n">
+        <v>0.3294117647058823</v>
+      </c>
+      <c r="F315" t="n">
+        <v>0.3544303797468354</v>
+      </c>
+      <c r="G315" t="n">
+        <v>0.3188405797101449</v>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>0.3342 (0.0183)</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E316" t="n">
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="F316" t="n">
+        <v>0.358974358974359</v>
+      </c>
+      <c r="G316" t="n">
+        <v>0.4810126582278481</v>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>0.3949 (0.0749)</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D313" t="inlineStr">
+      <c r="D317" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E313" t="n">
+      <c r="E317" t="n">
         <v>0.2777777777777778</v>
       </c>
-      <c r="F313" t="n">
+      <c r="F317" t="n">
         <v>0.360655737704918</v>
       </c>
-      <c r="G313" t="n">
+      <c r="G317" t="n">
         <v>0.3448275862068966</v>
       </c>
-      <c r="H313" t="inlineStr">
+      <c r="H317" t="inlineStr">
         <is>
           <t>0.3278 (0.0440)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 04:31:06)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H317"/>
+  <dimension ref="A1:H319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8748,11 +8748,15 @@
       <c r="E232" t="n">
         <v>0.2133333333333333</v>
       </c>
-      <c r="F232" t="inlineStr"/>
-      <c r="G232" t="inlineStr"/>
+      <c r="F232" t="n">
+        <v>0.4418604651162791</v>
+      </c>
+      <c r="G232" t="n">
+        <v>0.3703703703703703</v>
+      </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>0.2133 (0.0000)</t>
+          <t>0.3419 (0.1169)</t>
         </is>
       </c>
     </row>
@@ -8764,31 +8768,27 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E233" t="n">
-        <v>0.08333333333333333</v>
-      </c>
-      <c r="F233" t="n">
-        <v>0.2307692307692308</v>
-      </c>
-      <c r="G233" t="n">
-        <v>0.3870967741935484</v>
-      </c>
+        <v>0.3174603174603174</v>
+      </c>
+      <c r="F233" t="inlineStr"/>
+      <c r="G233" t="inlineStr"/>
       <c r="H233" t="inlineStr">
         <is>
-          <t>0.2337 (0.1519)</t>
+          <t>0.3175 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -8800,7 +8800,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -8810,21 +8810,21 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E234" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.3364485981308411</v>
       </c>
       <c r="F234" t="n">
-        <v>0.48</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="G234" t="n">
-        <v>0.3870967741935484</v>
+        <v>0.3764705882352941</v>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>0.3681 (0.1225)</t>
+          <t>0.3873 (0.0570)</t>
         </is>
       </c>
     </row>
@@ -8841,7 +8841,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -8850,17 +8850,17 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>0.3</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F235" t="n">
-        <v>0.3714285714285714</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G235" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>0.3029 (0.0671)</t>
+          <t>0.2337 (0.1519)</t>
         </is>
       </c>
     </row>
@@ -8877,7 +8877,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -8886,17 +8886,17 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>0.4848484848484849</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="F236" t="n">
-        <v>0.5151515151515151</v>
+        <v>0.48</v>
       </c>
       <c r="G236" t="n">
-        <v>0.4</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>0.4667 (0.0597)</t>
+          <t>0.3681 (0.1225)</t>
         </is>
       </c>
     </row>
@@ -8913,7 +8913,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -8922,17 +8922,17 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>0.0975609756097561</v>
+        <v>0.3</v>
       </c>
       <c r="F237" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.3714285714285714</v>
       </c>
       <c r="G237" t="n">
-        <v>0.3214285714285715</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>0.2166 (0.1126)</t>
+          <t>0.3029 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -8944,27 +8944,31 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E238" t="n">
-        <v>0.2307692307692308</v>
-      </c>
-      <c r="F238" t="inlineStr"/>
-      <c r="G238" t="inlineStr"/>
+        <v>0.4848484848484849</v>
+      </c>
+      <c r="F238" t="n">
+        <v>0.5151515151515151</v>
+      </c>
+      <c r="G238" t="n">
+        <v>0.4</v>
+      </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>0.2308 (0.0000)</t>
+          <t>0.4667 (0.0597)</t>
         </is>
       </c>
     </row>
@@ -8976,31 +8980,31 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>0.3116883116883117</v>
+        <v>0.0975609756097561</v>
       </c>
       <c r="F239" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G239" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3214285714285715</v>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>0.3581 (0.0492)</t>
+          <t>0.2166 (0.1126)</t>
         </is>
       </c>
     </row>
@@ -9017,7 +9021,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -9026,17 +9030,17 @@
         </is>
       </c>
       <c r="E240" t="n">
-        <v>0.3050847457627119</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="F240" t="n">
-        <v>0.3278688524590164</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="G240" t="n">
-        <v>0.3050847457627119</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>0.3127 (0.0132)</t>
+          <t>0.3785 (0.1301)</t>
         </is>
       </c>
     </row>
@@ -9053,7 +9057,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -9062,15 +9066,17 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>0.3666666666666666</v>
+        <v>0.3116883116883117</v>
       </c>
       <c r="F241" t="n">
-        <v>0.5161290322580645</v>
-      </c>
-      <c r="G241" t="inlineStr"/>
+        <v>0.4096385542168675</v>
+      </c>
+      <c r="G241" t="n">
+        <v>0.3529411764705883</v>
+      </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>0.4414 (0.1057)</t>
+          <t>0.3581 (0.0492)</t>
         </is>
       </c>
     </row>
@@ -9087,7 +9093,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -9096,87 +9102,89 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.3050847457627119</v>
       </c>
       <c r="F242" t="n">
-        <v>0.2692307692307692</v>
-      </c>
-      <c r="G242" t="inlineStr"/>
+        <v>0.3278688524590164</v>
+      </c>
+      <c r="G242" t="n">
+        <v>0.3050847457627119</v>
+      </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>0.1801 (0.1261)</t>
+          <t>0.3127 (0.0132)</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E243" t="n">
-        <v>0.3106796116504854</v>
+        <v>0.3666666666666666</v>
       </c>
       <c r="F243" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.5161290322580645</v>
       </c>
       <c r="G243" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>0.3618 (0.0444)</t>
+          <t>0.4119 (0.0905)</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E244" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="F244" t="n">
-        <v>0.3863636363636364</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="G244" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.3934426229508197</v>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>0.3811 (0.0259)</t>
+          <t>0.2512 (0.1521)</t>
         </is>
       </c>
     </row>
@@ -9193,7 +9201,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -9202,17 +9210,17 @@
         </is>
       </c>
       <c r="E245" t="n">
-        <v>0.2365591397849462</v>
+        <v>0.3106796116504854</v>
       </c>
       <c r="F245" t="n">
-        <v>0.275</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G245" t="n">
-        <v>0.3595505617977528</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>0.2904 (0.0629)</t>
+          <t>0.3618 (0.0444)</t>
         </is>
       </c>
     </row>
@@ -9229,7 +9237,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -9238,17 +9246,17 @@
         </is>
       </c>
       <c r="E246" t="n">
-        <v>0.4912280701754386</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F246" t="n">
-        <v>0.345679012345679</v>
+        <v>0.3863636363636364</v>
       </c>
       <c r="G246" t="n">
-        <v>0.459016393442623</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>0.4320 (0.0764)</t>
+          <t>0.3811 (0.0259)</t>
         </is>
       </c>
     </row>
@@ -9265,7 +9273,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -9274,17 +9282,17 @@
         </is>
       </c>
       <c r="E247" t="n">
-        <v>0.24</v>
+        <v>0.2365591397849462</v>
       </c>
       <c r="F247" t="n">
-        <v>0.25</v>
+        <v>0.275</v>
       </c>
       <c r="G247" t="n">
-        <v>0.4466019417475728</v>
+        <v>0.3595505617977528</v>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>0.3122 (0.1165)</t>
+          <t>0.2904 (0.0629)</t>
         </is>
       </c>
     </row>
@@ -9296,31 +9304,31 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E248" t="n">
-        <v>0.367816091954023</v>
+        <v>0.4912280701754386</v>
       </c>
       <c r="F248" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.345679012345679</v>
       </c>
       <c r="G248" t="n">
-        <v>0.3953488372093023</v>
+        <v>0.459016393442623</v>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>0.3826 (0.0139)</t>
+          <t>0.4320 (0.0764)</t>
         </is>
       </c>
     </row>
@@ -9332,31 +9340,31 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E249" t="n">
-        <v>0.3260869565217391</v>
+        <v>0.24</v>
       </c>
       <c r="F249" t="n">
-        <v>0.4086021505376344</v>
+        <v>0.25</v>
       </c>
       <c r="G249" t="n">
-        <v>0.449438202247191</v>
+        <v>0.4466019417475728</v>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>0.3947 (0.0628)</t>
+          <t>0.3122 (0.1165)</t>
         </is>
       </c>
     </row>
@@ -9373,7 +9381,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -9382,17 +9390,17 @@
         </is>
       </c>
       <c r="E250" t="n">
-        <v>0.247191011235955</v>
+        <v>0.367816091954023</v>
       </c>
       <c r="F250" t="n">
-        <v>0.3376623376623377</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G250" t="n">
-        <v>0.2716049382716049</v>
+        <v>0.3953488372093023</v>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>0.2855 (0.0468)</t>
+          <t>0.3826 (0.0139)</t>
         </is>
       </c>
     </row>
@@ -9409,7 +9417,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -9418,17 +9426,17 @@
         </is>
       </c>
       <c r="E251" t="n">
-        <v>0.5045045045045045</v>
+        <v>0.3260869565217391</v>
       </c>
       <c r="F251" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.4086021505376344</v>
       </c>
       <c r="G251" t="n">
-        <v>0.4554455445544555</v>
+        <v>0.449438202247191</v>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>0.4599 (0.0426)</t>
+          <t>0.3947 (0.0628)</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9453,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -9454,17 +9462,17 @@
         </is>
       </c>
       <c r="E252" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.247191011235955</v>
       </c>
       <c r="F252" t="n">
-        <v>0.3235294117647059</v>
+        <v>0.3376623376623377</v>
       </c>
       <c r="G252" t="n">
-        <v>0.48</v>
+        <v>0.2716049382716049</v>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>0.3691 (0.0965)</t>
+          <t>0.2855 (0.0468)</t>
         </is>
       </c>
     </row>
@@ -9476,31 +9484,31 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E253" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.5045045045045045</v>
       </c>
       <c r="F253" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G253" t="n">
-        <v>0.3655913978494624</v>
+        <v>0.4554455445544555</v>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>0.3654 (0.0124)</t>
+          <t>0.4599 (0.0426)</t>
         </is>
       </c>
     </row>
@@ -9512,31 +9520,31 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>0.4</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F254" t="n">
-        <v>0.4885496183206107</v>
+        <v>0.3235294117647059</v>
       </c>
       <c r="G254" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.48</v>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>0.4443 (0.0443)</t>
+          <t>0.3691 (0.0965)</t>
         </is>
       </c>
     </row>
@@ -9553,7 +9561,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -9562,17 +9570,17 @@
         </is>
       </c>
       <c r="E255" t="n">
-        <v>0.3963963963963964</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F255" t="n">
-        <v>0.2823529411764706</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G255" t="n">
-        <v>0.3505154639175257</v>
+        <v>0.3655913978494624</v>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>0.3431 (0.0574)</t>
+          <t>0.3654 (0.0124)</t>
         </is>
       </c>
     </row>
@@ -9589,7 +9597,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -9598,17 +9606,17 @@
         </is>
       </c>
       <c r="E256" t="n">
-        <v>0.4905660377358491</v>
+        <v>0.4</v>
       </c>
       <c r="F256" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.4885496183206107</v>
       </c>
       <c r="G256" t="n">
-        <v>0.4888888888888889</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>0.4524 (0.0646)</t>
+          <t>0.4443 (0.0443)</t>
         </is>
       </c>
     </row>
@@ -9625,7 +9633,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -9634,17 +9642,17 @@
         </is>
       </c>
       <c r="E257" t="n">
-        <v>0.3423423423423423</v>
+        <v>0.3963963963963964</v>
       </c>
       <c r="F257" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2823529411764706</v>
       </c>
       <c r="G257" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>0.3306 (0.0403)</t>
+          <t>0.3431 (0.0574)</t>
         </is>
       </c>
     </row>
@@ -9656,31 +9664,31 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E258" t="n">
-        <v>0.4369747899159664</v>
+        <v>0.4905660377358491</v>
       </c>
       <c r="F258" t="n">
-        <v>0.3013698630136986</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G258" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.4888888888888889</v>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>0.3850 (0.0731)</t>
+          <t>0.4524 (0.0646)</t>
         </is>
       </c>
     </row>
@@ -9692,31 +9700,31 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>0.3505154639175257</v>
+        <v>0.3423423423423423</v>
       </c>
       <c r="F259" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G259" t="n">
-        <v>0.4050632911392405</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>0.3819 (0.0282)</t>
+          <t>0.3306 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -9733,7 +9741,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -9742,17 +9750,17 @@
         </is>
       </c>
       <c r="E260" t="n">
-        <v>0.2619047619047619</v>
+        <v>0.4369747899159664</v>
       </c>
       <c r="F260" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.3013698630136986</v>
       </c>
       <c r="G260" t="n">
-        <v>0.2318840579710145</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>0.2501 (0.0160)</t>
+          <t>0.3850 (0.0731)</t>
         </is>
       </c>
     </row>
@@ -9769,7 +9777,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -9778,17 +9786,17 @@
         </is>
       </c>
       <c r="E261" t="n">
-        <v>0.5546218487394958</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="F261" t="n">
-        <v>0.5217391304347826</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="G261" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.4050632911392405</v>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>0.5084 (0.0541)</t>
+          <t>0.3819 (0.0282)</t>
         </is>
       </c>
     </row>
@@ -9805,7 +9813,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -9814,17 +9822,17 @@
         </is>
       </c>
       <c r="E262" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.2619047619047619</v>
       </c>
       <c r="F262" t="n">
-        <v>0.1875</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="G262" t="n">
-        <v>0.32</v>
+        <v>0.2318840579710145</v>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>0.2136 (0.0960)</t>
+          <t>0.2501 (0.0160)</t>
         </is>
       </c>
     </row>
@@ -9836,31 +9844,31 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E263" t="n">
+        <v>0.5546218487394958</v>
+      </c>
+      <c r="F263" t="n">
+        <v>0.5217391304347826</v>
+      </c>
+      <c r="G263" t="n">
         <v>0.4489795918367347</v>
       </c>
-      <c r="F263" t="n">
-        <v>0.4155844155844156</v>
-      </c>
-      <c r="G263" t="n">
-        <v>0.4470588235294118</v>
-      </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>0.4372 (0.0188)</t>
+          <t>0.5084 (0.0541)</t>
         </is>
       </c>
     </row>
@@ -9872,31 +9880,31 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E264" t="n">
-        <v>0.4117647058823529</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="F264" t="n">
-        <v>0.3958333333333333</v>
+        <v>0.1875</v>
       </c>
       <c r="G264" t="n">
-        <v>0.4044943820224719</v>
+        <v>0.32</v>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>0.4040 (0.0080)</t>
+          <t>0.2136 (0.0960)</t>
         </is>
       </c>
     </row>
@@ -9913,7 +9921,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -9922,17 +9930,17 @@
         </is>
       </c>
       <c r="E265" t="n">
-        <v>0.2888888888888889</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F265" t="n">
-        <v>0.2077922077922078</v>
+        <v>0.4155844155844156</v>
       </c>
       <c r="G265" t="n">
-        <v>0.3908045977011494</v>
+        <v>0.4470588235294118</v>
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>0.2958 (0.0917)</t>
+          <t>0.4372 (0.0188)</t>
         </is>
       </c>
     </row>
@@ -9949,7 +9957,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -9958,17 +9966,17 @@
         </is>
       </c>
       <c r="E266" t="n">
-        <v>0.4835164835164835</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="F266" t="n">
-        <v>0.3950617283950617</v>
+        <v>0.3958333333333333</v>
       </c>
       <c r="G266" t="n">
-        <v>0.4946236559139785</v>
+        <v>0.4044943820224719</v>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>0.4577 (0.0546)</t>
+          <t>0.4040 (0.0080)</t>
         </is>
       </c>
     </row>
@@ -9985,7 +9993,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -9994,89 +10002,89 @@
         </is>
       </c>
       <c r="E267" t="n">
-        <v>0.1578947368421053</v>
+        <v>0.2888888888888889</v>
       </c>
       <c r="F267" t="n">
-        <v>0.2121212121212121</v>
+        <v>0.2077922077922078</v>
       </c>
       <c r="G267" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.3908045977011494</v>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>0.2706 (0.1508)</t>
+          <t>0.2958 (0.0917)</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>0.1558441558441558</v>
+        <v>0.4835164835164835</v>
       </c>
       <c r="F268" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.3950617283950617</v>
       </c>
       <c r="G268" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.4946236559139785</v>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>0.2654 (0.1127)</t>
+          <t>0.4577 (0.0546)</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>0.2037037037037037</v>
+        <v>0.1578947368421053</v>
       </c>
       <c r="F269" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.2121212121212121</v>
       </c>
       <c r="G269" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>0.2974 (0.0906)</t>
+          <t>0.2706 (0.1508)</t>
         </is>
       </c>
     </row>
@@ -10093,7 +10101,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -10102,17 +10110,17 @@
         </is>
       </c>
       <c r="E270" t="n">
-        <v>0.0625</v>
+        <v>0.1558441558441558</v>
       </c>
       <c r="F270" t="n">
-        <v>0.2898550724637681</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="G270" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>0.2110 (0.1287)</t>
+          <t>0.2654 (0.1127)</t>
         </is>
       </c>
     </row>
@@ -10129,7 +10137,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -10138,17 +10146,17 @@
         </is>
       </c>
       <c r="E271" t="n">
-        <v>0.2769230769230769</v>
+        <v>0.2037037037037037</v>
       </c>
       <c r="F271" t="n">
-        <v>0.3661971830985916</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G271" t="n">
-        <v>0.208955223880597</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>0.2840 (0.0789)</t>
+          <t>0.2974 (0.0906)</t>
         </is>
       </c>
     </row>
@@ -10165,7 +10173,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -10174,17 +10182,17 @@
         </is>
       </c>
       <c r="E272" t="n">
-        <v>0.1212121212121212</v>
+        <v>0.0625</v>
       </c>
       <c r="F272" t="n">
-        <v>0.2424242424242424</v>
+        <v>0.2898550724637681</v>
       </c>
       <c r="G272" t="n">
-        <v>0.2432432432432433</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>0.2023 (0.0702)</t>
+          <t>0.2110 (0.1287)</t>
         </is>
       </c>
     </row>
@@ -10196,31 +10204,31 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>0.2325581395348837</v>
+        <v>0.2769230769230769</v>
       </c>
       <c r="F273" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3661971830985916</v>
       </c>
       <c r="G273" t="n">
-        <v>0.2553191489361702</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>0.2579 (0.0267)</t>
+          <t>0.2840 (0.0789)</t>
         </is>
       </c>
     </row>
@@ -10232,31 +10240,31 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.1212121212121212</v>
       </c>
       <c r="F274" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.2424242424242424</v>
       </c>
       <c r="G274" t="n">
-        <v>0.3137254901960784</v>
+        <v>0.2432432432432433</v>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>0.2751 (0.0418)</t>
+          <t>0.2023 (0.0702)</t>
         </is>
       </c>
     </row>
@@ -10273,7 +10281,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -10282,17 +10290,17 @@
         </is>
       </c>
       <c r="E275" t="n">
-        <v>0.08</v>
+        <v>0.2325581395348837</v>
       </c>
       <c r="F275" t="n">
-        <v>0.1176470588235294</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G275" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.2553191489361702</v>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>0.1528 (0.0954)</t>
+          <t>0.2579 (0.0267)</t>
         </is>
       </c>
     </row>
@@ -10309,7 +10317,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -10318,17 +10326,17 @@
         </is>
       </c>
       <c r="E276" t="n">
-        <v>0.28125</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="F276" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="G276" t="n">
-        <v>0.2181818181818182</v>
+        <v>0.3137254901960784</v>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>0.2814 (0.0633)</t>
+          <t>0.2751 (0.0418)</t>
         </is>
       </c>
     </row>
@@ -10345,7 +10353,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -10354,17 +10362,17 @@
         </is>
       </c>
       <c r="E277" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.08</v>
       </c>
       <c r="F277" t="n">
-        <v>0.1621621621621622</v>
+        <v>0.1176470588235294</v>
       </c>
       <c r="G277" t="n">
-        <v>0.2790697674418605</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>0.1831 (0.0874)</t>
+          <t>0.1528 (0.0954)</t>
         </is>
       </c>
     </row>
@@ -10376,31 +10384,31 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>0.1754385964912281</v>
+        <v>0.28125</v>
       </c>
       <c r="F278" t="n">
-        <v>0.34375</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="G278" t="n">
-        <v>0.3508771929824561</v>
+        <v>0.2181818181818182</v>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>0.2900 (0.0993)</t>
+          <t>0.2814 (0.0633)</t>
         </is>
       </c>
     </row>
@@ -10412,31 +10420,31 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>0.1839080459770115</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="F279" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.1621621621621622</v>
       </c>
       <c r="G279" t="n">
-        <v>0.2702702702702703</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>0.2690 (0.0845)</t>
+          <t>0.1831 (0.0874)</t>
         </is>
       </c>
     </row>
@@ -10453,7 +10461,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -10462,17 +10470,17 @@
         </is>
       </c>
       <c r="E280" t="n">
-        <v>0.09230769230769231</v>
+        <v>0.1754385964912281</v>
       </c>
       <c r="F280" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.34375</v>
       </c>
       <c r="G280" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.3508771929824561</v>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>0.1654 (0.0725)</t>
+          <t>0.2900 (0.0993)</t>
         </is>
       </c>
     </row>
@@ -10489,7 +10497,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -10498,17 +10506,17 @@
         </is>
       </c>
       <c r="E281" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.1839080459770115</v>
       </c>
       <c r="F281" t="n">
-        <v>0.4307692307692308</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="G281" t="n">
-        <v>0.3076923076923077</v>
+        <v>0.2702702702702703</v>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>0.3342 (0.0864)</t>
+          <t>0.2690 (0.0845)</t>
         </is>
       </c>
     </row>
@@ -10525,7 +10533,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -10534,17 +10542,17 @@
         </is>
       </c>
       <c r="E282" t="n">
-        <v>0.1639344262295082</v>
+        <v>0.09230769230769231</v>
       </c>
       <c r="F282" t="n">
-        <v>0.2962962962962963</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="G282" t="n">
-        <v>0.2295081967213115</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>0.2299 (0.0662)</t>
+          <t>0.1654 (0.0725)</t>
         </is>
       </c>
     </row>
@@ -10556,31 +10564,31 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>0.1777777777777778</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F283" t="n">
-        <v>0.2272727272727273</v>
+        <v>0.4307692307692308</v>
       </c>
       <c r="G283" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>0.2205 (0.0398)</t>
+          <t>0.3342 (0.0864)</t>
         </is>
       </c>
     </row>
@@ -10592,31 +10600,31 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>0.2790697674418605</v>
+        <v>0.1639344262295082</v>
       </c>
       <c r="F284" t="n">
-        <v>0.3859649122807017</v>
+        <v>0.2962962962962963</v>
       </c>
       <c r="G284" t="n">
-        <v>0.3673469387755102</v>
+        <v>0.2295081967213115</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>0.3441 (0.0571)</t>
+          <t>0.2299 (0.0662)</t>
         </is>
       </c>
     </row>
@@ -10633,7 +10641,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -10642,17 +10650,17 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="F285" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.2272727272727273</v>
       </c>
       <c r="G285" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>0.1530 (0.0500)</t>
+          <t>0.2205 (0.0398)</t>
         </is>
       </c>
     </row>
@@ -10669,7 +10677,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -10678,17 +10686,17 @@
         </is>
       </c>
       <c r="E286" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="F286" t="n">
-        <v>0.4</v>
+        <v>0.3859649122807017</v>
       </c>
       <c r="G286" t="n">
-        <v>0.3571428571428572</v>
+        <v>0.3673469387755102</v>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>0.3226 (0.0994)</t>
+          <t>0.3441 (0.0571)</t>
         </is>
       </c>
     </row>
@@ -10705,7 +10713,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -10714,17 +10722,17 @@
         </is>
       </c>
       <c r="E287" t="n">
-        <v>0.0975609756097561</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="F287" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G287" t="n">
-        <v>0.25</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>0.1462 (0.0900)</t>
+          <t>0.1530 (0.0500)</t>
         </is>
       </c>
     </row>
@@ -10736,31 +10744,31 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>0.2380952380952381</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="F288" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.4</v>
       </c>
       <c r="G288" t="n">
-        <v>0.3478260869565217</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>0.2429 (0.1026)</t>
+          <t>0.3226 (0.0994)</t>
         </is>
       </c>
     </row>
@@ -10772,31 +10780,31 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>0.24</v>
+        <v>0.0975609756097561</v>
       </c>
       <c r="F289" t="n">
-        <v>0.303030303030303</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="G289" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.25</v>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>0.2708 (0.0315)</t>
+          <t>0.1462 (0.0900)</t>
         </is>
       </c>
     </row>
@@ -10813,7 +10821,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -10822,17 +10830,17 @@
         </is>
       </c>
       <c r="E290" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.2380952380952381</v>
       </c>
       <c r="F290" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="G290" t="n">
-        <v>0.2173913043478261</v>
+        <v>0.3478260869565217</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>0.1515 (0.0671)</t>
+          <t>0.2429 (0.1026)</t>
         </is>
       </c>
     </row>
@@ -10849,7 +10857,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -10858,17 +10866,17 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="F291" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G291" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>0.2998 (0.0581)</t>
+          <t>0.2708 (0.0315)</t>
         </is>
       </c>
     </row>
@@ -10885,7 +10893,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
@@ -10894,89 +10902,89 @@
         </is>
       </c>
       <c r="E292" t="n">
-        <v>0.25</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F292" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="G292" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>0.2146 (0.0939)</t>
+          <t>0.1515 (0.0671)</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>0.2391304347826087</v>
+        <v>0.25</v>
       </c>
       <c r="F293" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="G293" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>0.3070 (0.0589)</t>
+          <t>0.2998 (0.0581)</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>0.3168316831683168</v>
+        <v>0.25</v>
       </c>
       <c r="F294" t="n">
-        <v>0.3454545454545455</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="G294" t="n">
-        <v>0.3793103448275862</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>0.3472 (0.0313)</t>
+          <t>0.2146 (0.0939)</t>
         </is>
       </c>
     </row>
@@ -10993,7 +11001,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
@@ -11002,17 +11010,17 @@
         </is>
       </c>
       <c r="E295" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.2391304347826087</v>
       </c>
       <c r="F295" t="n">
-        <v>0.4303797468354431</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="G295" t="n">
-        <v>0.3820224719101123</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>0.4054 (0.0242)</t>
+          <t>0.3070 (0.0589)</t>
         </is>
       </c>
     </row>
@@ -11029,7 +11037,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -11038,17 +11046,17 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>0.4036697247706422</v>
+        <v>0.3168316831683168</v>
       </c>
       <c r="F296" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.3454545454545455</v>
       </c>
       <c r="G296" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.3793103448275862</v>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>0.4326 (0.0256)</t>
+          <t>0.3472 (0.0313)</t>
         </is>
       </c>
     </row>
@@ -11065,7 +11073,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
@@ -11074,17 +11082,17 @@
         </is>
       </c>
       <c r="E297" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="F297" t="n">
-        <v>0.2117647058823529</v>
+        <v>0.4303797468354431</v>
       </c>
       <c r="G297" t="n">
-        <v>0.2921348314606741</v>
+        <v>0.3820224719101123</v>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>0.2538 (0.0403)</t>
+          <t>0.4054 (0.0242)</t>
         </is>
       </c>
     </row>
@@ -11096,27 +11104,31 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>0.2285714285714286</v>
-      </c>
-      <c r="F298" t="inlineStr"/>
-      <c r="G298" t="inlineStr"/>
+        <v>0.4036697247706422</v>
+      </c>
+      <c r="F298" t="n">
+        <v>0.4523809523809524</v>
+      </c>
+      <c r="G298" t="n">
+        <v>0.4418604651162791</v>
+      </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>0.2286 (0.0000)</t>
+          <t>0.4326 (0.0256)</t>
         </is>
       </c>
     </row>
@@ -11128,31 +11140,31 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>0.3023255813953488</v>
+        <v>0.2574257425742574</v>
       </c>
       <c r="F299" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.2117647058823529</v>
       </c>
       <c r="G299" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.2921348314606741</v>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>0.3677 (0.0598)</t>
+          <t>0.2538 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -11169,7 +11181,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
@@ -11178,17 +11190,15 @@
         </is>
       </c>
       <c r="E300" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.2285714285714286</v>
       </c>
       <c r="F300" t="n">
-        <v>0.2597402597402597</v>
-      </c>
-      <c r="G300" t="n">
-        <v>0.2608695652173913</v>
-      </c>
+        <v>0.3142857142857143</v>
+      </c>
+      <c r="G300" t="inlineStr"/>
       <c r="H300" t="inlineStr">
         <is>
-          <t>0.3101 (0.0862)</t>
+          <t>0.2714 (0.0606)</t>
         </is>
       </c>
     </row>
@@ -11205,7 +11215,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
@@ -11214,15 +11224,17 @@
         </is>
       </c>
       <c r="E301" t="n">
-        <v>0.4356435643564356</v>
+        <v>0.3023255813953488</v>
       </c>
       <c r="F301" t="n">
-        <v>0.4878048780487805</v>
-      </c>
-      <c r="G301" t="inlineStr"/>
+        <v>0.4197530864197531</v>
+      </c>
+      <c r="G301" t="n">
+        <v>0.3809523809523809</v>
+      </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>0.4617 (0.0369)</t>
+          <t>0.3677 (0.0598)</t>
         </is>
       </c>
     </row>
@@ -11239,7 +11251,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
@@ -11248,13 +11260,17 @@
         </is>
       </c>
       <c r="E302" t="n">
-        <v>0.3235294117647059</v>
-      </c>
-      <c r="F302" t="inlineStr"/>
-      <c r="G302" t="inlineStr"/>
+        <v>0.4096385542168675</v>
+      </c>
+      <c r="F302" t="n">
+        <v>0.2597402597402597</v>
+      </c>
+      <c r="G302" t="n">
+        <v>0.2608695652173913</v>
+      </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>0.3235 (0.0000)</t>
+          <t>0.3101 (0.0862)</t>
         </is>
       </c>
     </row>
@@ -11266,29 +11282,29 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>0.2736842105263158</v>
+        <v>0.4356435643564356</v>
       </c>
       <c r="F303" t="n">
-        <v>0.3736263736263736</v>
+        <v>0.4878048780487805</v>
       </c>
       <c r="G303" t="inlineStr"/>
       <c r="H303" t="inlineStr">
         <is>
-          <t>0.3237 (0.0707)</t>
+          <t>0.4617 (0.0369)</t>
         </is>
       </c>
     </row>
@@ -11300,31 +11316,27 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>0.3760683760683761</v>
-      </c>
-      <c r="F304" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="G304" t="n">
-        <v>0.4081632653061225</v>
-      </c>
+        <v>0.3235294117647059</v>
+      </c>
+      <c r="F304" t="inlineStr"/>
+      <c r="G304" t="inlineStr"/>
       <c r="H304" t="inlineStr">
         <is>
-          <t>0.4147 (0.0424)</t>
+          <t>0.3235 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -11341,7 +11353,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
@@ -11350,17 +11362,17 @@
         </is>
       </c>
       <c r="E305" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.2736842105263158</v>
       </c>
       <c r="F305" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.3736263736263736</v>
       </c>
       <c r="G305" t="n">
-        <v>0.3838383838383838</v>
+        <v>0.3855421686746988</v>
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>0.3236 (0.0634)</t>
+          <t>0.3443 (0.0614)</t>
         </is>
       </c>
     </row>
@@ -11377,7 +11389,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
@@ -11386,15 +11398,17 @@
         </is>
       </c>
       <c r="E306" t="n">
-        <v>0.4791666666666667</v>
+        <v>0.3760683760683761</v>
       </c>
       <c r="F306" t="n">
-        <v>0.4285714285714285</v>
-      </c>
-      <c r="G306" t="inlineStr"/>
+        <v>0.46</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0.4081632653061225</v>
+      </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>0.4539 (0.0358)</t>
+          <t>0.4147 (0.0424)</t>
         </is>
       </c>
     </row>
@@ -11411,7 +11425,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
@@ -11420,15 +11434,17 @@
         </is>
       </c>
       <c r="E307" t="n">
-        <v>0.3125</v>
+        <v>0.2574257425742574</v>
       </c>
       <c r="F307" t="n">
-        <v>0.4337349397590362</v>
-      </c>
-      <c r="G307" t="inlineStr"/>
+        <v>0.3294117647058823</v>
+      </c>
+      <c r="G307" t="n">
+        <v>0.3838383838383838</v>
+      </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>0.3731 (0.0857)</t>
+          <t>0.3236 (0.0634)</t>
         </is>
       </c>
     </row>
@@ -11440,31 +11456,31 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E308" t="n">
-        <v>0.1724137931034483</v>
+        <v>0.4791666666666667</v>
       </c>
       <c r="F308" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="G308" t="n">
-        <v>0.3384615384615385</v>
+        <v>0.4</v>
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>0.2572 (0.0831)</t>
+          <t>0.4359 (0.0401)</t>
         </is>
       </c>
     </row>
@@ -11476,31 +11492,31 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E309" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.3125</v>
       </c>
       <c r="F309" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.4337349397590362</v>
       </c>
       <c r="G309" t="n">
-        <v>0.3611111111111111</v>
+        <v>0.4269662921348314</v>
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>0.3582 (0.0530)</t>
+          <t>0.3911 (0.0681)</t>
         </is>
       </c>
     </row>
@@ -11517,7 +11533,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
@@ -11526,17 +11542,17 @@
         </is>
       </c>
       <c r="E310" t="n">
-        <v>0.2</v>
+        <v>0.1724137931034483</v>
       </c>
       <c r="F310" t="n">
-        <v>0.2571428571428571</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="G310" t="n">
-        <v>0.253968253968254</v>
+        <v>0.3384615384615385</v>
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>0.2370 (0.0321)</t>
+          <t>0.2572 (0.0831)</t>
         </is>
       </c>
     </row>
@@ -11553,7 +11569,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
@@ -11562,17 +11578,17 @@
         </is>
       </c>
       <c r="E311" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F311" t="n">
-        <v>0.4395604395604396</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="G311" t="n">
-        <v>0.4594594594594595</v>
+        <v>0.3611111111111111</v>
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>0.4493 (0.0100)</t>
+          <t>0.3582 (0.0530)</t>
         </is>
       </c>
     </row>
@@ -11589,7 +11605,7 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
@@ -11598,17 +11614,17 @@
         </is>
       </c>
       <c r="E312" t="n">
-        <v>0.1153846153846154</v>
+        <v>0.2</v>
       </c>
       <c r="F312" t="n">
-        <v>0.125</v>
+        <v>0.2571428571428571</v>
       </c>
       <c r="G312" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.253968253968254</v>
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>0.1771 (0.0987)</t>
+          <t>0.2370 (0.0321)</t>
         </is>
       </c>
     </row>
@@ -11620,31 +11636,31 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E313" t="n">
-        <v>0.2253521126760563</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F313" t="n">
-        <v>0.3188405797101449</v>
+        <v>0.4395604395604396</v>
       </c>
       <c r="G313" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.4594594594594595</v>
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>0.3203 (0.0957)</t>
+          <t>0.4493 (0.0100)</t>
         </is>
       </c>
     </row>
@@ -11656,31 +11672,31 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E314" t="n">
-        <v>0.3296703296703297</v>
+        <v>0.1153846153846154</v>
       </c>
       <c r="F314" t="n">
-        <v>0.4871794871794872</v>
+        <v>0.125</v>
       </c>
       <c r="G314" t="n">
-        <v>0.4137931034482759</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>0.4102 (0.0788)</t>
+          <t>0.1771 (0.0987)</t>
         </is>
       </c>
     </row>
@@ -11697,7 +11713,7 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -11706,17 +11722,17 @@
         </is>
       </c>
       <c r="E315" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.2253521126760563</v>
       </c>
       <c r="F315" t="n">
-        <v>0.3544303797468354</v>
+        <v>0.3188405797101449</v>
       </c>
       <c r="G315" t="n">
-        <v>0.3188405797101449</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>0.3342 (0.0183)</t>
+          <t>0.3203 (0.0957)</t>
         </is>
       </c>
     </row>
@@ -11733,7 +11749,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
@@ -11742,17 +11758,17 @@
         </is>
       </c>
       <c r="E316" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.3296703296703297</v>
       </c>
       <c r="F316" t="n">
-        <v>0.358974358974359</v>
+        <v>0.4871794871794872</v>
       </c>
       <c r="G316" t="n">
-        <v>0.4810126582278481</v>
+        <v>0.4137931034482759</v>
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>0.3949 (0.0749)</t>
+          <t>0.4102 (0.0788)</t>
         </is>
       </c>
     </row>
@@ -11769,24 +11785,96 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E317" t="n">
+        <v>0.3294117647058823</v>
+      </c>
+      <c r="F317" t="n">
+        <v>0.3544303797468354</v>
+      </c>
+      <c r="G317" t="n">
+        <v>0.3188405797101449</v>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>0.3342 (0.0183)</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E318" t="n">
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="F318" t="n">
+        <v>0.358974358974359</v>
+      </c>
+      <c r="G318" t="n">
+        <v>0.4810126582278481</v>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>0.3949 (0.0749)</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D317" t="inlineStr">
+      <c r="D319" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E317" t="n">
+      <c r="E319" t="n">
         <v>0.2777777777777778</v>
       </c>
-      <c r="F317" t="n">
+      <c r="F319" t="n">
         <v>0.360655737704918</v>
       </c>
-      <c r="G317" t="n">
+      <c r="G319" t="n">
         <v>0.3448275862068966</v>
       </c>
-      <c r="H317" t="inlineStr">
+      <c r="H319" t="inlineStr">
         <is>
           <t>0.3278 (0.0440)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 05:31:24)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H319"/>
+  <dimension ref="A1:H320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8784,11 +8784,13 @@
       <c r="E233" t="n">
         <v>0.3174603174603174</v>
       </c>
-      <c r="F233" t="inlineStr"/>
+      <c r="F233" t="n">
+        <v>0.35</v>
+      </c>
       <c r="G233" t="inlineStr"/>
       <c r="H233" t="inlineStr">
         <is>
-          <t>0.3175 (0.0000)</t>
+          <t>0.3337 (0.0230)</t>
         </is>
       </c>
     </row>
@@ -8836,31 +8838,29 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E235" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.367816091954023</v>
       </c>
       <c r="F235" t="n">
-        <v>0.2307692307692308</v>
-      </c>
-      <c r="G235" t="n">
-        <v>0.3870967741935484</v>
-      </c>
+        <v>0.3421052631578947</v>
+      </c>
+      <c r="G235" t="inlineStr"/>
       <c r="H235" t="inlineStr">
         <is>
-          <t>0.2337 (0.1519)</t>
+          <t>0.3550 (0.0182)</t>
         </is>
       </c>
     </row>
@@ -8877,7 +8877,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -8886,17 +8886,17 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F236" t="n">
-        <v>0.48</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G236" t="n">
         <v>0.3870967741935484</v>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>0.3681 (0.1225)</t>
+          <t>0.2337 (0.1519)</t>
         </is>
       </c>
     </row>
@@ -8913,7 +8913,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -8922,17 +8922,17 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>0.3</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="F237" t="n">
-        <v>0.3714285714285714</v>
+        <v>0.48</v>
       </c>
       <c r="G237" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>0.3029 (0.0671)</t>
+          <t>0.3681 (0.1225)</t>
         </is>
       </c>
     </row>
@@ -8949,7 +8949,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -8958,17 +8958,17 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>0.4848484848484849</v>
+        <v>0.3</v>
       </c>
       <c r="F238" t="n">
-        <v>0.5151515151515151</v>
+        <v>0.3714285714285714</v>
       </c>
       <c r="G238" t="n">
-        <v>0.4</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>0.4667 (0.0597)</t>
+          <t>0.3029 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -8985,7 +8985,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -8994,17 +8994,17 @@
         </is>
       </c>
       <c r="E239" t="n">
-        <v>0.0975609756097561</v>
+        <v>0.4848484848484849</v>
       </c>
       <c r="F239" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.5151515151515151</v>
       </c>
       <c r="G239" t="n">
-        <v>0.3214285714285715</v>
+        <v>0.4</v>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>0.2166 (0.1126)</t>
+          <t>0.4667 (0.0597)</t>
         </is>
       </c>
     </row>
@@ -9016,31 +9016,31 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E240" t="n">
+        <v>0.0975609756097561</v>
+      </c>
+      <c r="F240" t="n">
         <v>0.2307692307692308</v>
       </c>
-      <c r="F240" t="n">
-        <v>0.4761904761904762</v>
-      </c>
       <c r="G240" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.3214285714285715</v>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>0.3785 (0.1301)</t>
+          <t>0.2166 (0.1126)</t>
         </is>
       </c>
     </row>
@@ -9057,7 +9057,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -9066,17 +9066,17 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>0.3116883116883117</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="F241" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="G241" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>0.3581 (0.0492)</t>
+          <t>0.3785 (0.1301)</t>
         </is>
       </c>
     </row>
@@ -9093,7 +9093,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -9102,17 +9102,17 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>0.3050847457627119</v>
+        <v>0.3116883116883117</v>
       </c>
       <c r="F242" t="n">
-        <v>0.3278688524590164</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="G242" t="n">
-        <v>0.3050847457627119</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>0.3127 (0.0132)</t>
+          <t>0.3581 (0.0492)</t>
         </is>
       </c>
     </row>
@@ -9129,7 +9129,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -9138,17 +9138,17 @@
         </is>
       </c>
       <c r="E243" t="n">
-        <v>0.3666666666666666</v>
+        <v>0.3050847457627119</v>
       </c>
       <c r="F243" t="n">
-        <v>0.5161290322580645</v>
+        <v>0.3278688524590164</v>
       </c>
       <c r="G243" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3050847457627119</v>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>0.4119 (0.0905)</t>
+          <t>0.3127 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -9174,53 +9174,53 @@
         </is>
       </c>
       <c r="E244" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.3666666666666666</v>
       </c>
       <c r="F244" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.5161290322580645</v>
       </c>
       <c r="G244" t="n">
-        <v>0.3934426229508197</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>0.2512 (0.1521)</t>
+          <t>0.4119 (0.0905)</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E245" t="n">
-        <v>0.3106796116504854</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="F245" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="G245" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.3934426229508197</v>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>0.3618 (0.0444)</t>
+          <t>0.2512 (0.1521)</t>
         </is>
       </c>
     </row>
@@ -9237,7 +9237,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -9246,17 +9246,17 @@
         </is>
       </c>
       <c r="E246" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3106796116504854</v>
       </c>
       <c r="F246" t="n">
-        <v>0.3863636363636364</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G246" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>0.3811 (0.0259)</t>
+          <t>0.3618 (0.0444)</t>
         </is>
       </c>
     </row>
@@ -9273,7 +9273,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -9282,17 +9282,17 @@
         </is>
       </c>
       <c r="E247" t="n">
-        <v>0.2365591397849462</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F247" t="n">
-        <v>0.275</v>
+        <v>0.3863636363636364</v>
       </c>
       <c r="G247" t="n">
-        <v>0.3595505617977528</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>0.2904 (0.0629)</t>
+          <t>0.3811 (0.0259)</t>
         </is>
       </c>
     </row>
@@ -9309,7 +9309,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -9318,17 +9318,17 @@
         </is>
       </c>
       <c r="E248" t="n">
-        <v>0.4912280701754386</v>
+        <v>0.2365591397849462</v>
       </c>
       <c r="F248" t="n">
-        <v>0.345679012345679</v>
+        <v>0.275</v>
       </c>
       <c r="G248" t="n">
-        <v>0.459016393442623</v>
+        <v>0.3595505617977528</v>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>0.4320 (0.0764)</t>
+          <t>0.2904 (0.0629)</t>
         </is>
       </c>
     </row>
@@ -9345,7 +9345,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -9354,17 +9354,17 @@
         </is>
       </c>
       <c r="E249" t="n">
-        <v>0.24</v>
+        <v>0.4912280701754386</v>
       </c>
       <c r="F249" t="n">
-        <v>0.25</v>
+        <v>0.345679012345679</v>
       </c>
       <c r="G249" t="n">
-        <v>0.4466019417475728</v>
+        <v>0.459016393442623</v>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>0.3122 (0.1165)</t>
+          <t>0.4320 (0.0764)</t>
         </is>
       </c>
     </row>
@@ -9376,31 +9376,31 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E250" t="n">
-        <v>0.367816091954023</v>
+        <v>0.24</v>
       </c>
       <c r="F250" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.25</v>
       </c>
       <c r="G250" t="n">
-        <v>0.3953488372093023</v>
+        <v>0.4466019417475728</v>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>0.3826 (0.0139)</t>
+          <t>0.3122 (0.1165)</t>
         </is>
       </c>
     </row>
@@ -9417,7 +9417,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -9426,17 +9426,17 @@
         </is>
       </c>
       <c r="E251" t="n">
-        <v>0.3260869565217391</v>
+        <v>0.367816091954023</v>
       </c>
       <c r="F251" t="n">
-        <v>0.4086021505376344</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G251" t="n">
-        <v>0.449438202247191</v>
+        <v>0.3953488372093023</v>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>0.3947 (0.0628)</t>
+          <t>0.3826 (0.0139)</t>
         </is>
       </c>
     </row>
@@ -9453,7 +9453,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -9462,17 +9462,17 @@
         </is>
       </c>
       <c r="E252" t="n">
-        <v>0.247191011235955</v>
+        <v>0.3260869565217391</v>
       </c>
       <c r="F252" t="n">
-        <v>0.3376623376623377</v>
+        <v>0.4086021505376344</v>
       </c>
       <c r="G252" t="n">
-        <v>0.2716049382716049</v>
+        <v>0.449438202247191</v>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>0.2855 (0.0468)</t>
+          <t>0.3947 (0.0628)</t>
         </is>
       </c>
     </row>
@@ -9489,7 +9489,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -9498,17 +9498,17 @@
         </is>
       </c>
       <c r="E253" t="n">
-        <v>0.5045045045045045</v>
+        <v>0.247191011235955</v>
       </c>
       <c r="F253" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.3376623376623377</v>
       </c>
       <c r="G253" t="n">
-        <v>0.4554455445544555</v>
+        <v>0.2716049382716049</v>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>0.4599 (0.0426)</t>
+          <t>0.2855 (0.0468)</t>
         </is>
       </c>
     </row>
@@ -9525,7 +9525,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -9534,17 +9534,17 @@
         </is>
       </c>
       <c r="E254" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.5045045045045045</v>
       </c>
       <c r="F254" t="n">
-        <v>0.3235294117647059</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G254" t="n">
-        <v>0.48</v>
+        <v>0.4554455445544555</v>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>0.3691 (0.0965)</t>
+          <t>0.4599 (0.0426)</t>
         </is>
       </c>
     </row>
@@ -9556,31 +9556,31 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E255" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F255" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.3235294117647059</v>
       </c>
       <c r="G255" t="n">
-        <v>0.3655913978494624</v>
+        <v>0.48</v>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>0.3654 (0.0124)</t>
+          <t>0.3691 (0.0965)</t>
         </is>
       </c>
     </row>
@@ -9597,7 +9597,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -9606,17 +9606,17 @@
         </is>
       </c>
       <c r="E256" t="n">
-        <v>0.4</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F256" t="n">
-        <v>0.4885496183206107</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G256" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.3655913978494624</v>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>0.4443 (0.0443)</t>
+          <t>0.3654 (0.0124)</t>
         </is>
       </c>
     </row>
@@ -9633,7 +9633,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -9642,17 +9642,17 @@
         </is>
       </c>
       <c r="E257" t="n">
-        <v>0.3963963963963964</v>
+        <v>0.4</v>
       </c>
       <c r="F257" t="n">
-        <v>0.2823529411764706</v>
+        <v>0.4885496183206107</v>
       </c>
       <c r="G257" t="n">
-        <v>0.3505154639175257</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>0.3431 (0.0574)</t>
+          <t>0.4443 (0.0443)</t>
         </is>
       </c>
     </row>
@@ -9669,7 +9669,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -9678,17 +9678,17 @@
         </is>
       </c>
       <c r="E258" t="n">
-        <v>0.4905660377358491</v>
+        <v>0.3963963963963964</v>
       </c>
       <c r="F258" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.2823529411764706</v>
       </c>
       <c r="G258" t="n">
-        <v>0.4888888888888889</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>0.4524 (0.0646)</t>
+          <t>0.3431 (0.0574)</t>
         </is>
       </c>
     </row>
@@ -9705,7 +9705,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -9714,17 +9714,17 @@
         </is>
       </c>
       <c r="E259" t="n">
-        <v>0.3423423423423423</v>
+        <v>0.4905660377358491</v>
       </c>
       <c r="F259" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G259" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.4888888888888889</v>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>0.3306 (0.0403)</t>
+          <t>0.4524 (0.0646)</t>
         </is>
       </c>
     </row>
@@ -9736,31 +9736,31 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E260" t="n">
-        <v>0.4369747899159664</v>
+        <v>0.3423423423423423</v>
       </c>
       <c r="F260" t="n">
-        <v>0.3013698630136986</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G260" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>0.3850 (0.0731)</t>
+          <t>0.3306 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -9777,7 +9777,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -9786,17 +9786,17 @@
         </is>
       </c>
       <c r="E261" t="n">
-        <v>0.3505154639175257</v>
+        <v>0.4369747899159664</v>
       </c>
       <c r="F261" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.3013698630136986</v>
       </c>
       <c r="G261" t="n">
-        <v>0.4050632911392405</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>0.3819 (0.0282)</t>
+          <t>0.3850 (0.0731)</t>
         </is>
       </c>
     </row>
@@ -9813,7 +9813,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -9822,17 +9822,17 @@
         </is>
       </c>
       <c r="E262" t="n">
-        <v>0.2619047619047619</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="F262" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="G262" t="n">
-        <v>0.2318840579710145</v>
+        <v>0.4050632911392405</v>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>0.2501 (0.0160)</t>
+          <t>0.3819 (0.0282)</t>
         </is>
       </c>
     </row>
@@ -9849,7 +9849,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -9858,17 +9858,17 @@
         </is>
       </c>
       <c r="E263" t="n">
-        <v>0.5546218487394958</v>
+        <v>0.2619047619047619</v>
       </c>
       <c r="F263" t="n">
-        <v>0.5217391304347826</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="G263" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.2318840579710145</v>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>0.5084 (0.0541)</t>
+          <t>0.2501 (0.0160)</t>
         </is>
       </c>
     </row>
@@ -9885,7 +9885,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -9894,17 +9894,17 @@
         </is>
       </c>
       <c r="E264" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.5546218487394958</v>
       </c>
       <c r="F264" t="n">
-        <v>0.1875</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="G264" t="n">
-        <v>0.32</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>0.2136 (0.0960)</t>
+          <t>0.5084 (0.0541)</t>
         </is>
       </c>
     </row>
@@ -9916,31 +9916,31 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E265" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="F265" t="n">
-        <v>0.4155844155844156</v>
+        <v>0.1875</v>
       </c>
       <c r="G265" t="n">
-        <v>0.4470588235294118</v>
+        <v>0.32</v>
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>0.4372 (0.0188)</t>
+          <t>0.2136 (0.0960)</t>
         </is>
       </c>
     </row>
@@ -9957,7 +9957,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -9966,17 +9966,17 @@
         </is>
       </c>
       <c r="E266" t="n">
-        <v>0.4117647058823529</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F266" t="n">
-        <v>0.3958333333333333</v>
+        <v>0.4155844155844156</v>
       </c>
       <c r="G266" t="n">
-        <v>0.4044943820224719</v>
+        <v>0.4470588235294118</v>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>0.4040 (0.0080)</t>
+          <t>0.4372 (0.0188)</t>
         </is>
       </c>
     </row>
@@ -9993,7 +9993,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -10002,17 +10002,17 @@
         </is>
       </c>
       <c r="E267" t="n">
-        <v>0.2888888888888889</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="F267" t="n">
-        <v>0.2077922077922078</v>
+        <v>0.3958333333333333</v>
       </c>
       <c r="G267" t="n">
-        <v>0.3908045977011494</v>
+        <v>0.4044943820224719</v>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>0.2958 (0.0917)</t>
+          <t>0.4040 (0.0080)</t>
         </is>
       </c>
     </row>
@@ -10029,7 +10029,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -10038,17 +10038,17 @@
         </is>
       </c>
       <c r="E268" t="n">
-        <v>0.4835164835164835</v>
+        <v>0.2888888888888889</v>
       </c>
       <c r="F268" t="n">
-        <v>0.3950617283950617</v>
+        <v>0.2077922077922078</v>
       </c>
       <c r="G268" t="n">
-        <v>0.4946236559139785</v>
+        <v>0.3908045977011494</v>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>0.4577 (0.0546)</t>
+          <t>0.2958 (0.0917)</t>
         </is>
       </c>
     </row>
@@ -10065,7 +10065,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -10074,53 +10074,53 @@
         </is>
       </c>
       <c r="E269" t="n">
-        <v>0.1578947368421053</v>
+        <v>0.4835164835164835</v>
       </c>
       <c r="F269" t="n">
-        <v>0.2121212121212121</v>
+        <v>0.3950617283950617</v>
       </c>
       <c r="G269" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.4946236559139785</v>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>0.2706 (0.1508)</t>
+          <t>0.4577 (0.0546)</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>0.1558441558441558</v>
+        <v>0.1578947368421053</v>
       </c>
       <c r="F270" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.2121212121212121</v>
       </c>
       <c r="G270" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>0.2654 (0.1127)</t>
+          <t>0.2706 (0.1508)</t>
         </is>
       </c>
     </row>
@@ -10137,7 +10137,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -10146,17 +10146,17 @@
         </is>
       </c>
       <c r="E271" t="n">
-        <v>0.2037037037037037</v>
+        <v>0.1558441558441558</v>
       </c>
       <c r="F271" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="G271" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>0.2974 (0.0906)</t>
+          <t>0.2654 (0.1127)</t>
         </is>
       </c>
     </row>
@@ -10173,7 +10173,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -10182,17 +10182,17 @@
         </is>
       </c>
       <c r="E272" t="n">
-        <v>0.0625</v>
+        <v>0.2037037037037037</v>
       </c>
       <c r="F272" t="n">
-        <v>0.2898550724637681</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G272" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>0.2110 (0.1287)</t>
+          <t>0.2974 (0.0906)</t>
         </is>
       </c>
     </row>
@@ -10209,7 +10209,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -10218,17 +10218,17 @@
         </is>
       </c>
       <c r="E273" t="n">
-        <v>0.2769230769230769</v>
+        <v>0.0625</v>
       </c>
       <c r="F273" t="n">
-        <v>0.3661971830985916</v>
+        <v>0.2898550724637681</v>
       </c>
       <c r="G273" t="n">
-        <v>0.208955223880597</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>0.2840 (0.0789)</t>
+          <t>0.2110 (0.1287)</t>
         </is>
       </c>
     </row>
@@ -10245,7 +10245,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -10254,17 +10254,17 @@
         </is>
       </c>
       <c r="E274" t="n">
-        <v>0.1212121212121212</v>
+        <v>0.2769230769230769</v>
       </c>
       <c r="F274" t="n">
-        <v>0.2424242424242424</v>
+        <v>0.3661971830985916</v>
       </c>
       <c r="G274" t="n">
-        <v>0.2432432432432433</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>0.2023 (0.0702)</t>
+          <t>0.2840 (0.0789)</t>
         </is>
       </c>
     </row>
@@ -10276,31 +10276,31 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>0.2325581395348837</v>
+        <v>0.1212121212121212</v>
       </c>
       <c r="F275" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2424242424242424</v>
       </c>
       <c r="G275" t="n">
-        <v>0.2553191489361702</v>
+        <v>0.2432432432432433</v>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>0.2579 (0.0267)</t>
+          <t>0.2023 (0.0702)</t>
         </is>
       </c>
     </row>
@@ -10317,7 +10317,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -10326,17 +10326,17 @@
         </is>
       </c>
       <c r="E276" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2325581395348837</v>
       </c>
       <c r="F276" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G276" t="n">
-        <v>0.3137254901960784</v>
+        <v>0.2553191489361702</v>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>0.2751 (0.0418)</t>
+          <t>0.2579 (0.0267)</t>
         </is>
       </c>
     </row>
@@ -10353,7 +10353,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -10362,17 +10362,17 @@
         </is>
       </c>
       <c r="E277" t="n">
-        <v>0.08</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="F277" t="n">
-        <v>0.1176470588235294</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="G277" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.3137254901960784</v>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>0.1528 (0.0954)</t>
+          <t>0.2751 (0.0418)</t>
         </is>
       </c>
     </row>
@@ -10389,7 +10389,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -10398,17 +10398,17 @@
         </is>
       </c>
       <c r="E278" t="n">
-        <v>0.28125</v>
+        <v>0.08</v>
       </c>
       <c r="F278" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.1176470588235294</v>
       </c>
       <c r="G278" t="n">
-        <v>0.2181818181818182</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>0.2814 (0.0633)</t>
+          <t>0.1528 (0.0954)</t>
         </is>
       </c>
     </row>
@@ -10425,7 +10425,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -10434,17 +10434,17 @@
         </is>
       </c>
       <c r="E279" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.28125</v>
       </c>
       <c r="F279" t="n">
-        <v>0.1621621621621622</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="G279" t="n">
-        <v>0.2790697674418605</v>
+        <v>0.2181818181818182</v>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>0.1831 (0.0874)</t>
+          <t>0.2814 (0.0633)</t>
         </is>
       </c>
     </row>
@@ -10456,31 +10456,31 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>0.1754385964912281</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="F280" t="n">
-        <v>0.34375</v>
+        <v>0.1621621621621622</v>
       </c>
       <c r="G280" t="n">
-        <v>0.3508771929824561</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>0.2900 (0.0993)</t>
+          <t>0.1831 (0.0874)</t>
         </is>
       </c>
     </row>
@@ -10497,7 +10497,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -10506,17 +10506,17 @@
         </is>
       </c>
       <c r="E281" t="n">
-        <v>0.1839080459770115</v>
+        <v>0.1754385964912281</v>
       </c>
       <c r="F281" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.34375</v>
       </c>
       <c r="G281" t="n">
-        <v>0.2702702702702703</v>
+        <v>0.3508771929824561</v>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>0.2690 (0.0845)</t>
+          <t>0.2900 (0.0993)</t>
         </is>
       </c>
     </row>
@@ -10533,7 +10533,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -10542,17 +10542,17 @@
         </is>
       </c>
       <c r="E282" t="n">
-        <v>0.09230769230769231</v>
+        <v>0.1839080459770115</v>
       </c>
       <c r="F282" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="G282" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.2702702702702703</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>0.1654 (0.0725)</t>
+          <t>0.2690 (0.0845)</t>
         </is>
       </c>
     </row>
@@ -10569,7 +10569,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -10578,17 +10578,17 @@
         </is>
       </c>
       <c r="E283" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.09230769230769231</v>
       </c>
       <c r="F283" t="n">
-        <v>0.4307692307692308</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="G283" t="n">
-        <v>0.3076923076923077</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>0.3342 (0.0864)</t>
+          <t>0.1654 (0.0725)</t>
         </is>
       </c>
     </row>
@@ -10605,7 +10605,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -10614,17 +10614,17 @@
         </is>
       </c>
       <c r="E284" t="n">
-        <v>0.1639344262295082</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F284" t="n">
-        <v>0.2962962962962963</v>
+        <v>0.4307692307692308</v>
       </c>
       <c r="G284" t="n">
-        <v>0.2295081967213115</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>0.2299 (0.0662)</t>
+          <t>0.3342 (0.0864)</t>
         </is>
       </c>
     </row>
@@ -10636,31 +10636,31 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>0.1777777777777778</v>
+        <v>0.1639344262295082</v>
       </c>
       <c r="F285" t="n">
-        <v>0.2272727272727273</v>
+        <v>0.2962962962962963</v>
       </c>
       <c r="G285" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.2295081967213115</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>0.2205 (0.0398)</t>
+          <t>0.2299 (0.0662)</t>
         </is>
       </c>
     </row>
@@ -10677,7 +10677,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -10686,17 +10686,17 @@
         </is>
       </c>
       <c r="E286" t="n">
-        <v>0.2790697674418605</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="F286" t="n">
-        <v>0.3859649122807017</v>
+        <v>0.2272727272727273</v>
       </c>
       <c r="G286" t="n">
-        <v>0.3673469387755102</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>0.3441 (0.0571)</t>
+          <t>0.2205 (0.0398)</t>
         </is>
       </c>
     </row>
@@ -10713,7 +10713,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -10722,17 +10722,17 @@
         </is>
       </c>
       <c r="E287" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="F287" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3859649122807017</v>
       </c>
       <c r="G287" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3673469387755102</v>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>0.1530 (0.0500)</t>
+          <t>0.3441 (0.0571)</t>
         </is>
       </c>
     </row>
@@ -10749,7 +10749,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -10758,17 +10758,17 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="F288" t="n">
-        <v>0.4</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G288" t="n">
-        <v>0.3571428571428572</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>0.3226 (0.0994)</t>
+          <t>0.1530 (0.0500)</t>
         </is>
       </c>
     </row>
@@ -10785,7 +10785,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -10794,17 +10794,17 @@
         </is>
       </c>
       <c r="E289" t="n">
-        <v>0.0975609756097561</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="F289" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.4</v>
       </c>
       <c r="G289" t="n">
-        <v>0.25</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>0.1462 (0.0900)</t>
+          <t>0.3226 (0.0994)</t>
         </is>
       </c>
     </row>
@@ -10816,31 +10816,31 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>0.2380952380952381</v>
+        <v>0.0975609756097561</v>
       </c>
       <c r="F290" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="G290" t="n">
-        <v>0.3478260869565217</v>
+        <v>0.25</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>0.2429 (0.1026)</t>
+          <t>0.1462 (0.0900)</t>
         </is>
       </c>
     </row>
@@ -10857,7 +10857,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -10866,17 +10866,17 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>0.24</v>
+        <v>0.2380952380952381</v>
       </c>
       <c r="F291" t="n">
-        <v>0.303030303030303</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="G291" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.3478260869565217</v>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>0.2708 (0.0315)</t>
+          <t>0.2429 (0.1026)</t>
         </is>
       </c>
     </row>
@@ -10893,7 +10893,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
@@ -10902,17 +10902,17 @@
         </is>
       </c>
       <c r="E292" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.24</v>
       </c>
       <c r="F292" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G292" t="n">
-        <v>0.2173913043478261</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>0.1515 (0.0671)</t>
+          <t>0.2708 (0.0315)</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10929,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
@@ -10938,17 +10938,17 @@
         </is>
       </c>
       <c r="E293" t="n">
-        <v>0.25</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F293" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="G293" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>0.2998 (0.0581)</t>
+          <t>0.1515 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -10965,7 +10965,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -10977,50 +10977,50 @@
         <v>0.25</v>
       </c>
       <c r="F294" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="G294" t="n">
         <v>0.2857142857142857</v>
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>0.2146 (0.0939)</t>
+          <t>0.2998 (0.0581)</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>0.2391304347826087</v>
+        <v>0.25</v>
       </c>
       <c r="F295" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="G295" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>0.3070 (0.0589)</t>
+          <t>0.2146 (0.0939)</t>
         </is>
       </c>
     </row>
@@ -11037,7 +11037,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -11046,17 +11046,17 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>0.3168316831683168</v>
+        <v>0.2391304347826087</v>
       </c>
       <c r="F296" t="n">
-        <v>0.3454545454545455</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="G296" t="n">
-        <v>0.3793103448275862</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>0.3472 (0.0313)</t>
+          <t>0.3070 (0.0589)</t>
         </is>
       </c>
     </row>
@@ -11073,7 +11073,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
@@ -11082,17 +11082,17 @@
         </is>
       </c>
       <c r="E297" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.3168316831683168</v>
       </c>
       <c r="F297" t="n">
-        <v>0.4303797468354431</v>
+        <v>0.3454545454545455</v>
       </c>
       <c r="G297" t="n">
-        <v>0.3820224719101123</v>
+        <v>0.3793103448275862</v>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>0.4054 (0.0242)</t>
+          <t>0.3472 (0.0313)</t>
         </is>
       </c>
     </row>
@@ -11109,7 +11109,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
@@ -11118,17 +11118,17 @@
         </is>
       </c>
       <c r="E298" t="n">
-        <v>0.4036697247706422</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="F298" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.4303797468354431</v>
       </c>
       <c r="G298" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.3820224719101123</v>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>0.4326 (0.0256)</t>
+          <t>0.4054 (0.0242)</t>
         </is>
       </c>
     </row>
@@ -11145,7 +11145,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
@@ -11154,17 +11154,17 @@
         </is>
       </c>
       <c r="E299" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.4036697247706422</v>
       </c>
       <c r="F299" t="n">
-        <v>0.2117647058823529</v>
+        <v>0.4523809523809524</v>
       </c>
       <c r="G299" t="n">
-        <v>0.2921348314606741</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>0.2538 (0.0403)</t>
+          <t>0.4326 (0.0256)</t>
         </is>
       </c>
     </row>
@@ -11176,29 +11176,31 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>0.2285714285714286</v>
+        <v>0.2574257425742574</v>
       </c>
       <c r="F300" t="n">
-        <v>0.3142857142857143</v>
-      </c>
-      <c r="G300" t="inlineStr"/>
+        <v>0.2117647058823529</v>
+      </c>
+      <c r="G300" t="n">
+        <v>0.2921348314606741</v>
+      </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>0.2714 (0.0606)</t>
+          <t>0.2538 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -11215,7 +11217,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
@@ -11224,17 +11226,15 @@
         </is>
       </c>
       <c r="E301" t="n">
-        <v>0.3023255813953488</v>
+        <v>0.2285714285714286</v>
       </c>
       <c r="F301" t="n">
-        <v>0.4197530864197531</v>
-      </c>
-      <c r="G301" t="n">
-        <v>0.3809523809523809</v>
-      </c>
+        <v>0.3142857142857143</v>
+      </c>
+      <c r="G301" t="inlineStr"/>
       <c r="H301" t="inlineStr">
         <is>
-          <t>0.3677 (0.0598)</t>
+          <t>0.2714 (0.0606)</t>
         </is>
       </c>
     </row>
@@ -11251,7 +11251,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
@@ -11260,17 +11260,17 @@
         </is>
       </c>
       <c r="E302" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.3023255813953488</v>
       </c>
       <c r="F302" t="n">
-        <v>0.2597402597402597</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G302" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>0.3101 (0.0862)</t>
+          <t>0.3677 (0.0598)</t>
         </is>
       </c>
     </row>
@@ -11287,7 +11287,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
@@ -11296,15 +11296,17 @@
         </is>
       </c>
       <c r="E303" t="n">
-        <v>0.4356435643564356</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="F303" t="n">
-        <v>0.4878048780487805</v>
-      </c>
-      <c r="G303" t="inlineStr"/>
+        <v>0.2597402597402597</v>
+      </c>
+      <c r="G303" t="n">
+        <v>0.2608695652173913</v>
+      </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>0.4617 (0.0369)</t>
+          <t>0.3101 (0.0862)</t>
         </is>
       </c>
     </row>
@@ -11321,7 +11323,7 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
@@ -11330,13 +11332,17 @@
         </is>
       </c>
       <c r="E304" t="n">
-        <v>0.3235294117647059</v>
-      </c>
-      <c r="F304" t="inlineStr"/>
-      <c r="G304" t="inlineStr"/>
+        <v>0.4356435643564356</v>
+      </c>
+      <c r="F304" t="n">
+        <v>0.4878048780487805</v>
+      </c>
+      <c r="G304" t="n">
+        <v>0.4057971014492754</v>
+      </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>0.3235 (0.0000)</t>
+          <t>0.4431 (0.0415)</t>
         </is>
       </c>
     </row>
@@ -11348,31 +11354,29 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>0.2736842105263158</v>
+        <v>0.3235294117647059</v>
       </c>
       <c r="F305" t="n">
-        <v>0.3736263736263736</v>
-      </c>
-      <c r="G305" t="n">
-        <v>0.3855421686746988</v>
-      </c>
+        <v>0.1851851851851852</v>
+      </c>
+      <c r="G305" t="inlineStr"/>
       <c r="H305" t="inlineStr">
         <is>
-          <t>0.3443 (0.0614)</t>
+          <t>0.2544 (0.0978)</t>
         </is>
       </c>
     </row>
@@ -11389,7 +11393,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
@@ -11398,17 +11402,17 @@
         </is>
       </c>
       <c r="E306" t="n">
-        <v>0.3760683760683761</v>
+        <v>0.2736842105263158</v>
       </c>
       <c r="F306" t="n">
-        <v>0.46</v>
+        <v>0.3736263736263736</v>
       </c>
       <c r="G306" t="n">
-        <v>0.4081632653061225</v>
+        <v>0.3855421686746988</v>
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>0.4147 (0.0424)</t>
+          <t>0.3443 (0.0614)</t>
         </is>
       </c>
     </row>
@@ -11425,7 +11429,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
@@ -11434,17 +11438,17 @@
         </is>
       </c>
       <c r="E307" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.3760683760683761</v>
       </c>
       <c r="F307" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.46</v>
       </c>
       <c r="G307" t="n">
-        <v>0.3838383838383838</v>
+        <v>0.4081632653061225</v>
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>0.3236 (0.0634)</t>
+          <t>0.4147 (0.0424)</t>
         </is>
       </c>
     </row>
@@ -11461,7 +11465,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
@@ -11470,17 +11474,17 @@
         </is>
       </c>
       <c r="E308" t="n">
-        <v>0.4791666666666667</v>
+        <v>0.2574257425742574</v>
       </c>
       <c r="F308" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.3294117647058823</v>
       </c>
       <c r="G308" t="n">
-        <v>0.4</v>
+        <v>0.3838383838383838</v>
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>0.4359 (0.0401)</t>
+          <t>0.3236 (0.0634)</t>
         </is>
       </c>
     </row>
@@ -11497,7 +11501,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
@@ -11506,17 +11510,17 @@
         </is>
       </c>
       <c r="E309" t="n">
-        <v>0.3125</v>
+        <v>0.4791666666666667</v>
       </c>
       <c r="F309" t="n">
-        <v>0.4337349397590362</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="G309" t="n">
-        <v>0.4269662921348314</v>
+        <v>0.4</v>
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>0.3911 (0.0681)</t>
+          <t>0.4359 (0.0401)</t>
         </is>
       </c>
     </row>
@@ -11528,31 +11532,31 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E310" t="n">
-        <v>0.1724137931034483</v>
+        <v>0.3125</v>
       </c>
       <c r="F310" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.4337349397590362</v>
       </c>
       <c r="G310" t="n">
-        <v>0.3384615384615385</v>
+        <v>0.4269662921348314</v>
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>0.2572 (0.0831)</t>
+          <t>0.3911 (0.0681)</t>
         </is>
       </c>
     </row>
@@ -11569,7 +11573,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
@@ -11578,17 +11582,17 @@
         </is>
       </c>
       <c r="E311" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.1724137931034483</v>
       </c>
       <c r="F311" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="G311" t="n">
-        <v>0.3611111111111111</v>
+        <v>0.3384615384615385</v>
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>0.3582 (0.0530)</t>
+          <t>0.2572 (0.0831)</t>
         </is>
       </c>
     </row>
@@ -11605,7 +11609,7 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
@@ -11614,17 +11618,17 @@
         </is>
       </c>
       <c r="E312" t="n">
-        <v>0.2</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F312" t="n">
-        <v>0.2571428571428571</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="G312" t="n">
-        <v>0.253968253968254</v>
+        <v>0.3611111111111111</v>
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>0.2370 (0.0321)</t>
+          <t>0.3582 (0.0530)</t>
         </is>
       </c>
     </row>
@@ -11641,7 +11645,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
@@ -11650,17 +11654,17 @@
         </is>
       </c>
       <c r="E313" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.2</v>
       </c>
       <c r="F313" t="n">
-        <v>0.4395604395604396</v>
+        <v>0.2571428571428571</v>
       </c>
       <c r="G313" t="n">
-        <v>0.4594594594594595</v>
+        <v>0.253968253968254</v>
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>0.4493 (0.0100)</t>
+          <t>0.2370 (0.0321)</t>
         </is>
       </c>
     </row>
@@ -11677,7 +11681,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
@@ -11686,17 +11690,17 @@
         </is>
       </c>
       <c r="E314" t="n">
-        <v>0.1153846153846154</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F314" t="n">
-        <v>0.125</v>
+        <v>0.4395604395604396</v>
       </c>
       <c r="G314" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.4594594594594595</v>
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>0.1771 (0.0987)</t>
+          <t>0.4493 (0.0100)</t>
         </is>
       </c>
     </row>
@@ -11708,31 +11712,31 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E315" t="n">
-        <v>0.2253521126760563</v>
+        <v>0.1153846153846154</v>
       </c>
       <c r="F315" t="n">
-        <v>0.3188405797101449</v>
+        <v>0.125</v>
       </c>
       <c r="G315" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>0.3203 (0.0957)</t>
+          <t>0.1771 (0.0987)</t>
         </is>
       </c>
     </row>
@@ -11749,7 +11753,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
@@ -11758,17 +11762,17 @@
         </is>
       </c>
       <c r="E316" t="n">
-        <v>0.3296703296703297</v>
+        <v>0.2253521126760563</v>
       </c>
       <c r="F316" t="n">
-        <v>0.4871794871794872</v>
+        <v>0.3188405797101449</v>
       </c>
       <c r="G316" t="n">
-        <v>0.4137931034482759</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>0.4102 (0.0788)</t>
+          <t>0.3203 (0.0957)</t>
         </is>
       </c>
     </row>
@@ -11785,7 +11789,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
@@ -11794,17 +11798,17 @@
         </is>
       </c>
       <c r="E317" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.3296703296703297</v>
       </c>
       <c r="F317" t="n">
-        <v>0.3544303797468354</v>
+        <v>0.4871794871794872</v>
       </c>
       <c r="G317" t="n">
-        <v>0.3188405797101449</v>
+        <v>0.4137931034482759</v>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>0.3342 (0.0183)</t>
+          <t>0.4102 (0.0788)</t>
         </is>
       </c>
     </row>
@@ -11821,7 +11825,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
@@ -11830,17 +11834,17 @@
         </is>
       </c>
       <c r="E318" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.3294117647058823</v>
       </c>
       <c r="F318" t="n">
-        <v>0.358974358974359</v>
+        <v>0.3544303797468354</v>
       </c>
       <c r="G318" t="n">
-        <v>0.4810126582278481</v>
+        <v>0.3188405797101449</v>
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>0.3949 (0.0749)</t>
+          <t>0.3342 (0.0183)</t>
         </is>
       </c>
     </row>
@@ -11857,24 +11861,60 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E319" t="n">
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="F319" t="n">
+        <v>0.358974358974359</v>
+      </c>
+      <c r="G319" t="n">
+        <v>0.4810126582278481</v>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>0.3949 (0.0749)</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D319" t="inlineStr">
+      <c r="D320" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E319" t="n">
+      <c r="E320" t="n">
         <v>0.2777777777777778</v>
       </c>
-      <c r="F319" t="n">
+      <c r="F320" t="n">
         <v>0.360655737704918</v>
       </c>
-      <c r="G319" t="n">
+      <c r="G320" t="n">
         <v>0.3448275862068966</v>
       </c>
-      <c r="H319" t="inlineStr">
+      <c r="H320" t="inlineStr">
         <is>
           <t>0.3278 (0.0440)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 06:31:42)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H320"/>
+  <dimension ref="A1:H336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8737,7 +8737,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -8746,17 +8746,13 @@
         </is>
       </c>
       <c r="E232" t="n">
-        <v>0.2133333333333333</v>
-      </c>
-      <c r="F232" t="n">
-        <v>0.4418604651162791</v>
-      </c>
-      <c r="G232" t="n">
-        <v>0.3703703703703703</v>
-      </c>
+        <v>0.2264150943396226</v>
+      </c>
+      <c r="F232" t="inlineStr"/>
+      <c r="G232" t="inlineStr"/>
       <c r="H232" t="inlineStr">
         <is>
-          <t>0.3419 (0.1169)</t>
+          <t>0.2264 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -8773,7 +8769,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -8782,15 +8778,17 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>0.3174603174603174</v>
+        <v>0.2133333333333333</v>
       </c>
       <c r="F233" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="G233" t="inlineStr"/>
+        <v>0.4418604651162791</v>
+      </c>
+      <c r="G233" t="n">
+        <v>0.3703703703703703</v>
+      </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>0.3337 (0.0230)</t>
+          <t>0.3419 (0.1169)</t>
         </is>
       </c>
     </row>
@@ -8802,31 +8800,31 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E234" t="n">
-        <v>0.3364485981308411</v>
+        <v>0.3174603174603174</v>
       </c>
       <c r="F234" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.35</v>
       </c>
       <c r="G234" t="n">
-        <v>0.3764705882352941</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>0.3873 (0.0570)</t>
+          <t>0.3114 (0.0420)</t>
         </is>
       </c>
     </row>
@@ -8838,29 +8836,27 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E235" t="n">
-        <v>0.367816091954023</v>
-      </c>
-      <c r="F235" t="n">
-        <v>0.3421052631578947</v>
-      </c>
+        <v>0.4262295081967213</v>
+      </c>
+      <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr"/>
       <c r="H235" t="inlineStr">
         <is>
-          <t>0.3550 (0.0182)</t>
+          <t>0.4262 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -8872,7 +8868,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -8882,21 +8878,17 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E236" t="n">
-        <v>0.08333333333333333</v>
-      </c>
-      <c r="F236" t="n">
-        <v>0.2307692307692308</v>
-      </c>
-      <c r="G236" t="n">
-        <v>0.3870967741935484</v>
-      </c>
+        <v>0.2318840579710145</v>
+      </c>
+      <c r="F236" t="inlineStr"/>
+      <c r="G236" t="inlineStr"/>
       <c r="H236" t="inlineStr">
         <is>
-          <t>0.2337 (0.1519)</t>
+          <t>0.2319 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -8908,7 +8900,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -8918,21 +8910,21 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E237" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.3364485981308411</v>
       </c>
       <c r="F237" t="n">
-        <v>0.48</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="G237" t="n">
-        <v>0.3870967741935484</v>
+        <v>0.3764705882352941</v>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>0.3681 (0.1225)</t>
+          <t>0.3873 (0.0570)</t>
         </is>
       </c>
     </row>
@@ -8944,7 +8936,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -8954,21 +8946,21 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E238" t="n">
-        <v>0.3</v>
+        <v>0.367816091954023</v>
       </c>
       <c r="F238" t="n">
-        <v>0.3714285714285714</v>
+        <v>0.3421052631578947</v>
       </c>
       <c r="G238" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.3283582089552239</v>
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>0.3029 (0.0671)</t>
+          <t>0.3461 (0.0200)</t>
         </is>
       </c>
     </row>
@@ -8980,7 +8972,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -8990,21 +8982,17 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>0.4848484848484849</v>
-      </c>
-      <c r="F239" t="n">
-        <v>0.5151515151515151</v>
-      </c>
-      <c r="G239" t="n">
-        <v>0.4</v>
-      </c>
+        <v>0.3870967741935484</v>
+      </c>
+      <c r="F239" t="inlineStr"/>
+      <c r="G239" t="inlineStr"/>
       <c r="H239" t="inlineStr">
         <is>
-          <t>0.4667 (0.0597)</t>
+          <t>0.3871 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -9016,7 +9004,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -9026,21 +9014,17 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E240" t="n">
-        <v>0.0975609756097561</v>
-      </c>
-      <c r="F240" t="n">
-        <v>0.2307692307692308</v>
-      </c>
-      <c r="G240" t="n">
-        <v>0.3214285714285715</v>
-      </c>
+        <v>0.1904761904761905</v>
+      </c>
+      <c r="F240" t="inlineStr"/>
+      <c r="G240" t="inlineStr"/>
       <c r="H240" t="inlineStr">
         <is>
-          <t>0.2166 (0.1126)</t>
+          <t>0.1905 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -9052,7 +9036,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -9062,21 +9046,21 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E241" t="n">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="F241" t="n">
         <v>0.2307692307692308</v>
       </c>
-      <c r="F241" t="n">
-        <v>0.4761904761904762</v>
-      </c>
       <c r="G241" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>0.3785 (0.1301)</t>
+          <t>0.2337 (0.1519)</t>
         </is>
       </c>
     </row>
@@ -9088,7 +9072,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -9098,21 +9082,21 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E242" t="n">
-        <v>0.3116883116883117</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="F242" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.48</v>
       </c>
       <c r="G242" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>0.3581 (0.0492)</t>
+          <t>0.3681 (0.1225)</t>
         </is>
       </c>
     </row>
@@ -9124,7 +9108,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -9134,21 +9118,21 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E243" t="n">
-        <v>0.3050847457627119</v>
+        <v>0.3</v>
       </c>
       <c r="F243" t="n">
-        <v>0.3278688524590164</v>
+        <v>0.3714285714285714</v>
       </c>
       <c r="G243" t="n">
-        <v>0.3050847457627119</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>0.3127 (0.0132)</t>
+          <t>0.3029 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -9160,7 +9144,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -9170,21 +9154,21 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E244" t="n">
-        <v>0.3666666666666666</v>
+        <v>0.4848484848484849</v>
       </c>
       <c r="F244" t="n">
-        <v>0.5161290322580645</v>
+        <v>0.5151515151515151</v>
       </c>
       <c r="G244" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.4</v>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>0.4119 (0.0905)</t>
+          <t>0.4667 (0.0597)</t>
         </is>
       </c>
     </row>
@@ -9196,7 +9180,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -9206,33 +9190,33 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E245" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.0975609756097561</v>
       </c>
       <c r="F245" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G245" t="n">
-        <v>0.3934426229508197</v>
+        <v>0.3214285714285715</v>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>0.2512 (0.1521)</t>
+          <t>0.2166 (0.1126)</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -9242,33 +9226,33 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E246" t="n">
-        <v>0.3106796116504854</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="F246" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="G246" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>0.3618 (0.0444)</t>
+          <t>0.3785 (0.1301)</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -9278,33 +9262,33 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E247" t="n">
+        <v>0.3116883116883117</v>
+      </c>
+      <c r="F247" t="n">
+        <v>0.4096385542168675</v>
+      </c>
+      <c r="G247" t="n">
         <v>0.3529411764705883</v>
       </c>
-      <c r="F247" t="n">
-        <v>0.3863636363636364</v>
-      </c>
-      <c r="G247" t="n">
-        <v>0.4038461538461539</v>
-      </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>0.3811 (0.0259)</t>
+          <t>0.3581 (0.0492)</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -9314,33 +9298,33 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E248" t="n">
-        <v>0.2365591397849462</v>
+        <v>0.3050847457627119</v>
       </c>
       <c r="F248" t="n">
-        <v>0.275</v>
+        <v>0.3278688524590164</v>
       </c>
       <c r="G248" t="n">
-        <v>0.3595505617977528</v>
+        <v>0.3050847457627119</v>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>0.2904 (0.0629)</t>
+          <t>0.3127 (0.0132)</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -9350,33 +9334,33 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E249" t="n">
-        <v>0.4912280701754386</v>
+        <v>0.3666666666666666</v>
       </c>
       <c r="F249" t="n">
-        <v>0.345679012345679</v>
+        <v>0.5161290322580645</v>
       </c>
       <c r="G249" t="n">
-        <v>0.459016393442623</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>0.4320 (0.0764)</t>
+          <t>0.4119 (0.0905)</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -9386,21 +9370,21 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E250" t="n">
-        <v>0.24</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="F250" t="n">
-        <v>0.25</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="G250" t="n">
-        <v>0.4466019417475728</v>
+        <v>0.3934426229508197</v>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>0.3122 (0.1165)</t>
+          <t>0.2512 (0.1521)</t>
         </is>
       </c>
     </row>
@@ -9412,7 +9396,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -9422,21 +9406,21 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E251" t="n">
-        <v>0.367816091954023</v>
+        <v>0.3106796116504854</v>
       </c>
       <c r="F251" t="n">
         <v>0.3846153846153846</v>
       </c>
       <c r="G251" t="n">
-        <v>0.3953488372093023</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>0.3826 (0.0139)</t>
+          <t>0.3618 (0.0444)</t>
         </is>
       </c>
     </row>
@@ -9448,7 +9432,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -9458,21 +9442,21 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>0.3260869565217391</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F252" t="n">
-        <v>0.4086021505376344</v>
+        <v>0.3863636363636364</v>
       </c>
       <c r="G252" t="n">
-        <v>0.449438202247191</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>0.3947 (0.0628)</t>
+          <t>0.3811 (0.0259)</t>
         </is>
       </c>
     </row>
@@ -9484,7 +9468,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -9494,21 +9478,21 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E253" t="n">
-        <v>0.247191011235955</v>
+        <v>0.2365591397849462</v>
       </c>
       <c r="F253" t="n">
-        <v>0.3376623376623377</v>
+        <v>0.275</v>
       </c>
       <c r="G253" t="n">
-        <v>0.2716049382716049</v>
+        <v>0.3595505617977528</v>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>0.2855 (0.0468)</t>
+          <t>0.2904 (0.0629)</t>
         </is>
       </c>
     </row>
@@ -9520,7 +9504,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -9530,21 +9514,21 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>0.5045045045045045</v>
+        <v>0.4912280701754386</v>
       </c>
       <c r="F254" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.345679012345679</v>
       </c>
       <c r="G254" t="n">
-        <v>0.4554455445544555</v>
+        <v>0.459016393442623</v>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>0.4599 (0.0426)</t>
+          <t>0.4320 (0.0764)</t>
         </is>
       </c>
     </row>
@@ -9556,7 +9540,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -9566,21 +9550,21 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E255" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.24</v>
       </c>
       <c r="F255" t="n">
-        <v>0.3235294117647059</v>
+        <v>0.25</v>
       </c>
       <c r="G255" t="n">
-        <v>0.48</v>
+        <v>0.4466019417475728</v>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>0.3691 (0.0965)</t>
+          <t>0.3122 (0.1165)</t>
         </is>
       </c>
     </row>
@@ -9592,7 +9576,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -9602,21 +9586,21 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.367816091954023</v>
       </c>
       <c r="F256" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G256" t="n">
-        <v>0.3655913978494624</v>
+        <v>0.3953488372093023</v>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>0.3654 (0.0124)</t>
+          <t>0.3826 (0.0139)</t>
         </is>
       </c>
     </row>
@@ -9628,7 +9612,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -9638,21 +9622,21 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E257" t="n">
-        <v>0.4</v>
+        <v>0.3260869565217391</v>
       </c>
       <c r="F257" t="n">
-        <v>0.4885496183206107</v>
+        <v>0.4086021505376344</v>
       </c>
       <c r="G257" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.449438202247191</v>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>0.4443 (0.0443)</t>
+          <t>0.3947 (0.0628)</t>
         </is>
       </c>
     </row>
@@ -9664,7 +9648,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -9674,21 +9658,21 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E258" t="n">
-        <v>0.3963963963963964</v>
+        <v>0.247191011235955</v>
       </c>
       <c r="F258" t="n">
-        <v>0.2823529411764706</v>
+        <v>0.3376623376623377</v>
       </c>
       <c r="G258" t="n">
-        <v>0.3505154639175257</v>
+        <v>0.2716049382716049</v>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>0.3431 (0.0574)</t>
+          <t>0.2855 (0.0468)</t>
         </is>
       </c>
     </row>
@@ -9700,7 +9684,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -9710,21 +9694,21 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>0.4905660377358491</v>
+        <v>0.5045045045045045</v>
       </c>
       <c r="F259" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G259" t="n">
-        <v>0.4888888888888889</v>
+        <v>0.4554455445544555</v>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>0.4524 (0.0646)</t>
+          <t>0.4599 (0.0426)</t>
         </is>
       </c>
     </row>
@@ -9736,7 +9720,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -9746,21 +9730,21 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E260" t="n">
-        <v>0.3423423423423423</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F260" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3235294117647059</v>
       </c>
       <c r="G260" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.48</v>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>0.3306 (0.0403)</t>
+          <t>0.3691 (0.0965)</t>
         </is>
       </c>
     </row>
@@ -9772,7 +9756,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -9782,21 +9766,21 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E261" t="n">
-        <v>0.4369747899159664</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F261" t="n">
-        <v>0.3013698630136986</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G261" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.3655913978494624</v>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>0.3850 (0.0731)</t>
+          <t>0.3654 (0.0124)</t>
         </is>
       </c>
     </row>
@@ -9808,7 +9792,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -9818,21 +9802,21 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E262" t="n">
-        <v>0.3505154639175257</v>
+        <v>0.4</v>
       </c>
       <c r="F262" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.4885496183206107</v>
       </c>
       <c r="G262" t="n">
-        <v>0.4050632911392405</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>0.3819 (0.0282)</t>
+          <t>0.4443 (0.0443)</t>
         </is>
       </c>
     </row>
@@ -9844,7 +9828,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -9854,21 +9838,21 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E263" t="n">
-        <v>0.2619047619047619</v>
+        <v>0.3963963963963964</v>
       </c>
       <c r="F263" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.2823529411764706</v>
       </c>
       <c r="G263" t="n">
-        <v>0.2318840579710145</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>0.2501 (0.0160)</t>
+          <t>0.3431 (0.0574)</t>
         </is>
       </c>
     </row>
@@ -9880,7 +9864,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -9890,21 +9874,21 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E264" t="n">
-        <v>0.5546218487394958</v>
+        <v>0.4905660377358491</v>
       </c>
       <c r="F264" t="n">
-        <v>0.5217391304347826</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G264" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.4888888888888889</v>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>0.5084 (0.0541)</t>
+          <t>0.4524 (0.0646)</t>
         </is>
       </c>
     </row>
@@ -9916,7 +9900,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -9926,21 +9910,21 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E265" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.3423423423423423</v>
       </c>
       <c r="F265" t="n">
-        <v>0.1875</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G265" t="n">
-        <v>0.32</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>0.2136 (0.0960)</t>
+          <t>0.3306 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -9952,7 +9936,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -9962,21 +9946,21 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E266" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.4369747899159664</v>
       </c>
       <c r="F266" t="n">
-        <v>0.4155844155844156</v>
+        <v>0.3013698630136986</v>
       </c>
       <c r="G266" t="n">
-        <v>0.4470588235294118</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>0.4372 (0.0188)</t>
+          <t>0.3850 (0.0731)</t>
         </is>
       </c>
     </row>
@@ -9988,7 +9972,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -9998,21 +9982,21 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>0.4117647058823529</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="F267" t="n">
-        <v>0.3958333333333333</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="G267" t="n">
-        <v>0.4044943820224719</v>
+        <v>0.4050632911392405</v>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>0.4040 (0.0080)</t>
+          <t>0.3819 (0.0282)</t>
         </is>
       </c>
     </row>
@@ -10024,7 +10008,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -10034,21 +10018,21 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>0.2888888888888889</v>
+        <v>0.2619047619047619</v>
       </c>
       <c r="F268" t="n">
-        <v>0.2077922077922078</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="G268" t="n">
-        <v>0.3908045977011494</v>
+        <v>0.2318840579710145</v>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>0.2958 (0.0917)</t>
+          <t>0.2501 (0.0160)</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10044,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -10070,21 +10054,21 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>0.4835164835164835</v>
+        <v>0.5546218487394958</v>
       </c>
       <c r="F269" t="n">
-        <v>0.3950617283950617</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="G269" t="n">
-        <v>0.4946236559139785</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>0.4577 (0.0546)</t>
+          <t>0.5084 (0.0541)</t>
         </is>
       </c>
     </row>
@@ -10096,7 +10080,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -10106,33 +10090,33 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>0.1578947368421053</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="F270" t="n">
-        <v>0.2121212121212121</v>
+        <v>0.1875</v>
       </c>
       <c r="G270" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.32</v>
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>0.2706 (0.1508)</t>
+          <t>0.2136 (0.0960)</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -10142,33 +10126,33 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E271" t="n">
-        <v>0.1558441558441558</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F271" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.4155844155844156</v>
       </c>
       <c r="G271" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.4470588235294118</v>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>0.2654 (0.1127)</t>
+          <t>0.4372 (0.0188)</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -10178,33 +10162,33 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>0.2037037037037037</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="F272" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.3958333333333333</v>
       </c>
       <c r="G272" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.4044943820224719</v>
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>0.2974 (0.0906)</t>
+          <t>0.4040 (0.0080)</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -10214,33 +10198,33 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>0.0625</v>
+        <v>0.2888888888888889</v>
       </c>
       <c r="F273" t="n">
-        <v>0.2898550724637681</v>
+        <v>0.2077922077922078</v>
       </c>
       <c r="G273" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.3908045977011494</v>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>0.2110 (0.1287)</t>
+          <t>0.2958 (0.0917)</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -10250,33 +10234,33 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>0.2769230769230769</v>
+        <v>0.4835164835164835</v>
       </c>
       <c r="F274" t="n">
-        <v>0.3661971830985916</v>
+        <v>0.3950617283950617</v>
       </c>
       <c r="G274" t="n">
-        <v>0.208955223880597</v>
+        <v>0.4946236559139785</v>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>0.2840 (0.0789)</t>
+          <t>0.4577 (0.0546)</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -10286,21 +10270,21 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>0.1212121212121212</v>
+        <v>0.1578947368421053</v>
       </c>
       <c r="F275" t="n">
-        <v>0.2424242424242424</v>
+        <v>0.2121212121212121</v>
       </c>
       <c r="G275" t="n">
-        <v>0.2432432432432433</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>0.2023 (0.0702)</t>
+          <t>0.2706 (0.1508)</t>
         </is>
       </c>
     </row>
@@ -10312,7 +10296,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -10322,21 +10306,21 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>0.2325581395348837</v>
+        <v>0.1558441558441558</v>
       </c>
       <c r="F276" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="G276" t="n">
-        <v>0.2553191489361702</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>0.2579 (0.0267)</t>
+          <t>0.2654 (0.1127)</t>
         </is>
       </c>
     </row>
@@ -10348,7 +10332,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -10358,21 +10342,21 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2037037037037037</v>
       </c>
       <c r="F277" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G277" t="n">
-        <v>0.3137254901960784</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>0.2751 (0.0418)</t>
+          <t>0.2974 (0.0906)</t>
         </is>
       </c>
     </row>
@@ -10384,7 +10368,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -10394,21 +10378,21 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>0.08</v>
+        <v>0.0625</v>
       </c>
       <c r="F278" t="n">
-        <v>0.1176470588235294</v>
+        <v>0.2898550724637681</v>
       </c>
       <c r="G278" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>0.1528 (0.0954)</t>
+          <t>0.2110 (0.1287)</t>
         </is>
       </c>
     </row>
@@ -10420,7 +10404,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -10430,21 +10414,21 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>0.28125</v>
+        <v>0.2769230769230769</v>
       </c>
       <c r="F279" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.3661971830985916</v>
       </c>
       <c r="G279" t="n">
-        <v>0.2181818181818182</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>0.2814 (0.0633)</t>
+          <t>0.2840 (0.0789)</t>
         </is>
       </c>
     </row>
@@ -10456,7 +10440,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -10466,21 +10450,21 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.1212121212121212</v>
       </c>
       <c r="F280" t="n">
-        <v>0.1621621621621622</v>
+        <v>0.2424242424242424</v>
       </c>
       <c r="G280" t="n">
-        <v>0.2790697674418605</v>
+        <v>0.2432432432432433</v>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>0.1831 (0.0874)</t>
+          <t>0.2023 (0.0702)</t>
         </is>
       </c>
     </row>
@@ -10492,7 +10476,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -10502,21 +10486,21 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>0.1754385964912281</v>
+        <v>0.2325581395348837</v>
       </c>
       <c r="F281" t="n">
-        <v>0.34375</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G281" t="n">
-        <v>0.3508771929824561</v>
+        <v>0.2553191489361702</v>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>0.2900 (0.0993)</t>
+          <t>0.2579 (0.0267)</t>
         </is>
       </c>
     </row>
@@ -10528,7 +10512,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10538,21 +10522,21 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>0.1839080459770115</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="F282" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="G282" t="n">
-        <v>0.2702702702702703</v>
+        <v>0.3137254901960784</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>0.2690 (0.0845)</t>
+          <t>0.2751 (0.0418)</t>
         </is>
       </c>
     </row>
@@ -10564,7 +10548,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -10574,21 +10558,21 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>0.09230769230769231</v>
+        <v>0.08</v>
       </c>
       <c r="F283" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.1176470588235294</v>
       </c>
       <c r="G283" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>0.1654 (0.0725)</t>
+          <t>0.1528 (0.0954)</t>
         </is>
       </c>
     </row>
@@ -10600,7 +10584,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -10610,21 +10594,21 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.28125</v>
       </c>
       <c r="F284" t="n">
-        <v>0.4307692307692308</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="G284" t="n">
-        <v>0.3076923076923077</v>
+        <v>0.2181818181818182</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>0.3342 (0.0864)</t>
+          <t>0.2814 (0.0633)</t>
         </is>
       </c>
     </row>
@@ -10636,7 +10620,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -10646,21 +10630,21 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>0.1639344262295082</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="F285" t="n">
-        <v>0.2962962962962963</v>
+        <v>0.1621621621621622</v>
       </c>
       <c r="G285" t="n">
-        <v>0.2295081967213115</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>0.2299 (0.0662)</t>
+          <t>0.1831 (0.0874)</t>
         </is>
       </c>
     </row>
@@ -10672,7 +10656,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -10682,21 +10666,21 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E286" t="n">
-        <v>0.1777777777777778</v>
+        <v>0.1754385964912281</v>
       </c>
       <c r="F286" t="n">
-        <v>0.2272727272727273</v>
+        <v>0.34375</v>
       </c>
       <c r="G286" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.3508771929824561</v>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>0.2205 (0.0398)</t>
+          <t>0.2900 (0.0993)</t>
         </is>
       </c>
     </row>
@@ -10708,7 +10692,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -10718,21 +10702,21 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>0.2790697674418605</v>
+        <v>0.1839080459770115</v>
       </c>
       <c r="F287" t="n">
-        <v>0.3859649122807017</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="G287" t="n">
-        <v>0.3673469387755102</v>
+        <v>0.2702702702702703</v>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>0.3441 (0.0571)</t>
+          <t>0.2690 (0.0845)</t>
         </is>
       </c>
     </row>
@@ -10744,7 +10728,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -10754,21 +10738,21 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.09230769230769231</v>
       </c>
       <c r="F288" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="G288" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>0.1530 (0.0500)</t>
+          <t>0.1654 (0.0725)</t>
         </is>
       </c>
     </row>
@@ -10780,7 +10764,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -10790,21 +10774,21 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F289" t="n">
-        <v>0.4</v>
+        <v>0.4307692307692308</v>
       </c>
       <c r="G289" t="n">
-        <v>0.3571428571428572</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>0.3226 (0.0994)</t>
+          <t>0.3342 (0.0864)</t>
         </is>
       </c>
     </row>
@@ -10816,7 +10800,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -10826,21 +10810,21 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>0.0975609756097561</v>
+        <v>0.1639344262295082</v>
       </c>
       <c r="F290" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2962962962962963</v>
       </c>
       <c r="G290" t="n">
-        <v>0.25</v>
+        <v>0.2295081967213115</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>0.1462 (0.0900)</t>
+          <t>0.2299 (0.0662)</t>
         </is>
       </c>
     </row>
@@ -10852,7 +10836,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -10862,21 +10846,21 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>0.2380952380952381</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="F291" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.2272727272727273</v>
       </c>
       <c r="G291" t="n">
-        <v>0.3478260869565217</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>0.2429 (0.1026)</t>
+          <t>0.2205 (0.0398)</t>
         </is>
       </c>
     </row>
@@ -10888,7 +10872,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -10898,21 +10882,21 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>0.24</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="F292" t="n">
-        <v>0.303030303030303</v>
+        <v>0.3859649122807017</v>
       </c>
       <c r="G292" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.3673469387755102</v>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>0.2708 (0.0315)</t>
+          <t>0.3441 (0.0571)</t>
         </is>
       </c>
     </row>
@@ -10924,7 +10908,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -10934,21 +10918,21 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="F293" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G293" t="n">
-        <v>0.2173913043478261</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>0.1515 (0.0671)</t>
+          <t>0.1530 (0.0500)</t>
         </is>
       </c>
     </row>
@@ -10960,7 +10944,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -10970,21 +10954,21 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>0.25</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="F294" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.4</v>
       </c>
       <c r="G294" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>0.2998 (0.0581)</t>
+          <t>0.3226 (0.0994)</t>
         </is>
       </c>
     </row>
@@ -10996,7 +10980,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11006,33 +10990,33 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E295" t="n">
+        <v>0.0975609756097561</v>
+      </c>
+      <c r="F295" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="G295" t="n">
         <v>0.25</v>
       </c>
-      <c r="F295" t="n">
-        <v>0.1081081081081081</v>
-      </c>
-      <c r="G295" t="n">
-        <v>0.2857142857142857</v>
-      </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>0.2146 (0.0939)</t>
+          <t>0.1462 (0.0900)</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11042,33 +11026,33 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>0.2391304347826087</v>
+        <v>0.2380952380952381</v>
       </c>
       <c r="F296" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="G296" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.3478260869565217</v>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>0.3070 (0.0589)</t>
+          <t>0.2429 (0.1026)</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11078,33 +11062,33 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>0.3168316831683168</v>
+        <v>0.24</v>
       </c>
       <c r="F297" t="n">
-        <v>0.3454545454545455</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G297" t="n">
-        <v>0.3793103448275862</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>0.3472 (0.0313)</t>
+          <t>0.2708 (0.0315)</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11114,33 +11098,33 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F298" t="n">
-        <v>0.4303797468354431</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="G298" t="n">
-        <v>0.3820224719101123</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>0.4054 (0.0242)</t>
+          <t>0.1515 (0.0671)</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11150,33 +11134,33 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>0.4036697247706422</v>
+        <v>0.25</v>
       </c>
       <c r="F299" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="G299" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>0.4326 (0.0256)</t>
+          <t>0.2998 (0.0581)</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11186,21 +11170,21 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.25</v>
       </c>
       <c r="F300" t="n">
-        <v>0.2117647058823529</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="G300" t="n">
-        <v>0.2921348314606741</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>0.2538 (0.0403)</t>
+          <t>0.2146 (0.0939)</t>
         </is>
       </c>
     </row>
@@ -11212,7 +11196,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11222,19 +11206,21 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>0.2285714285714286</v>
+        <v>0.2391304347826087</v>
       </c>
       <c r="F301" t="n">
-        <v>0.3142857142857143</v>
-      </c>
-      <c r="G301" t="inlineStr"/>
+        <v>0.3370786516853932</v>
+      </c>
+      <c r="G301" t="n">
+        <v>0.3448275862068966</v>
+      </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>0.2714 (0.0606)</t>
+          <t>0.3070 (0.0589)</t>
         </is>
       </c>
     </row>
@@ -11246,7 +11232,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11256,21 +11242,21 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E302" t="n">
-        <v>0.3023255813953488</v>
+        <v>0.3168316831683168</v>
       </c>
       <c r="F302" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.3454545454545455</v>
       </c>
       <c r="G302" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.3793103448275862</v>
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>0.3677 (0.0598)</t>
+          <t>0.3472 (0.0313)</t>
         </is>
       </c>
     </row>
@@ -11282,7 +11268,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11292,21 +11278,21 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="F303" t="n">
-        <v>0.2597402597402597</v>
+        <v>0.4303797468354431</v>
       </c>
       <c r="G303" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.3820224719101123</v>
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>0.3101 (0.0862)</t>
+          <t>0.4054 (0.0242)</t>
         </is>
       </c>
     </row>
@@ -11318,7 +11304,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11328,21 +11314,21 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>0.4356435643564356</v>
+        <v>0.4036697247706422</v>
       </c>
       <c r="F304" t="n">
-        <v>0.4878048780487805</v>
+        <v>0.4523809523809524</v>
       </c>
       <c r="G304" t="n">
-        <v>0.4057971014492754</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>0.4431 (0.0415)</t>
+          <t>0.4326 (0.0256)</t>
         </is>
       </c>
     </row>
@@ -11354,7 +11340,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11364,19 +11350,21 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>0.3235294117647059</v>
+        <v>0.2574257425742574</v>
       </c>
       <c r="F305" t="n">
-        <v>0.1851851851851852</v>
-      </c>
-      <c r="G305" t="inlineStr"/>
+        <v>0.2117647058823529</v>
+      </c>
+      <c r="G305" t="n">
+        <v>0.2921348314606741</v>
+      </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>0.2544 (0.0978)</t>
+          <t>0.2538 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -11388,7 +11376,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11398,21 +11386,19 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E306" t="n">
-        <v>0.2736842105263158</v>
+        <v>0.2285714285714286</v>
       </c>
       <c r="F306" t="n">
-        <v>0.3736263736263736</v>
-      </c>
-      <c r="G306" t="n">
-        <v>0.3855421686746988</v>
-      </c>
+        <v>0.3142857142857143</v>
+      </c>
+      <c r="G306" t="inlineStr"/>
       <c r="H306" t="inlineStr">
         <is>
-          <t>0.3443 (0.0614)</t>
+          <t>0.2714 (0.0606)</t>
         </is>
       </c>
     </row>
@@ -11424,7 +11410,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11434,21 +11420,21 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E307" t="n">
-        <v>0.3760683760683761</v>
+        <v>0.3023255813953488</v>
       </c>
       <c r="F307" t="n">
-        <v>0.46</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G307" t="n">
-        <v>0.4081632653061225</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>0.4147 (0.0424)</t>
+          <t>0.3677 (0.0598)</t>
         </is>
       </c>
     </row>
@@ -11460,7 +11446,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11470,21 +11456,21 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E308" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="F308" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.2597402597402597</v>
       </c>
       <c r="G308" t="n">
-        <v>0.3838383838383838</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>0.3236 (0.0634)</t>
+          <t>0.3101 (0.0862)</t>
         </is>
       </c>
     </row>
@@ -11496,7 +11482,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -11506,21 +11492,21 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E309" t="n">
-        <v>0.4791666666666667</v>
+        <v>0.4356435643564356</v>
       </c>
       <c r="F309" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.4878048780487805</v>
       </c>
       <c r="G309" t="n">
-        <v>0.4</v>
+        <v>0.4057971014492754</v>
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>0.4359 (0.0401)</t>
+          <t>0.4431 (0.0415)</t>
         </is>
       </c>
     </row>
@@ -11532,7 +11518,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -11542,21 +11528,19 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E310" t="n">
-        <v>0.3125</v>
+        <v>0.3235294117647059</v>
       </c>
       <c r="F310" t="n">
-        <v>0.4337349397590362</v>
-      </c>
-      <c r="G310" t="n">
-        <v>0.4269662921348314</v>
-      </c>
+        <v>0.1851851851851852</v>
+      </c>
+      <c r="G310" t="inlineStr"/>
       <c r="H310" t="inlineStr">
         <is>
-          <t>0.3911 (0.0681)</t>
+          <t>0.2544 (0.0978)</t>
         </is>
       </c>
     </row>
@@ -11568,7 +11552,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -11578,21 +11562,21 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E311" t="n">
-        <v>0.1724137931034483</v>
+        <v>0.2736842105263158</v>
       </c>
       <c r="F311" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.3736263736263736</v>
       </c>
       <c r="G311" t="n">
-        <v>0.3384615384615385</v>
+        <v>0.3855421686746988</v>
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>0.2572 (0.0831)</t>
+          <t>0.3443 (0.0614)</t>
         </is>
       </c>
     </row>
@@ -11604,7 +11588,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -11614,21 +11598,21 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E312" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.3760683760683761</v>
       </c>
       <c r="F312" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.46</v>
       </c>
       <c r="G312" t="n">
-        <v>0.3611111111111111</v>
+        <v>0.4081632653061225</v>
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>0.3582 (0.0530)</t>
+          <t>0.4147 (0.0424)</t>
         </is>
       </c>
     </row>
@@ -11640,7 +11624,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -11650,21 +11634,21 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E313" t="n">
-        <v>0.2</v>
+        <v>0.2574257425742574</v>
       </c>
       <c r="F313" t="n">
-        <v>0.2571428571428571</v>
+        <v>0.3294117647058823</v>
       </c>
       <c r="G313" t="n">
-        <v>0.253968253968254</v>
+        <v>0.3838383838383838</v>
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>0.2370 (0.0321)</t>
+          <t>0.3236 (0.0634)</t>
         </is>
       </c>
     </row>
@@ -11676,7 +11660,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -11686,21 +11670,21 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E314" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.4791666666666667</v>
       </c>
       <c r="F314" t="n">
-        <v>0.4395604395604396</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="G314" t="n">
-        <v>0.4594594594594595</v>
+        <v>0.4</v>
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>0.4493 (0.0100)</t>
+          <t>0.4359 (0.0401)</t>
         </is>
       </c>
     </row>
@@ -11712,7 +11696,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -11722,21 +11706,21 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E315" t="n">
-        <v>0.1153846153846154</v>
+        <v>0.3125</v>
       </c>
       <c r="F315" t="n">
-        <v>0.125</v>
+        <v>0.4337349397590362</v>
       </c>
       <c r="G315" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.4269662921348314</v>
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>0.1771 (0.0987)</t>
+          <t>0.3911 (0.0681)</t>
         </is>
       </c>
     </row>
@@ -11748,7 +11732,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -11758,21 +11742,21 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E316" t="n">
-        <v>0.2253521126760563</v>
+        <v>0.1724137931034483</v>
       </c>
       <c r="F316" t="n">
-        <v>0.3188405797101449</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="G316" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.3384615384615385</v>
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>0.3203 (0.0957)</t>
+          <t>0.2572 (0.0831)</t>
         </is>
       </c>
     </row>
@@ -11784,7 +11768,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -11794,21 +11778,21 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E317" t="n">
-        <v>0.3296703296703297</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F317" t="n">
-        <v>0.4871794871794872</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="G317" t="n">
-        <v>0.4137931034482759</v>
+        <v>0.3611111111111111</v>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>0.4102 (0.0788)</t>
+          <t>0.3582 (0.0530)</t>
         </is>
       </c>
     </row>
@@ -11820,7 +11804,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -11830,21 +11814,21 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E318" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.2</v>
       </c>
       <c r="F318" t="n">
-        <v>0.3544303797468354</v>
+        <v>0.2571428571428571</v>
       </c>
       <c r="G318" t="n">
-        <v>0.3188405797101449</v>
+        <v>0.253968253968254</v>
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>0.3342 (0.0183)</t>
+          <t>0.2370 (0.0321)</t>
         </is>
       </c>
     </row>
@@ -11856,7 +11840,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -11866,21 +11850,21 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E319" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F319" t="n">
-        <v>0.358974358974359</v>
+        <v>0.4395604395604396</v>
       </c>
       <c r="G319" t="n">
-        <v>0.4810126582278481</v>
+        <v>0.4594594594594595</v>
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>0.3949 (0.0749)</t>
+          <t>0.4493 (0.0100)</t>
         </is>
       </c>
     </row>
@@ -11892,31 +11876,607 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E320" t="n">
+        <v>0.1153846153846154</v>
+      </c>
+      <c r="F320" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="G320" t="n">
+        <v>0.2909090909090909</v>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>0.1771 (0.0987)</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
           <t>xgb</t>
         </is>
       </c>
-      <c r="C320" t="inlineStr">
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E321" t="n">
+        <v>0.2253521126760563</v>
+      </c>
+      <c r="F321" t="n">
+        <v>0.3188405797101449</v>
+      </c>
+      <c r="G321" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>0.3203 (0.0957)</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E322" t="n">
+        <v>0.3296703296703297</v>
+      </c>
+      <c r="F322" t="n">
+        <v>0.4871794871794872</v>
+      </c>
+      <c r="G322" t="n">
+        <v>0.4137931034482759</v>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>0.4102 (0.0788)</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E323" t="n">
+        <v>0.3294117647058823</v>
+      </c>
+      <c r="F323" t="n">
+        <v>0.3544303797468354</v>
+      </c>
+      <c r="G323" t="n">
+        <v>0.3188405797101449</v>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>0.3342 (0.0183)</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E324" t="n">
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="F324" t="n">
+        <v>0.358974358974359</v>
+      </c>
+      <c r="G324" t="n">
+        <v>0.4810126582278481</v>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>0.3949 (0.0749)</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>BSK_hDFCGF_VCAM1</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
         <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D320" t="inlineStr">
+      <c r="D325" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E320" t="n">
+      <c r="E325" t="n">
         <v>0.2777777777777778</v>
       </c>
-      <c r="F320" t="n">
+      <c r="F325" t="n">
         <v>0.360655737704918</v>
       </c>
-      <c r="G320" t="n">
+      <c r="G325" t="n">
         <v>0.3448275862068966</v>
       </c>
-      <c r="H320" t="inlineStr">
+      <c r="H325" t="inlineStr">
         <is>
           <t>0.3278 (0.0440)</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E326" t="n">
+        <v>0</v>
+      </c>
+      <c r="F326" t="n">
+        <v>0</v>
+      </c>
+      <c r="G326" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>0.0952 (0.1650)</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E327" t="n">
+        <v>0</v>
+      </c>
+      <c r="F327" t="n">
+        <v>0</v>
+      </c>
+      <c r="G327" t="n">
+        <v>1</v>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E328" t="n">
+        <v>0</v>
+      </c>
+      <c r="F328" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="G328" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>0.3556 (0.3355)</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E329" t="n">
+        <v>0</v>
+      </c>
+      <c r="F329" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G329" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>0.1944 (0.1735)</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E330" t="n">
+        <v>0</v>
+      </c>
+      <c r="F330" t="n">
+        <v>0</v>
+      </c>
+      <c r="G330" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>0.0952 (0.1650)</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E331" t="n">
+        <v>0</v>
+      </c>
+      <c r="F331" t="n">
+        <v>0</v>
+      </c>
+      <c r="G331" t="n">
+        <v>1</v>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E332" t="n">
+        <v>0</v>
+      </c>
+      <c r="F332" t="n">
+        <v>0</v>
+      </c>
+      <c r="G332" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E333" t="n">
+        <v>0</v>
+      </c>
+      <c r="F333" t="n">
+        <v>0</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E334" t="n">
+        <v>0</v>
+      </c>
+      <c r="F334" t="n">
+        <v>0</v>
+      </c>
+      <c r="G334" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E335" t="n">
+        <v>0</v>
+      </c>
+      <c r="F335" t="n">
+        <v>0</v>
+      </c>
+      <c r="G335" t="n">
+        <v>1</v>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E336" t="n">
+        <v>0</v>
+      </c>
+      <c r="F336" t="n">
+        <v>0</v>
+      </c>
+      <c r="G336" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 07:32:01)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H336"/>
+  <dimension ref="A1:H340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8868,27 +8868,27 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E236" t="n">
-        <v>0.2318840579710145</v>
+        <v>0.04545454545454546</v>
       </c>
       <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr"/>
       <c r="H236" t="inlineStr">
         <is>
-          <t>0.2319 (0.0000)</t>
+          <t>0.0455 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -8905,7 +8905,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -8914,17 +8914,13 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>0.3364485981308411</v>
-      </c>
-      <c r="F237" t="n">
-        <v>0.4489795918367347</v>
-      </c>
-      <c r="G237" t="n">
-        <v>0.3764705882352941</v>
-      </c>
+        <v>0.2318840579710145</v>
+      </c>
+      <c r="F237" t="inlineStr"/>
+      <c r="G237" t="inlineStr"/>
       <c r="H237" t="inlineStr">
         <is>
-          <t>0.3873 (0.0570)</t>
+          <t>0.2319 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -8941,7 +8937,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -8950,17 +8946,17 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>0.367816091954023</v>
+        <v>0.3364485981308411</v>
       </c>
       <c r="F238" t="n">
-        <v>0.3421052631578947</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="G238" t="n">
-        <v>0.3283582089552239</v>
+        <v>0.3764705882352941</v>
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>0.3461 (0.0200)</t>
+          <t>0.3873 (0.0570)</t>
         </is>
       </c>
     </row>
@@ -8977,7 +8973,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -8986,13 +8982,17 @@
         </is>
       </c>
       <c r="E239" t="n">
-        <v>0.3870967741935484</v>
-      </c>
-      <c r="F239" t="inlineStr"/>
-      <c r="G239" t="inlineStr"/>
+        <v>0.367816091954023</v>
+      </c>
+      <c r="F239" t="n">
+        <v>0.3421052631578947</v>
+      </c>
+      <c r="G239" t="n">
+        <v>0.3283582089552239</v>
+      </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>0.3871 (0.0000)</t>
+          <t>0.3461 (0.0200)</t>
         </is>
       </c>
     </row>
@@ -9009,7 +9009,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -9018,13 +9018,15 @@
         </is>
       </c>
       <c r="E240" t="n">
-        <v>0.1904761904761905</v>
-      </c>
-      <c r="F240" t="inlineStr"/>
+        <v>0.3870967741935484</v>
+      </c>
+      <c r="F240" t="n">
+        <v>0.4935064935064935</v>
+      </c>
       <c r="G240" t="inlineStr"/>
       <c r="H240" t="inlineStr">
         <is>
-          <t>0.1905 (0.0000)</t>
+          <t>0.4403 (0.0752)</t>
         </is>
       </c>
     </row>
@@ -9036,31 +9038,29 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E241" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.1904761904761905</v>
       </c>
       <c r="F241" t="n">
-        <v>0.2307692307692308</v>
-      </c>
-      <c r="G241" t="n">
-        <v>0.3870967741935484</v>
-      </c>
+        <v>0.3611111111111111</v>
+      </c>
+      <c r="G241" t="inlineStr"/>
       <c r="H241" t="inlineStr">
         <is>
-          <t>0.2337 (0.1519)</t>
+          <t>0.2758 (0.1207)</t>
         </is>
       </c>
     </row>
@@ -9077,7 +9077,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -9086,17 +9086,17 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F242" t="n">
-        <v>0.48</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G242" t="n">
         <v>0.3870967741935484</v>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>0.3681 (0.1225)</t>
+          <t>0.2337 (0.1519)</t>
         </is>
       </c>
     </row>
@@ -9113,7 +9113,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -9122,17 +9122,17 @@
         </is>
       </c>
       <c r="E243" t="n">
-        <v>0.3</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="F243" t="n">
-        <v>0.3714285714285714</v>
+        <v>0.48</v>
       </c>
       <c r="G243" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>0.3029 (0.0671)</t>
+          <t>0.3681 (0.1225)</t>
         </is>
       </c>
     </row>
@@ -9149,7 +9149,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -9158,17 +9158,17 @@
         </is>
       </c>
       <c r="E244" t="n">
-        <v>0.4848484848484849</v>
+        <v>0.3</v>
       </c>
       <c r="F244" t="n">
-        <v>0.5151515151515151</v>
+        <v>0.3714285714285714</v>
       </c>
       <c r="G244" t="n">
-        <v>0.4</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>0.4667 (0.0597)</t>
+          <t>0.3029 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -9185,7 +9185,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -9194,17 +9194,17 @@
         </is>
       </c>
       <c r="E245" t="n">
-        <v>0.0975609756097561</v>
+        <v>0.4848484848484849</v>
       </c>
       <c r="F245" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.5151515151515151</v>
       </c>
       <c r="G245" t="n">
-        <v>0.3214285714285715</v>
+        <v>0.4</v>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>0.2166 (0.1126)</t>
+          <t>0.4667 (0.0597)</t>
         </is>
       </c>
     </row>
@@ -9216,31 +9216,31 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E246" t="n">
+        <v>0.0975609756097561</v>
+      </c>
+      <c r="F246" t="n">
         <v>0.2307692307692308</v>
       </c>
-      <c r="F246" t="n">
-        <v>0.4761904761904762</v>
-      </c>
       <c r="G246" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.3214285714285715</v>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>0.3785 (0.1301)</t>
+          <t>0.2166 (0.1126)</t>
         </is>
       </c>
     </row>
@@ -9257,7 +9257,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -9266,17 +9266,17 @@
         </is>
       </c>
       <c r="E247" t="n">
-        <v>0.3116883116883117</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="F247" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="G247" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>0.3581 (0.0492)</t>
+          <t>0.3785 (0.1301)</t>
         </is>
       </c>
     </row>
@@ -9293,7 +9293,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -9302,17 +9302,17 @@
         </is>
       </c>
       <c r="E248" t="n">
-        <v>0.3050847457627119</v>
+        <v>0.3116883116883117</v>
       </c>
       <c r="F248" t="n">
-        <v>0.3278688524590164</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="G248" t="n">
-        <v>0.3050847457627119</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>0.3127 (0.0132)</t>
+          <t>0.3581 (0.0492)</t>
         </is>
       </c>
     </row>
@@ -9329,7 +9329,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -9338,17 +9338,17 @@
         </is>
       </c>
       <c r="E249" t="n">
-        <v>0.3666666666666666</v>
+        <v>0.3050847457627119</v>
       </c>
       <c r="F249" t="n">
-        <v>0.5161290322580645</v>
+        <v>0.3278688524590164</v>
       </c>
       <c r="G249" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3050847457627119</v>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>0.4119 (0.0905)</t>
+          <t>0.3127 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -9365,7 +9365,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -9374,53 +9374,53 @@
         </is>
       </c>
       <c r="E250" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.3666666666666666</v>
       </c>
       <c r="F250" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.5161290322580645</v>
       </c>
       <c r="G250" t="n">
-        <v>0.3934426229508197</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>0.2512 (0.1521)</t>
+          <t>0.4119 (0.0905)</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_PAI1</t>
+          <t>BSK_KF3CT_TIMP2</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E251" t="n">
-        <v>0.3106796116504854</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="F251" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="G251" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.3934426229508197</v>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>0.3618 (0.0444)</t>
+          <t>0.2512 (0.1521)</t>
         </is>
       </c>
     </row>
@@ -9437,7 +9437,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -9446,17 +9446,17 @@
         </is>
       </c>
       <c r="E252" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3106796116504854</v>
       </c>
       <c r="F252" t="n">
-        <v>0.3863636363636364</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G252" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>0.3811 (0.0259)</t>
+          <t>0.3618 (0.0444)</t>
         </is>
       </c>
     </row>
@@ -9473,7 +9473,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -9482,17 +9482,17 @@
         </is>
       </c>
       <c r="E253" t="n">
-        <v>0.2365591397849462</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F253" t="n">
-        <v>0.275</v>
+        <v>0.3863636363636364</v>
       </c>
       <c r="G253" t="n">
-        <v>0.3595505617977528</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>0.2904 (0.0629)</t>
+          <t>0.3811 (0.0259)</t>
         </is>
       </c>
     </row>
@@ -9509,7 +9509,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -9518,17 +9518,17 @@
         </is>
       </c>
       <c r="E254" t="n">
-        <v>0.4912280701754386</v>
+        <v>0.2365591397849462</v>
       </c>
       <c r="F254" t="n">
-        <v>0.345679012345679</v>
+        <v>0.275</v>
       </c>
       <c r="G254" t="n">
-        <v>0.459016393442623</v>
+        <v>0.3595505617977528</v>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>0.4320 (0.0764)</t>
+          <t>0.2904 (0.0629)</t>
         </is>
       </c>
     </row>
@@ -9545,7 +9545,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -9554,17 +9554,17 @@
         </is>
       </c>
       <c r="E255" t="n">
-        <v>0.24</v>
+        <v>0.4912280701754386</v>
       </c>
       <c r="F255" t="n">
-        <v>0.25</v>
+        <v>0.345679012345679</v>
       </c>
       <c r="G255" t="n">
-        <v>0.4466019417475728</v>
+        <v>0.459016393442623</v>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>0.3122 (0.1165)</t>
+          <t>0.4320 (0.0764)</t>
         </is>
       </c>
     </row>
@@ -9576,31 +9576,31 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>0.367816091954023</v>
+        <v>0.24</v>
       </c>
       <c r="F256" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.25</v>
       </c>
       <c r="G256" t="n">
-        <v>0.3953488372093023</v>
+        <v>0.4466019417475728</v>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>0.3826 (0.0139)</t>
+          <t>0.3122 (0.1165)</t>
         </is>
       </c>
     </row>
@@ -9617,7 +9617,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -9626,17 +9626,17 @@
         </is>
       </c>
       <c r="E257" t="n">
-        <v>0.3260869565217391</v>
+        <v>0.367816091954023</v>
       </c>
       <c r="F257" t="n">
-        <v>0.4086021505376344</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G257" t="n">
-        <v>0.449438202247191</v>
+        <v>0.3953488372093023</v>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>0.3947 (0.0628)</t>
+          <t>0.3826 (0.0139)</t>
         </is>
       </c>
     </row>
@@ -9653,7 +9653,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -9662,17 +9662,17 @@
         </is>
       </c>
       <c r="E258" t="n">
-        <v>0.247191011235955</v>
+        <v>0.3260869565217391</v>
       </c>
       <c r="F258" t="n">
-        <v>0.3376623376623377</v>
+        <v>0.4086021505376344</v>
       </c>
       <c r="G258" t="n">
-        <v>0.2716049382716049</v>
+        <v>0.449438202247191</v>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>0.2855 (0.0468)</t>
+          <t>0.3947 (0.0628)</t>
         </is>
       </c>
     </row>
@@ -9689,7 +9689,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -9698,17 +9698,17 @@
         </is>
       </c>
       <c r="E259" t="n">
-        <v>0.5045045045045045</v>
+        <v>0.247191011235955</v>
       </c>
       <c r="F259" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.3376623376623377</v>
       </c>
       <c r="G259" t="n">
-        <v>0.4554455445544555</v>
+        <v>0.2716049382716049</v>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>0.4599 (0.0426)</t>
+          <t>0.2855 (0.0468)</t>
         </is>
       </c>
     </row>
@@ -9725,7 +9725,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -9734,17 +9734,17 @@
         </is>
       </c>
       <c r="E260" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.5045045045045045</v>
       </c>
       <c r="F260" t="n">
-        <v>0.3235294117647059</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G260" t="n">
-        <v>0.48</v>
+        <v>0.4554455445544555</v>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>0.3691 (0.0965)</t>
+          <t>0.4599 (0.0426)</t>
         </is>
       </c>
     </row>
@@ -9756,31 +9756,31 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E261" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F261" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.3235294117647059</v>
       </c>
       <c r="G261" t="n">
-        <v>0.3655913978494624</v>
+        <v>0.48</v>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>0.3654 (0.0124)</t>
+          <t>0.3691 (0.0965)</t>
         </is>
       </c>
     </row>
@@ -9797,7 +9797,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -9806,17 +9806,17 @@
         </is>
       </c>
       <c r="E262" t="n">
-        <v>0.4</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F262" t="n">
-        <v>0.4885496183206107</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G262" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.3655913978494624</v>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>0.4443 (0.0443)</t>
+          <t>0.3654 (0.0124)</t>
         </is>
       </c>
     </row>
@@ -9833,7 +9833,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -9842,17 +9842,17 @@
         </is>
       </c>
       <c r="E263" t="n">
-        <v>0.3963963963963964</v>
+        <v>0.4</v>
       </c>
       <c r="F263" t="n">
-        <v>0.2823529411764706</v>
+        <v>0.4885496183206107</v>
       </c>
       <c r="G263" t="n">
-        <v>0.3505154639175257</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>0.3431 (0.0574)</t>
+          <t>0.4443 (0.0443)</t>
         </is>
       </c>
     </row>
@@ -9869,7 +9869,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -9878,17 +9878,17 @@
         </is>
       </c>
       <c r="E264" t="n">
-        <v>0.4905660377358491</v>
+        <v>0.3963963963963964</v>
       </c>
       <c r="F264" t="n">
-        <v>0.3777777777777778</v>
+        <v>0.2823529411764706</v>
       </c>
       <c r="G264" t="n">
-        <v>0.4888888888888889</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>0.4524 (0.0646)</t>
+          <t>0.3431 (0.0574)</t>
         </is>
       </c>
     </row>
@@ -9905,7 +9905,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -9914,17 +9914,17 @@
         </is>
       </c>
       <c r="E265" t="n">
-        <v>0.3423423423423423</v>
+        <v>0.4905660377358491</v>
       </c>
       <c r="F265" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="G265" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.4888888888888889</v>
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>0.3306 (0.0403)</t>
+          <t>0.4524 (0.0646)</t>
         </is>
       </c>
     </row>
@@ -9936,31 +9936,31 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E266" t="n">
-        <v>0.4369747899159664</v>
+        <v>0.3423423423423423</v>
       </c>
       <c r="F266" t="n">
-        <v>0.3013698630136986</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G266" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>0.3850 (0.0731)</t>
+          <t>0.3306 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -9977,7 +9977,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -9986,17 +9986,17 @@
         </is>
       </c>
       <c r="E267" t="n">
-        <v>0.3505154639175257</v>
+        <v>0.4369747899159664</v>
       </c>
       <c r="F267" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.3013698630136986</v>
       </c>
       <c r="G267" t="n">
-        <v>0.4050632911392405</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>0.3819 (0.0282)</t>
+          <t>0.3850 (0.0731)</t>
         </is>
       </c>
     </row>
@@ -10013,7 +10013,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -10022,17 +10022,17 @@
         </is>
       </c>
       <c r="E268" t="n">
-        <v>0.2619047619047619</v>
+        <v>0.3505154639175257</v>
       </c>
       <c r="F268" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="G268" t="n">
-        <v>0.2318840579710145</v>
+        <v>0.4050632911392405</v>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>0.2501 (0.0160)</t>
+          <t>0.3819 (0.0282)</t>
         </is>
       </c>
     </row>
@@ -10049,7 +10049,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -10058,17 +10058,17 @@
         </is>
       </c>
       <c r="E269" t="n">
-        <v>0.5546218487394958</v>
+        <v>0.2619047619047619</v>
       </c>
       <c r="F269" t="n">
-        <v>0.5217391304347826</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="G269" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.2318840579710145</v>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>0.5084 (0.0541)</t>
+          <t>0.2501 (0.0160)</t>
         </is>
       </c>
     </row>
@@ -10085,7 +10085,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -10094,17 +10094,17 @@
         </is>
       </c>
       <c r="E270" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.5546218487394958</v>
       </c>
       <c r="F270" t="n">
-        <v>0.1875</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="G270" t="n">
-        <v>0.32</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>0.2136 (0.0960)</t>
+          <t>0.5084 (0.0541)</t>
         </is>
       </c>
     </row>
@@ -10116,31 +10116,31 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E271" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="F271" t="n">
-        <v>0.4155844155844156</v>
+        <v>0.1875</v>
       </c>
       <c r="G271" t="n">
-        <v>0.4470588235294118</v>
+        <v>0.32</v>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>0.4372 (0.0188)</t>
+          <t>0.2136 (0.0960)</t>
         </is>
       </c>
     </row>
@@ -10157,7 +10157,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -10166,17 +10166,17 @@
         </is>
       </c>
       <c r="E272" t="n">
-        <v>0.4117647058823529</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F272" t="n">
-        <v>0.3958333333333333</v>
+        <v>0.4155844155844156</v>
       </c>
       <c r="G272" t="n">
-        <v>0.4044943820224719</v>
+        <v>0.4470588235294118</v>
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>0.4040 (0.0080)</t>
+          <t>0.4372 (0.0188)</t>
         </is>
       </c>
     </row>
@@ -10193,7 +10193,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -10202,17 +10202,17 @@
         </is>
       </c>
       <c r="E273" t="n">
-        <v>0.2888888888888889</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="F273" t="n">
-        <v>0.2077922077922078</v>
+        <v>0.3958333333333333</v>
       </c>
       <c r="G273" t="n">
-        <v>0.3908045977011494</v>
+        <v>0.4044943820224719</v>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>0.2958 (0.0917)</t>
+          <t>0.4040 (0.0080)</t>
         </is>
       </c>
     </row>
@@ -10229,7 +10229,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -10238,17 +10238,17 @@
         </is>
       </c>
       <c r="E274" t="n">
-        <v>0.4835164835164835</v>
+        <v>0.2888888888888889</v>
       </c>
       <c r="F274" t="n">
-        <v>0.3950617283950617</v>
+        <v>0.2077922077922078</v>
       </c>
       <c r="G274" t="n">
-        <v>0.4946236559139785</v>
+        <v>0.3908045977011494</v>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>0.4577 (0.0546)</t>
+          <t>0.2958 (0.0917)</t>
         </is>
       </c>
     </row>
@@ -10265,7 +10265,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -10274,53 +10274,53 @@
         </is>
       </c>
       <c r="E275" t="n">
-        <v>0.1578947368421053</v>
+        <v>0.4835164835164835</v>
       </c>
       <c r="F275" t="n">
-        <v>0.2121212121212121</v>
+        <v>0.3950617283950617</v>
       </c>
       <c r="G275" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.4946236559139785</v>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>0.2706 (0.1508)</t>
+          <t>0.4577 (0.0546)</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_TIMP1</t>
+          <t>BSK_hDFCGF_PAI1</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>0.1558441558441558</v>
+        <v>0.1578947368421053</v>
       </c>
       <c r="F276" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.2121212121212121</v>
       </c>
       <c r="G276" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>0.2654 (0.1127)</t>
+          <t>0.2706 (0.1508)</t>
         </is>
       </c>
     </row>
@@ -10337,7 +10337,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -10346,17 +10346,17 @@
         </is>
       </c>
       <c r="E277" t="n">
-        <v>0.2037037037037037</v>
+        <v>0.1558441558441558</v>
       </c>
       <c r="F277" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="G277" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>0.2974 (0.0906)</t>
+          <t>0.2654 (0.1127)</t>
         </is>
       </c>
     </row>
@@ -10373,7 +10373,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -10382,17 +10382,17 @@
         </is>
       </c>
       <c r="E278" t="n">
-        <v>0.0625</v>
+        <v>0.2037037037037037</v>
       </c>
       <c r="F278" t="n">
-        <v>0.2898550724637681</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G278" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>0.2110 (0.1287)</t>
+          <t>0.2974 (0.0906)</t>
         </is>
       </c>
     </row>
@@ -10409,7 +10409,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -10418,17 +10418,17 @@
         </is>
       </c>
       <c r="E279" t="n">
-        <v>0.2769230769230769</v>
+        <v>0.0625</v>
       </c>
       <c r="F279" t="n">
-        <v>0.3661971830985916</v>
+        <v>0.2898550724637681</v>
       </c>
       <c r="G279" t="n">
-        <v>0.208955223880597</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>0.2840 (0.0789)</t>
+          <t>0.2110 (0.1287)</t>
         </is>
       </c>
     </row>
@@ -10445,7 +10445,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -10454,17 +10454,17 @@
         </is>
       </c>
       <c r="E280" t="n">
-        <v>0.1212121212121212</v>
+        <v>0.2769230769230769</v>
       </c>
       <c r="F280" t="n">
-        <v>0.2424242424242424</v>
+        <v>0.3661971830985916</v>
       </c>
       <c r="G280" t="n">
-        <v>0.2432432432432433</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>0.2023 (0.0702)</t>
+          <t>0.2840 (0.0789)</t>
         </is>
       </c>
     </row>
@@ -10476,31 +10476,31 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>0.2325581395348837</v>
+        <v>0.1212121212121212</v>
       </c>
       <c r="F281" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2424242424242424</v>
       </c>
       <c r="G281" t="n">
-        <v>0.2553191489361702</v>
+        <v>0.2432432432432433</v>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>0.2579 (0.0267)</t>
+          <t>0.2023 (0.0702)</t>
         </is>
       </c>
     </row>
@@ -10517,7 +10517,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -10526,17 +10526,17 @@
         </is>
       </c>
       <c r="E282" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2325581395348837</v>
       </c>
       <c r="F282" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G282" t="n">
-        <v>0.3137254901960784</v>
+        <v>0.2553191489361702</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>0.2751 (0.0418)</t>
+          <t>0.2579 (0.0267)</t>
         </is>
       </c>
     </row>
@@ -10553,7 +10553,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -10562,17 +10562,17 @@
         </is>
       </c>
       <c r="E283" t="n">
-        <v>0.08</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="F283" t="n">
-        <v>0.1176470588235294</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="G283" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.3137254901960784</v>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>0.1528 (0.0954)</t>
+          <t>0.2751 (0.0418)</t>
         </is>
       </c>
     </row>
@@ -10589,7 +10589,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -10598,17 +10598,17 @@
         </is>
       </c>
       <c r="E284" t="n">
-        <v>0.28125</v>
+        <v>0.08</v>
       </c>
       <c r="F284" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.1176470588235294</v>
       </c>
       <c r="G284" t="n">
-        <v>0.2181818181818182</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>0.2814 (0.0633)</t>
+          <t>0.1528 (0.0954)</t>
         </is>
       </c>
     </row>
@@ -10625,7 +10625,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -10634,17 +10634,17 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.28125</v>
       </c>
       <c r="F285" t="n">
-        <v>0.1621621621621622</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="G285" t="n">
-        <v>0.2790697674418605</v>
+        <v>0.2181818181818182</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>0.1831 (0.0874)</t>
+          <t>0.2814 (0.0633)</t>
         </is>
       </c>
     </row>
@@ -10656,31 +10656,31 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E286" t="n">
-        <v>0.1754385964912281</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="F286" t="n">
-        <v>0.34375</v>
+        <v>0.1621621621621622</v>
       </c>
       <c r="G286" t="n">
-        <v>0.3508771929824561</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>0.2900 (0.0993)</t>
+          <t>0.1831 (0.0874)</t>
         </is>
       </c>
     </row>
@@ -10697,7 +10697,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -10706,17 +10706,17 @@
         </is>
       </c>
       <c r="E287" t="n">
-        <v>0.1839080459770115</v>
+        <v>0.1754385964912281</v>
       </c>
       <c r="F287" t="n">
-        <v>0.3529411764705883</v>
+        <v>0.34375</v>
       </c>
       <c r="G287" t="n">
-        <v>0.2702702702702703</v>
+        <v>0.3508771929824561</v>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>0.2690 (0.0845)</t>
+          <t>0.2900 (0.0993)</t>
         </is>
       </c>
     </row>
@@ -10733,7 +10733,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -10742,17 +10742,17 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>0.09230769230769231</v>
+        <v>0.1839080459770115</v>
       </c>
       <c r="F288" t="n">
-        <v>0.2372881355932203</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="G288" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.2702702702702703</v>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>0.1654 (0.0725)</t>
+          <t>0.2690 (0.0845)</t>
         </is>
       </c>
     </row>
@@ -10769,7 +10769,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -10778,17 +10778,17 @@
         </is>
       </c>
       <c r="E289" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.09230769230769231</v>
       </c>
       <c r="F289" t="n">
-        <v>0.4307692307692308</v>
+        <v>0.2372881355932203</v>
       </c>
       <c r="G289" t="n">
-        <v>0.3076923076923077</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>0.3342 (0.0864)</t>
+          <t>0.1654 (0.0725)</t>
         </is>
       </c>
     </row>
@@ -10805,7 +10805,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -10814,17 +10814,17 @@
         </is>
       </c>
       <c r="E290" t="n">
-        <v>0.1639344262295082</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F290" t="n">
-        <v>0.2962962962962963</v>
+        <v>0.4307692307692308</v>
       </c>
       <c r="G290" t="n">
-        <v>0.2295081967213115</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>0.2299 (0.0662)</t>
+          <t>0.3342 (0.0864)</t>
         </is>
       </c>
     </row>
@@ -10836,31 +10836,31 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>0.1777777777777778</v>
+        <v>0.1639344262295082</v>
       </c>
       <c r="F291" t="n">
-        <v>0.2272727272727273</v>
+        <v>0.2962962962962963</v>
       </c>
       <c r="G291" t="n">
-        <v>0.2564102564102564</v>
+        <v>0.2295081967213115</v>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>0.2205 (0.0398)</t>
+          <t>0.2299 (0.0662)</t>
         </is>
       </c>
     </row>
@@ -10877,7 +10877,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
@@ -10886,17 +10886,17 @@
         </is>
       </c>
       <c r="E292" t="n">
-        <v>0.2790697674418605</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="F292" t="n">
-        <v>0.3859649122807017</v>
+        <v>0.2272727272727273</v>
       </c>
       <c r="G292" t="n">
-        <v>0.3673469387755102</v>
+        <v>0.2564102564102564</v>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>0.3441 (0.0571)</t>
+          <t>0.2205 (0.0398)</t>
         </is>
       </c>
     </row>
@@ -10913,7 +10913,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
@@ -10922,17 +10922,17 @@
         </is>
       </c>
       <c r="E293" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="F293" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3859649122807017</v>
       </c>
       <c r="G293" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3673469387755102</v>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>0.1530 (0.0500)</t>
+          <t>0.3441 (0.0571)</t>
         </is>
       </c>
     </row>
@@ -10949,7 +10949,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -10958,17 +10958,17 @@
         </is>
       </c>
       <c r="E294" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="F294" t="n">
-        <v>0.4</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G294" t="n">
-        <v>0.3571428571428572</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>0.3226 (0.0994)</t>
+          <t>0.1530 (0.0500)</t>
         </is>
       </c>
     </row>
@@ -10985,7 +10985,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
@@ -10994,17 +10994,17 @@
         </is>
       </c>
       <c r="E295" t="n">
-        <v>0.0975609756097561</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="F295" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.4</v>
       </c>
       <c r="G295" t="n">
-        <v>0.25</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>0.1462 (0.0900)</t>
+          <t>0.3226 (0.0994)</t>
         </is>
       </c>
     </row>
@@ -11016,31 +11016,31 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>0.2380952380952381</v>
+        <v>0.0975609756097561</v>
       </c>
       <c r="F296" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="G296" t="n">
-        <v>0.3478260869565217</v>
+        <v>0.25</v>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>0.2429 (0.1026)</t>
+          <t>0.1462 (0.0900)</t>
         </is>
       </c>
     </row>
@@ -11057,7 +11057,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
@@ -11066,17 +11066,17 @@
         </is>
       </c>
       <c r="E297" t="n">
-        <v>0.24</v>
+        <v>0.2380952380952381</v>
       </c>
       <c r="F297" t="n">
-        <v>0.303030303030303</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="G297" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.3478260869565217</v>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>0.2708 (0.0315)</t>
+          <t>0.2429 (0.1026)</t>
         </is>
       </c>
     </row>
@@ -11093,7 +11093,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
@@ -11102,17 +11102,17 @@
         </is>
       </c>
       <c r="E298" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.24</v>
       </c>
       <c r="F298" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G298" t="n">
-        <v>0.2173913043478261</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>0.1515 (0.0671)</t>
+          <t>0.2708 (0.0315)</t>
         </is>
       </c>
     </row>
@@ -11129,7 +11129,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
@@ -11138,17 +11138,17 @@
         </is>
       </c>
       <c r="E299" t="n">
-        <v>0.25</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F299" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="G299" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>0.2998 (0.0581)</t>
+          <t>0.1515 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -11165,7 +11165,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
@@ -11177,50 +11177,50 @@
         <v>0.25</v>
       </c>
       <c r="F300" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="G300" t="n">
         <v>0.2857142857142857</v>
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>0.2146 (0.0939)</t>
+          <t>0.2998 (0.0581)</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>BSK_hDFCGF_VCAM1</t>
+          <t>BSK_hDFCGF_TIMP1</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>0.2391304347826087</v>
+        <v>0.25</v>
       </c>
       <c r="F301" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="G301" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>0.3070 (0.0589)</t>
+          <t>0.2146 (0.0939)</t>
         </is>
       </c>
     </row>
@@ -11237,7 +11237,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
@@ -11246,17 +11246,17 @@
         </is>
       </c>
       <c r="E302" t="n">
-        <v>0.3168316831683168</v>
+        <v>0.2391304347826087</v>
       </c>
       <c r="F302" t="n">
-        <v>0.3454545454545455</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="G302" t="n">
-        <v>0.3793103448275862</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>0.3472 (0.0313)</t>
+          <t>0.3070 (0.0589)</t>
         </is>
       </c>
     </row>
@@ -11273,7 +11273,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
@@ -11282,17 +11282,17 @@
         </is>
       </c>
       <c r="E303" t="n">
-        <v>0.4038461538461539</v>
+        <v>0.3168316831683168</v>
       </c>
       <c r="F303" t="n">
-        <v>0.4303797468354431</v>
+        <v>0.3454545454545455</v>
       </c>
       <c r="G303" t="n">
-        <v>0.3820224719101123</v>
+        <v>0.3793103448275862</v>
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>0.4054 (0.0242)</t>
+          <t>0.3472 (0.0313)</t>
         </is>
       </c>
     </row>
@@ -11309,7 +11309,7 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
@@ -11318,17 +11318,17 @@
         </is>
       </c>
       <c r="E304" t="n">
-        <v>0.4036697247706422</v>
+        <v>0.4038461538461539</v>
       </c>
       <c r="F304" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.4303797468354431</v>
       </c>
       <c r="G304" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.3820224719101123</v>
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>0.4326 (0.0256)</t>
+          <t>0.4054 (0.0242)</t>
         </is>
       </c>
     </row>
@@ -11345,7 +11345,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
@@ -11354,17 +11354,17 @@
         </is>
       </c>
       <c r="E305" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.4036697247706422</v>
       </c>
       <c r="F305" t="n">
-        <v>0.2117647058823529</v>
+        <v>0.4523809523809524</v>
       </c>
       <c r="G305" t="n">
-        <v>0.2921348314606741</v>
+        <v>0.4418604651162791</v>
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>0.2538 (0.0403)</t>
+          <t>0.4326 (0.0256)</t>
         </is>
       </c>
     </row>
@@ -11376,29 +11376,31 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E306" t="n">
-        <v>0.2285714285714286</v>
+        <v>0.2574257425742574</v>
       </c>
       <c r="F306" t="n">
-        <v>0.3142857142857143</v>
-      </c>
-      <c r="G306" t="inlineStr"/>
+        <v>0.2117647058823529</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0.2921348314606741</v>
+      </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>0.2714 (0.0606)</t>
+          <t>0.2538 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -11415,7 +11417,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
@@ -11424,17 +11426,17 @@
         </is>
       </c>
       <c r="E307" t="n">
-        <v>0.3023255813953488</v>
+        <v>0.2285714285714286</v>
       </c>
       <c r="F307" t="n">
-        <v>0.4197530864197531</v>
+        <v>0.3142857142857143</v>
       </c>
       <c r="G307" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.4864864864864865</v>
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>0.3677 (0.0598)</t>
+          <t>0.3431 (0.1314)</t>
         </is>
       </c>
     </row>
@@ -11451,7 +11453,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
@@ -11460,17 +11462,17 @@
         </is>
       </c>
       <c r="E308" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.3023255813953488</v>
       </c>
       <c r="F308" t="n">
-        <v>0.2597402597402597</v>
+        <v>0.4197530864197531</v>
       </c>
       <c r="G308" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>0.3101 (0.0862)</t>
+          <t>0.3677 (0.0598)</t>
         </is>
       </c>
     </row>
@@ -11487,7 +11489,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
@@ -11496,17 +11498,17 @@
         </is>
       </c>
       <c r="E309" t="n">
-        <v>0.4356435643564356</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="F309" t="n">
-        <v>0.4878048780487805</v>
+        <v>0.2597402597402597</v>
       </c>
       <c r="G309" t="n">
-        <v>0.4057971014492754</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>0.4431 (0.0415)</t>
+          <t>0.3101 (0.0862)</t>
         </is>
       </c>
     </row>
@@ -11523,7 +11525,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
@@ -11532,15 +11534,17 @@
         </is>
       </c>
       <c r="E310" t="n">
-        <v>0.3235294117647059</v>
+        <v>0.4356435643564356</v>
       </c>
       <c r="F310" t="n">
-        <v>0.1851851851851852</v>
-      </c>
-      <c r="G310" t="inlineStr"/>
+        <v>0.4878048780487805</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0.4057971014492754</v>
+      </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>0.2544 (0.0978)</t>
+          <t>0.4431 (0.0415)</t>
         </is>
       </c>
     </row>
@@ -11552,31 +11556,29 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E311" t="n">
-        <v>0.2736842105263158</v>
+        <v>0.3235294117647059</v>
       </c>
       <c r="F311" t="n">
-        <v>0.3736263736263736</v>
-      </c>
-      <c r="G311" t="n">
-        <v>0.3855421686746988</v>
-      </c>
+        <v>0.1851851851851852</v>
+      </c>
+      <c r="G311" t="inlineStr"/>
       <c r="H311" t="inlineStr">
         <is>
-          <t>0.3443 (0.0614)</t>
+          <t>0.2544 (0.0978)</t>
         </is>
       </c>
     </row>
@@ -11593,7 +11595,7 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
@@ -11602,17 +11604,17 @@
         </is>
       </c>
       <c r="E312" t="n">
-        <v>0.3760683760683761</v>
+        <v>0.2736842105263158</v>
       </c>
       <c r="F312" t="n">
-        <v>0.46</v>
+        <v>0.3736263736263736</v>
       </c>
       <c r="G312" t="n">
-        <v>0.4081632653061225</v>
+        <v>0.3855421686746988</v>
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>0.4147 (0.0424)</t>
+          <t>0.3443 (0.0614)</t>
         </is>
       </c>
     </row>
@@ -11629,7 +11631,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
@@ -11638,17 +11640,17 @@
         </is>
       </c>
       <c r="E313" t="n">
-        <v>0.2574257425742574</v>
+        <v>0.3760683760683761</v>
       </c>
       <c r="F313" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.46</v>
       </c>
       <c r="G313" t="n">
-        <v>0.3838383838383838</v>
+        <v>0.4081632653061225</v>
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>0.3236 (0.0634)</t>
+          <t>0.4147 (0.0424)</t>
         </is>
       </c>
     </row>
@@ -11665,7 +11667,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
@@ -11674,17 +11676,17 @@
         </is>
       </c>
       <c r="E314" t="n">
-        <v>0.4791666666666667</v>
+        <v>0.2574257425742574</v>
       </c>
       <c r="F314" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.3294117647058823</v>
       </c>
       <c r="G314" t="n">
-        <v>0.4</v>
+        <v>0.3838383838383838</v>
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>0.4359 (0.0401)</t>
+          <t>0.3236 (0.0634)</t>
         </is>
       </c>
     </row>
@@ -11701,7 +11703,7 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -11710,17 +11712,17 @@
         </is>
       </c>
       <c r="E315" t="n">
-        <v>0.3125</v>
+        <v>0.4791666666666667</v>
       </c>
       <c r="F315" t="n">
-        <v>0.4337349397590362</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="G315" t="n">
-        <v>0.4269662921348314</v>
+        <v>0.4</v>
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>0.3911 (0.0681)</t>
+          <t>0.4359 (0.0401)</t>
         </is>
       </c>
     </row>
@@ -11732,31 +11734,31 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E316" t="n">
-        <v>0.1724137931034483</v>
+        <v>0.3125</v>
       </c>
       <c r="F316" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.4337349397590362</v>
       </c>
       <c r="G316" t="n">
-        <v>0.3384615384615385</v>
+        <v>0.4269662921348314</v>
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>0.2572 (0.0831)</t>
+          <t>0.3911 (0.0681)</t>
         </is>
       </c>
     </row>
@@ -11773,7 +11775,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
@@ -11782,17 +11784,17 @@
         </is>
       </c>
       <c r="E317" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.1724137931034483</v>
       </c>
       <c r="F317" t="n">
-        <v>0.4096385542168675</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="G317" t="n">
-        <v>0.3611111111111111</v>
+        <v>0.3384615384615385</v>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>0.3582 (0.0530)</t>
+          <t>0.2572 (0.0831)</t>
         </is>
       </c>
     </row>
@@ -11809,7 +11811,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
@@ -11818,17 +11820,17 @@
         </is>
       </c>
       <c r="E318" t="n">
-        <v>0.2</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="F318" t="n">
-        <v>0.2571428571428571</v>
+        <v>0.4096385542168675</v>
       </c>
       <c r="G318" t="n">
-        <v>0.253968253968254</v>
+        <v>0.3611111111111111</v>
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>0.2370 (0.0321)</t>
+          <t>0.3582 (0.0530)</t>
         </is>
       </c>
     </row>
@@ -11845,7 +11847,7 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -11854,17 +11856,17 @@
         </is>
       </c>
       <c r="E319" t="n">
-        <v>0.4489795918367347</v>
+        <v>0.2</v>
       </c>
       <c r="F319" t="n">
-        <v>0.4395604395604396</v>
+        <v>0.2571428571428571</v>
       </c>
       <c r="G319" t="n">
-        <v>0.4594594594594595</v>
+        <v>0.253968253968254</v>
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>0.4493 (0.0100)</t>
+          <t>0.2370 (0.0321)</t>
         </is>
       </c>
     </row>
@@ -11881,7 +11883,7 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -11890,17 +11892,17 @@
         </is>
       </c>
       <c r="E320" t="n">
-        <v>0.1153846153846154</v>
+        <v>0.4489795918367347</v>
       </c>
       <c r="F320" t="n">
-        <v>0.125</v>
+        <v>0.4395604395604396</v>
       </c>
       <c r="G320" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.4594594594594595</v>
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>0.1771 (0.0987)</t>
+          <t>0.4493 (0.0100)</t>
         </is>
       </c>
     </row>
@@ -11912,31 +11914,31 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E321" t="n">
-        <v>0.2253521126760563</v>
+        <v>0.1153846153846154</v>
       </c>
       <c r="F321" t="n">
-        <v>0.3188405797101449</v>
+        <v>0.125</v>
       </c>
       <c r="G321" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>0.3203 (0.0957)</t>
+          <t>0.1771 (0.0987)</t>
         </is>
       </c>
     </row>
@@ -11953,7 +11955,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -11962,17 +11964,17 @@
         </is>
       </c>
       <c r="E322" t="n">
-        <v>0.3296703296703297</v>
+        <v>0.2253521126760563</v>
       </c>
       <c r="F322" t="n">
-        <v>0.4871794871794872</v>
+        <v>0.3188405797101449</v>
       </c>
       <c r="G322" t="n">
-        <v>0.4137931034482759</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t>0.4102 (0.0788)</t>
+          <t>0.3203 (0.0957)</t>
         </is>
       </c>
     </row>
@@ -11989,7 +11991,7 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
@@ -11998,17 +12000,17 @@
         </is>
       </c>
       <c r="E323" t="n">
-        <v>0.3294117647058823</v>
+        <v>0.3296703296703297</v>
       </c>
       <c r="F323" t="n">
-        <v>0.3544303797468354</v>
+        <v>0.4871794871794872</v>
       </c>
       <c r="G323" t="n">
-        <v>0.3188405797101449</v>
+        <v>0.4137931034482759</v>
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>0.3342 (0.0183)</t>
+          <t>0.4102 (0.0788)</t>
         </is>
       </c>
     </row>
@@ -12025,7 +12027,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
@@ -12034,17 +12036,17 @@
         </is>
       </c>
       <c r="E324" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.3294117647058823</v>
       </c>
       <c r="F324" t="n">
-        <v>0.358974358974359</v>
+        <v>0.3544303797468354</v>
       </c>
       <c r="G324" t="n">
-        <v>0.4810126582278481</v>
+        <v>0.3188405797101449</v>
       </c>
       <c r="H324" t="inlineStr">
         <is>
-          <t>0.3949 (0.0749)</t>
+          <t>0.3342 (0.0183)</t>
         </is>
       </c>
     </row>
@@ -12061,7 +12063,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
@@ -12070,53 +12072,53 @@
         </is>
       </c>
       <c r="E325" t="n">
-        <v>0.2777777777777778</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="F325" t="n">
-        <v>0.360655737704918</v>
+        <v>0.358974358974359</v>
       </c>
       <c r="G325" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.4810126582278481</v>
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t>0.3278 (0.0440)</t>
+          <t>0.3949 (0.0749)</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>BSK_hDFCGF_VCAM1</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E326" t="n">
-        <v>0</v>
+        <v>0.2777777777777778</v>
       </c>
       <c r="F326" t="n">
-        <v>0</v>
+        <v>0.360655737704918</v>
       </c>
       <c r="G326" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.3278 (0.0440)</t>
         </is>
       </c>
     </row>
@@ -12133,7 +12135,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
@@ -12148,11 +12150,11 @@
         <v>0</v>
       </c>
       <c r="G327" t="n">
-        <v>1</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -12169,7 +12171,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
@@ -12181,14 +12183,14 @@
         <v>0</v>
       </c>
       <c r="F328" t="n">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="G328" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -12205,7 +12207,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
@@ -12217,14 +12219,14 @@
         <v>0</v>
       </c>
       <c r="F329" t="n">
-        <v>0.25</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G329" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t>0.1944 (0.1735)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -12241,7 +12243,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
@@ -12253,14 +12255,14 @@
         <v>0</v>
       </c>
       <c r="F330" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G330" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.1944 (0.1735)</t>
         </is>
       </c>
     </row>
@@ -12272,17 +12274,17 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E331" t="n">
@@ -12292,11 +12294,11 @@
         <v>0</v>
       </c>
       <c r="G331" t="n">
-        <v>1</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H331" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -12313,7 +12315,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
@@ -12328,11 +12330,11 @@
         <v>0</v>
       </c>
       <c r="G332" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H332" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -12349,7 +12351,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
@@ -12364,11 +12366,11 @@
         <v>0</v>
       </c>
       <c r="G333" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -12385,7 +12387,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
@@ -12421,7 +12423,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
@@ -12436,11 +12438,11 @@
         <v>0</v>
       </c>
       <c r="G335" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.2222 (0.3849)</t>
         </is>
       </c>
     </row>
@@ -12452,17 +12454,17 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E336" t="n">
@@ -12472,11 +12474,151 @@
         <v>0</v>
       </c>
       <c r="G336" t="n">
+        <v>1</v>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E337" t="n">
+        <v>0</v>
+      </c>
+      <c r="F337" t="n">
+        <v>0</v>
+      </c>
+      <c r="G337" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="H336" t="inlineStr">
+      <c r="H337" t="inlineStr">
         <is>
           <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E338" t="n">
+        <v>0</v>
+      </c>
+      <c r="F338" t="n">
+        <v>0</v>
+      </c>
+      <c r="G338" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E339" t="n">
+        <v>0</v>
+      </c>
+      <c r="F339" t="n">
+        <v>0</v>
+      </c>
+      <c r="G339" t="inlineStr"/>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>0.0000 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E340" t="n">
+        <v>0</v>
+      </c>
+      <c r="F340" t="n">
+        <v>0</v>
+      </c>
+      <c r="G340" t="inlineStr"/>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>0.0000 (0.0000)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 08:32:23)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H340"/>
+  <dimension ref="A1:H355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8852,11 +8852,13 @@
       <c r="E235" t="n">
         <v>0.4262295081967213</v>
       </c>
-      <c r="F235" t="inlineStr"/>
+      <c r="F235" t="n">
+        <v>0.4927536231884058</v>
+      </c>
       <c r="G235" t="inlineStr"/>
       <c r="H235" t="inlineStr">
         <is>
-          <t>0.4262 (0.0000)</t>
+          <t>0.4595 (0.0470)</t>
         </is>
       </c>
     </row>
@@ -8916,11 +8918,13 @@
       <c r="E237" t="n">
         <v>0.2318840579710145</v>
       </c>
-      <c r="F237" t="inlineStr"/>
+      <c r="F237" t="n">
+        <v>0.4651162790697674</v>
+      </c>
       <c r="G237" t="inlineStr"/>
       <c r="H237" t="inlineStr">
         <is>
-          <t>0.2319 (0.0000)</t>
+          <t>0.3485 (0.1649)</t>
         </is>
       </c>
     </row>
@@ -9023,10 +9027,12 @@
       <c r="F240" t="n">
         <v>0.4935064935064935</v>
       </c>
-      <c r="G240" t="inlineStr"/>
+      <c r="G240" t="n">
+        <v>0.3835616438356164</v>
+      </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>0.4403 (0.0752)</t>
+          <t>0.4214 (0.0625)</t>
         </is>
       </c>
     </row>
@@ -9057,10 +9063,12 @@
       <c r="F241" t="n">
         <v>0.3611111111111111</v>
       </c>
-      <c r="G241" t="inlineStr"/>
+      <c r="G241" t="n">
+        <v>0.3333333333333333</v>
+      </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>0.2758 (0.1207)</t>
+          <t>0.2950 (0.0916)</t>
         </is>
       </c>
     </row>
@@ -11575,10 +11583,12 @@
       <c r="F311" t="n">
         <v>0.1851851851851852</v>
       </c>
-      <c r="G311" t="inlineStr"/>
+      <c r="G311" t="n">
+        <v>0.2222222222222222</v>
+      </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>0.2544 (0.0978)</t>
+          <t>0.2436 (0.0716)</t>
         </is>
       </c>
     </row>
@@ -12125,7 +12135,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -12135,7 +12145,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
@@ -12144,24 +12154,24 @@
         </is>
       </c>
       <c r="E327" t="n">
-        <v>0</v>
+        <v>0.5074626865671642</v>
       </c>
       <c r="F327" t="n">
-        <v>0</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G327" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.6391752577319587</v>
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5658 (0.0671)</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -12171,7 +12181,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
@@ -12180,24 +12190,24 @@
         </is>
       </c>
       <c r="E328" t="n">
-        <v>0</v>
+        <v>0.6736842105263158</v>
       </c>
       <c r="F328" t="n">
-        <v>0</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="G328" t="n">
-        <v>1</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.6502 (0.0208)</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
@@ -12207,7 +12217,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
@@ -12216,24 +12226,20 @@
         </is>
       </c>
       <c r="E329" t="n">
-        <v>0</v>
-      </c>
-      <c r="F329" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="G329" t="n">
-        <v>0.4</v>
-      </c>
+        <v>0.6741573033707865</v>
+      </c>
+      <c r="F329" t="inlineStr"/>
+      <c r="G329" t="inlineStr"/>
       <c r="H329" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.6742 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
@@ -12243,7 +12249,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
@@ -12252,17 +12258,13 @@
         </is>
       </c>
       <c r="E330" t="n">
-        <v>0</v>
-      </c>
-      <c r="F330" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G330" t="n">
-        <v>0.3333333333333333</v>
-      </c>
+        <v>0.5263157894736842</v>
+      </c>
+      <c r="F330" t="inlineStr"/>
+      <c r="G330" t="inlineStr"/>
       <c r="H330" t="inlineStr">
         <is>
-          <t>0.1944 (0.1735)</t>
+          <t>0.5263 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12279,7 +12281,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
@@ -12310,17 +12312,17 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E332" t="n">
@@ -12346,31 +12348,31 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E333" t="n">
         <v>0</v>
       </c>
       <c r="F333" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G333" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -12382,31 +12384,31 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E334" t="n">
         <v>0</v>
       </c>
       <c r="F334" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G334" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H334" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1944 (0.1735)</t>
         </is>
       </c>
     </row>
@@ -12418,17 +12420,17 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E335" t="n">
@@ -12438,11 +12440,11 @@
         <v>0</v>
       </c>
       <c r="G335" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -12454,17 +12456,17 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E336" t="n">
@@ -12473,12 +12475,10 @@
       <c r="F336" t="n">
         <v>0</v>
       </c>
-      <c r="G336" t="n">
-        <v>1</v>
-      </c>
+      <c r="G336" t="inlineStr"/>
       <c r="H336" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.0000 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12490,7 +12490,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -12500,21 +12500,21 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E337" t="n">
         <v>0</v>
       </c>
       <c r="F337" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G337" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -12526,7 +12526,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -12536,7 +12536,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E338" t="n">
@@ -12546,11 +12546,11 @@
         <v>0</v>
       </c>
       <c r="G338" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -12562,7 +12562,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E339" t="n">
@@ -12596,7 +12596,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -12606,7 +12606,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E340" t="n">
@@ -12619,6 +12619,544 @@
       <c r="H340" t="inlineStr">
         <is>
           <t>0.0000 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E341" t="n">
+        <v>0</v>
+      </c>
+      <c r="F341" t="n">
+        <v>0</v>
+      </c>
+      <c r="G341" t="inlineStr"/>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>0.0000 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E342" t="n">
+        <v>0</v>
+      </c>
+      <c r="F342" t="n">
+        <v>0</v>
+      </c>
+      <c r="G342" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>0.1333 (0.2309)</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E343" t="n">
+        <v>0</v>
+      </c>
+      <c r="F343" t="n">
+        <v>0</v>
+      </c>
+      <c r="G343" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>0.1333 (0.2309)</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E344" t="n">
+        <v>0</v>
+      </c>
+      <c r="F344" t="n">
+        <v>0</v>
+      </c>
+      <c r="G344" t="n">
+        <v>0</v>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>0.0000 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E345" t="n">
+        <v>0</v>
+      </c>
+      <c r="F345" t="n">
+        <v>0</v>
+      </c>
+      <c r="G345" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E346" t="n">
+        <v>0</v>
+      </c>
+      <c r="F346" t="n">
+        <v>0</v>
+      </c>
+      <c r="G346" t="n">
+        <v>1</v>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E347" t="n">
+        <v>0</v>
+      </c>
+      <c r="F347" t="n">
+        <v>0</v>
+      </c>
+      <c r="G347" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E348" t="n">
+        <v>0</v>
+      </c>
+      <c r="F348" t="n">
+        <v>0</v>
+      </c>
+      <c r="G348" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E349" t="n">
+        <v>0</v>
+      </c>
+      <c r="F349" t="n">
+        <v>0</v>
+      </c>
+      <c r="G349" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E350" t="n">
+        <v>0</v>
+      </c>
+      <c r="F350" t="n">
+        <v>0</v>
+      </c>
+      <c r="G350" t="n">
+        <v>1</v>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E351" t="n">
+        <v>0</v>
+      </c>
+      <c r="F351" t="n">
+        <v>0</v>
+      </c>
+      <c r="G351" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E352" t="n">
+        <v>0</v>
+      </c>
+      <c r="F352" t="n">
+        <v>0</v>
+      </c>
+      <c r="G352" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E353" t="n">
+        <v>0</v>
+      </c>
+      <c r="F353" t="n">
+        <v>0</v>
+      </c>
+      <c r="G353" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E354" t="n">
+        <v>0</v>
+      </c>
+      <c r="F354" t="n">
+        <v>0</v>
+      </c>
+      <c r="G354" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>0.1111 (0.1925)</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E355" t="n">
+        <v>0</v>
+      </c>
+      <c r="F355" t="n">
+        <v>0</v>
+      </c>
+      <c r="G355" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 09:32:43)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H355"/>
+  <dimension ref="A1:H369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8748,11 +8748,13 @@
       <c r="E232" t="n">
         <v>0.2264150943396226</v>
       </c>
-      <c r="F232" t="inlineStr"/>
+      <c r="F232" t="n">
+        <v>0.4137931034482759</v>
+      </c>
       <c r="G232" t="inlineStr"/>
       <c r="H232" t="inlineStr">
         <is>
-          <t>0.2264 (0.0000)</t>
+          <t>0.3201 (0.1325)</t>
         </is>
       </c>
     </row>
@@ -8855,10 +8857,12 @@
       <c r="F235" t="n">
         <v>0.4927536231884058</v>
       </c>
-      <c r="G235" t="inlineStr"/>
+      <c r="G235" t="n">
+        <v>0.3714285714285714</v>
+      </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>0.4595 (0.0470)</t>
+          <t>0.4301 (0.0608)</t>
         </is>
       </c>
     </row>
@@ -8921,10 +8925,12 @@
       <c r="F237" t="n">
         <v>0.4651162790697674</v>
       </c>
-      <c r="G237" t="inlineStr"/>
+      <c r="G237" t="n">
+        <v>0.4473684210526316</v>
+      </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>0.3485 (0.1649)</t>
+          <t>0.3815 (0.1298)</t>
         </is>
       </c>
     </row>
@@ -12145,7 +12151,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
@@ -12154,17 +12160,17 @@
         </is>
       </c>
       <c r="E327" t="n">
-        <v>0.5074626865671642</v>
+        <v>0.6486486486486487</v>
       </c>
       <c r="F327" t="n">
-        <v>0.5507246376811594</v>
+        <v>0.5</v>
       </c>
       <c r="G327" t="n">
-        <v>0.6391752577319587</v>
+        <v>0.6129032258064516</v>
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>0.5658 (0.0671)</t>
+          <t>0.5872 (0.0776)</t>
         </is>
       </c>
     </row>
@@ -12181,7 +12187,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
@@ -12190,17 +12196,17 @@
         </is>
       </c>
       <c r="E328" t="n">
-        <v>0.6736842105263158</v>
+        <v>0.5074626865671642</v>
       </c>
       <c r="F328" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G328" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.6391752577319587</v>
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>0.6502 (0.0208)</t>
+          <t>0.5658 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -12217,7 +12223,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
@@ -12226,13 +12232,17 @@
         </is>
       </c>
       <c r="E329" t="n">
-        <v>0.6741573033707865</v>
-      </c>
-      <c r="F329" t="inlineStr"/>
-      <c r="G329" t="inlineStr"/>
+        <v>0.6736842105263158</v>
+      </c>
+      <c r="F329" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="G329" t="n">
+        <v>0.6341463414634146</v>
+      </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t>0.6742 (0.0000)</t>
+          <t>0.6502 (0.0208)</t>
         </is>
       </c>
     </row>
@@ -12249,7 +12259,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
@@ -12258,20 +12268,24 @@
         </is>
       </c>
       <c r="E330" t="n">
-        <v>0.5263157894736842</v>
-      </c>
-      <c r="F330" t="inlineStr"/>
-      <c r="G330" t="inlineStr"/>
+        <v>0.6741573033707865</v>
+      </c>
+      <c r="F330" t="n">
+        <v>0.5789473684210527</v>
+      </c>
+      <c r="G330" t="n">
+        <v>0.6744186046511628</v>
+      </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>0.5263 (0.0000)</t>
+          <t>0.6425 (0.0550)</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -12281,7 +12295,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
@@ -12290,29 +12304,29 @@
         </is>
       </c>
       <c r="E331" t="n">
-        <v>0</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="F331" t="n">
-        <v>0</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="G331" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.5901639344262295</v>
       </c>
       <c r="H331" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5817 (0.0517)</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12322,33 +12336,33 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E332" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="F332" t="n">
-        <v>0</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="G332" t="n">
-        <v>1</v>
+        <v>0.5573770491803278</v>
       </c>
       <c r="H332" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.5747 (0.0224)</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12358,409 +12372,405 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E333" t="n">
-        <v>0</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F333" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6</v>
       </c>
       <c r="G333" t="n">
-        <v>0.4</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.6026 (0.0325)</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E334" t="n">
-        <v>0</v>
+        <v>0.5822784810126582</v>
       </c>
       <c r="F334" t="n">
-        <v>0.25</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G334" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H334" t="inlineStr">
         <is>
-          <t>0.1944 (0.1735)</t>
+          <t>0.5554 (0.0248)</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E335" t="n">
-        <v>0</v>
+        <v>0.64</v>
       </c>
       <c r="F335" t="n">
-        <v>0</v>
+        <v>0.5588235294117647</v>
       </c>
       <c r="G335" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.6016 (0.0408)</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E336" t="n">
-        <v>0</v>
+        <v>0.6578947368421053</v>
       </c>
       <c r="F336" t="n">
-        <v>0</v>
-      </c>
-      <c r="G336" t="inlineStr"/>
+        <v>0.5079365079365079</v>
+      </c>
+      <c r="G336" t="n">
+        <v>0.5714285714285714</v>
+      </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>0.0000 (0.0000)</t>
+          <t>0.5791 (0.0753)</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E337" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F337" t="n">
-        <v>0.4</v>
+        <v>0.5633802816901409</v>
       </c>
       <c r="G337" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6567164179104478</v>
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.6289 (0.0570)</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E338" t="n">
-        <v>0</v>
+        <v>0.6436781609195402</v>
       </c>
       <c r="F338" t="n">
-        <v>0</v>
+        <v>0.6410256410256411</v>
       </c>
       <c r="G338" t="n">
-        <v>0.4</v>
+        <v>0.6756756756756757</v>
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.6535 (0.0193)</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E339" t="n">
-        <v>0</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F339" t="n">
-        <v>0</v>
-      </c>
-      <c r="G339" t="inlineStr"/>
+        <v>0.576271186440678</v>
+      </c>
+      <c r="G339" t="n">
+        <v>0.4150943396226415</v>
+      </c>
       <c r="H339" t="inlineStr">
         <is>
-          <t>0.0000 (0.0000)</t>
+          <t>0.5249 (0.0952)</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E340" t="n">
-        <v>0</v>
-      </c>
-      <c r="F340" t="n">
-        <v>0</v>
-      </c>
+        <v>0.5373134328358209</v>
+      </c>
+      <c r="F340" t="inlineStr"/>
       <c r="G340" t="inlineStr"/>
       <c r="H340" t="inlineStr">
         <is>
-          <t>0.0000 (0.0000)</t>
+          <t>0.5373 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E341" t="n">
-        <v>0</v>
+        <v>0.6197183098591549</v>
       </c>
       <c r="F341" t="n">
-        <v>0</v>
-      </c>
-      <c r="G341" t="inlineStr"/>
+        <v>0.5396825396825397</v>
+      </c>
+      <c r="G341" t="n">
+        <v>0.5423728813559322</v>
+      </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>0.0000 (0.0000)</t>
+          <t>0.5673 (0.0455)</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E342" t="n">
-        <v>0</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="F342" t="n">
-        <v>0</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="G342" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.5541 (0.0469)</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E343" t="n">
-        <v>0</v>
-      </c>
-      <c r="F343" t="n">
-        <v>0</v>
-      </c>
-      <c r="G343" t="n">
-        <v>0.4</v>
-      </c>
+        <v>0.675</v>
+      </c>
+      <c r="F343" t="inlineStr"/>
+      <c r="G343" t="inlineStr"/>
       <c r="H343" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.6750 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E344" t="n">
-        <v>0</v>
-      </c>
-      <c r="F344" t="n">
-        <v>0</v>
-      </c>
-      <c r="G344" t="n">
-        <v>0</v>
-      </c>
+        <v>0.5070422535211268</v>
+      </c>
+      <c r="F344" t="inlineStr"/>
+      <c r="G344" t="inlineStr"/>
       <c r="H344" t="inlineStr">
         <is>
-          <t>0.0000 (0.0000)</t>
+          <t>0.5070 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12772,17 +12782,17 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E345" t="n">
@@ -12792,11 +12802,11 @@
         <v>0</v>
       </c>
       <c r="G345" t="n">
-        <v>0.5</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -12808,17 +12818,17 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E346" t="n">
@@ -12844,31 +12854,31 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E347" t="n">
         <v>0</v>
       </c>
       <c r="F347" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G347" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -12880,31 +12890,31 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E348" t="n">
         <v>0</v>
       </c>
       <c r="F348" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G348" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1944 (0.1735)</t>
         </is>
       </c>
     </row>
@@ -12916,17 +12926,17 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E349" t="n">
@@ -12936,11 +12946,11 @@
         <v>0</v>
       </c>
       <c r="G349" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -12952,17 +12962,17 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E350" t="n">
@@ -12972,11 +12982,11 @@
         <v>0</v>
       </c>
       <c r="G350" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H350" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -12988,31 +12998,31 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E351" t="n">
         <v>0</v>
       </c>
       <c r="F351" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G351" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -13024,17 +13034,17 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E352" t="n">
@@ -13044,11 +13054,11 @@
         <v>0</v>
       </c>
       <c r="G352" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H352" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -13060,17 +13070,17 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E353" t="n">
@@ -13080,11 +13090,11 @@
         <v>0</v>
       </c>
       <c r="G353" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13106,17 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E354" t="n">
@@ -13116,11 +13126,11 @@
         <v>0</v>
       </c>
       <c r="G354" t="n">
-        <v>0.3333333333333333</v>
+        <v>1</v>
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>0.1111 (0.1925)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -13132,17 +13142,17 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E355" t="n">
@@ -13152,9 +13162,513 @@
         <v>0</v>
       </c>
       <c r="G355" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E356" t="n">
+        <v>0</v>
+      </c>
+      <c r="F356" t="n">
+        <v>0</v>
+      </c>
+      <c r="G356" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>0.1333 (0.2309)</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E357" t="n">
+        <v>0</v>
+      </c>
+      <c r="F357" t="n">
+        <v>0</v>
+      </c>
+      <c r="G357" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>0.1333 (0.2309)</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E358" t="n">
+        <v>0</v>
+      </c>
+      <c r="F358" t="n">
+        <v>0</v>
+      </c>
+      <c r="G358" t="n">
+        <v>0</v>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>0.0000 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E359" t="n">
+        <v>0</v>
+      </c>
+      <c r="F359" t="n">
+        <v>0</v>
+      </c>
+      <c r="G359" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E360" t="n">
+        <v>0</v>
+      </c>
+      <c r="F360" t="n">
+        <v>0</v>
+      </c>
+      <c r="G360" t="n">
+        <v>1</v>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E361" t="n">
+        <v>0</v>
+      </c>
+      <c r="F361" t="n">
+        <v>0</v>
+      </c>
+      <c r="G361" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E362" t="n">
+        <v>0</v>
+      </c>
+      <c r="F362" t="n">
+        <v>0</v>
+      </c>
+      <c r="G362" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="H355" t="inlineStr">
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E363" t="n">
+        <v>0</v>
+      </c>
+      <c r="F363" t="n">
+        <v>0</v>
+      </c>
+      <c r="G363" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E364" t="n">
+        <v>0</v>
+      </c>
+      <c r="F364" t="n">
+        <v>0</v>
+      </c>
+      <c r="G364" t="n">
+        <v>1</v>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E365" t="n">
+        <v>0</v>
+      </c>
+      <c r="F365" t="n">
+        <v>0</v>
+      </c>
+      <c r="G365" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E366" t="n">
+        <v>0</v>
+      </c>
+      <c r="F366" t="n">
+        <v>0</v>
+      </c>
+      <c r="G366" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E367" t="n">
+        <v>0</v>
+      </c>
+      <c r="F367" t="n">
+        <v>0</v>
+      </c>
+      <c r="G367" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E368" t="n">
+        <v>0</v>
+      </c>
+      <c r="F368" t="n">
+        <v>0</v>
+      </c>
+      <c r="G368" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>0.1111 (0.1925)</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E369" t="n">
+        <v>0</v>
+      </c>
+      <c r="F369" t="n">
+        <v>0</v>
+      </c>
+      <c r="G369" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H369" t="inlineStr">
         <is>
           <t>0.2222 (0.3849)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 10:33:05)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H369"/>
+  <dimension ref="A1:H384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8890,11 +8890,13 @@
       <c r="E236" t="n">
         <v>0.04545454545454546</v>
       </c>
-      <c r="F236" t="inlineStr"/>
+      <c r="F236" t="n">
+        <v>0.4444444444444444</v>
+      </c>
       <c r="G236" t="inlineStr"/>
       <c r="H236" t="inlineStr">
         <is>
-          <t>0.0455 (0.0000)</t>
+          <t>0.2449 (0.2821)</t>
         </is>
       </c>
     </row>
@@ -12141,7 +12143,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -12160,24 +12162,24 @@
         </is>
       </c>
       <c r="E327" t="n">
-        <v>0.6486486486486487</v>
+        <v>0.25</v>
       </c>
       <c r="F327" t="n">
-        <v>0.5</v>
+        <v>0.3243243243243243</v>
       </c>
       <c r="G327" t="n">
-        <v>0.6129032258064516</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>0.5872 (0.0776)</t>
+          <t>0.2359 (0.0963)</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -12196,24 +12198,24 @@
         </is>
       </c>
       <c r="E328" t="n">
-        <v>0.5074626865671642</v>
+        <v>0.3225806451612903</v>
       </c>
       <c r="F328" t="n">
-        <v>0.5507246376811594</v>
+        <v>0.0625</v>
       </c>
       <c r="G328" t="n">
-        <v>0.6391752577319587</v>
+        <v>0.06896551724137931</v>
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>0.5658 (0.0671)</t>
+          <t>0.1513 (0.1483)</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
@@ -12232,24 +12234,24 @@
         </is>
       </c>
       <c r="E329" t="n">
-        <v>0.6736842105263158</v>
+        <v>0.392156862745098</v>
       </c>
       <c r="F329" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.25</v>
       </c>
       <c r="G329" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t>0.6502 (0.0208)</t>
+          <t>0.2617 (0.1251)</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
@@ -12268,24 +12270,24 @@
         </is>
       </c>
       <c r="E330" t="n">
-        <v>0.6741573033707865</v>
+        <v>0.2926829268292683</v>
       </c>
       <c r="F330" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G330" t="n">
-        <v>0.6744186046511628</v>
+        <v>0.1764705882352941</v>
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>0.6425 (0.0550)</t>
+          <t>0.2846 (0.1043)</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -12304,29 +12306,29 @@
         </is>
       </c>
       <c r="E331" t="n">
-        <v>0.5263157894736842</v>
+        <v>0.1875</v>
       </c>
       <c r="F331" t="n">
-        <v>0.6285714285714286</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="G331" t="n">
-        <v>0.5901639344262295</v>
+        <v>0.125</v>
       </c>
       <c r="H331" t="inlineStr">
         <is>
-          <t>0.5817 (0.0517)</t>
+          <t>0.1412 (0.0407)</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12336,33 +12338,31 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E332" t="n">
-        <v>0.6</v>
+        <v>0.4324324324324325</v>
       </c>
       <c r="F332" t="n">
-        <v>0.5666666666666667</v>
-      </c>
-      <c r="G332" t="n">
-        <v>0.5573770491803278</v>
-      </c>
+        <v>0.16</v>
+      </c>
+      <c r="G332" t="inlineStr"/>
       <c r="H332" t="inlineStr">
         <is>
-          <t>0.5747 (0.0224)</t>
+          <t>0.2962 (0.1926)</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12372,57 +12372,49 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E333" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="F333" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G333" t="n">
-        <v>0.6363636363636364</v>
-      </c>
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="F333" t="inlineStr"/>
+      <c r="G333" t="inlineStr"/>
       <c r="H333" t="inlineStr">
         <is>
-          <t>0.6026 (0.0325)</t>
+          <t>0.2632 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E334" t="n">
-        <v>0.5822784810126582</v>
-      </c>
-      <c r="F334" t="n">
-        <v>0.5507246376811594</v>
-      </c>
-      <c r="G334" t="n">
-        <v>0.5333333333333333</v>
-      </c>
+        <v>0.3636363636363636</v>
+      </c>
+      <c r="F334" t="inlineStr"/>
+      <c r="G334" t="inlineStr"/>
       <c r="H334" t="inlineStr">
         <is>
-          <t>0.5554 (0.0248)</t>
+          <t>0.3636 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12434,7 +12426,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12444,21 +12436,21 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E335" t="n">
-        <v>0.64</v>
+        <v>0.6486486486486487</v>
       </c>
       <c r="F335" t="n">
-        <v>0.5588235294117647</v>
+        <v>0.5</v>
       </c>
       <c r="G335" t="n">
-        <v>0.6060606060606061</v>
+        <v>0.6129032258064516</v>
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>0.6016 (0.0408)</t>
+          <t>0.5872 (0.0776)</t>
         </is>
       </c>
     </row>
@@ -12470,7 +12462,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -12480,21 +12472,21 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E336" t="n">
-        <v>0.6578947368421053</v>
+        <v>0.5074626865671642</v>
       </c>
       <c r="F336" t="n">
-        <v>0.5079365079365079</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G336" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.6391752577319587</v>
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>0.5791 (0.0753)</t>
+          <t>0.5658 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -12506,7 +12498,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -12516,21 +12508,21 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E337" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6736842105263158</v>
       </c>
       <c r="F337" t="n">
-        <v>0.5633802816901409</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="G337" t="n">
-        <v>0.6567164179104478</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>0.6289 (0.0570)</t>
+          <t>0.6502 (0.0208)</t>
         </is>
       </c>
     </row>
@@ -12542,7 +12534,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -12552,21 +12544,21 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E338" t="n">
-        <v>0.6436781609195402</v>
+        <v>0.6741573033707865</v>
       </c>
       <c r="F338" t="n">
-        <v>0.6410256410256411</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="G338" t="n">
-        <v>0.6756756756756757</v>
+        <v>0.6744186046511628</v>
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>0.6535 (0.0193)</t>
+          <t>0.6425 (0.0550)</t>
         </is>
       </c>
     </row>
@@ -12578,7 +12570,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -12588,21 +12580,21 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E339" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="F339" t="n">
-        <v>0.576271186440678</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="G339" t="n">
-        <v>0.4150943396226415</v>
+        <v>0.5901639344262295</v>
       </c>
       <c r="H339" t="inlineStr">
         <is>
-          <t>0.5249 (0.0952)</t>
+          <t>0.5817 (0.0517)</t>
         </is>
       </c>
     </row>
@@ -12614,7 +12606,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -12624,17 +12616,17 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E340" t="n">
-        <v>0.5373134328358209</v>
+        <v>0.4307692307692308</v>
       </c>
       <c r="F340" t="inlineStr"/>
       <c r="G340" t="inlineStr"/>
       <c r="H340" t="inlineStr">
         <is>
-          <t>0.5373 (0.0000)</t>
+          <t>0.4308 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12646,7 +12638,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -12656,21 +12648,21 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E341" t="n">
-        <v>0.6197183098591549</v>
+        <v>0.6</v>
       </c>
       <c r="F341" t="n">
-        <v>0.5396825396825397</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="G341" t="n">
-        <v>0.5423728813559322</v>
+        <v>0.5573770491803278</v>
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>0.5673 (0.0455)</t>
+          <t>0.5747 (0.0224)</t>
         </is>
       </c>
     </row>
@@ -12682,7 +12674,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -12692,21 +12684,21 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E342" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F342" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.6</v>
       </c>
       <c r="G342" t="n">
-        <v>0.5</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t>0.5541 (0.0469)</t>
+          <t>0.6026 (0.0325)</t>
         </is>
       </c>
     </row>
@@ -12718,7 +12710,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -12728,17 +12720,19 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E343" t="n">
-        <v>0.675</v>
-      </c>
-      <c r="F343" t="inlineStr"/>
+        <v>0.6279069767441861</v>
+      </c>
+      <c r="F343" t="n">
+        <v>0.5555555555555556</v>
+      </c>
       <c r="G343" t="inlineStr"/>
       <c r="H343" t="inlineStr">
         <is>
-          <t>0.6750 (0.0000)</t>
+          <t>0.5917 (0.0512)</t>
         </is>
       </c>
     </row>
@@ -12750,7 +12744,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -12760,29 +12754,29 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E344" t="n">
-        <v>0.5070422535211268</v>
+        <v>0.5915492957746479</v>
       </c>
       <c r="F344" t="inlineStr"/>
       <c r="G344" t="inlineStr"/>
       <c r="H344" t="inlineStr">
         <is>
-          <t>0.5070 (0.0000)</t>
+          <t>0.5915 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -12792,33 +12786,29 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E345" t="n">
-        <v>0</v>
-      </c>
-      <c r="F345" t="n">
-        <v>0</v>
-      </c>
-      <c r="G345" t="n">
-        <v>0.2857142857142857</v>
-      </c>
+        <v>0.5079365079365079</v>
+      </c>
+      <c r="F345" t="inlineStr"/>
+      <c r="G345" t="inlineStr"/>
       <c r="H345" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5079 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -12828,33 +12818,33 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E346" t="n">
-        <v>0</v>
+        <v>0.5822784810126582</v>
       </c>
       <c r="F346" t="n">
-        <v>0</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G346" t="n">
-        <v>1</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.5554 (0.0248)</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -12864,33 +12854,33 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E347" t="n">
-        <v>0</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="F347" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="G347" t="n">
-        <v>0.4</v>
+        <v>0.53125</v>
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.6157 (0.0770)</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -12900,33 +12890,31 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E348" t="n">
-        <v>0</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="F348" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G348" t="n">
-        <v>0.3333333333333333</v>
-      </c>
+        <v>0.5753424657534246</v>
+      </c>
+      <c r="G348" t="inlineStr"/>
       <c r="H348" t="inlineStr">
         <is>
-          <t>0.1944 (0.1735)</t>
+          <t>0.6091 (0.0477)</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -12936,33 +12924,33 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E349" t="n">
-        <v>0</v>
+        <v>0.631578947368421</v>
       </c>
       <c r="F349" t="n">
-        <v>0</v>
+        <v>0.6268656716417911</v>
       </c>
       <c r="G349" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5943 (0.0605)</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -12972,33 +12960,33 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E350" t="n">
-        <v>0</v>
+        <v>0.64</v>
       </c>
       <c r="F350" t="n">
-        <v>0</v>
+        <v>0.5588235294117647</v>
       </c>
       <c r="G350" t="n">
-        <v>0.5</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="H350" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.6016 (0.0408)</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -13008,33 +12996,33 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E351" t="n">
-        <v>0</v>
+        <v>0.6578947368421053</v>
       </c>
       <c r="F351" t="n">
-        <v>0.4</v>
+        <v>0.5079365079365079</v>
       </c>
       <c r="G351" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.5791 (0.0753)</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -13044,33 +13032,33 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E352" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F352" t="n">
-        <v>0</v>
+        <v>0.5633802816901409</v>
       </c>
       <c r="G352" t="n">
-        <v>0.4</v>
+        <v>0.6567164179104478</v>
       </c>
       <c r="H352" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.6289 (0.0570)</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -13080,33 +13068,33 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E353" t="n">
-        <v>0</v>
+        <v>0.6436781609195402</v>
       </c>
       <c r="F353" t="n">
-        <v>0</v>
+        <v>0.6410256410256411</v>
       </c>
       <c r="G353" t="n">
-        <v>0.4</v>
+        <v>0.6756756756756757</v>
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.6535 (0.0193)</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -13116,33 +13104,33 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E354" t="n">
-        <v>0</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F354" t="n">
-        <v>0</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="G354" t="n">
-        <v>1</v>
+        <v>0.4150943396226415</v>
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.5249 (0.0952)</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -13152,33 +13140,33 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E355" t="n">
-        <v>0</v>
+        <v>0.5373134328358209</v>
       </c>
       <c r="F355" t="n">
-        <v>0</v>
+        <v>0.4918032786885246</v>
       </c>
       <c r="G355" t="n">
-        <v>0.5</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.5351 (0.0423)</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -13188,33 +13176,33 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E356" t="n">
-        <v>0</v>
+        <v>0.6197183098591549</v>
       </c>
       <c r="F356" t="n">
-        <v>0</v>
+        <v>0.5396825396825397</v>
       </c>
       <c r="G356" t="n">
-        <v>0.4</v>
+        <v>0.5423728813559322</v>
       </c>
       <c r="H356" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.5673 (0.0455)</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -13224,33 +13212,33 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E357" t="n">
-        <v>0</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="F357" t="n">
-        <v>0</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="G357" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.5541 (0.0469)</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -13260,33 +13248,33 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E358" t="n">
-        <v>0</v>
+        <v>0.675</v>
       </c>
       <c r="F358" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G358" t="n">
-        <v>0</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H358" t="inlineStr">
         <is>
-          <t>0.0000 (0.0000)</t>
+          <t>0.6028 (0.0709)</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -13296,21 +13284,21 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E359" t="n">
-        <v>0</v>
+        <v>0.5070422535211268</v>
       </c>
       <c r="F359" t="n">
-        <v>0</v>
+        <v>0.5806451612903226</v>
       </c>
       <c r="G359" t="n">
-        <v>0.5</v>
+        <v>0.4528301886792453</v>
       </c>
       <c r="H359" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.5135 (0.0642)</t>
         </is>
       </c>
     </row>
@@ -13322,7 +13310,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -13332,7 +13320,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E360" t="n">
@@ -13342,11 +13330,11 @@
         <v>0</v>
       </c>
       <c r="G360" t="n">
-        <v>1</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H360" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -13358,7 +13346,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -13368,7 +13356,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E361" t="n">
@@ -13378,11 +13366,11 @@
         <v>0</v>
       </c>
       <c r="G361" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -13394,7 +13382,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -13404,21 +13392,21 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E362" t="n">
         <v>0</v>
       </c>
       <c r="F362" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G362" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H362" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -13430,7 +13418,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -13440,21 +13428,21 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E363" t="n">
         <v>0</v>
       </c>
       <c r="F363" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G363" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1944 (0.1735)</t>
         </is>
       </c>
     </row>
@@ -13466,7 +13454,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -13476,7 +13464,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E364" t="n">
@@ -13486,11 +13474,11 @@
         <v>0</v>
       </c>
       <c r="G364" t="n">
-        <v>1</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H364" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -13502,7 +13490,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -13512,7 +13500,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E365" t="n">
@@ -13522,11 +13510,11 @@
         <v>0</v>
       </c>
       <c r="G365" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="H365" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -13538,7 +13526,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -13548,21 +13536,21 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E366" t="n">
         <v>0</v>
       </c>
       <c r="F366" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G366" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="H366" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -13574,7 +13562,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -13584,7 +13572,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E367" t="n">
@@ -13594,11 +13582,11 @@
         <v>0</v>
       </c>
       <c r="G367" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -13610,7 +13598,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -13620,7 +13608,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E368" t="n">
@@ -13630,11 +13618,11 @@
         <v>0</v>
       </c>
       <c r="G368" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>0.1111 (0.1925)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -13646,7 +13634,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -13656,7 +13644,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E369" t="n">
@@ -13666,9 +13654,549 @@
         <v>0</v>
       </c>
       <c r="G369" t="n">
+        <v>1</v>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E370" t="n">
+        <v>0</v>
+      </c>
+      <c r="F370" t="n">
+        <v>0</v>
+      </c>
+      <c r="G370" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E371" t="n">
+        <v>0</v>
+      </c>
+      <c r="F371" t="n">
+        <v>0</v>
+      </c>
+      <c r="G371" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>0.1333 (0.2309)</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E372" t="n">
+        <v>0</v>
+      </c>
+      <c r="F372" t="n">
+        <v>0</v>
+      </c>
+      <c r="G372" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>0.1333 (0.2309)</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E373" t="n">
+        <v>0</v>
+      </c>
+      <c r="F373" t="n">
+        <v>0</v>
+      </c>
+      <c r="G373" t="n">
+        <v>0</v>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>0.0000 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E374" t="n">
+        <v>0</v>
+      </c>
+      <c r="F374" t="n">
+        <v>0</v>
+      </c>
+      <c r="G374" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E375" t="n">
+        <v>0</v>
+      </c>
+      <c r="F375" t="n">
+        <v>0</v>
+      </c>
+      <c r="G375" t="n">
+        <v>1</v>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E376" t="n">
+        <v>0</v>
+      </c>
+      <c r="F376" t="n">
+        <v>0</v>
+      </c>
+      <c r="G376" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E377" t="n">
+        <v>0</v>
+      </c>
+      <c r="F377" t="n">
+        <v>0</v>
+      </c>
+      <c r="G377" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="H369" t="inlineStr">
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E378" t="n">
+        <v>0</v>
+      </c>
+      <c r="F378" t="n">
+        <v>0</v>
+      </c>
+      <c r="G378" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E379" t="n">
+        <v>0</v>
+      </c>
+      <c r="F379" t="n">
+        <v>0</v>
+      </c>
+      <c r="G379" t="n">
+        <v>1</v>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E380" t="n">
+        <v>0</v>
+      </c>
+      <c r="F380" t="n">
+        <v>0</v>
+      </c>
+      <c r="G380" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E381" t="n">
+        <v>0</v>
+      </c>
+      <c r="F381" t="n">
+        <v>0</v>
+      </c>
+      <c r="G381" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E382" t="n">
+        <v>0</v>
+      </c>
+      <c r="F382" t="n">
+        <v>0</v>
+      </c>
+      <c r="G382" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E383" t="n">
+        <v>0</v>
+      </c>
+      <c r="F383" t="n">
+        <v>0</v>
+      </c>
+      <c r="G383" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>0.1111 (0.1925)</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E384" t="n">
+        <v>0</v>
+      </c>
+      <c r="F384" t="n">
+        <v>0</v>
+      </c>
+      <c r="G384" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H384" t="inlineStr">
         <is>
           <t>0.2222 (0.3849)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 11:33:27)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H384"/>
+  <dimension ref="A1:H393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8751,10 +8751,12 @@
       <c r="F232" t="n">
         <v>0.4137931034482759</v>
       </c>
-      <c r="G232" t="inlineStr"/>
+      <c r="G232" t="n">
+        <v>0.3508771929824561</v>
+      </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>0.3201 (0.1325)</t>
+          <t>0.3304 (0.0954)</t>
         </is>
       </c>
     </row>
@@ -12328,7 +12330,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12338,19 +12340,21 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E332" t="n">
-        <v>0.4324324324324325</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="F332" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="G332" t="inlineStr"/>
+        <v>0.125</v>
+      </c>
+      <c r="G332" t="n">
+        <v>0</v>
+      </c>
       <c r="H332" t="inlineStr">
         <is>
-          <t>0.2962 (0.1926)</t>
+          <t>0.1629 (0.1848)</t>
         </is>
       </c>
     </row>
@@ -12362,7 +12366,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12372,17 +12376,17 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E333" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.3</v>
       </c>
       <c r="F333" t="inlineStr"/>
       <c r="G333" t="inlineStr"/>
       <c r="H333" t="inlineStr">
         <is>
-          <t>0.2632 (0.0000)</t>
+          <t>0.3000 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12399,7 +12403,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
@@ -12408,331 +12412,329 @@
         </is>
       </c>
       <c r="E334" t="n">
-        <v>0.3636363636363636</v>
-      </c>
-      <c r="F334" t="inlineStr"/>
-      <c r="G334" t="inlineStr"/>
+        <v>0.3125</v>
+      </c>
+      <c r="F334" t="n">
+        <v>0</v>
+      </c>
+      <c r="G334" t="n">
+        <v>0</v>
+      </c>
       <c r="H334" t="inlineStr">
         <is>
-          <t>0.3636 (0.0000)</t>
+          <t>0.1042 (0.1804)</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E335" t="n">
-        <v>0.6486486486486487</v>
+        <v>0.4324324324324325</v>
       </c>
       <c r="F335" t="n">
-        <v>0.5</v>
+        <v>0.16</v>
       </c>
       <c r="G335" t="n">
-        <v>0.6129032258064516</v>
+        <v>0</v>
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>0.5872 (0.0776)</t>
+          <t>0.1975 (0.2186)</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E336" t="n">
-        <v>0.5074626865671642</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F336" t="n">
-        <v>0.5507246376811594</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="G336" t="n">
-        <v>0.6391752577319587</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>0.5658 (0.0671)</t>
+          <t>0.1498 (0.0982)</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E337" t="n">
-        <v>0.6736842105263158</v>
+        <v>0.4680851063829787</v>
       </c>
       <c r="F337" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.3225806451612903</v>
       </c>
       <c r="G337" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.1052631578947368</v>
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>0.6502 (0.0208)</t>
+          <t>0.2986 (0.1826)</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E338" t="n">
-        <v>0.6741573033707865</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="F338" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="G338" t="n">
-        <v>0.6744186046511628</v>
+        <v>0</v>
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>0.6425 (0.0550)</t>
+          <t>0.1953 (0.1833)</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E339" t="n">
-        <v>0.5263157894736842</v>
-      </c>
-      <c r="F339" t="n">
-        <v>0.6285714285714286</v>
-      </c>
-      <c r="G339" t="n">
-        <v>0.5901639344262295</v>
-      </c>
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="F339" t="inlineStr"/>
+      <c r="G339" t="inlineStr"/>
       <c r="H339" t="inlineStr">
         <is>
-          <t>0.5817 (0.0517)</t>
+          <t>0.3448 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E340" t="n">
-        <v>0.4307692307692308</v>
-      </c>
-      <c r="F340" t="inlineStr"/>
-      <c r="G340" t="inlineStr"/>
+        <v>0.3529411764705883</v>
+      </c>
+      <c r="F340" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="G340" t="n">
+        <v>0</v>
+      </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>0.4308 (0.0000)</t>
+          <t>0.1593 (0.1790)</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E341" t="n">
-        <v>0.6</v>
+        <v>0.3157894736842105</v>
       </c>
       <c r="F341" t="n">
-        <v>0.5666666666666667</v>
+        <v>0</v>
       </c>
       <c r="G341" t="n">
-        <v>0.5573770491803278</v>
+        <v>0</v>
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>0.5747 (0.0224)</t>
+          <t>0.1053 (0.1823)</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E342" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="F342" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G342" t="n">
-        <v>0.6363636363636364</v>
-      </c>
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="F342" t="inlineStr"/>
+      <c r="G342" t="inlineStr"/>
       <c r="H342" t="inlineStr">
         <is>
-          <t>0.6026 (0.0325)</t>
+          <t>0.3448 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E343" t="n">
-        <v>0.6279069767441861</v>
-      </c>
-      <c r="F343" t="n">
-        <v>0.5555555555555556</v>
-      </c>
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F343" t="inlineStr"/>
       <c r="G343" t="inlineStr"/>
       <c r="H343" t="inlineStr">
         <is>
-          <t>0.5917 (0.0512)</t>
+          <t>0.3333 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12744,27 +12746,31 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E344" t="n">
-        <v>0.5915492957746479</v>
-      </c>
-      <c r="F344" t="inlineStr"/>
-      <c r="G344" t="inlineStr"/>
+        <v>0.6486486486486487</v>
+      </c>
+      <c r="F344" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G344" t="n">
+        <v>0.6129032258064516</v>
+      </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t>0.5915 (0.0000)</t>
+          <t>0.5872 (0.0776)</t>
         </is>
       </c>
     </row>
@@ -12776,27 +12782,31 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E345" t="n">
-        <v>0.5079365079365079</v>
-      </c>
-      <c r="F345" t="inlineStr"/>
-      <c r="G345" t="inlineStr"/>
+        <v>0.5074626865671642</v>
+      </c>
+      <c r="F345" t="n">
+        <v>0.5507246376811594</v>
+      </c>
+      <c r="G345" t="n">
+        <v>0.6391752577319587</v>
+      </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>0.5079 (0.0000)</t>
+          <t>0.5658 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -12808,31 +12818,31 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E346" t="n">
-        <v>0.5822784810126582</v>
+        <v>0.6736842105263158</v>
       </c>
       <c r="F346" t="n">
-        <v>0.5507246376811594</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="G346" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>0.5554 (0.0248)</t>
+          <t>0.6502 (0.0208)</t>
         </is>
       </c>
     </row>
@@ -12844,31 +12854,31 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E347" t="n">
-        <v>0.6818181818181818</v>
+        <v>0.6741573033707865</v>
       </c>
       <c r="F347" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="G347" t="n">
-        <v>0.53125</v>
+        <v>0.6744186046511628</v>
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>0.6157 (0.0770)</t>
+          <t>0.6425 (0.0550)</t>
         </is>
       </c>
     </row>
@@ -12880,29 +12890,31 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E348" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="F348" t="n">
-        <v>0.5753424657534246</v>
-      </c>
-      <c r="G348" t="inlineStr"/>
+        <v>0.6285714285714286</v>
+      </c>
+      <c r="G348" t="n">
+        <v>0.5901639344262295</v>
+      </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>0.6091 (0.0477)</t>
+          <t>0.5817 (0.0517)</t>
         </is>
       </c>
     </row>
@@ -12914,31 +12926,29 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E349" t="n">
-        <v>0.631578947368421</v>
+        <v>0.4307692307692308</v>
       </c>
       <c r="F349" t="n">
-        <v>0.6268656716417911</v>
-      </c>
-      <c r="G349" t="n">
-        <v>0.5245901639344263</v>
-      </c>
+        <v>0.6</v>
+      </c>
+      <c r="G349" t="inlineStr"/>
       <c r="H349" t="inlineStr">
         <is>
-          <t>0.5943 (0.0605)</t>
+          <t>0.5154 (0.1197)</t>
         </is>
       </c>
     </row>
@@ -12950,31 +12960,31 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E350" t="n">
-        <v>0.64</v>
+        <v>0.6</v>
       </c>
       <c r="F350" t="n">
-        <v>0.5588235294117647</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="G350" t="n">
-        <v>0.6060606060606061</v>
+        <v>0.5573770491803278</v>
       </c>
       <c r="H350" t="inlineStr">
         <is>
-          <t>0.6016 (0.0408)</t>
+          <t>0.5747 (0.0224)</t>
         </is>
       </c>
     </row>
@@ -12986,31 +12996,31 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E351" t="n">
-        <v>0.6578947368421053</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F351" t="n">
-        <v>0.5079365079365079</v>
+        <v>0.6</v>
       </c>
       <c r="G351" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t>0.5791 (0.0753)</t>
+          <t>0.6026 (0.0325)</t>
         </is>
       </c>
     </row>
@@ -13022,31 +13032,31 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E352" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6279069767441861</v>
       </c>
       <c r="F352" t="n">
-        <v>0.5633802816901409</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="G352" t="n">
-        <v>0.6567164179104478</v>
+        <v>0.6101694915254238</v>
       </c>
       <c r="H352" t="inlineStr">
         <is>
-          <t>0.6289 (0.0570)</t>
+          <t>0.5979 (0.0377)</t>
         </is>
       </c>
     </row>
@@ -13058,31 +13068,29 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E353" t="n">
-        <v>0.6436781609195402</v>
+        <v>0.5915492957746479</v>
       </c>
       <c r="F353" t="n">
-        <v>0.6410256410256411</v>
-      </c>
-      <c r="G353" t="n">
-        <v>0.6756756756756757</v>
-      </c>
+        <v>0.4482758620689655</v>
+      </c>
+      <c r="G353" t="inlineStr"/>
       <c r="H353" t="inlineStr">
         <is>
-          <t>0.6535 (0.0193)</t>
+          <t>0.5199 (0.1013)</t>
         </is>
       </c>
     </row>
@@ -13094,31 +13102,31 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E354" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5079365079365079</v>
       </c>
       <c r="F354" t="n">
-        <v>0.576271186440678</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="G354" t="n">
-        <v>0.4150943396226415</v>
+        <v>0.5846153846153846</v>
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>0.5249 (0.0952)</t>
+          <t>0.5390 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -13130,31 +13138,31 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E355" t="n">
-        <v>0.5373134328358209</v>
+        <v>0.5822784810126582</v>
       </c>
       <c r="F355" t="n">
-        <v>0.4918032786885246</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G355" t="n">
-        <v>0.576271186440678</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t>0.5351 (0.0423)</t>
+          <t>0.5554 (0.0248)</t>
         </is>
       </c>
     </row>
@@ -13166,31 +13174,31 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E356" t="n">
-        <v>0.6197183098591549</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="F356" t="n">
-        <v>0.5396825396825397</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="G356" t="n">
-        <v>0.5423728813559322</v>
+        <v>0.53125</v>
       </c>
       <c r="H356" t="inlineStr">
         <is>
-          <t>0.5673 (0.0455)</t>
+          <t>0.6157 (0.0770)</t>
         </is>
       </c>
     </row>
@@ -13202,31 +13210,31 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E357" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="F357" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5753424657534246</v>
       </c>
       <c r="G357" t="n">
-        <v>0.5</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>0.5541 (0.0469)</t>
+          <t>0.5648 (0.0838)</t>
         </is>
       </c>
     </row>
@@ -13238,31 +13246,31 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E358" t="n">
-        <v>0.675</v>
+        <v>0.631578947368421</v>
       </c>
       <c r="F358" t="n">
-        <v>0.6</v>
+        <v>0.6268656716417911</v>
       </c>
       <c r="G358" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="H358" t="inlineStr">
         <is>
-          <t>0.6028 (0.0709)</t>
+          <t>0.5943 (0.0605)</t>
         </is>
       </c>
     </row>
@@ -13274,355 +13282,355 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E359" t="n">
-        <v>0.5070422535211268</v>
+        <v>0.64</v>
       </c>
       <c r="F359" t="n">
-        <v>0.5806451612903226</v>
+        <v>0.5588235294117647</v>
       </c>
       <c r="G359" t="n">
-        <v>0.4528301886792453</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="H359" t="inlineStr">
         <is>
-          <t>0.5135 (0.0642)</t>
+          <t>0.6016 (0.0408)</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E360" t="n">
-        <v>0</v>
+        <v>0.6578947368421053</v>
       </c>
       <c r="F360" t="n">
-        <v>0</v>
+        <v>0.5079365079365079</v>
       </c>
       <c r="G360" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="H360" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5791 (0.0753)</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E361" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F361" t="n">
-        <v>0</v>
+        <v>0.5633802816901409</v>
       </c>
       <c r="G361" t="n">
-        <v>1</v>
+        <v>0.6567164179104478</v>
       </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.6289 (0.0570)</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E362" t="n">
-        <v>0</v>
+        <v>0.6436781609195402</v>
       </c>
       <c r="F362" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6410256410256411</v>
       </c>
       <c r="G362" t="n">
-        <v>0.4</v>
+        <v>0.6756756756756757</v>
       </c>
       <c r="H362" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.6535 (0.0193)</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E363" t="n">
-        <v>0</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F363" t="n">
-        <v>0.25</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="G363" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4150943396226415</v>
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t>0.1944 (0.1735)</t>
+          <t>0.5249 (0.0952)</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E364" t="n">
-        <v>0</v>
+        <v>0.5373134328358209</v>
       </c>
       <c r="F364" t="n">
-        <v>0</v>
+        <v>0.4918032786885246</v>
       </c>
       <c r="G364" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="H364" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5351 (0.0423)</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E365" t="n">
-        <v>0</v>
+        <v>0.6197183098591549</v>
       </c>
       <c r="F365" t="n">
-        <v>0</v>
+        <v>0.5396825396825397</v>
       </c>
       <c r="G365" t="n">
-        <v>0.5</v>
+        <v>0.5423728813559322</v>
       </c>
       <c r="H365" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.5673 (0.0455)</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E366" t="n">
-        <v>0</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="F366" t="n">
-        <v>0.4</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="G366" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="H366" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.5541 (0.0469)</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E367" t="n">
-        <v>0</v>
+        <v>0.675</v>
       </c>
       <c r="F367" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G367" t="n">
-        <v>0.4</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.6028 (0.0709)</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E368" t="n">
-        <v>0</v>
+        <v>0.5070422535211268</v>
       </c>
       <c r="F368" t="n">
-        <v>0</v>
+        <v>0.5806451612903226</v>
       </c>
       <c r="G368" t="n">
-        <v>0.4</v>
+        <v>0.4528301886792453</v>
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.5135 (0.0642)</t>
         </is>
       </c>
     </row>
@@ -13634,17 +13642,17 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E369" t="n">
@@ -13654,11 +13662,11 @@
         <v>0</v>
       </c>
       <c r="G369" t="n">
-        <v>1</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -13670,17 +13678,17 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E370" t="n">
@@ -13690,11 +13698,11 @@
         <v>0</v>
       </c>
       <c r="G370" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H370" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -13706,31 +13714,31 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E371" t="n">
         <v>0</v>
       </c>
       <c r="F371" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G371" t="n">
         <v>0.4</v>
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -13742,31 +13750,31 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E372" t="n">
         <v>0</v>
       </c>
       <c r="F372" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G372" t="n">
-        <v>0.4</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.1944 (0.1735)</t>
         </is>
       </c>
     </row>
@@ -13778,17 +13786,17 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E373" t="n">
@@ -13798,11 +13806,11 @@
         <v>0</v>
       </c>
       <c r="G373" t="n">
-        <v>0</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>0.0000 (0.0000)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -13814,17 +13822,17 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E374" t="n">
@@ -13850,31 +13858,31 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E375" t="n">
         <v>0</v>
       </c>
       <c r="F375" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G375" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -13886,17 +13894,17 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E376" t="n">
@@ -13906,11 +13914,11 @@
         <v>0</v>
       </c>
       <c r="G376" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -13922,17 +13930,17 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E377" t="n">
@@ -13942,11 +13950,11 @@
         <v>0</v>
       </c>
       <c r="G377" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -13958,17 +13966,17 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E378" t="n">
@@ -13978,11 +13986,11 @@
         <v>0</v>
       </c>
       <c r="G378" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -13994,17 +14002,17 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E379" t="n">
@@ -14014,11 +14022,11 @@
         <v>0</v>
       </c>
       <c r="G379" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H379" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -14030,17 +14038,17 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D380" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E380" t="n">
@@ -14050,11 +14058,11 @@
         <v>0</v>
       </c>
       <c r="G380" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H380" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -14066,17 +14074,17 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E381" t="n">
@@ -14086,11 +14094,11 @@
         <v>0</v>
       </c>
       <c r="G381" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -14102,17 +14110,17 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E382" t="n">
@@ -14122,11 +14130,11 @@
         <v>0</v>
       </c>
       <c r="G382" t="n">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.0000 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -14138,17 +14146,17 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E383" t="n">
@@ -14158,11 +14166,11 @@
         <v>0</v>
       </c>
       <c r="G383" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="H383" t="inlineStr">
         <is>
-          <t>0.1111 (0.1925)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -14174,17 +14182,17 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E384" t="n">
@@ -14194,9 +14202,333 @@
         <v>0</v>
       </c>
       <c r="G384" t="n">
+        <v>1</v>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E385" t="n">
+        <v>0</v>
+      </c>
+      <c r="F385" t="n">
+        <v>0</v>
+      </c>
+      <c r="G385" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E386" t="n">
+        <v>0</v>
+      </c>
+      <c r="F386" t="n">
+        <v>0</v>
+      </c>
+      <c r="G386" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="H384" t="inlineStr">
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E387" t="n">
+        <v>0</v>
+      </c>
+      <c r="F387" t="n">
+        <v>0</v>
+      </c>
+      <c r="G387" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E388" t="n">
+        <v>0</v>
+      </c>
+      <c r="F388" t="n">
+        <v>0</v>
+      </c>
+      <c r="G388" t="n">
+        <v>1</v>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E389" t="n">
+        <v>0</v>
+      </c>
+      <c r="F389" t="n">
+        <v>0</v>
+      </c>
+      <c r="G389" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E390" t="n">
+        <v>0</v>
+      </c>
+      <c r="F390" t="n">
+        <v>0</v>
+      </c>
+      <c r="G390" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E391" t="n">
+        <v>0</v>
+      </c>
+      <c r="F391" t="n">
+        <v>0</v>
+      </c>
+      <c r="G391" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E392" t="n">
+        <v>0</v>
+      </c>
+      <c r="F392" t="n">
+        <v>0</v>
+      </c>
+      <c r="G392" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>0.1111 (0.1925)</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E393" t="n">
+        <v>0</v>
+      </c>
+      <c r="F393" t="n">
+        <v>0</v>
+      </c>
+      <c r="G393" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H393" t="inlineStr">
         <is>
           <t>0.2222 (0.3849)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 12:33:47)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H393"/>
+  <dimension ref="A1:H409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12335,7 +12335,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
@@ -12344,17 +12344,13 @@
         </is>
       </c>
       <c r="E332" t="n">
-        <v>0.3636363636363636</v>
-      </c>
-      <c r="F332" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="G332" t="n">
-        <v>0</v>
-      </c>
+        <v>0.3571428571428572</v>
+      </c>
+      <c r="F332" t="inlineStr"/>
+      <c r="G332" t="inlineStr"/>
       <c r="H332" t="inlineStr">
         <is>
-          <t>0.1629 (0.1848)</t>
+          <t>0.3571 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12371,7 +12367,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
@@ -12380,13 +12376,17 @@
         </is>
       </c>
       <c r="E333" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F333" t="inlineStr"/>
-      <c r="G333" t="inlineStr"/>
+        <v>0.3636363636363636</v>
+      </c>
+      <c r="F333" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0</v>
+      </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t>0.3000 (0.0000)</t>
+          <t>0.1629 (0.1848)</t>
         </is>
       </c>
     </row>
@@ -12398,21 +12398,21 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E334" t="n">
-        <v>0.3125</v>
+        <v>0.3</v>
       </c>
       <c r="F334" t="n">
         <v>0</v>
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H334" t="inlineStr">
         <is>
-          <t>0.1042 (0.1804)</t>
+          <t>0.1000 (0.1732)</t>
         </is>
       </c>
     </row>
@@ -12434,31 +12434,27 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E335" t="n">
-        <v>0.4324324324324325</v>
-      </c>
-      <c r="F335" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="G335" t="n">
-        <v>0</v>
-      </c>
+        <v>0.4242424242424243</v>
+      </c>
+      <c r="F335" t="inlineStr"/>
+      <c r="G335" t="inlineStr"/>
       <c r="H335" t="inlineStr">
         <is>
-          <t>0.1975 (0.2186)</t>
+          <t>0.4242 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12470,31 +12466,27 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E336" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F336" t="n">
-        <v>0.09090909090909091</v>
-      </c>
-      <c r="G336" t="n">
-        <v>0.09523809523809523</v>
-      </c>
+        <v>0.4117647058823529</v>
+      </c>
+      <c r="F336" t="inlineStr"/>
+      <c r="G336" t="inlineStr"/>
       <c r="H336" t="inlineStr">
         <is>
-          <t>0.1498 (0.0982)</t>
+          <t>0.4118 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12506,31 +12498,27 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E337" t="n">
-        <v>0.4680851063829787</v>
-      </c>
-      <c r="F337" t="n">
-        <v>0.3225806451612903</v>
-      </c>
-      <c r="G337" t="n">
-        <v>0.1052631578947368</v>
-      </c>
+        <v>0.3529411764705883</v>
+      </c>
+      <c r="F337" t="inlineStr"/>
+      <c r="G337" t="inlineStr"/>
       <c r="H337" t="inlineStr">
         <is>
-          <t>0.2986 (0.1826)</t>
+          <t>0.3529 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12542,31 +12530,31 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E338" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="F338" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="G338" t="n">
-        <v>0</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>0.1953 (0.1833)</t>
+          <t>0.2354 (0.1845)</t>
         </is>
       </c>
     </row>
@@ -12578,27 +12566,31 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E339" t="n">
-        <v>0.3448275862068966</v>
-      </c>
-      <c r="F339" t="inlineStr"/>
-      <c r="G339" t="inlineStr"/>
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F339" t="n">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="G339" t="n">
+        <v>0.09523809523809523</v>
+      </c>
       <c r="H339" t="inlineStr">
         <is>
-          <t>0.3448 (0.0000)</t>
+          <t>0.1799 (0.1331)</t>
         </is>
       </c>
     </row>
@@ -12610,31 +12602,27 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E340" t="n">
-        <v>0.3529411764705883</v>
-      </c>
-      <c r="F340" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="G340" t="n">
-        <v>0</v>
-      </c>
+        <v>0.3125</v>
+      </c>
+      <c r="F340" t="inlineStr"/>
+      <c r="G340" t="inlineStr"/>
       <c r="H340" t="inlineStr">
         <is>
-          <t>0.1593 (0.1790)</t>
+          <t>0.3125 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12646,31 +12634,27 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E341" t="n">
-        <v>0.3157894736842105</v>
-      </c>
-      <c r="F341" t="n">
-        <v>0</v>
-      </c>
-      <c r="G341" t="n">
-        <v>0</v>
-      </c>
+        <v>0.5128205128205128</v>
+      </c>
+      <c r="F341" t="inlineStr"/>
+      <c r="G341" t="inlineStr"/>
       <c r="H341" t="inlineStr">
         <is>
-          <t>0.1053 (0.1823)</t>
+          <t>0.5128 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -12682,27 +12666,31 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E342" t="n">
-        <v>0.3448275862068966</v>
-      </c>
-      <c r="F342" t="inlineStr"/>
-      <c r="G342" t="inlineStr"/>
+        <v>0.3125</v>
+      </c>
+      <c r="F342" t="n">
+        <v>0</v>
+      </c>
+      <c r="G342" t="n">
+        <v>0</v>
+      </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t>0.3448 (0.0000)</t>
+          <t>0.1042 (0.1804)</t>
         </is>
       </c>
     </row>
@@ -12714,570 +12702,578 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E343" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="F343" t="inlineStr"/>
-      <c r="G343" t="inlineStr"/>
+        <v>0.4324324324324325</v>
+      </c>
+      <c r="F343" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G343" t="n">
+        <v>0</v>
+      </c>
       <c r="H343" t="inlineStr">
         <is>
-          <t>0.3333 (0.0000)</t>
+          <t>0.1975 (0.2186)</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E344" t="n">
-        <v>0.6486486486486487</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F344" t="n">
-        <v>0.5</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="G344" t="n">
-        <v>0.6129032258064516</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t>0.5872 (0.0776)</t>
+          <t>0.1498 (0.0982)</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E345" t="n">
-        <v>0.5074626865671642</v>
+        <v>0.4680851063829787</v>
       </c>
       <c r="F345" t="n">
-        <v>0.5507246376811594</v>
+        <v>0.3225806451612903</v>
       </c>
       <c r="G345" t="n">
-        <v>0.6391752577319587</v>
+        <v>0.1052631578947368</v>
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>0.5658 (0.0671)</t>
+          <t>0.2986 (0.1826)</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E346" t="n">
-        <v>0.6736842105263158</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="F346" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="G346" t="n">
-        <v>0.6341463414634146</v>
+        <v>0</v>
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>0.6502 (0.0208)</t>
+          <t>0.1953 (0.1833)</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E347" t="n">
-        <v>0.6741573033707865</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="F347" t="n">
-        <v>0.5789473684210527</v>
+        <v>0</v>
       </c>
       <c r="G347" t="n">
-        <v>0.6744186046511628</v>
+        <v>0</v>
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>0.6425 (0.0550)</t>
+          <t>0.1149 (0.1991)</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E348" t="n">
-        <v>0.5263157894736842</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="F348" t="n">
-        <v>0.6285714285714286</v>
+        <v>0.125</v>
       </c>
       <c r="G348" t="n">
-        <v>0.5901639344262295</v>
+        <v>0</v>
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>0.5817 (0.0517)</t>
+          <t>0.1593 (0.1790)</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E349" t="n">
-        <v>0.4307692307692308</v>
+        <v>0.3157894736842105</v>
       </c>
       <c r="F349" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G349" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="G349" t="n">
+        <v>0</v>
+      </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>0.5154 (0.1197)</t>
+          <t>0.1053 (0.1823)</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E350" t="n">
-        <v>0.6</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="F350" t="n">
-        <v>0.5666666666666667</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G350" t="n">
-        <v>0.5573770491803278</v>
+        <v>0</v>
       </c>
       <c r="H350" t="inlineStr">
         <is>
-          <t>0.5747 (0.0224)</t>
+          <t>0.1919 (0.1757)</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRADIOL</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E351" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F351" t="n">
-        <v>0.6</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="G351" t="n">
-        <v>0.6363636363636364</v>
+        <v>0</v>
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t>0.6026 (0.0325)</t>
+          <t>0.1556 (0.1678)</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E352" t="n">
-        <v>0.6279069767441861</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F352" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.5161290322580645</v>
       </c>
       <c r="G352" t="n">
-        <v>0.6101694915254238</v>
+        <v>0.2</v>
       </c>
       <c r="H352" t="inlineStr">
         <is>
-          <t>0.5979 (0.0377)</t>
+          <t>0.3738 (0.1604)</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E353" t="n">
-        <v>0.5915492957746479</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="F353" t="n">
-        <v>0.4482758620689655</v>
-      </c>
-      <c r="G353" t="inlineStr"/>
+        <v>0.3076923076923077</v>
+      </c>
+      <c r="G353" t="n">
+        <v>0.1739130434782609</v>
+      </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t>0.5199 (0.1013)</t>
+          <t>0.2887 (0.1066)</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E354" t="n">
-        <v>0.5079365079365079</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="F354" t="n">
-        <v>0.5245901639344263</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="G354" t="n">
-        <v>0.5846153846153846</v>
+        <v>0</v>
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>0.5390 (0.0403)</t>
+          <t>0.1255 (0.1460)</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E355" t="n">
-        <v>0.5822784810126582</v>
+        <v>0.4857142857142857</v>
       </c>
       <c r="F355" t="n">
-        <v>0.5507246376811594</v>
+        <v>0.2790697674418605</v>
       </c>
       <c r="G355" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.1176470588235294</v>
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t>0.5554 (0.0248)</t>
+          <t>0.2941 (0.1845)</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E356" t="n">
-        <v>0.6818181818181818</v>
+        <v>0.1739130434782609</v>
       </c>
       <c r="F356" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="G356" t="n">
-        <v>0.53125</v>
+        <v>0.08695652173913043</v>
       </c>
       <c r="H356" t="inlineStr">
         <is>
-          <t>0.6157 (0.0770)</t>
+          <t>0.1382 (0.0455)</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E357" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="F357" t="n">
-        <v>0.5753424657534246</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="G357" t="n">
-        <v>0.4761904761904762</v>
+        <v>0.08695652173913043</v>
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>0.5648 (0.0838)</t>
+          <t>0.2243 (0.1384)</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E358" t="n">
-        <v>0.631578947368421</v>
+        <v>0.456140350877193</v>
       </c>
       <c r="F358" t="n">
-        <v>0.6268656716417911</v>
+        <v>0.07692307692307693</v>
       </c>
       <c r="G358" t="n">
-        <v>0.5245901639344263</v>
+        <v>0</v>
       </c>
       <c r="H358" t="inlineStr">
         <is>
-          <t>0.5943 (0.0605)</t>
+          <t>0.1777 (0.2442)</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
@@ -13287,7 +13283,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
@@ -13296,17 +13292,15 @@
         </is>
       </c>
       <c r="E359" t="n">
-        <v>0.64</v>
+        <v>0.2</v>
       </c>
       <c r="F359" t="n">
-        <v>0.5588235294117647</v>
-      </c>
-      <c r="G359" t="n">
-        <v>0.6060606060606061</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G359" t="inlineStr"/>
       <c r="H359" t="inlineStr">
         <is>
-          <t>0.6016 (0.0408)</t>
+          <t>0.1000 (0.1414)</t>
         </is>
       </c>
     </row>
@@ -13318,31 +13312,31 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E360" t="n">
-        <v>0.6578947368421053</v>
+        <v>0.6486486486486487</v>
       </c>
       <c r="F360" t="n">
-        <v>0.5079365079365079</v>
+        <v>0.5</v>
       </c>
       <c r="G360" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.6129032258064516</v>
       </c>
       <c r="H360" t="inlineStr">
         <is>
-          <t>0.5791 (0.0753)</t>
+          <t>0.5872 (0.0776)</t>
         </is>
       </c>
     </row>
@@ -13354,31 +13348,31 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E361" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5074626865671642</v>
       </c>
       <c r="F361" t="n">
-        <v>0.5633802816901409</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G361" t="n">
-        <v>0.6567164179104478</v>
+        <v>0.6391752577319587</v>
       </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t>0.6289 (0.0570)</t>
+          <t>0.5658 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -13390,31 +13384,31 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E362" t="n">
-        <v>0.6436781609195402</v>
+        <v>0.6736842105263158</v>
       </c>
       <c r="F362" t="n">
-        <v>0.6410256410256411</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="G362" t="n">
-        <v>0.6756756756756757</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="H362" t="inlineStr">
         <is>
-          <t>0.6535 (0.0193)</t>
+          <t>0.6502 (0.0208)</t>
         </is>
       </c>
     </row>
@@ -13426,31 +13420,31 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E363" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.6741573033707865</v>
       </c>
       <c r="F363" t="n">
-        <v>0.576271186440678</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="G363" t="n">
-        <v>0.4150943396226415</v>
+        <v>0.6744186046511628</v>
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t>0.5249 (0.0952)</t>
+          <t>0.6425 (0.0550)</t>
         </is>
       </c>
     </row>
@@ -13462,31 +13456,31 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E364" t="n">
-        <v>0.5373134328358209</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="F364" t="n">
-        <v>0.4918032786885246</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="G364" t="n">
-        <v>0.576271186440678</v>
+        <v>0.5901639344262295</v>
       </c>
       <c r="H364" t="inlineStr">
         <is>
-          <t>0.5351 (0.0423)</t>
+          <t>0.5817 (0.0517)</t>
         </is>
       </c>
     </row>
@@ -13498,31 +13492,31 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E365" t="n">
-        <v>0.6197183098591549</v>
+        <v>0.4307692307692308</v>
       </c>
       <c r="F365" t="n">
-        <v>0.5396825396825397</v>
+        <v>0.6</v>
       </c>
       <c r="G365" t="n">
-        <v>0.5423728813559322</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="H365" t="inlineStr">
         <is>
-          <t>0.5673 (0.0455)</t>
+          <t>0.4718 (0.1134)</t>
         </is>
       </c>
     </row>
@@ -13534,31 +13528,31 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E366" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.6</v>
       </c>
       <c r="F366" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="G366" t="n">
-        <v>0.5</v>
+        <v>0.5573770491803278</v>
       </c>
       <c r="H366" t="inlineStr">
         <is>
-          <t>0.5541 (0.0469)</t>
+          <t>0.5747 (0.0224)</t>
         </is>
       </c>
     </row>
@@ -13570,31 +13564,31 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E367" t="n">
-        <v>0.675</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F367" t="n">
         <v>0.6</v>
       </c>
       <c r="G367" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>0.6028 (0.0709)</t>
+          <t>0.6026 (0.0325)</t>
         </is>
       </c>
     </row>
@@ -13606,607 +13600,607 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E368" t="n">
-        <v>0.5070422535211268</v>
+        <v>0.6279069767441861</v>
       </c>
       <c r="F368" t="n">
-        <v>0.5806451612903226</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="G368" t="n">
-        <v>0.4528301886792453</v>
+        <v>0.6101694915254238</v>
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>0.5135 (0.0642)</t>
+          <t>0.5979 (0.0377)</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E369" t="n">
-        <v>0</v>
+        <v>0.5915492957746479</v>
       </c>
       <c r="F369" t="n">
-        <v>0</v>
+        <v>0.4482758620689655</v>
       </c>
       <c r="G369" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.4814814814814815</v>
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5071 (0.0750)</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E370" t="n">
-        <v>0</v>
+        <v>0.5079365079365079</v>
       </c>
       <c r="F370" t="n">
-        <v>0</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="G370" t="n">
-        <v>1</v>
+        <v>0.5846153846153846</v>
       </c>
       <c r="H370" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.5390 (0.0403)</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E371" t="n">
-        <v>0</v>
+        <v>0.5822784810126582</v>
       </c>
       <c r="F371" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G371" t="n">
-        <v>0.4</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.5554 (0.0248)</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E372" t="n">
-        <v>0</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="F372" t="n">
-        <v>0.25</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="G372" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.53125</v>
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>0.1944 (0.1735)</t>
+          <t>0.6157 (0.0770)</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E373" t="n">
-        <v>0</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="F373" t="n">
-        <v>0</v>
+        <v>0.5753424657534246</v>
       </c>
       <c r="G373" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5648 (0.0838)</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E374" t="n">
-        <v>0</v>
+        <v>0.631578947368421</v>
       </c>
       <c r="F374" t="n">
-        <v>0</v>
+        <v>0.6268656716417911</v>
       </c>
       <c r="G374" t="n">
-        <v>0.5</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.5943 (0.0605)</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E375" t="n">
-        <v>0</v>
+        <v>0.64</v>
       </c>
       <c r="F375" t="n">
-        <v>0.4</v>
+        <v>0.5588235294117647</v>
       </c>
       <c r="G375" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.6016 (0.0408)</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E376" t="n">
-        <v>0</v>
+        <v>0.6578947368421053</v>
       </c>
       <c r="F376" t="n">
-        <v>0</v>
+        <v>0.5079365079365079</v>
       </c>
       <c r="G376" t="n">
-        <v>0.4</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.5791 (0.0753)</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E377" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F377" t="n">
-        <v>0</v>
+        <v>0.5633802816901409</v>
       </c>
       <c r="G377" t="n">
-        <v>0.4</v>
+        <v>0.6567164179104478</v>
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.6289 (0.0570)</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E378" t="n">
-        <v>0</v>
+        <v>0.6436781609195402</v>
       </c>
       <c r="F378" t="n">
-        <v>0</v>
+        <v>0.6410256410256411</v>
       </c>
       <c r="G378" t="n">
-        <v>1</v>
+        <v>0.6756756756756757</v>
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.6535 (0.0193)</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E379" t="n">
-        <v>0</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F379" t="n">
-        <v>0</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="G379" t="n">
-        <v>0.5</v>
+        <v>0.4150943396226415</v>
       </c>
       <c r="H379" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.5249 (0.0952)</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D380" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E380" t="n">
-        <v>0</v>
+        <v>0.5373134328358209</v>
       </c>
       <c r="F380" t="n">
-        <v>0</v>
+        <v>0.4918032786885246</v>
       </c>
       <c r="G380" t="n">
-        <v>0.4</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="H380" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.5351 (0.0423)</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E381" t="n">
-        <v>0</v>
+        <v>0.6197183098591549</v>
       </c>
       <c r="F381" t="n">
-        <v>0</v>
+        <v>0.5396825396825397</v>
       </c>
       <c r="G381" t="n">
-        <v>0.4</v>
+        <v>0.5423728813559322</v>
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.5673 (0.0455)</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E382" t="n">
-        <v>0</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="F382" t="n">
-        <v>0</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="G382" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t>0.0000 (0.0000)</t>
+          <t>0.5541 (0.0469)</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E383" t="n">
-        <v>0</v>
+        <v>0.675</v>
       </c>
       <c r="F383" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G383" t="n">
-        <v>0.5</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H383" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.6028 (0.0709)</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E384" t="n">
-        <v>0</v>
+        <v>0.5070422535211268</v>
       </c>
       <c r="F384" t="n">
-        <v>0</v>
+        <v>0.5806451612903226</v>
       </c>
       <c r="G384" t="n">
-        <v>1</v>
+        <v>0.4528301886792453</v>
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.5135 (0.0642)</t>
         </is>
       </c>
     </row>
@@ -14218,17 +14212,17 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E385" t="n">
@@ -14238,11 +14232,11 @@
         <v>0</v>
       </c>
       <c r="G385" t="n">
-        <v>0.5</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H385" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -14254,17 +14248,17 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E386" t="n">
@@ -14274,11 +14268,11 @@
         <v>0</v>
       </c>
       <c r="G386" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="H386" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -14290,31 +14284,31 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E387" t="n">
         <v>0</v>
       </c>
       <c r="F387" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G387" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H387" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -14326,31 +14320,31 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E388" t="n">
         <v>0</v>
       </c>
       <c r="F388" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G388" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H388" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.1944 (0.1735)</t>
         </is>
       </c>
     </row>
@@ -14362,17 +14356,17 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E389" t="n">
@@ -14382,11 +14376,11 @@
         <v>0</v>
       </c>
       <c r="G389" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -14398,17 +14392,17 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E390" t="n">
@@ -14418,11 +14412,11 @@
         <v>0</v>
       </c>
       <c r="G390" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -14434,31 +14428,31 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E391" t="n">
         <v>0</v>
       </c>
       <c r="F391" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G391" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="H391" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -14470,17 +14464,17 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E392" t="n">
@@ -14490,11 +14484,11 @@
         <v>0</v>
       </c>
       <c r="G392" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>0.1111 (0.1925)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -14506,17 +14500,17 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E393" t="n">
@@ -14526,9 +14520,585 @@
         <v>0</v>
       </c>
       <c r="G393" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>0.1333 (0.2309)</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>gbt</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>GradientBoosting</t>
+        </is>
+      </c>
+      <c r="E394" t="n">
+        <v>0</v>
+      </c>
+      <c r="F394" t="n">
+        <v>0</v>
+      </c>
+      <c r="G394" t="n">
+        <v>1</v>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E395" t="n">
+        <v>0</v>
+      </c>
+      <c r="F395" t="n">
+        <v>0</v>
+      </c>
+      <c r="G395" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E396" t="n">
+        <v>0</v>
+      </c>
+      <c r="F396" t="n">
+        <v>0</v>
+      </c>
+      <c r="G396" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>0.1333 (0.2309)</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E397" t="n">
+        <v>0</v>
+      </c>
+      <c r="F397" t="n">
+        <v>0</v>
+      </c>
+      <c r="G397" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>0.1333 (0.2309)</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E398" t="n">
+        <v>0</v>
+      </c>
+      <c r="F398" t="n">
+        <v>0</v>
+      </c>
+      <c r="G398" t="n">
+        <v>0</v>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>0.0000 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E399" t="n">
+        <v>0</v>
+      </c>
+      <c r="F399" t="n">
+        <v>0</v>
+      </c>
+      <c r="G399" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E400" t="n">
+        <v>0</v>
+      </c>
+      <c r="F400" t="n">
+        <v>0</v>
+      </c>
+      <c r="G400" t="n">
+        <v>1</v>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E401" t="n">
+        <v>0</v>
+      </c>
+      <c r="F401" t="n">
+        <v>0</v>
+      </c>
+      <c r="G401" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E402" t="n">
+        <v>0</v>
+      </c>
+      <c r="F402" t="n">
+        <v>0</v>
+      </c>
+      <c r="G402" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="H393" t="inlineStr">
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E403" t="n">
+        <v>0</v>
+      </c>
+      <c r="F403" t="n">
+        <v>0</v>
+      </c>
+      <c r="G403" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E404" t="n">
+        <v>0</v>
+      </c>
+      <c r="F404" t="n">
+        <v>0</v>
+      </c>
+      <c r="G404" t="n">
+        <v>1</v>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E405" t="n">
+        <v>0</v>
+      </c>
+      <c r="F405" t="n">
+        <v>0</v>
+      </c>
+      <c r="G405" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E406" t="n">
+        <v>0</v>
+      </c>
+      <c r="F406" t="n">
+        <v>0</v>
+      </c>
+      <c r="G406" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E407" t="n">
+        <v>0</v>
+      </c>
+      <c r="F407" t="n">
+        <v>0</v>
+      </c>
+      <c r="G407" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E408" t="n">
+        <v>0</v>
+      </c>
+      <c r="F408" t="n">
+        <v>0</v>
+      </c>
+      <c r="G408" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>0.1111 (0.1925)</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E409" t="n">
+        <v>0</v>
+      </c>
+      <c r="F409" t="n">
+        <v>0</v>
+      </c>
+      <c r="G409" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H409" t="inlineStr">
         <is>
           <t>0.2222 (0.3849)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 13:34:07)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H409"/>
+  <dimension ref="A1:H418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8895,10 +8895,12 @@
       <c r="F236" t="n">
         <v>0.4444444444444444</v>
       </c>
-      <c r="G236" t="inlineStr"/>
+      <c r="G236" t="n">
+        <v>0.3846153846153846</v>
+      </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>0.2449 (0.2821)</t>
+          <t>0.2915 (0.2152)</t>
         </is>
       </c>
     </row>
@@ -12346,11 +12348,13 @@
       <c r="E332" t="n">
         <v>0.3571428571428572</v>
       </c>
-      <c r="F332" t="inlineStr"/>
+      <c r="F332" t="n">
+        <v>0</v>
+      </c>
       <c r="G332" t="inlineStr"/>
       <c r="H332" t="inlineStr">
         <is>
-          <t>0.3571 (0.0000)</t>
+          <t>0.1786 (0.2525)</t>
         </is>
       </c>
     </row>
@@ -12450,11 +12454,15 @@
       <c r="E335" t="n">
         <v>0.4242424242424243</v>
       </c>
-      <c r="F335" t="inlineStr"/>
-      <c r="G335" t="inlineStr"/>
+      <c r="F335" t="n">
+        <v>0.3846153846153846</v>
+      </c>
+      <c r="G335" t="n">
+        <v>0</v>
+      </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>0.4242 (0.0000)</t>
+          <t>0.2696 (0.2343)</t>
         </is>
       </c>
     </row>
@@ -12514,11 +12522,15 @@
       <c r="E337" t="n">
         <v>0.3529411764705883</v>
       </c>
-      <c r="F337" t="inlineStr"/>
-      <c r="G337" t="inlineStr"/>
+      <c r="F337" t="n">
+        <v>0</v>
+      </c>
+      <c r="G337" t="n">
+        <v>0</v>
+      </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>0.3529 (0.0000)</t>
+          <t>0.1176 (0.2038)</t>
         </is>
       </c>
     </row>
@@ -12618,11 +12630,15 @@
       <c r="E340" t="n">
         <v>0.3125</v>
       </c>
-      <c r="F340" t="inlineStr"/>
-      <c r="G340" t="inlineStr"/>
+      <c r="F340" t="n">
+        <v>0.2727272727272727</v>
+      </c>
+      <c r="G340" t="n">
+        <v>0.1818181818181818</v>
+      </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>0.3125 (0.0000)</t>
+          <t>0.2557 (0.0670)</t>
         </is>
       </c>
     </row>
@@ -12650,11 +12666,15 @@
       <c r="E341" t="n">
         <v>0.5128205128205128</v>
       </c>
-      <c r="F341" t="inlineStr"/>
-      <c r="G341" t="inlineStr"/>
+      <c r="F341" t="n">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="G341" t="n">
+        <v>0.1666666666666667</v>
+      </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>0.5128 (0.0000)</t>
+          <t>0.2635 (0.2177)</t>
         </is>
       </c>
     </row>
@@ -13206,7 +13226,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -13216,21 +13236,21 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E357" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F357" t="n">
         <v>0.3636363636363636</v>
       </c>
-      <c r="F357" t="n">
-        <v>0.2222222222222222</v>
-      </c>
       <c r="G357" t="n">
-        <v>0.08695652173913043</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>0.2243 (0.1384)</t>
+          <t>0.2879 (0.1061)</t>
         </is>
       </c>
     </row>
@@ -13242,7 +13262,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -13252,21 +13272,17 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E358" t="n">
-        <v>0.456140350877193</v>
-      </c>
-      <c r="F358" t="n">
-        <v>0.07692307692307693</v>
-      </c>
-      <c r="G358" t="n">
-        <v>0</v>
-      </c>
+        <v>0.3076923076923077</v>
+      </c>
+      <c r="F358" t="inlineStr"/>
+      <c r="G358" t="inlineStr"/>
       <c r="H358" t="inlineStr">
         <is>
-          <t>0.1777 (0.2442)</t>
+          <t>0.3077 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -13283,7 +13299,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
@@ -13292,339 +13308,329 @@
         </is>
       </c>
       <c r="E359" t="n">
-        <v>0.2</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="F359" t="n">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="G359" t="n">
         <v>0</v>
       </c>
-      <c r="G359" t="inlineStr"/>
       <c r="H359" t="inlineStr">
         <is>
-          <t>0.1000 (0.1414)</t>
+          <t>0.2201 (0.3118)</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E360" t="n">
-        <v>0.6486486486486487</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="F360" t="n">
-        <v>0.5</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="G360" t="n">
-        <v>0.6129032258064516</v>
+        <v>0.08695652173913043</v>
       </c>
       <c r="H360" t="inlineStr">
         <is>
-          <t>0.5872 (0.0776)</t>
+          <t>0.2243 (0.1384)</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E361" t="n">
-        <v>0.5074626865671642</v>
+        <v>0.456140350877193</v>
       </c>
       <c r="F361" t="n">
-        <v>0.5507246376811594</v>
+        <v>0.07692307692307693</v>
       </c>
       <c r="G361" t="n">
-        <v>0.6391752577319587</v>
+        <v>0</v>
       </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t>0.5658 (0.0671)</t>
+          <t>0.1777 (0.2442)</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E362" t="n">
-        <v>0.6736842105263158</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="F362" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="G362" t="n">
-        <v>0.6341463414634146</v>
+        <v>0</v>
       </c>
       <c r="H362" t="inlineStr">
         <is>
-          <t>0.6502 (0.0208)</t>
+          <t>0.1978 (0.1717)</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E363" t="n">
-        <v>0.6741573033707865</v>
+        <v>0.2</v>
       </c>
       <c r="F363" t="n">
-        <v>0.5789473684210527</v>
+        <v>0</v>
       </c>
       <c r="G363" t="n">
-        <v>0.6744186046511628</v>
+        <v>0</v>
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t>0.6425 (0.0550)</t>
+          <t>0.0667 (0.1155)</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E364" t="n">
-        <v>0.5263157894736842</v>
-      </c>
-      <c r="F364" t="n">
-        <v>0.6285714285714286</v>
-      </c>
-      <c r="G364" t="n">
-        <v>0.5901639344262295</v>
-      </c>
+        <v>0.4090909090909091</v>
+      </c>
+      <c r="F364" t="inlineStr"/>
+      <c r="G364" t="inlineStr"/>
       <c r="H364" t="inlineStr">
         <is>
-          <t>0.5817 (0.0517)</t>
+          <t>0.4091 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E365" t="n">
-        <v>0.4307692307692308</v>
+        <v>0.2926829268292683</v>
       </c>
       <c r="F365" t="n">
-        <v>0.6</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="G365" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="H365" t="inlineStr">
         <is>
-          <t>0.4718 (0.1134)</t>
+          <t>0.2682 (0.1098)</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E366" t="n">
-        <v>0.6</v>
+        <v>0.3111111111111111</v>
       </c>
       <c r="F366" t="n">
-        <v>0.5666666666666667</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="G366" t="n">
-        <v>0.5573770491803278</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H366" t="inlineStr">
         <is>
-          <t>0.5747 (0.0224)</t>
+          <t>0.1799 (0.1152)</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E367" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="F367" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G367" t="n">
-        <v>0.6363636363636364</v>
-      </c>
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F367" t="inlineStr"/>
+      <c r="G367" t="inlineStr"/>
       <c r="H367" t="inlineStr">
         <is>
-          <t>0.6026 (0.0325)</t>
+          <t>0.3333 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E368" t="n">
-        <v>0.6279069767441861</v>
-      </c>
-      <c r="F368" t="n">
-        <v>0.5555555555555556</v>
-      </c>
-      <c r="G368" t="n">
-        <v>0.6101694915254238</v>
-      </c>
+        <v>0.2105263157894737</v>
+      </c>
+      <c r="F368" t="inlineStr"/>
+      <c r="G368" t="inlineStr"/>
       <c r="H368" t="inlineStr">
         <is>
-          <t>0.5979 (0.0377)</t>
+          <t>0.2105 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -13636,31 +13642,31 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E369" t="n">
-        <v>0.5915492957746479</v>
+        <v>0.6486486486486487</v>
       </c>
       <c r="F369" t="n">
-        <v>0.4482758620689655</v>
+        <v>0.5</v>
       </c>
       <c r="G369" t="n">
-        <v>0.4814814814814815</v>
+        <v>0.6129032258064516</v>
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>0.5071 (0.0750)</t>
+          <t>0.5872 (0.0776)</t>
         </is>
       </c>
     </row>
@@ -13672,31 +13678,31 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E370" t="n">
-        <v>0.5079365079365079</v>
+        <v>0.5074626865671642</v>
       </c>
       <c r="F370" t="n">
-        <v>0.5245901639344263</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G370" t="n">
-        <v>0.5846153846153846</v>
+        <v>0.6391752577319587</v>
       </c>
       <c r="H370" t="inlineStr">
         <is>
-          <t>0.5390 (0.0403)</t>
+          <t>0.5658 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -13708,31 +13714,31 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E371" t="n">
-        <v>0.5822784810126582</v>
+        <v>0.6736842105263158</v>
       </c>
       <c r="F371" t="n">
-        <v>0.5507246376811594</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="G371" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>0.5554 (0.0248)</t>
+          <t>0.6502 (0.0208)</t>
         </is>
       </c>
     </row>
@@ -13744,31 +13750,31 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E372" t="n">
-        <v>0.6818181818181818</v>
+        <v>0.6741573033707865</v>
       </c>
       <c r="F372" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="G372" t="n">
-        <v>0.53125</v>
+        <v>0.6744186046511628</v>
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>0.6157 (0.0770)</t>
+          <t>0.6425 (0.0550)</t>
         </is>
       </c>
     </row>
@@ -13780,31 +13786,31 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E373" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="F373" t="n">
-        <v>0.5753424657534246</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="G373" t="n">
-        <v>0.4761904761904762</v>
+        <v>0.5901639344262295</v>
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>0.5648 (0.0838)</t>
+          <t>0.5817 (0.0517)</t>
         </is>
       </c>
     </row>
@@ -13816,31 +13822,31 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E374" t="n">
-        <v>0.631578947368421</v>
+        <v>0.4307692307692308</v>
       </c>
       <c r="F374" t="n">
-        <v>0.6268656716417911</v>
+        <v>0.6</v>
       </c>
       <c r="G374" t="n">
-        <v>0.5245901639344263</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t>0.5943 (0.0605)</t>
+          <t>0.4718 (0.1134)</t>
         </is>
       </c>
     </row>
@@ -13852,31 +13858,31 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E375" t="n">
-        <v>0.64</v>
+        <v>0.6</v>
       </c>
       <c r="F375" t="n">
-        <v>0.5588235294117647</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="G375" t="n">
-        <v>0.6060606060606061</v>
+        <v>0.5573770491803278</v>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>0.6016 (0.0408)</t>
+          <t>0.5747 (0.0224)</t>
         </is>
       </c>
     </row>
@@ -13888,31 +13894,31 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E376" t="n">
-        <v>0.6578947368421053</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F376" t="n">
-        <v>0.5079365079365079</v>
+        <v>0.6</v>
       </c>
       <c r="G376" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>0.5791 (0.0753)</t>
+          <t>0.6026 (0.0325)</t>
         </is>
       </c>
     </row>
@@ -13924,31 +13930,31 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E377" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6279069767441861</v>
       </c>
       <c r="F377" t="n">
-        <v>0.5633802816901409</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="G377" t="n">
-        <v>0.6567164179104478</v>
+        <v>0.6101694915254238</v>
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t>0.6289 (0.0570)</t>
+          <t>0.5979 (0.0377)</t>
         </is>
       </c>
     </row>
@@ -13960,31 +13966,31 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E378" t="n">
-        <v>0.6436781609195402</v>
+        <v>0.5915492957746479</v>
       </c>
       <c r="F378" t="n">
-        <v>0.6410256410256411</v>
+        <v>0.4482758620689655</v>
       </c>
       <c r="G378" t="n">
-        <v>0.6756756756756757</v>
+        <v>0.4814814814814815</v>
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t>0.6535 (0.0193)</t>
+          <t>0.5071 (0.0750)</t>
         </is>
       </c>
     </row>
@@ -13996,31 +14002,31 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E379" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5079365079365079</v>
       </c>
       <c r="F379" t="n">
-        <v>0.576271186440678</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="G379" t="n">
-        <v>0.4150943396226415</v>
+        <v>0.5846153846153846</v>
       </c>
       <c r="H379" t="inlineStr">
         <is>
-          <t>0.5249 (0.0952)</t>
+          <t>0.5390 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -14032,31 +14038,31 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D380" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E380" t="n">
-        <v>0.5373134328358209</v>
+        <v>0.5822784810126582</v>
       </c>
       <c r="F380" t="n">
-        <v>0.4918032786885246</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G380" t="n">
-        <v>0.576271186440678</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H380" t="inlineStr">
         <is>
-          <t>0.5351 (0.0423)</t>
+          <t>0.5554 (0.0248)</t>
         </is>
       </c>
     </row>
@@ -14068,31 +14074,31 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E381" t="n">
-        <v>0.6197183098591549</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="F381" t="n">
-        <v>0.5396825396825397</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="G381" t="n">
-        <v>0.5423728813559322</v>
+        <v>0.53125</v>
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t>0.5673 (0.0455)</t>
+          <t>0.6157 (0.0770)</t>
         </is>
       </c>
     </row>
@@ -14104,31 +14110,31 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E382" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="F382" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5753424657534246</v>
       </c>
       <c r="G382" t="n">
-        <v>0.5</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t>0.5541 (0.0469)</t>
+          <t>0.5648 (0.0838)</t>
         </is>
       </c>
     </row>
@@ -14140,31 +14146,31 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E383" t="n">
-        <v>0.675</v>
+        <v>0.631578947368421</v>
       </c>
       <c r="F383" t="n">
-        <v>0.6</v>
+        <v>0.6268656716417911</v>
       </c>
       <c r="G383" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="H383" t="inlineStr">
         <is>
-          <t>0.6028 (0.0709)</t>
+          <t>0.5943 (0.0605)</t>
         </is>
       </c>
     </row>
@@ -14176,355 +14182,355 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E384" t="n">
-        <v>0.5070422535211268</v>
+        <v>0.64</v>
       </c>
       <c r="F384" t="n">
-        <v>0.5806451612903226</v>
+        <v>0.5588235294117647</v>
       </c>
       <c r="G384" t="n">
-        <v>0.4528301886792453</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t>0.5135 (0.0642)</t>
+          <t>0.6016 (0.0408)</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E385" t="n">
-        <v>0</v>
+        <v>0.6578947368421053</v>
       </c>
       <c r="F385" t="n">
-        <v>0</v>
+        <v>0.5079365079365079</v>
       </c>
       <c r="G385" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="H385" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5791 (0.0753)</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E386" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F386" t="n">
-        <v>0</v>
+        <v>0.5633802816901409</v>
       </c>
       <c r="G386" t="n">
-        <v>1</v>
+        <v>0.6567164179104478</v>
       </c>
       <c r="H386" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.6289 (0.0570)</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E387" t="n">
-        <v>0</v>
+        <v>0.6436781609195402</v>
       </c>
       <c r="F387" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6410256410256411</v>
       </c>
       <c r="G387" t="n">
-        <v>0.4</v>
+        <v>0.6756756756756757</v>
       </c>
       <c r="H387" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.6535 (0.0193)</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E388" t="n">
-        <v>0</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F388" t="n">
-        <v>0.25</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="G388" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4150943396226415</v>
       </c>
       <c r="H388" t="inlineStr">
         <is>
-          <t>0.1944 (0.1735)</t>
+          <t>0.5249 (0.0952)</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E389" t="n">
-        <v>0</v>
+        <v>0.5373134328358209</v>
       </c>
       <c r="F389" t="n">
-        <v>0</v>
+        <v>0.4918032786885246</v>
       </c>
       <c r="G389" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5351 (0.0423)</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E390" t="n">
-        <v>0</v>
+        <v>0.6197183098591549</v>
       </c>
       <c r="F390" t="n">
-        <v>0</v>
+        <v>0.5396825396825397</v>
       </c>
       <c r="G390" t="n">
-        <v>0.5</v>
+        <v>0.5423728813559322</v>
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.5673 (0.0455)</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E391" t="n">
-        <v>0</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="F391" t="n">
-        <v>0.4</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="G391" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="H391" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.5541 (0.0469)</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E392" t="n">
-        <v>0</v>
+        <v>0.675</v>
       </c>
       <c r="F392" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G392" t="n">
-        <v>0.4</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.6028 (0.0709)</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E393" t="n">
-        <v>0</v>
+        <v>0.5070422535211268</v>
       </c>
       <c r="F393" t="n">
-        <v>0</v>
+        <v>0.5806451612903226</v>
       </c>
       <c r="G393" t="n">
-        <v>0.4</v>
+        <v>0.4528301886792453</v>
       </c>
       <c r="H393" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.5135 (0.0642)</t>
         </is>
       </c>
     </row>
@@ -14536,17 +14542,17 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E394" t="n">
@@ -14556,11 +14562,11 @@
         <v>0</v>
       </c>
       <c r="G394" t="n">
-        <v>1</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H394" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -14572,17 +14578,17 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E395" t="n">
@@ -14592,11 +14598,11 @@
         <v>0</v>
       </c>
       <c r="G395" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -14608,31 +14614,31 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E396" t="n">
         <v>0</v>
       </c>
       <c r="F396" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G396" t="n">
         <v>0.4</v>
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -14644,31 +14650,31 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E397" t="n">
         <v>0</v>
       </c>
       <c r="F397" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G397" t="n">
-        <v>0.4</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.1944 (0.1735)</t>
         </is>
       </c>
     </row>
@@ -14680,17 +14686,17 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E398" t="n">
@@ -14700,11 +14706,11 @@
         <v>0</v>
       </c>
       <c r="G398" t="n">
-        <v>0</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t>0.0000 (0.0000)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -14716,17 +14722,17 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E399" t="n">
@@ -14752,31 +14758,31 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E400" t="n">
         <v>0</v>
       </c>
       <c r="F400" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G400" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -14788,17 +14794,17 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E401" t="n">
@@ -14808,11 +14814,11 @@
         <v>0</v>
       </c>
       <c r="G401" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -14824,17 +14830,17 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E402" t="n">
@@ -14844,11 +14850,11 @@
         <v>0</v>
       </c>
       <c r="G402" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -14860,17 +14866,17 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E403" t="n">
@@ -14880,11 +14886,11 @@
         <v>0</v>
       </c>
       <c r="G403" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="H403" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -14896,17 +14902,17 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E404" t="n">
@@ -14916,11 +14922,11 @@
         <v>0</v>
       </c>
       <c r="G404" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H404" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -14932,17 +14938,17 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E405" t="n">
@@ -14952,11 +14958,11 @@
         <v>0</v>
       </c>
       <c r="G405" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -14968,17 +14974,17 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E406" t="n">
@@ -14988,11 +14994,11 @@
         <v>0</v>
       </c>
       <c r="G406" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H406" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -15004,17 +15010,17 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E407" t="n">
@@ -15024,11 +15030,11 @@
         <v>0</v>
       </c>
       <c r="G407" t="n">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.0000 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -15040,17 +15046,17 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E408" t="n">
@@ -15060,11 +15066,11 @@
         <v>0</v>
       </c>
       <c r="G408" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="H408" t="inlineStr">
         <is>
-          <t>0.1111 (0.1925)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -15076,17 +15082,17 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E409" t="n">
@@ -15096,9 +15102,333 @@
         <v>0</v>
       </c>
       <c r="G409" t="n">
+        <v>1</v>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E410" t="n">
+        <v>0</v>
+      </c>
+      <c r="F410" t="n">
+        <v>0</v>
+      </c>
+      <c r="G410" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E411" t="n">
+        <v>0</v>
+      </c>
+      <c r="F411" t="n">
+        <v>0</v>
+      </c>
+      <c r="G411" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="H409" t="inlineStr">
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E412" t="n">
+        <v>0</v>
+      </c>
+      <c r="F412" t="n">
+        <v>0</v>
+      </c>
+      <c r="G412" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E413" t="n">
+        <v>0</v>
+      </c>
+      <c r="F413" t="n">
+        <v>0</v>
+      </c>
+      <c r="G413" t="n">
+        <v>1</v>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E414" t="n">
+        <v>0</v>
+      </c>
+      <c r="F414" t="n">
+        <v>0</v>
+      </c>
+      <c r="G414" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E415" t="n">
+        <v>0</v>
+      </c>
+      <c r="F415" t="n">
+        <v>0</v>
+      </c>
+      <c r="G415" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E416" t="n">
+        <v>0</v>
+      </c>
+      <c r="F416" t="n">
+        <v>0</v>
+      </c>
+      <c r="G416" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E417" t="n">
+        <v>0</v>
+      </c>
+      <c r="F417" t="n">
+        <v>0</v>
+      </c>
+      <c r="G417" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>0.1111 (0.1925)</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E418" t="n">
+        <v>0</v>
+      </c>
+      <c r="F418" t="n">
+        <v>0</v>
+      </c>
+      <c r="G418" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H418" t="inlineStr">
         <is>
           <t>0.2222 (0.3849)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 14:34:25)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H418"/>
+  <dimension ref="A1:H432"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12351,10 +12351,12 @@
       <c r="F332" t="n">
         <v>0</v>
       </c>
-      <c r="G332" t="inlineStr"/>
+      <c r="G332" t="n">
+        <v>0</v>
+      </c>
       <c r="H332" t="inlineStr">
         <is>
-          <t>0.1786 (0.2525)</t>
+          <t>0.1190 (0.2062)</t>
         </is>
       </c>
     </row>
@@ -12490,11 +12492,13 @@
       <c r="E336" t="n">
         <v>0.4117647058823529</v>
       </c>
-      <c r="F336" t="inlineStr"/>
+      <c r="F336" t="n">
+        <v>0.3809523809523809</v>
+      </c>
       <c r="G336" t="inlineStr"/>
       <c r="H336" t="inlineStr">
         <is>
-          <t>0.4118 (0.0000)</t>
+          <t>0.3964 (0.0218)</t>
         </is>
       </c>
     </row>
@@ -13231,7 +13235,7 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
@@ -13240,17 +13244,13 @@
         </is>
       </c>
       <c r="E357" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="F357" t="n">
-        <v>0.3636363636363636</v>
-      </c>
-      <c r="G357" t="n">
-        <v>0.1666666666666667</v>
-      </c>
+        <v>0.358974358974359</v>
+      </c>
+      <c r="F357" t="inlineStr"/>
+      <c r="G357" t="inlineStr"/>
       <c r="H357" t="inlineStr">
         <is>
-          <t>0.2879 (0.1061)</t>
+          <t>0.3590 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -13267,7 +13267,7 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
@@ -13276,13 +13276,17 @@
         </is>
       </c>
       <c r="E358" t="n">
-        <v>0.3076923076923077</v>
-      </c>
-      <c r="F358" t="inlineStr"/>
-      <c r="G358" t="inlineStr"/>
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F358" t="n">
+        <v>0.3636363636363636</v>
+      </c>
+      <c r="G358" t="n">
+        <v>0.1666666666666667</v>
+      </c>
       <c r="H358" t="inlineStr">
         <is>
-          <t>0.3077 (0.0000)</t>
+          <t>0.2879 (0.1061)</t>
         </is>
       </c>
     </row>
@@ -13294,31 +13298,31 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E359" t="n">
-        <v>0.5769230769230769</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="F359" t="n">
         <v>0.08333333333333333</v>
       </c>
       <c r="G359" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="H359" t="inlineStr">
         <is>
-          <t>0.2201 (0.3118)</t>
+          <t>0.1720 (0.1193)</t>
         </is>
       </c>
     </row>
@@ -13330,31 +13334,27 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E360" t="n">
-        <v>0.3636363636363636</v>
-      </c>
-      <c r="F360" t="n">
-        <v>0.2222222222222222</v>
-      </c>
-      <c r="G360" t="n">
-        <v>0.08695652173913043</v>
-      </c>
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F360" t="inlineStr"/>
+      <c r="G360" t="inlineStr"/>
       <c r="H360" t="inlineStr">
         <is>
-          <t>0.2243 (0.1384)</t>
+          <t>0.3333 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -13366,31 +13366,27 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E361" t="n">
-        <v>0.456140350877193</v>
-      </c>
-      <c r="F361" t="n">
-        <v>0.07692307692307693</v>
-      </c>
-      <c r="G361" t="n">
-        <v>0</v>
-      </c>
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="F361" t="inlineStr"/>
+      <c r="G361" t="inlineStr"/>
       <c r="H361" t="inlineStr">
         <is>
-          <t>0.1777 (0.2442)</t>
+          <t>0.2632 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -13402,31 +13398,31 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E362" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3</v>
       </c>
       <c r="F362" t="n">
-        <v>0.3076923076923077</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="G362" t="n">
-        <v>0</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="H362" t="inlineStr">
         <is>
-          <t>0.1978 (0.1717)</t>
+          <t>0.2849 (0.1351)</t>
         </is>
       </c>
     </row>
@@ -13438,31 +13434,31 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E363" t="n">
-        <v>0.2</v>
+        <v>0.3018867924528302</v>
       </c>
       <c r="F363" t="n">
-        <v>0</v>
+        <v>0.2142857142857143</v>
       </c>
       <c r="G363" t="n">
-        <v>0</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t>0.0667 (0.1155)</t>
+          <t>0.1998 (0.1100)</t>
         </is>
       </c>
     </row>
@@ -13474,27 +13470,27 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E364" t="n">
-        <v>0.4090909090909091</v>
+        <v>0.3720930232558139</v>
       </c>
       <c r="F364" t="inlineStr"/>
       <c r="G364" t="inlineStr"/>
       <c r="H364" t="inlineStr">
         <is>
-          <t>0.4091 (0.0000)</t>
+          <t>0.3721 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -13506,31 +13502,27 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E365" t="n">
-        <v>0.2926829268292683</v>
-      </c>
-      <c r="F365" t="n">
-        <v>0.3636363636363636</v>
-      </c>
-      <c r="G365" t="n">
-        <v>0.1481481481481481</v>
-      </c>
+        <v>0.3404255319148936</v>
+      </c>
+      <c r="F365" t="inlineStr"/>
+      <c r="G365" t="inlineStr"/>
       <c r="H365" t="inlineStr">
         <is>
-          <t>0.2682 (0.1098)</t>
+          <t>0.3404 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -13542,31 +13534,31 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E366" t="n">
-        <v>0.3111111111111111</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="F366" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="G366" t="n">
-        <v>0.1333333333333333</v>
+        <v>0</v>
       </c>
       <c r="H366" t="inlineStr">
         <is>
-          <t>0.1799 (0.1152)</t>
+          <t>0.2201 (0.3118)</t>
         </is>
       </c>
     </row>
@@ -13578,27 +13570,31 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E367" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="F367" t="inlineStr"/>
-      <c r="G367" t="inlineStr"/>
+        <v>0.3636363636363636</v>
+      </c>
+      <c r="F367" t="n">
+        <v>0.2222222222222222</v>
+      </c>
+      <c r="G367" t="n">
+        <v>0.08695652173913043</v>
+      </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>0.3333 (0.0000)</t>
+          <t>0.2243 (0.1384)</t>
         </is>
       </c>
     </row>
@@ -13610,279 +13606,283 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E368" t="n">
-        <v>0.2105263157894737</v>
-      </c>
-      <c r="F368" t="inlineStr"/>
-      <c r="G368" t="inlineStr"/>
+        <v>0.456140350877193</v>
+      </c>
+      <c r="F368" t="n">
+        <v>0.07692307692307693</v>
+      </c>
+      <c r="G368" t="n">
+        <v>0</v>
+      </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>0.2105 (0.0000)</t>
+          <t>0.1777 (0.2442)</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E369" t="n">
-        <v>0.6486486486486487</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="F369" t="n">
-        <v>0.5</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="G369" t="n">
-        <v>0.6129032258064516</v>
+        <v>0</v>
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>0.5872 (0.0776)</t>
+          <t>0.1978 (0.1717)</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E370" t="n">
-        <v>0.5074626865671642</v>
+        <v>0.2</v>
       </c>
       <c r="F370" t="n">
-        <v>0.5507246376811594</v>
+        <v>0</v>
       </c>
       <c r="G370" t="n">
-        <v>0.6391752577319587</v>
+        <v>0</v>
       </c>
       <c r="H370" t="inlineStr">
         <is>
-          <t>0.5658 (0.0671)</t>
+          <t>0.0667 (0.1155)</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E371" t="n">
-        <v>0.6736842105263158</v>
+        <v>0.4090909090909091</v>
       </c>
       <c r="F371" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="G371" t="n">
-        <v>0.6341463414634146</v>
+        <v>0</v>
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>0.6502 (0.0208)</t>
+          <t>0.2233 (0.2071)</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E372" t="n">
-        <v>0.6741573033707865</v>
+        <v>0.2926829268292683</v>
       </c>
       <c r="F372" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="G372" t="n">
-        <v>0.6744186046511628</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>0.6425 (0.0550)</t>
+          <t>0.2682 (0.1098)</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E373" t="n">
-        <v>0.5263157894736842</v>
+        <v>0.3111111111111111</v>
       </c>
       <c r="F373" t="n">
-        <v>0.6285714285714286</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="G373" t="n">
-        <v>0.5901639344262295</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>0.5817 (0.0517)</t>
+          <t>0.1799 (0.1152)</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E374" t="n">
-        <v>0.4307692307692308</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F374" t="n">
-        <v>0.6</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G374" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t>0.4718 (0.1134)</t>
+          <t>0.2508 (0.1045)</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E375" t="n">
-        <v>0.6</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="F375" t="n">
-        <v>0.5666666666666667</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="G375" t="n">
-        <v>0.5573770491803278</v>
+        <v>0</v>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>0.5747 (0.0224)</t>
+          <t>0.1072 (0.1053)</t>
         </is>
       </c>
     </row>
@@ -13894,31 +13894,31 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E376" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.6486486486486487</v>
       </c>
       <c r="F376" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="G376" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.6129032258064516</v>
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>0.6026 (0.0325)</t>
+          <t>0.5872 (0.0776)</t>
         </is>
       </c>
     </row>
@@ -13930,31 +13930,31 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E377" t="n">
-        <v>0.6279069767441861</v>
+        <v>0.5074626865671642</v>
       </c>
       <c r="F377" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G377" t="n">
-        <v>0.6101694915254238</v>
+        <v>0.6391752577319587</v>
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t>0.5979 (0.0377)</t>
+          <t>0.5658 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -13966,31 +13966,31 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E378" t="n">
-        <v>0.5915492957746479</v>
+        <v>0.6736842105263158</v>
       </c>
       <c r="F378" t="n">
-        <v>0.4482758620689655</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="G378" t="n">
-        <v>0.4814814814814815</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t>0.5071 (0.0750)</t>
+          <t>0.6502 (0.0208)</t>
         </is>
       </c>
     </row>
@@ -14002,31 +14002,31 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E379" t="n">
-        <v>0.5079365079365079</v>
+        <v>0.6741573033707865</v>
       </c>
       <c r="F379" t="n">
-        <v>0.5245901639344263</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="G379" t="n">
-        <v>0.5846153846153846</v>
+        <v>0.6744186046511628</v>
       </c>
       <c r="H379" t="inlineStr">
         <is>
-          <t>0.5390 (0.0403)</t>
+          <t>0.6425 (0.0550)</t>
         </is>
       </c>
     </row>
@@ -14038,31 +14038,31 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D380" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E380" t="n">
-        <v>0.5822784810126582</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="F380" t="n">
-        <v>0.5507246376811594</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="G380" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5901639344262295</v>
       </c>
       <c r="H380" t="inlineStr">
         <is>
-          <t>0.5554 (0.0248)</t>
+          <t>0.5817 (0.0517)</t>
         </is>
       </c>
     </row>
@@ -14074,31 +14074,31 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E381" t="n">
-        <v>0.6818181818181818</v>
+        <v>0.4307692307692308</v>
       </c>
       <c r="F381" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.6</v>
       </c>
       <c r="G381" t="n">
-        <v>0.53125</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t>0.6157 (0.0770)</t>
+          <t>0.4718 (0.1134)</t>
         </is>
       </c>
     </row>
@@ -14110,31 +14110,31 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E382" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.6</v>
       </c>
       <c r="F382" t="n">
-        <v>0.5753424657534246</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="G382" t="n">
-        <v>0.4761904761904762</v>
+        <v>0.5573770491803278</v>
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t>0.5648 (0.0838)</t>
+          <t>0.5747 (0.0224)</t>
         </is>
       </c>
     </row>
@@ -14146,31 +14146,31 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E383" t="n">
-        <v>0.631578947368421</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F383" t="n">
-        <v>0.6268656716417911</v>
+        <v>0.6</v>
       </c>
       <c r="G383" t="n">
-        <v>0.5245901639344263</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="H383" t="inlineStr">
         <is>
-          <t>0.5943 (0.0605)</t>
+          <t>0.6026 (0.0325)</t>
         </is>
       </c>
     </row>
@@ -14182,31 +14182,31 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E384" t="n">
-        <v>0.64</v>
+        <v>0.6279069767441861</v>
       </c>
       <c r="F384" t="n">
-        <v>0.5588235294117647</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="G384" t="n">
-        <v>0.6060606060606061</v>
+        <v>0.6101694915254238</v>
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t>0.6016 (0.0408)</t>
+          <t>0.5979 (0.0377)</t>
         </is>
       </c>
     </row>
@@ -14218,31 +14218,31 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E385" t="n">
-        <v>0.6578947368421053</v>
+        <v>0.5915492957746479</v>
       </c>
       <c r="F385" t="n">
-        <v>0.5079365079365079</v>
+        <v>0.4482758620689655</v>
       </c>
       <c r="G385" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.4814814814814815</v>
       </c>
       <c r="H385" t="inlineStr">
         <is>
-          <t>0.5791 (0.0753)</t>
+          <t>0.5071 (0.0750)</t>
         </is>
       </c>
     </row>
@@ -14254,31 +14254,31 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E386" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5079365079365079</v>
       </c>
       <c r="F386" t="n">
-        <v>0.5633802816901409</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="G386" t="n">
-        <v>0.6567164179104478</v>
+        <v>0.5846153846153846</v>
       </c>
       <c r="H386" t="inlineStr">
         <is>
-          <t>0.6289 (0.0570)</t>
+          <t>0.5390 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -14290,31 +14290,31 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E387" t="n">
-        <v>0.6436781609195402</v>
+        <v>0.5822784810126582</v>
       </c>
       <c r="F387" t="n">
-        <v>0.6410256410256411</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G387" t="n">
-        <v>0.6756756756756757</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H387" t="inlineStr">
         <is>
-          <t>0.6535 (0.0193)</t>
+          <t>0.5554 (0.0248)</t>
         </is>
       </c>
     </row>
@@ -14326,31 +14326,31 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E388" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="F388" t="n">
-        <v>0.576271186440678</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="G388" t="n">
-        <v>0.4150943396226415</v>
+        <v>0.53125</v>
       </c>
       <c r="H388" t="inlineStr">
         <is>
-          <t>0.5249 (0.0952)</t>
+          <t>0.6157 (0.0770)</t>
         </is>
       </c>
     </row>
@@ -14362,31 +14362,31 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E389" t="n">
-        <v>0.5373134328358209</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="F389" t="n">
-        <v>0.4918032786885246</v>
+        <v>0.5753424657534246</v>
       </c>
       <c r="G389" t="n">
-        <v>0.576271186440678</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t>0.5351 (0.0423)</t>
+          <t>0.5648 (0.0838)</t>
         </is>
       </c>
     </row>
@@ -14398,31 +14398,31 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E390" t="n">
-        <v>0.6197183098591549</v>
+        <v>0.631578947368421</v>
       </c>
       <c r="F390" t="n">
-        <v>0.5396825396825397</v>
+        <v>0.6268656716417911</v>
       </c>
       <c r="G390" t="n">
-        <v>0.5423728813559322</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t>0.5673 (0.0455)</t>
+          <t>0.5943 (0.0605)</t>
         </is>
       </c>
     </row>
@@ -14434,31 +14434,31 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E391" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.64</v>
       </c>
       <c r="F391" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5588235294117647</v>
       </c>
       <c r="G391" t="n">
-        <v>0.5</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="H391" t="inlineStr">
         <is>
-          <t>0.5541 (0.0469)</t>
+          <t>0.6016 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -14470,31 +14470,31 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E392" t="n">
-        <v>0.675</v>
+        <v>0.6578947368421053</v>
       </c>
       <c r="F392" t="n">
-        <v>0.6</v>
+        <v>0.5079365079365079</v>
       </c>
       <c r="G392" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>0.6028 (0.0709)</t>
+          <t>0.5791 (0.0753)</t>
         </is>
       </c>
     </row>
@@ -14506,535 +14506,529 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E393" t="n">
-        <v>0.5070422535211268</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F393" t="n">
-        <v>0.5806451612903226</v>
+        <v>0.5633802816901409</v>
       </c>
       <c r="G393" t="n">
-        <v>0.4528301886792453</v>
+        <v>0.6567164179104478</v>
       </c>
       <c r="H393" t="inlineStr">
         <is>
-          <t>0.5135 (0.0642)</t>
+          <t>0.6289 (0.0570)</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E394" t="n">
-        <v>0</v>
+        <v>0.6436781609195402</v>
       </c>
       <c r="F394" t="n">
-        <v>0</v>
+        <v>0.6410256410256411</v>
       </c>
       <c r="G394" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.6756756756756757</v>
       </c>
       <c r="H394" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.6535 (0.0193)</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E395" t="n">
-        <v>0</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F395" t="n">
-        <v>0</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="G395" t="n">
-        <v>1</v>
+        <v>0.4150943396226415</v>
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.5249 (0.0952)</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E396" t="n">
-        <v>0</v>
+        <v>0.5373134328358209</v>
       </c>
       <c r="F396" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4918032786885246</v>
       </c>
       <c r="G396" t="n">
-        <v>0.4</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.5351 (0.0423)</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E397" t="n">
-        <v>0</v>
+        <v>0.6197183098591549</v>
       </c>
       <c r="F397" t="n">
-        <v>0.25</v>
+        <v>0.5396825396825397</v>
       </c>
       <c r="G397" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5423728813559322</v>
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t>0.1944 (0.1735)</t>
+          <t>0.5673 (0.0455)</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E398" t="n">
-        <v>0</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="F398" t="n">
-        <v>0</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="G398" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.5</v>
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5541 (0.0469)</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E399" t="n">
-        <v>0</v>
+        <v>0.675</v>
       </c>
       <c r="F399" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G399" t="n">
-        <v>0.5</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.6028 (0.0709)</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E400" t="n">
-        <v>0</v>
+        <v>0.5070422535211268</v>
       </c>
       <c r="F400" t="n">
-        <v>0.4</v>
+        <v>0.5806451612903226</v>
       </c>
       <c r="G400" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4528301886792453</v>
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.5135 (0.0642)</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E401" t="n">
-        <v>0</v>
+        <v>0.5316455696202531</v>
       </c>
       <c r="F401" t="n">
-        <v>0</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="G401" t="n">
-        <v>0.4</v>
+        <v>0.5070422535211268</v>
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.5314 (0.0243)</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E402" t="n">
-        <v>0</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F402" t="n">
-        <v>0</v>
+        <v>0.4313725490196079</v>
       </c>
       <c r="G402" t="n">
-        <v>0.4</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.5082 (0.0710)</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E403" t="n">
-        <v>0</v>
+        <v>0.4477611940298508</v>
       </c>
       <c r="F403" t="n">
-        <v>0</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="G403" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H403" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.3908 (0.0572)</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E404" t="n">
-        <v>0</v>
+        <v>0.5365853658536586</v>
       </c>
       <c r="F404" t="n">
-        <v>0</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="G404" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="H404" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.5809 (0.0385)</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E405" t="n">
-        <v>0</v>
+        <v>0.6470588235294118</v>
       </c>
       <c r="F405" t="n">
-        <v>0</v>
+        <v>0.4067796610169492</v>
       </c>
       <c r="G405" t="n">
-        <v>0.4</v>
+        <v>0.5416666666666666</v>
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.5318 (0.1204)</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E406" t="n">
-        <v>0</v>
+        <v>0.547945205479452</v>
       </c>
       <c r="F406" t="n">
-        <v>0</v>
-      </c>
-      <c r="G406" t="n">
-        <v>0.4</v>
-      </c>
+        <v>0.5106382978723404</v>
+      </c>
+      <c r="G406" t="inlineStr"/>
       <c r="H406" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.5293 (0.0264)</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E407" t="n">
-        <v>0</v>
-      </c>
-      <c r="F407" t="n">
-        <v>0</v>
-      </c>
-      <c r="G407" t="n">
-        <v>0</v>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="F407" t="inlineStr"/>
+      <c r="G407" t="inlineStr"/>
       <c r="H407" t="inlineStr">
         <is>
-          <t>0.0000 (0.0000)</t>
+          <t>0.5000 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -15046,17 +15040,17 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E408" t="n">
@@ -15066,11 +15060,11 @@
         <v>0</v>
       </c>
       <c r="G408" t="n">
-        <v>0.5</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H408" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -15082,17 +15076,17 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E409" t="n">
@@ -15118,31 +15112,31 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E410" t="n">
         <v>0</v>
       </c>
       <c r="F410" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G410" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -15154,31 +15148,31 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E411" t="n">
         <v>0</v>
       </c>
       <c r="F411" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G411" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1944 (0.1735)</t>
         </is>
       </c>
     </row>
@@ -15190,17 +15184,17 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E412" t="n">
@@ -15210,11 +15204,11 @@
         <v>0</v>
       </c>
       <c r="G412" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -15226,17 +15220,17 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E413" t="n">
@@ -15246,11 +15240,11 @@
         <v>0</v>
       </c>
       <c r="G413" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -15262,31 +15256,31 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E414" t="n">
         <v>0</v>
       </c>
       <c r="F414" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G414" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -15298,17 +15292,17 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E415" t="n">
@@ -15318,11 +15312,11 @@
         <v>0</v>
       </c>
       <c r="G415" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H415" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -15334,17 +15328,17 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E416" t="n">
@@ -15354,11 +15348,11 @@
         <v>0</v>
       </c>
       <c r="G416" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -15370,17 +15364,17 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E417" t="n">
@@ -15390,11 +15384,11 @@
         <v>0</v>
       </c>
       <c r="G417" t="n">
-        <v>0.3333333333333333</v>
+        <v>1</v>
       </c>
       <c r="H417" t="inlineStr">
         <is>
-          <t>0.1111 (0.1925)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -15406,17 +15400,17 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E418" t="n">
@@ -15426,9 +15420,513 @@
         <v>0</v>
       </c>
       <c r="G418" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E419" t="n">
+        <v>0</v>
+      </c>
+      <c r="F419" t="n">
+        <v>0</v>
+      </c>
+      <c r="G419" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>0.1333 (0.2309)</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E420" t="n">
+        <v>0</v>
+      </c>
+      <c r="F420" t="n">
+        <v>0</v>
+      </c>
+      <c r="G420" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>0.1333 (0.2309)</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E421" t="n">
+        <v>0</v>
+      </c>
+      <c r="F421" t="n">
+        <v>0</v>
+      </c>
+      <c r="G421" t="n">
+        <v>0</v>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>0.0000 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E422" t="n">
+        <v>0</v>
+      </c>
+      <c r="F422" t="n">
+        <v>0</v>
+      </c>
+      <c r="G422" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E423" t="n">
+        <v>0</v>
+      </c>
+      <c r="F423" t="n">
+        <v>0</v>
+      </c>
+      <c r="G423" t="n">
+        <v>1</v>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E424" t="n">
+        <v>0</v>
+      </c>
+      <c r="F424" t="n">
+        <v>0</v>
+      </c>
+      <c r="G424" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E425" t="n">
+        <v>0</v>
+      </c>
+      <c r="F425" t="n">
+        <v>0</v>
+      </c>
+      <c r="G425" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="H418" t="inlineStr">
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E426" t="n">
+        <v>0</v>
+      </c>
+      <c r="F426" t="n">
+        <v>0</v>
+      </c>
+      <c r="G426" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E427" t="n">
+        <v>0</v>
+      </c>
+      <c r="F427" t="n">
+        <v>0</v>
+      </c>
+      <c r="G427" t="n">
+        <v>1</v>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E428" t="n">
+        <v>0</v>
+      </c>
+      <c r="F428" t="n">
+        <v>0</v>
+      </c>
+      <c r="G428" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E429" t="n">
+        <v>0</v>
+      </c>
+      <c r="F429" t="n">
+        <v>0</v>
+      </c>
+      <c r="G429" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E430" t="n">
+        <v>0</v>
+      </c>
+      <c r="F430" t="n">
+        <v>0</v>
+      </c>
+      <c r="G430" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E431" t="n">
+        <v>0</v>
+      </c>
+      <c r="F431" t="n">
+        <v>0</v>
+      </c>
+      <c r="G431" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>0.1111 (0.1925)</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E432" t="n">
+        <v>0</v>
+      </c>
+      <c r="F432" t="n">
+        <v>0</v>
+      </c>
+      <c r="G432" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H432" t="inlineStr">
         <is>
           <t>0.2222 (0.3849)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 15:34:45)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H432"/>
+  <dimension ref="A1:H443"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12495,10 +12495,12 @@
       <c r="F336" t="n">
         <v>0.3809523809523809</v>
       </c>
-      <c r="G336" t="inlineStr"/>
+      <c r="G336" t="n">
+        <v>0</v>
+      </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>0.3964 (0.0218)</t>
+          <t>0.2642 (0.2294)</t>
         </is>
       </c>
     </row>
@@ -13246,11 +13248,13 @@
       <c r="E357" t="n">
         <v>0.358974358974359</v>
       </c>
-      <c r="F357" t="inlineStr"/>
+      <c r="F357" t="n">
+        <v>0.1666666666666667</v>
+      </c>
       <c r="G357" t="inlineStr"/>
       <c r="H357" t="inlineStr">
         <is>
-          <t>0.3590 (0.0000)</t>
+          <t>0.2628 (0.1360)</t>
         </is>
       </c>
     </row>
@@ -13350,11 +13354,15 @@
       <c r="E360" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="F360" t="inlineStr"/>
-      <c r="G360" t="inlineStr"/>
+      <c r="F360" t="n">
+        <v>0.2758620689655172</v>
+      </c>
+      <c r="G360" t="n">
+        <v>0.125</v>
+      </c>
       <c r="H360" t="inlineStr">
         <is>
-          <t>0.3333 (0.0000)</t>
+          <t>0.2447 (0.1076)</t>
         </is>
       </c>
     </row>
@@ -13403,7 +13411,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
@@ -13412,17 +13420,17 @@
         </is>
       </c>
       <c r="E362" t="n">
-        <v>0.3</v>
+        <v>0.44</v>
       </c>
       <c r="F362" t="n">
-        <v>0.4117647058823529</v>
+        <v>0.3225806451612903</v>
       </c>
       <c r="G362" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H362" t="inlineStr">
         <is>
-          <t>0.2849 (0.1351)</t>
+          <t>0.3494 (0.0806)</t>
         </is>
       </c>
     </row>
@@ -13439,7 +13447,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
@@ -13448,17 +13456,17 @@
         </is>
       </c>
       <c r="E363" t="n">
-        <v>0.3018867924528302</v>
+        <v>0.3</v>
       </c>
       <c r="F363" t="n">
-        <v>0.2142857142857143</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="G363" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t>0.1998 (0.1100)</t>
+          <t>0.2849 (0.1351)</t>
         </is>
       </c>
     </row>
@@ -13475,7 +13483,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
@@ -13484,13 +13492,17 @@
         </is>
       </c>
       <c r="E364" t="n">
-        <v>0.3720930232558139</v>
-      </c>
-      <c r="F364" t="inlineStr"/>
-      <c r="G364" t="inlineStr"/>
+        <v>0.3018867924528302</v>
+      </c>
+      <c r="F364" t="n">
+        <v>0.2142857142857143</v>
+      </c>
+      <c r="G364" t="n">
+        <v>0.08333333333333333</v>
+      </c>
       <c r="H364" t="inlineStr">
         <is>
-          <t>0.3721 (0.0000)</t>
+          <t>0.1998 (0.1100)</t>
         </is>
       </c>
     </row>
@@ -13507,7 +13519,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
@@ -13516,13 +13528,17 @@
         </is>
       </c>
       <c r="E365" t="n">
-        <v>0.3404255319148936</v>
-      </c>
-      <c r="F365" t="inlineStr"/>
-      <c r="G365" t="inlineStr"/>
+        <v>0.3720930232558139</v>
+      </c>
+      <c r="F365" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="G365" t="n">
+        <v>0.09523809523809523</v>
+      </c>
       <c r="H365" t="inlineStr">
         <is>
-          <t>0.3404 (0.0000)</t>
+          <t>0.2447 (0.1397)</t>
         </is>
       </c>
     </row>
@@ -13534,31 +13550,31 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E366" t="n">
-        <v>0.5769230769230769</v>
+        <v>0.3404255319148936</v>
       </c>
       <c r="F366" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="G366" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H366" t="inlineStr">
         <is>
-          <t>0.2201 (0.3118)</t>
+          <t>0.2579 (0.1368)</t>
         </is>
       </c>
     </row>
@@ -13575,7 +13591,7 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
@@ -13584,17 +13600,17 @@
         </is>
       </c>
       <c r="E367" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="F367" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="G367" t="n">
-        <v>0.08695652173913043</v>
+        <v>0</v>
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>0.2243 (0.1384)</t>
+          <t>0.2201 (0.3118)</t>
         </is>
       </c>
     </row>
@@ -13611,7 +13627,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
@@ -13620,17 +13636,17 @@
         </is>
       </c>
       <c r="E368" t="n">
-        <v>0.456140350877193</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="F368" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="G368" t="n">
-        <v>0</v>
+        <v>0.08695652173913043</v>
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>0.1777 (0.2442)</t>
+          <t>0.2243 (0.1384)</t>
         </is>
       </c>
     </row>
@@ -13647,7 +13663,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
@@ -13656,17 +13672,17 @@
         </is>
       </c>
       <c r="E369" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.456140350877193</v>
       </c>
       <c r="F369" t="n">
-        <v>0.3076923076923077</v>
+        <v>0.07692307692307693</v>
       </c>
       <c r="G369" t="n">
         <v>0</v>
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>0.1978 (0.1717)</t>
+          <t>0.1777 (0.2442)</t>
         </is>
       </c>
     </row>
@@ -13683,7 +13699,7 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
@@ -13692,17 +13708,17 @@
         </is>
       </c>
       <c r="E370" t="n">
-        <v>0.2</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="F370" t="n">
-        <v>0</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="G370" t="n">
         <v>0</v>
       </c>
       <c r="H370" t="inlineStr">
         <is>
-          <t>0.0667 (0.1155)</t>
+          <t>0.1978 (0.1717)</t>
         </is>
       </c>
     </row>
@@ -13714,31 +13730,31 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E371" t="n">
-        <v>0.4090909090909091</v>
+        <v>0.2</v>
       </c>
       <c r="F371" t="n">
-        <v>0.2608695652173913</v>
+        <v>0</v>
       </c>
       <c r="G371" t="n">
         <v>0</v>
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>0.2233 (0.2071)</t>
+          <t>0.0667 (0.1155)</t>
         </is>
       </c>
     </row>
@@ -13755,7 +13771,7 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
@@ -13764,17 +13780,17 @@
         </is>
       </c>
       <c r="E372" t="n">
-        <v>0.2926829268292683</v>
+        <v>0.4090909090909091</v>
       </c>
       <c r="F372" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2608695652173913</v>
       </c>
       <c r="G372" t="n">
-        <v>0.1481481481481481</v>
+        <v>0</v>
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>0.2682 (0.1098)</t>
+          <t>0.2233 (0.2071)</t>
         </is>
       </c>
     </row>
@@ -13791,7 +13807,7 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
@@ -13800,17 +13816,17 @@
         </is>
       </c>
       <c r="E373" t="n">
-        <v>0.3111111111111111</v>
+        <v>0.2926829268292683</v>
       </c>
       <c r="F373" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="G373" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>0.1799 (0.1152)</t>
+          <t>0.2682 (0.1098)</t>
         </is>
       </c>
     </row>
@@ -13827,7 +13843,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D374" t="inlineStr">
@@ -13836,17 +13852,17 @@
         </is>
       </c>
       <c r="E374" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.3111111111111111</v>
       </c>
       <c r="F374" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="G374" t="n">
         <v>0.1333333333333333</v>
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t>0.2508 (0.1045)</t>
+          <t>0.1799 (0.1152)</t>
         </is>
       </c>
     </row>
@@ -13863,7 +13879,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D375" t="inlineStr">
@@ -13872,53 +13888,53 @@
         </is>
       </c>
       <c r="E375" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F375" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G375" t="n">
-        <v>0</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>0.1072 (0.1053)</t>
+          <t>0.2508 (0.1045)</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_OHPROG</t>
+          <t>CEETOX_H295R_ESTRONE</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E376" t="n">
-        <v>0.6486486486486487</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="F376" t="n">
-        <v>0.5</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="G376" t="n">
-        <v>0.6129032258064516</v>
+        <v>0</v>
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>0.5872 (0.0776)</t>
+          <t>0.1072 (0.1053)</t>
         </is>
       </c>
     </row>
@@ -13935,7 +13951,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
@@ -13944,17 +13960,17 @@
         </is>
       </c>
       <c r="E377" t="n">
-        <v>0.5074626865671642</v>
+        <v>0.6486486486486487</v>
       </c>
       <c r="F377" t="n">
-        <v>0.5507246376811594</v>
+        <v>0.5</v>
       </c>
       <c r="G377" t="n">
-        <v>0.6391752577319587</v>
+        <v>0.6129032258064516</v>
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t>0.5658 (0.0671)</t>
+          <t>0.5872 (0.0776)</t>
         </is>
       </c>
     </row>
@@ -13971,7 +13987,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D378" t="inlineStr">
@@ -13980,17 +13996,17 @@
         </is>
       </c>
       <c r="E378" t="n">
-        <v>0.6736842105263158</v>
+        <v>0.5074626865671642</v>
       </c>
       <c r="F378" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G378" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.6391752577319587</v>
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t>0.6502 (0.0208)</t>
+          <t>0.5658 (0.0671)</t>
         </is>
       </c>
     </row>
@@ -14007,7 +14023,7 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D379" t="inlineStr">
@@ -14016,17 +14032,17 @@
         </is>
       </c>
       <c r="E379" t="n">
-        <v>0.6741573033707865</v>
+        <v>0.6736842105263158</v>
       </c>
       <c r="F379" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="G379" t="n">
-        <v>0.6744186046511628</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="H379" t="inlineStr">
         <is>
-          <t>0.6425 (0.0550)</t>
+          <t>0.6502 (0.0208)</t>
         </is>
       </c>
     </row>
@@ -14043,7 +14059,7 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D380" t="inlineStr">
@@ -14052,17 +14068,17 @@
         </is>
       </c>
       <c r="E380" t="n">
-        <v>0.5263157894736842</v>
+        <v>0.6741573033707865</v>
       </c>
       <c r="F380" t="n">
-        <v>0.6285714285714286</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="G380" t="n">
-        <v>0.5901639344262295</v>
+        <v>0.6744186046511628</v>
       </c>
       <c r="H380" t="inlineStr">
         <is>
-          <t>0.5817 (0.0517)</t>
+          <t>0.6425 (0.0550)</t>
         </is>
       </c>
     </row>
@@ -14074,31 +14090,31 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E381" t="n">
-        <v>0.4307692307692308</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="F381" t="n">
-        <v>0.6</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="G381" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.5901639344262295</v>
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t>0.4718 (0.1134)</t>
+          <t>0.5817 (0.0517)</t>
         </is>
       </c>
     </row>
@@ -14115,7 +14131,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D382" t="inlineStr">
@@ -14124,17 +14140,17 @@
         </is>
       </c>
       <c r="E382" t="n">
+        <v>0.4307692307692308</v>
+      </c>
+      <c r="F382" t="n">
         <v>0.6</v>
       </c>
-      <c r="F382" t="n">
-        <v>0.5666666666666667</v>
-      </c>
       <c r="G382" t="n">
-        <v>0.5573770491803278</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t>0.5747 (0.0224)</t>
+          <t>0.4718 (0.1134)</t>
         </is>
       </c>
     </row>
@@ -14151,7 +14167,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D383" t="inlineStr">
@@ -14160,17 +14176,17 @@
         </is>
       </c>
       <c r="E383" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.6</v>
       </c>
       <c r="F383" t="n">
-        <v>0.6</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="G383" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.5573770491803278</v>
       </c>
       <c r="H383" t="inlineStr">
         <is>
-          <t>0.6026 (0.0325)</t>
+          <t>0.5747 (0.0224)</t>
         </is>
       </c>
     </row>
@@ -14187,7 +14203,7 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
@@ -14196,17 +14212,17 @@
         </is>
       </c>
       <c r="E384" t="n">
-        <v>0.6279069767441861</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F384" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.6</v>
       </c>
       <c r="G384" t="n">
-        <v>0.6101694915254238</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t>0.5979 (0.0377)</t>
+          <t>0.6026 (0.0325)</t>
         </is>
       </c>
     </row>
@@ -14223,7 +14239,7 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D385" t="inlineStr">
@@ -14232,17 +14248,17 @@
         </is>
       </c>
       <c r="E385" t="n">
-        <v>0.5915492957746479</v>
+        <v>0.6279069767441861</v>
       </c>
       <c r="F385" t="n">
-        <v>0.4482758620689655</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="G385" t="n">
-        <v>0.4814814814814815</v>
+        <v>0.6101694915254238</v>
       </c>
       <c r="H385" t="inlineStr">
         <is>
-          <t>0.5071 (0.0750)</t>
+          <t>0.5979 (0.0377)</t>
         </is>
       </c>
     </row>
@@ -14254,31 +14270,31 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E386" t="n">
-        <v>0.5079365079365079</v>
+        <v>0.5915492957746479</v>
       </c>
       <c r="F386" t="n">
-        <v>0.5245901639344263</v>
+        <v>0.4482758620689655</v>
       </c>
       <c r="G386" t="n">
-        <v>0.5846153846153846</v>
+        <v>0.4814814814814815</v>
       </c>
       <c r="H386" t="inlineStr">
         <is>
-          <t>0.5390 (0.0403)</t>
+          <t>0.5071 (0.0750)</t>
         </is>
       </c>
     </row>
@@ -14295,7 +14311,7 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
@@ -14304,17 +14320,17 @@
         </is>
       </c>
       <c r="E387" t="n">
-        <v>0.5822784810126582</v>
+        <v>0.5079365079365079</v>
       </c>
       <c r="F387" t="n">
-        <v>0.5507246376811594</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="G387" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5846153846153846</v>
       </c>
       <c r="H387" t="inlineStr">
         <is>
-          <t>0.5554 (0.0248)</t>
+          <t>0.5390 (0.0403)</t>
         </is>
       </c>
     </row>
@@ -14331,7 +14347,7 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
@@ -14340,17 +14356,17 @@
         </is>
       </c>
       <c r="E388" t="n">
-        <v>0.6818181818181818</v>
+        <v>0.5822784810126582</v>
       </c>
       <c r="F388" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.5507246376811594</v>
       </c>
       <c r="G388" t="n">
-        <v>0.53125</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H388" t="inlineStr">
         <is>
-          <t>0.6157 (0.0770)</t>
+          <t>0.5554 (0.0248)</t>
         </is>
       </c>
     </row>
@@ -14367,7 +14383,7 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D389" t="inlineStr">
@@ -14376,17 +14392,17 @@
         </is>
       </c>
       <c r="E389" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.6818181818181818</v>
       </c>
       <c r="F389" t="n">
-        <v>0.5753424657534246</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="G389" t="n">
-        <v>0.4761904761904762</v>
+        <v>0.53125</v>
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t>0.5648 (0.0838)</t>
+          <t>0.6157 (0.0770)</t>
         </is>
       </c>
     </row>
@@ -14403,7 +14419,7 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
@@ -14412,17 +14428,17 @@
         </is>
       </c>
       <c r="E390" t="n">
-        <v>0.631578947368421</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="F390" t="n">
-        <v>0.6268656716417911</v>
+        <v>0.5753424657534246</v>
       </c>
       <c r="G390" t="n">
-        <v>0.5245901639344263</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t>0.5943 (0.0605)</t>
+          <t>0.5648 (0.0838)</t>
         </is>
       </c>
     </row>
@@ -14434,31 +14450,31 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E391" t="n">
-        <v>0.64</v>
+        <v>0.631578947368421</v>
       </c>
       <c r="F391" t="n">
-        <v>0.5588235294117647</v>
+        <v>0.6268656716417911</v>
       </c>
       <c r="G391" t="n">
-        <v>0.6060606060606061</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="H391" t="inlineStr">
         <is>
-          <t>0.6016 (0.0408)</t>
+          <t>0.5943 (0.0605)</t>
         </is>
       </c>
     </row>
@@ -14475,7 +14491,7 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
@@ -14484,17 +14500,17 @@
         </is>
       </c>
       <c r="E392" t="n">
-        <v>0.6578947368421053</v>
+        <v>0.64</v>
       </c>
       <c r="F392" t="n">
-        <v>0.5079365079365079</v>
+        <v>0.5588235294117647</v>
       </c>
       <c r="G392" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>0.5791 (0.0753)</t>
+          <t>0.6016 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -14511,7 +14527,7 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
@@ -14520,17 +14536,17 @@
         </is>
       </c>
       <c r="E393" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6578947368421053</v>
       </c>
       <c r="F393" t="n">
-        <v>0.5633802816901409</v>
+        <v>0.5079365079365079</v>
       </c>
       <c r="G393" t="n">
-        <v>0.6567164179104478</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="H393" t="inlineStr">
         <is>
-          <t>0.6289 (0.0570)</t>
+          <t>0.5791 (0.0753)</t>
         </is>
       </c>
     </row>
@@ -14547,7 +14563,7 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
@@ -14556,17 +14572,17 @@
         </is>
       </c>
       <c r="E394" t="n">
-        <v>0.6436781609195402</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F394" t="n">
-        <v>0.6410256410256411</v>
+        <v>0.5633802816901409</v>
       </c>
       <c r="G394" t="n">
-        <v>0.6756756756756757</v>
+        <v>0.6567164179104478</v>
       </c>
       <c r="H394" t="inlineStr">
         <is>
-          <t>0.6535 (0.0193)</t>
+          <t>0.6289 (0.0570)</t>
         </is>
       </c>
     </row>
@@ -14583,7 +14599,7 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D395" t="inlineStr">
@@ -14592,17 +14608,17 @@
         </is>
       </c>
       <c r="E395" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.6436781609195402</v>
       </c>
       <c r="F395" t="n">
-        <v>0.576271186440678</v>
+        <v>0.6410256410256411</v>
       </c>
       <c r="G395" t="n">
-        <v>0.4150943396226415</v>
+        <v>0.6756756756756757</v>
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t>0.5249 (0.0952)</t>
+          <t>0.6535 (0.0193)</t>
         </is>
       </c>
     </row>
@@ -14614,31 +14630,31 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E396" t="n">
-        <v>0.5373134328358209</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F396" t="n">
-        <v>0.4918032786885246</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="G396" t="n">
-        <v>0.576271186440678</v>
+        <v>0.4150943396226415</v>
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t>0.5351 (0.0423)</t>
+          <t>0.5249 (0.0952)</t>
         </is>
       </c>
     </row>
@@ -14655,7 +14671,7 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D397" t="inlineStr">
@@ -14664,17 +14680,17 @@
         </is>
       </c>
       <c r="E397" t="n">
-        <v>0.6197183098591549</v>
+        <v>0.5373134328358209</v>
       </c>
       <c r="F397" t="n">
-        <v>0.5396825396825397</v>
+        <v>0.4918032786885246</v>
       </c>
       <c r="G397" t="n">
-        <v>0.5423728813559322</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t>0.5673 (0.0455)</t>
+          <t>0.5351 (0.0423)</t>
         </is>
       </c>
     </row>
@@ -14691,7 +14707,7 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D398" t="inlineStr">
@@ -14700,17 +14716,17 @@
         </is>
       </c>
       <c r="E398" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.6197183098591549</v>
       </c>
       <c r="F398" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5396825396825397</v>
       </c>
       <c r="G398" t="n">
-        <v>0.5</v>
+        <v>0.5423728813559322</v>
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t>0.5541 (0.0469)</t>
+          <t>0.5673 (0.0455)</t>
         </is>
       </c>
     </row>
@@ -14727,7 +14743,7 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
@@ -14736,17 +14752,17 @@
         </is>
       </c>
       <c r="E399" t="n">
-        <v>0.675</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="F399" t="n">
-        <v>0.6</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="G399" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t>0.6028 (0.0709)</t>
+          <t>0.5541 (0.0469)</t>
         </is>
       </c>
     </row>
@@ -14763,7 +14779,7 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D400" t="inlineStr">
@@ -14772,53 +14788,53 @@
         </is>
       </c>
       <c r="E400" t="n">
-        <v>0.5070422535211268</v>
+        <v>0.675</v>
       </c>
       <c r="F400" t="n">
-        <v>0.5806451612903226</v>
+        <v>0.6</v>
       </c>
       <c r="G400" t="n">
-        <v>0.4528301886792453</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t>0.5135 (0.0642)</t>
+          <t>0.6028 (0.0709)</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>CEETOX_H295R_PROG</t>
+          <t>CEETOX_H295R_OHPROG</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E401" t="n">
-        <v>0.5316455696202531</v>
+        <v>0.5070422535211268</v>
       </c>
       <c r="F401" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.5806451612903226</v>
       </c>
       <c r="G401" t="n">
-        <v>0.5070422535211268</v>
+        <v>0.4528301886792453</v>
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t>0.5314 (0.0243)</t>
+          <t>0.5135 (0.0642)</t>
         </is>
       </c>
     </row>
@@ -14835,7 +14851,7 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D402" t="inlineStr">
@@ -14844,17 +14860,17 @@
         </is>
       </c>
       <c r="E402" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.5316455696202531</v>
       </c>
       <c r="F402" t="n">
-        <v>0.4313725490196079</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="G402" t="n">
-        <v>0.5217391304347826</v>
+        <v>0.5070422535211268</v>
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t>0.5082 (0.0710)</t>
+          <t>0.5314 (0.0243)</t>
         </is>
       </c>
     </row>
@@ -14871,7 +14887,7 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D403" t="inlineStr">
@@ -14880,17 +14896,17 @@
         </is>
       </c>
       <c r="E403" t="n">
-        <v>0.4477611940298508</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F403" t="n">
-        <v>0.391304347826087</v>
+        <v>0.4313725490196079</v>
       </c>
       <c r="G403" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="H403" t="inlineStr">
         <is>
-          <t>0.3908 (0.0572)</t>
+          <t>0.5082 (0.0710)</t>
         </is>
       </c>
     </row>
@@ -14907,7 +14923,7 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D404" t="inlineStr">
@@ -14916,17 +14932,17 @@
         </is>
       </c>
       <c r="E404" t="n">
-        <v>0.5365853658536586</v>
+        <v>0.4477611940298508</v>
       </c>
       <c r="F404" t="n">
-        <v>0.6060606060606061</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="G404" t="n">
-        <v>0.6</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H404" t="inlineStr">
         <is>
-          <t>0.5809 (0.0385)</t>
+          <t>0.3908 (0.0572)</t>
         </is>
       </c>
     </row>
@@ -14943,7 +14959,7 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D405" t="inlineStr">
@@ -14952,17 +14968,17 @@
         </is>
       </c>
       <c r="E405" t="n">
-        <v>0.6470588235294118</v>
+        <v>0.5365853658536586</v>
       </c>
       <c r="F405" t="n">
-        <v>0.4067796610169492</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="G405" t="n">
-        <v>0.5416666666666666</v>
+        <v>0.6</v>
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t>0.5318 (0.1204)</t>
+          <t>0.5809 (0.0385)</t>
         </is>
       </c>
     </row>
@@ -14974,29 +14990,31 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E406" t="n">
-        <v>0.547945205479452</v>
+        <v>0.6470588235294118</v>
       </c>
       <c r="F406" t="n">
-        <v>0.5106382978723404</v>
-      </c>
-      <c r="G406" t="inlineStr"/>
+        <v>0.4067796610169492</v>
+      </c>
+      <c r="G406" t="n">
+        <v>0.5416666666666666</v>
+      </c>
       <c r="H406" t="inlineStr">
         <is>
-          <t>0.5293 (0.0264)</t>
+          <t>0.5318 (0.1204)</t>
         </is>
       </c>
     </row>
@@ -15008,423 +15026,411 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E407" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F407" t="inlineStr"/>
-      <c r="G407" t="inlineStr"/>
+        <v>0.5428571428571428</v>
+      </c>
+      <c r="F407" t="n">
+        <v>0.391304347826087</v>
+      </c>
+      <c r="G407" t="n">
+        <v>0.4888888888888889</v>
+      </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t>0.5000 (0.0000)</t>
+          <t>0.4744 (0.0768)</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E408" t="n">
-        <v>0</v>
-      </c>
-      <c r="F408" t="n">
-        <v>0</v>
-      </c>
-      <c r="G408" t="n">
-        <v>0.2857142857142857</v>
-      </c>
+        <v>0.5277777777777778</v>
+      </c>
+      <c r="F408" t="inlineStr"/>
+      <c r="G408" t="inlineStr"/>
       <c r="H408" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5278 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E409" t="n">
-        <v>0</v>
+        <v>0.6071428571428571</v>
       </c>
       <c r="F409" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G409" t="n">
-        <v>1</v>
+        <v>0.5531914893617021</v>
       </c>
       <c r="H409" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.5534 (0.0536)</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E410" t="n">
-        <v>0</v>
+        <v>0.547945205479452</v>
       </c>
       <c r="F410" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5106382978723404</v>
       </c>
       <c r="G410" t="n">
         <v>0.4</v>
       </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.4862 (0.0769)</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E411" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F411" t="n">
-        <v>0.25</v>
+        <v>0.4897959183673469</v>
       </c>
       <c r="G411" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.2978723404255319</v>
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>0.1944 (0.1735)</t>
+          <t>0.4292 (0.1139)</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E412" t="n">
-        <v>0</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="F412" t="n">
-        <v>0</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="G412" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.5396825396825397</v>
       </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.5746 (0.0474)</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E413" t="n">
-        <v>0</v>
+        <v>0.5614035087719298</v>
       </c>
       <c r="F413" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="G413" t="n">
-        <v>0.5</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.4521 (0.1143)</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E414" t="n">
-        <v>0</v>
-      </c>
-      <c r="F414" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G414" t="n">
-        <v>0.6666666666666666</v>
-      </c>
+        <v>0.5483870967741935</v>
+      </c>
+      <c r="F414" t="inlineStr"/>
+      <c r="G414" t="inlineStr"/>
       <c r="H414" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.5484 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E415" t="n">
-        <v>0</v>
+        <v>0.4864864864864865</v>
       </c>
       <c r="F415" t="n">
-        <v>0</v>
+        <v>0.32</v>
       </c>
       <c r="G415" t="n">
-        <v>0.4</v>
+        <v>0.3404255319148936</v>
       </c>
       <c r="H415" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.3823 (0.0908)</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E416" t="n">
-        <v>0</v>
+        <v>0.5588235294117647</v>
       </c>
       <c r="F416" t="n">
-        <v>0</v>
+        <v>0.5098039215686274</v>
       </c>
       <c r="G416" t="n">
-        <v>0.4</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.4155 (0.2073)</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E417" t="n">
-        <v>0</v>
-      </c>
-      <c r="F417" t="n">
-        <v>0</v>
-      </c>
-      <c r="G417" t="n">
-        <v>1</v>
-      </c>
+        <v>0.5901639344262295</v>
+      </c>
+      <c r="F417" t="inlineStr"/>
+      <c r="G417" t="inlineStr"/>
       <c r="H417" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.5902 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E418" t="n">
-        <v>0</v>
-      </c>
-      <c r="F418" t="n">
-        <v>0</v>
-      </c>
-      <c r="G418" t="n">
-        <v>0.5</v>
-      </c>
+        <v>0.5757575757575758</v>
+      </c>
+      <c r="F418" t="inlineStr"/>
+      <c r="G418" t="inlineStr"/>
       <c r="H418" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.5758 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -15436,17 +15442,17 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E419" t="n">
@@ -15456,11 +15462,11 @@
         <v>0</v>
       </c>
       <c r="G419" t="n">
-        <v>0.4</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -15472,17 +15478,17 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E420" t="n">
@@ -15492,11 +15498,11 @@
         <v>0</v>
       </c>
       <c r="G420" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -15508,31 +15514,31 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E421" t="n">
         <v>0</v>
       </c>
       <c r="F421" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G421" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="H421" t="inlineStr">
         <is>
-          <t>0.0000 (0.0000)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -15544,31 +15550,31 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E422" t="n">
         <v>0</v>
       </c>
       <c r="F422" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G422" t="n">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H422" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.1944 (0.1735)</t>
         </is>
       </c>
     </row>
@@ -15580,17 +15586,17 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E423" t="n">
@@ -15600,11 +15606,11 @@
         <v>0</v>
       </c>
       <c r="G423" t="n">
-        <v>1</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H423" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -15616,17 +15622,17 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E424" t="n">
@@ -15652,31 +15658,31 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E425" t="n">
         <v>0</v>
       </c>
       <c r="F425" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G425" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -15688,17 +15694,17 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E426" t="n">
@@ -15708,11 +15714,11 @@
         <v>0</v>
       </c>
       <c r="G426" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H426" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -15724,17 +15730,17 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E427" t="n">
@@ -15744,11 +15750,11 @@
         <v>0</v>
       </c>
       <c r="G427" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -15760,17 +15766,17 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E428" t="n">
@@ -15780,11 +15786,11 @@
         <v>0</v>
       </c>
       <c r="G428" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -15796,17 +15802,17 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E429" t="n">
@@ -15816,11 +15822,11 @@
         <v>0</v>
       </c>
       <c r="G429" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -15832,17 +15838,17 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E430" t="n">
@@ -15852,11 +15858,11 @@
         <v>0</v>
       </c>
       <c r="G430" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -15868,17 +15874,17 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E431" t="n">
@@ -15888,11 +15894,11 @@
         <v>0</v>
       </c>
       <c r="G431" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="H431" t="inlineStr">
         <is>
-          <t>0.1111 (0.1925)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -15904,17 +15910,17 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E432" t="n">
@@ -15924,9 +15930,405 @@
         <v>0</v>
       </c>
       <c r="G432" t="n">
+        <v>0</v>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>0.0000 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="E433" t="n">
+        <v>0</v>
+      </c>
+      <c r="F433" t="n">
+        <v>0</v>
+      </c>
+      <c r="G433" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E434" t="n">
+        <v>0</v>
+      </c>
+      <c r="F434" t="n">
+        <v>0</v>
+      </c>
+      <c r="G434" t="n">
+        <v>1</v>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E435" t="n">
+        <v>0</v>
+      </c>
+      <c r="F435" t="n">
+        <v>0</v>
+      </c>
+      <c r="G435" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E436" t="n">
+        <v>0</v>
+      </c>
+      <c r="F436" t="n">
+        <v>0</v>
+      </c>
+      <c r="G436" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="H432" t="inlineStr">
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E437" t="n">
+        <v>0</v>
+      </c>
+      <c r="F437" t="n">
+        <v>0</v>
+      </c>
+      <c r="G437" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E438" t="n">
+        <v>0</v>
+      </c>
+      <c r="F438" t="n">
+        <v>0</v>
+      </c>
+      <c r="G438" t="n">
+        <v>1</v>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E439" t="n">
+        <v>0</v>
+      </c>
+      <c r="F439" t="n">
+        <v>0</v>
+      </c>
+      <c r="G439" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E440" t="n">
+        <v>0</v>
+      </c>
+      <c r="F440" t="n">
+        <v>0</v>
+      </c>
+      <c r="G440" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E441" t="n">
+        <v>0</v>
+      </c>
+      <c r="F441" t="n">
+        <v>0</v>
+      </c>
+      <c r="G441" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E442" t="n">
+        <v>0</v>
+      </c>
+      <c r="F442" t="n">
+        <v>0</v>
+      </c>
+      <c r="G442" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>0.1111 (0.1925)</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E443" t="n">
+        <v>0</v>
+      </c>
+      <c r="F443" t="n">
+        <v>0</v>
+      </c>
+      <c r="G443" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H443" t="inlineStr">
         <is>
           <t>0.2222 (0.3849)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 16:35:06)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H443"/>
+  <dimension ref="A1:H454"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13251,10 +13251,12 @@
       <c r="F357" t="n">
         <v>0.1666666666666667</v>
       </c>
-      <c r="G357" t="inlineStr"/>
+      <c r="G357" t="n">
+        <v>0</v>
+      </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>0.2628 (0.1360)</t>
+          <t>0.1752 (0.1796)</t>
         </is>
       </c>
     </row>
@@ -13390,11 +13392,13 @@
       <c r="E361" t="n">
         <v>0.2631578947368421</v>
       </c>
-      <c r="F361" t="inlineStr"/>
+      <c r="F361" t="n">
+        <v>0.1176470588235294</v>
+      </c>
       <c r="G361" t="inlineStr"/>
       <c r="H361" t="inlineStr">
         <is>
-          <t>0.2632 (0.0000)</t>
+          <t>0.1904 (0.1029)</t>
         </is>
       </c>
     </row>
@@ -15031,7 +15035,7 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
@@ -15040,17 +15044,13 @@
         </is>
       </c>
       <c r="E407" t="n">
-        <v>0.5428571428571428</v>
-      </c>
-      <c r="F407" t="n">
-        <v>0.391304347826087</v>
-      </c>
-      <c r="G407" t="n">
-        <v>0.4888888888888889</v>
-      </c>
+        <v>0.5625</v>
+      </c>
+      <c r="F407" t="inlineStr"/>
+      <c r="G407" t="inlineStr"/>
       <c r="H407" t="inlineStr">
         <is>
-          <t>0.4744 (0.0768)</t>
+          <t>0.5625 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -15067,7 +15067,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D408" t="inlineStr">
@@ -15076,13 +15076,17 @@
         </is>
       </c>
       <c r="E408" t="n">
-        <v>0.5277777777777778</v>
-      </c>
-      <c r="F408" t="inlineStr"/>
-      <c r="G408" t="inlineStr"/>
+        <v>0.5428571428571428</v>
+      </c>
+      <c r="F408" t="n">
+        <v>0.391304347826087</v>
+      </c>
+      <c r="G408" t="n">
+        <v>0.4888888888888889</v>
+      </c>
       <c r="H408" t="inlineStr">
         <is>
-          <t>0.5278 (0.0000)</t>
+          <t>0.4744 (0.0768)</t>
         </is>
       </c>
     </row>
@@ -15094,31 +15098,31 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E409" t="n">
-        <v>0.6071428571428571</v>
+        <v>0.5277777777777778</v>
       </c>
       <c r="F409" t="n">
-        <v>0.5</v>
+        <v>0.5454545454545454</v>
       </c>
       <c r="G409" t="n">
-        <v>0.5531914893617021</v>
+        <v>0.2127659574468085</v>
       </c>
       <c r="H409" t="inlineStr">
         <is>
-          <t>0.5534 (0.0536)</t>
+          <t>0.4287 (0.1872)</t>
         </is>
       </c>
     </row>
@@ -15130,31 +15134,29 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E410" t="n">
-        <v>0.547945205479452</v>
+        <v>0.5135135135135135</v>
       </c>
       <c r="F410" t="n">
-        <v>0.5106382978723404</v>
-      </c>
-      <c r="G410" t="n">
-        <v>0.4</v>
-      </c>
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="G410" t="inlineStr"/>
       <c r="H410" t="inlineStr">
         <is>
-          <t>0.4862 (0.0769)</t>
+          <t>0.5425 (0.0410)</t>
         </is>
       </c>
     </row>
@@ -15166,31 +15168,27 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E411" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F411" t="n">
-        <v>0.4897959183673469</v>
-      </c>
-      <c r="G411" t="n">
-        <v>0.2978723404255319</v>
-      </c>
+        <v>0.59375</v>
+      </c>
+      <c r="F411" t="inlineStr"/>
+      <c r="G411" t="inlineStr"/>
       <c r="H411" t="inlineStr">
         <is>
-          <t>0.4292 (0.1139)</t>
+          <t>0.5938 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -15202,31 +15200,27 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E412" t="n">
-        <v>0.6285714285714286</v>
-      </c>
-      <c r="F412" t="n">
-        <v>0.5555555555555556</v>
-      </c>
-      <c r="G412" t="n">
-        <v>0.5396825396825397</v>
-      </c>
+        <v>0.360655737704918</v>
+      </c>
+      <c r="F412" t="inlineStr"/>
+      <c r="G412" t="inlineStr"/>
       <c r="H412" t="inlineStr">
         <is>
-          <t>0.5746 (0.0474)</t>
+          <t>0.3607 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -15238,31 +15232,31 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E413" t="n">
-        <v>0.5614035087719298</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="F413" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4193548387096774</v>
       </c>
       <c r="G413" t="n">
-        <v>0.4615384615384616</v>
+        <v>0.4074074074074074</v>
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t>0.4521 (0.1143)</t>
+          <t>0.4551 (0.0725)</t>
         </is>
       </c>
     </row>
@@ -15274,27 +15268,31 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E414" t="n">
-        <v>0.5483870967741935</v>
-      </c>
-      <c r="F414" t="inlineStr"/>
-      <c r="G414" t="inlineStr"/>
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="F414" t="n">
+        <v>0.5185185185185185</v>
+      </c>
+      <c r="G414" t="n">
+        <v>0.1818181818181818</v>
+      </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t>0.5484 (0.0000)</t>
+          <t>0.4239 (0.2113)</t>
         </is>
       </c>
     </row>
@@ -15306,31 +15304,29 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E415" t="n">
-        <v>0.4864864864864865</v>
+        <v>0.5373134328358209</v>
       </c>
       <c r="F415" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="G415" t="n">
-        <v>0.3404255319148936</v>
-      </c>
+        <v>0.5084745762711864</v>
+      </c>
+      <c r="G415" t="inlineStr"/>
       <c r="H415" t="inlineStr">
         <is>
-          <t>0.3823 (0.0908)</t>
+          <t>0.5229 (0.0204)</t>
         </is>
       </c>
     </row>
@@ -15342,31 +15338,29 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E416" t="n">
-        <v>0.5588235294117647</v>
+        <v>0.5753424657534246</v>
       </c>
       <c r="F416" t="n">
-        <v>0.5098039215686274</v>
-      </c>
-      <c r="G416" t="n">
-        <v>0.1777777777777778</v>
-      </c>
+        <v>0.392156862745098</v>
+      </c>
+      <c r="G416" t="inlineStr"/>
       <c r="H416" t="inlineStr">
         <is>
-          <t>0.4155 (0.2073)</t>
+          <t>0.4837 (0.1295)</t>
         </is>
       </c>
     </row>
@@ -15378,27 +15372,31 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E417" t="n">
-        <v>0.5901639344262295</v>
-      </c>
-      <c r="F417" t="inlineStr"/>
-      <c r="G417" t="inlineStr"/>
+        <v>0.6071428571428571</v>
+      </c>
+      <c r="F417" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G417" t="n">
+        <v>0.5531914893617021</v>
+      </c>
       <c r="H417" t="inlineStr">
         <is>
-          <t>0.5902 (0.0000)</t>
+          <t>0.5534 (0.0536)</t>
         </is>
       </c>
     </row>
@@ -15410,315 +15408,319 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E418" t="n">
-        <v>0.5757575757575758</v>
-      </c>
-      <c r="F418" t="inlineStr"/>
-      <c r="G418" t="inlineStr"/>
+        <v>0.547945205479452</v>
+      </c>
+      <c r="F418" t="n">
+        <v>0.5106382978723404</v>
+      </c>
+      <c r="G418" t="n">
+        <v>0.4</v>
+      </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t>0.5758 (0.0000)</t>
+          <t>0.4862 (0.0769)</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E419" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F419" t="n">
-        <v>0</v>
+        <v>0.4897959183673469</v>
       </c>
       <c r="G419" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2978723404255319</v>
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.4292 (0.1139)</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E420" t="n">
-        <v>0</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="F420" t="n">
-        <v>0</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="G420" t="n">
-        <v>1</v>
+        <v>0.5396825396825397</v>
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.5746 (0.0474)</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E421" t="n">
-        <v>0</v>
+        <v>0.5614035087719298</v>
       </c>
       <c r="F421" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="G421" t="n">
-        <v>0.4</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="H421" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.4521 (0.1143)</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E422" t="n">
-        <v>0</v>
+        <v>0.5483870967741935</v>
       </c>
       <c r="F422" t="n">
-        <v>0.25</v>
+        <v>0.4545454545454545</v>
       </c>
       <c r="G422" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.425531914893617</v>
       </c>
       <c r="H422" t="inlineStr">
         <is>
-          <t>0.1944 (0.1735)</t>
+          <t>0.4762 (0.0642)</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E423" t="n">
-        <v>0</v>
+        <v>0.4864864864864865</v>
       </c>
       <c r="F423" t="n">
-        <v>0</v>
+        <v>0.32</v>
       </c>
       <c r="G423" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3404255319148936</v>
       </c>
       <c r="H423" t="inlineStr">
         <is>
-          <t>0.0952 (0.1650)</t>
+          <t>0.3823 (0.0908)</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E424" t="n">
-        <v>0</v>
+        <v>0.5588235294117647</v>
       </c>
       <c r="F424" t="n">
-        <v>0</v>
+        <v>0.5098039215686274</v>
       </c>
       <c r="G424" t="n">
-        <v>0.5</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.4155 (0.2073)</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E425" t="n">
-        <v>0</v>
+        <v>0.5901639344262295</v>
       </c>
       <c r="F425" t="n">
-        <v>0.4</v>
+        <v>0.5925925925925926</v>
       </c>
       <c r="G425" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t>0.3556 (0.3355)</t>
+          <t>0.5691 (0.0386)</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>NVS_ENZ_hVEGFR3</t>
+          <t>CEETOX_H295R_PROG</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E426" t="n">
-        <v>0</v>
+        <v>0.5757575757575758</v>
       </c>
       <c r="F426" t="n">
-        <v>0</v>
+        <v>0.3720930232558139</v>
       </c>
       <c r="G426" t="n">
-        <v>0.4</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="H426" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.4464 (0.1125)</t>
         </is>
       </c>
     </row>
@@ -15730,17 +15732,17 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E427" t="n">
@@ -15750,11 +15752,11 @@
         <v>0</v>
       </c>
       <c r="G427" t="n">
-        <v>0.4</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -15766,17 +15768,17 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E428" t="n">
@@ -15802,31 +15804,31 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E429" t="n">
         <v>0</v>
       </c>
       <c r="F429" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G429" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -15838,31 +15840,31 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E430" t="n">
         <v>0</v>
       </c>
       <c r="F430" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G430" t="n">
-        <v>0.4</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.1944 (0.1735)</t>
         </is>
       </c>
     </row>
@@ -15874,17 +15876,17 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E431" t="n">
@@ -15894,11 +15896,11 @@
         <v>0</v>
       </c>
       <c r="G431" t="n">
-        <v>0.4</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="H431" t="inlineStr">
         <is>
-          <t>0.1333 (0.2309)</t>
+          <t>0.0952 (0.1650)</t>
         </is>
       </c>
     </row>
@@ -15910,17 +15912,17 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E432" t="n">
@@ -15930,11 +15932,11 @@
         <v>0</v>
       </c>
       <c r="G432" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t>0.0000 (0.0000)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -15946,31 +15948,31 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E433" t="n">
         <v>0</v>
       </c>
       <c r="F433" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G433" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="H433" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.3556 (0.3355)</t>
         </is>
       </c>
     </row>
@@ -15982,17 +15984,17 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E434" t="n">
@@ -16002,11 +16004,11 @@
         <v>0</v>
       </c>
       <c r="G434" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -16018,17 +16020,17 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E435" t="n">
@@ -16038,11 +16040,11 @@
         <v>0</v>
       </c>
       <c r="G435" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="H435" t="inlineStr">
         <is>
-          <t>0.1667 (0.2887)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -16054,17 +16056,17 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E436" t="n">
@@ -16074,11 +16076,11 @@
         <v>0</v>
       </c>
       <c r="G436" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="H436" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -16090,17 +16092,17 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E437" t="n">
@@ -16110,11 +16112,11 @@
         <v>0</v>
       </c>
       <c r="G437" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -16126,17 +16128,17 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E438" t="n">
@@ -16146,11 +16148,11 @@
         <v>0</v>
       </c>
       <c r="G438" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="H438" t="inlineStr">
         <is>
-          <t>0.3333 (0.5774)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -16162,17 +16164,17 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E439" t="n">
@@ -16182,11 +16184,11 @@
         <v>0</v>
       </c>
       <c r="G439" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H439" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1333 (0.2309)</t>
         </is>
       </c>
     </row>
@@ -16198,17 +16200,17 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E440" t="n">
@@ -16218,11 +16220,11 @@
         <v>0</v>
       </c>
       <c r="G440" t="n">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="H440" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.0000 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -16234,17 +16236,17 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E441" t="n">
@@ -16254,11 +16256,11 @@
         <v>0</v>
       </c>
       <c r="G441" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="H441" t="inlineStr">
         <is>
-          <t>0.2222 (0.3849)</t>
+          <t>0.1667 (0.2887)</t>
         </is>
       </c>
     </row>
@@ -16270,17 +16272,17 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E442" t="n">
@@ -16290,11 +16292,11 @@
         <v>0</v>
       </c>
       <c r="G442" t="n">
-        <v>0.3333333333333333</v>
+        <v>1</v>
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>0.1111 (0.1925)</t>
+          <t>0.3333 (0.5774)</t>
         </is>
       </c>
     </row>
@@ -16306,17 +16308,17 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E443" t="n">
@@ -16326,11 +16328,403 @@
         <v>0</v>
       </c>
       <c r="G443" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>0.1667 (0.2887)</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E444" t="n">
+        <v>0</v>
+      </c>
+      <c r="F444" t="n">
+        <v>0</v>
+      </c>
+      <c r="G444" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="H443" t="inlineStr">
+      <c r="H444" t="inlineStr">
         <is>
           <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E445" t="n">
+        <v>0</v>
+      </c>
+      <c r="F445" t="n">
+        <v>0</v>
+      </c>
+      <c r="G445" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E446" t="n">
+        <v>0</v>
+      </c>
+      <c r="F446" t="n">
+        <v>0</v>
+      </c>
+      <c r="G446" t="n">
+        <v>1</v>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>0.3333 (0.5774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E447" t="n">
+        <v>0</v>
+      </c>
+      <c r="F447" t="n">
+        <v>0</v>
+      </c>
+      <c r="G447" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E448" t="n">
+        <v>0</v>
+      </c>
+      <c r="F448" t="n">
+        <v>0</v>
+      </c>
+      <c r="G448" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E449" t="n">
+        <v>0</v>
+      </c>
+      <c r="F449" t="n">
+        <v>0</v>
+      </c>
+      <c r="G449" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E450" t="n">
+        <v>0</v>
+      </c>
+      <c r="F450" t="n">
+        <v>0</v>
+      </c>
+      <c r="G450" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>0.1111 (0.1925)</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>NVS_ENZ_hVEGFR3</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E451" t="n">
+        <v>0</v>
+      </c>
+      <c r="F451" t="n">
+        <v>0</v>
+      </c>
+      <c r="G451" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>0.2222 (0.3849)</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E452" t="n">
+        <v>0.3431952662721893</v>
+      </c>
+      <c r="F452" t="n">
+        <v>0.2333333333333333</v>
+      </c>
+      <c r="G452" t="n">
+        <v>0.2145593869731801</v>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>0.2637 (0.0695)</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E453" t="n">
+        <v>0.2584615384615385</v>
+      </c>
+      <c r="F453" t="n">
+        <v>0.2804428044280443</v>
+      </c>
+      <c r="G453" t="n">
+        <v>0.1886792452830189</v>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>0.2425 (0.0479)</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E454" t="n">
+        <v>0.2574850299401197</v>
+      </c>
+      <c r="F454" t="inlineStr"/>
+      <c r="G454" t="inlineStr"/>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>0.2575 (0.0000)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 17:35:25)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H454"/>
+  <dimension ref="A1:H463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13395,10 +13395,12 @@
       <c r="F361" t="n">
         <v>0.1176470588235294</v>
       </c>
-      <c r="G361" t="inlineStr"/>
+      <c r="G361" t="n">
+        <v>0</v>
+      </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t>0.1904 (0.1029)</t>
+          <t>0.1269 (0.1318)</t>
         </is>
       </c>
     </row>
@@ -15046,11 +15048,13 @@
       <c r="E407" t="n">
         <v>0.5625</v>
       </c>
-      <c r="F407" t="inlineStr"/>
+      <c r="F407" t="n">
+        <v>0.4705882352941176</v>
+      </c>
       <c r="G407" t="inlineStr"/>
       <c r="H407" t="inlineStr">
         <is>
-          <t>0.5625 (0.0000)</t>
+          <t>0.5165 (0.0650)</t>
         </is>
       </c>
     </row>
@@ -15153,10 +15157,12 @@
       <c r="F410" t="n">
         <v>0.5714285714285714</v>
       </c>
-      <c r="G410" t="inlineStr"/>
+      <c r="G410" t="n">
+        <v>0.4444444444444444</v>
+      </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t>0.5425 (0.0410)</t>
+          <t>0.5098 (0.0636)</t>
         </is>
       </c>
     </row>
@@ -15184,11 +15190,13 @@
       <c r="E411" t="n">
         <v>0.59375</v>
       </c>
-      <c r="F411" t="inlineStr"/>
+      <c r="F411" t="n">
+        <v>0.4545454545454545</v>
+      </c>
       <c r="G411" t="inlineStr"/>
       <c r="H411" t="inlineStr">
         <is>
-          <t>0.5938 (0.0000)</t>
+          <t>0.5241 (0.0984)</t>
         </is>
       </c>
     </row>
@@ -15216,11 +15224,15 @@
       <c r="E412" t="n">
         <v>0.360655737704918</v>
       </c>
-      <c r="F412" t="inlineStr"/>
-      <c r="G412" t="inlineStr"/>
+      <c r="F412" t="n">
+        <v>0.4912280701754386</v>
+      </c>
+      <c r="G412" t="n">
+        <v>0.4897959183673469</v>
+      </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t>0.3607 (0.0000)</t>
+          <t>0.4472 (0.0750)</t>
         </is>
       </c>
     </row>
@@ -15323,10 +15335,12 @@
       <c r="F415" t="n">
         <v>0.5084745762711864</v>
       </c>
-      <c r="G415" t="inlineStr"/>
+      <c r="G415" t="n">
+        <v>0.5357142857142857</v>
+      </c>
       <c r="H415" t="inlineStr">
         <is>
-          <t>0.5229 (0.0204)</t>
+          <t>0.5272 (0.0162)</t>
         </is>
       </c>
     </row>
@@ -15357,10 +15371,12 @@
       <c r="F416" t="n">
         <v>0.392156862745098</v>
       </c>
-      <c r="G416" t="inlineStr"/>
+      <c r="G416" t="n">
+        <v>0.4</v>
+      </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t>0.4837 (0.1295)</t>
+          <t>0.4558 (0.1036)</t>
         </is>
       </c>
     </row>
@@ -16637,7 +16653,7 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D452" t="inlineStr">
@@ -16646,17 +16662,17 @@
         </is>
       </c>
       <c r="E452" t="n">
-        <v>0.3431952662721893</v>
+        <v>0.2346041055718475</v>
       </c>
       <c r="F452" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2926829268292683</v>
       </c>
       <c r="G452" t="n">
-        <v>0.2145593869731801</v>
+        <v>0.28</v>
       </c>
       <c r="H452" t="inlineStr">
         <is>
-          <t>0.2637 (0.0695)</t>
+          <t>0.2691 (0.0305)</t>
         </is>
       </c>
     </row>
@@ -16673,7 +16689,7 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D453" t="inlineStr">
@@ -16682,17 +16698,17 @@
         </is>
       </c>
       <c r="E453" t="n">
-        <v>0.2584615384615385</v>
+        <v>0.3431952662721893</v>
       </c>
       <c r="F453" t="n">
-        <v>0.2804428044280443</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G453" t="n">
-        <v>0.1886792452830189</v>
+        <v>0.2145593869731801</v>
       </c>
       <c r="H453" t="inlineStr">
         <is>
-          <t>0.2425 (0.0479)</t>
+          <t>0.2637 (0.0695)</t>
         </is>
       </c>
     </row>
@@ -16709,22 +16725,346 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E454" t="n">
+        <v>0.2584615384615385</v>
+      </c>
+      <c r="F454" t="n">
+        <v>0.2804428044280443</v>
+      </c>
+      <c r="G454" t="n">
+        <v>0.1886792452830189</v>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>0.2425 (0.0479)</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E455" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F455" t="n">
+        <v>0.2671232876712329</v>
+      </c>
+      <c r="G455" t="n">
+        <v>0.2490566037735849</v>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>0.2787 (0.0369)</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D454" t="inlineStr">
+      <c r="D456" t="inlineStr">
         <is>
           <t>DecisionTree</t>
         </is>
       </c>
-      <c r="E454" t="n">
+      <c r="E456" t="n">
         <v>0.2574850299401197</v>
       </c>
-      <c r="F454" t="inlineStr"/>
-      <c r="G454" t="inlineStr"/>
-      <c r="H454" t="inlineStr">
-        <is>
-          <t>0.2575 (0.0000)</t>
+      <c r="F456" t="n">
+        <v>0.2148148148148148</v>
+      </c>
+      <c r="G456" t="n">
+        <v>0.2320819112627986</v>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>0.2348 (0.0215)</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E457" t="n">
+        <v>0.3007518796992481</v>
+      </c>
+      <c r="F457" t="n">
+        <v>0.1627906976744186</v>
+      </c>
+      <c r="G457" t="n">
+        <v>0.1818181818181818</v>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>0.2151 (0.0748)</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E458" t="n">
+        <v>0.3321033210332103</v>
+      </c>
+      <c r="F458" t="n">
+        <v>0.2543859649122807</v>
+      </c>
+      <c r="G458" t="n">
+        <v>0.2901554404145077</v>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>0.2922 (0.0389)</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E459" t="n">
+        <v>0.1209302325581395</v>
+      </c>
+      <c r="F459" t="n">
+        <v>0.1182795698924731</v>
+      </c>
+      <c r="G459" t="n">
+        <v>0.1548387096774194</v>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>0.1313 (0.0204)</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E460" t="n">
+        <v>0.391304347826087</v>
+      </c>
+      <c r="F460" t="n">
+        <v>0.3221476510067114</v>
+      </c>
+      <c r="G460" t="n">
+        <v>0.3011583011583012</v>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>0.3382 (0.0472)</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E461" t="n">
+        <v>0.2068965517241379</v>
+      </c>
+      <c r="F461" t="n">
+        <v>0.1837837837837838</v>
+      </c>
+      <c r="G461" t="n">
+        <v>0.2054794520547945</v>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>0.1987 (0.0130)</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E462" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F462" t="n">
+        <v>0.2698412698412698</v>
+      </c>
+      <c r="G462" t="n">
+        <v>0.2639593908629442</v>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>0.2821 (0.0265)</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E463" t="n">
+        <v>0.1818181818181818</v>
+      </c>
+      <c r="F463" t="inlineStr"/>
+      <c r="G463" t="inlineStr"/>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>0.1818 (0.0000)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 18:35:43)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H463"/>
+  <dimension ref="A1:H467"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15051,10 +15051,12 @@
       <c r="F407" t="n">
         <v>0.4705882352941176</v>
       </c>
-      <c r="G407" t="inlineStr"/>
+      <c r="G407" t="n">
+        <v>0.4489795918367347</v>
+      </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t>0.5165 (0.0650)</t>
+          <t>0.4940 (0.0603)</t>
         </is>
       </c>
     </row>
@@ -15193,10 +15195,12 @@
       <c r="F411" t="n">
         <v>0.4545454545454545</v>
       </c>
-      <c r="G411" t="inlineStr"/>
+      <c r="G411" t="n">
+        <v>0.3636363636363636</v>
+      </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>0.5241 (0.0984)</t>
+          <t>0.4706 (0.1159)</t>
         </is>
       </c>
     </row>
@@ -16828,31 +16832,27 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E457" t="n">
-        <v>0.3007518796992481</v>
-      </c>
-      <c r="F457" t="n">
-        <v>0.1627906976744186</v>
-      </c>
-      <c r="G457" t="n">
-        <v>0.1818181818181818</v>
-      </c>
+        <v>0.302013422818792</v>
+      </c>
+      <c r="F457" t="inlineStr"/>
+      <c r="G457" t="inlineStr"/>
       <c r="H457" t="inlineStr">
         <is>
-          <t>0.2151 (0.0748)</t>
+          <t>0.3020 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -16869,7 +16869,7 @@
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
@@ -16878,17 +16878,17 @@
         </is>
       </c>
       <c r="E458" t="n">
-        <v>0.3321033210332103</v>
+        <v>0.3007518796992481</v>
       </c>
       <c r="F458" t="n">
-        <v>0.2543859649122807</v>
+        <v>0.1627906976744186</v>
       </c>
       <c r="G458" t="n">
-        <v>0.2901554404145077</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H458" t="inlineStr">
         <is>
-          <t>0.2922 (0.0389)</t>
+          <t>0.2151 (0.0748)</t>
         </is>
       </c>
     </row>
@@ -16905,7 +16905,7 @@
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
@@ -16914,17 +16914,17 @@
         </is>
       </c>
       <c r="E459" t="n">
-        <v>0.1209302325581395</v>
+        <v>0.3321033210332103</v>
       </c>
       <c r="F459" t="n">
-        <v>0.1182795698924731</v>
+        <v>0.2543859649122807</v>
       </c>
       <c r="G459" t="n">
-        <v>0.1548387096774194</v>
+        <v>0.2901554404145077</v>
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>0.1313 (0.0204)</t>
+          <t>0.2922 (0.0389)</t>
         </is>
       </c>
     </row>
@@ -16941,7 +16941,7 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
@@ -16950,17 +16950,17 @@
         </is>
       </c>
       <c r="E460" t="n">
-        <v>0.391304347826087</v>
+        <v>0.1209302325581395</v>
       </c>
       <c r="F460" t="n">
-        <v>0.3221476510067114</v>
+        <v>0.1182795698924731</v>
       </c>
       <c r="G460" t="n">
-        <v>0.3011583011583012</v>
+        <v>0.1548387096774194</v>
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>0.3382 (0.0472)</t>
+          <t>0.1313 (0.0204)</t>
         </is>
       </c>
     </row>
@@ -16977,7 +16977,7 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
@@ -16986,17 +16986,17 @@
         </is>
       </c>
       <c r="E461" t="n">
-        <v>0.2068965517241379</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="F461" t="n">
-        <v>0.1837837837837838</v>
+        <v>0.3221476510067114</v>
       </c>
       <c r="G461" t="n">
-        <v>0.2054794520547945</v>
+        <v>0.3011583011583012</v>
       </c>
       <c r="H461" t="inlineStr">
         <is>
-          <t>0.1987 (0.0130)</t>
+          <t>0.3382 (0.0472)</t>
         </is>
       </c>
     </row>
@@ -17008,31 +17008,31 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E462" t="n">
-        <v>0.3125</v>
+        <v>0.2068965517241379</v>
       </c>
       <c r="F462" t="n">
-        <v>0.2698412698412698</v>
+        <v>0.1837837837837838</v>
       </c>
       <c r="G462" t="n">
-        <v>0.2639593908629442</v>
+        <v>0.2054794520547945</v>
       </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t>0.2821 (0.0265)</t>
+          <t>0.1987 (0.0130)</t>
         </is>
       </c>
     </row>
@@ -17049,7 +17049,7 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
@@ -17058,13 +17058,149 @@
         </is>
       </c>
       <c r="E463" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="F463" t="inlineStr"/>
       <c r="G463" t="inlineStr"/>
       <c r="H463" t="inlineStr">
         <is>
-          <t>0.1818 (0.0000)</t>
+          <t>0.3030 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E464" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F464" t="n">
+        <v>0.2698412698412698</v>
+      </c>
+      <c r="G464" t="n">
+        <v>0.2639593908629442</v>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>0.2821 (0.0265)</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E465" t="n">
+        <v>0.1818181818181818</v>
+      </c>
+      <c r="F465" t="n">
+        <v>0.1256544502617801</v>
+      </c>
+      <c r="G465" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>0.1692 (0.0388)</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E466" t="n">
+        <v>0.3709090909090909</v>
+      </c>
+      <c r="F466" t="inlineStr"/>
+      <c r="G466" t="inlineStr"/>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>0.3709 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E467" t="n">
+        <v>0.3135593220338983</v>
+      </c>
+      <c r="F467" t="inlineStr"/>
+      <c r="G467" t="inlineStr"/>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>0.3136 (0.0000)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 19:36:01)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H467"/>
+  <dimension ref="A1:H468"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16848,11 +16848,13 @@
       <c r="E457" t="n">
         <v>0.302013422818792</v>
       </c>
-      <c r="F457" t="inlineStr"/>
+      <c r="F457" t="n">
+        <v>0.296875</v>
+      </c>
       <c r="G457" t="inlineStr"/>
       <c r="H457" t="inlineStr">
         <is>
-          <t>0.3020 (0.0000)</t>
+          <t>0.2994 (0.0036)</t>
         </is>
       </c>
     </row>
@@ -16864,31 +16866,31 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E458" t="n">
-        <v>0.3007518796992481</v>
+        <v>0.3294573643410852</v>
       </c>
       <c r="F458" t="n">
-        <v>0.1627906976744186</v>
+        <v>0.3059360730593607</v>
       </c>
       <c r="G458" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="H458" t="inlineStr">
         <is>
-          <t>0.2151 (0.0748)</t>
+          <t>0.2859 (0.0564)</t>
         </is>
       </c>
     </row>
@@ -16905,7 +16907,7 @@
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
@@ -16914,17 +16916,17 @@
         </is>
       </c>
       <c r="E459" t="n">
-        <v>0.3321033210332103</v>
+        <v>0.3007518796992481</v>
       </c>
       <c r="F459" t="n">
-        <v>0.2543859649122807</v>
+        <v>0.1627906976744186</v>
       </c>
       <c r="G459" t="n">
-        <v>0.2901554404145077</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>0.2922 (0.0389)</t>
+          <t>0.2151 (0.0748)</t>
         </is>
       </c>
     </row>
@@ -16941,7 +16943,7 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
@@ -16950,17 +16952,17 @@
         </is>
       </c>
       <c r="E460" t="n">
-        <v>0.1209302325581395</v>
+        <v>0.3321033210332103</v>
       </c>
       <c r="F460" t="n">
-        <v>0.1182795698924731</v>
+        <v>0.2543859649122807</v>
       </c>
       <c r="G460" t="n">
-        <v>0.1548387096774194</v>
+        <v>0.2901554404145077</v>
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>0.1313 (0.0204)</t>
+          <t>0.2922 (0.0389)</t>
         </is>
       </c>
     </row>
@@ -16977,7 +16979,7 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
@@ -16986,17 +16988,17 @@
         </is>
       </c>
       <c r="E461" t="n">
-        <v>0.391304347826087</v>
+        <v>0.1209302325581395</v>
       </c>
       <c r="F461" t="n">
-        <v>0.3221476510067114</v>
+        <v>0.1182795698924731</v>
       </c>
       <c r="G461" t="n">
-        <v>0.3011583011583012</v>
+        <v>0.1548387096774194</v>
       </c>
       <c r="H461" t="inlineStr">
         <is>
-          <t>0.3382 (0.0472)</t>
+          <t>0.1313 (0.0204)</t>
         </is>
       </c>
     </row>
@@ -17013,7 +17015,7 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
@@ -17022,17 +17024,17 @@
         </is>
       </c>
       <c r="E462" t="n">
-        <v>0.2068965517241379</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="F462" t="n">
-        <v>0.1837837837837838</v>
+        <v>0.3221476510067114</v>
       </c>
       <c r="G462" t="n">
-        <v>0.2054794520547945</v>
+        <v>0.3011583011583012</v>
       </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t>0.1987 (0.0130)</t>
+          <t>0.3382 (0.0472)</t>
         </is>
       </c>
     </row>
@@ -17044,27 +17046,31 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E463" t="n">
-        <v>0.303030303030303</v>
-      </c>
-      <c r="F463" t="inlineStr"/>
-      <c r="G463" t="inlineStr"/>
+        <v>0.2068965517241379</v>
+      </c>
+      <c r="F463" t="n">
+        <v>0.1837837837837838</v>
+      </c>
+      <c r="G463" t="n">
+        <v>0.2054794520547945</v>
+      </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t>0.3030 (0.0000)</t>
+          <t>0.1987 (0.0130)</t>
         </is>
       </c>
     </row>
@@ -17081,7 +17087,7 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
@@ -17090,17 +17096,15 @@
         </is>
       </c>
       <c r="E464" t="n">
-        <v>0.3125</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="F464" t="n">
-        <v>0.2698412698412698</v>
-      </c>
-      <c r="G464" t="n">
-        <v>0.2639593908629442</v>
-      </c>
+        <v>0.2022471910112359</v>
+      </c>
+      <c r="G464" t="inlineStr"/>
       <c r="H464" t="inlineStr">
         <is>
-          <t>0.2821 (0.0265)</t>
+          <t>0.2526 (0.0713)</t>
         </is>
       </c>
     </row>
@@ -17117,7 +17121,7 @@
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
@@ -17126,17 +17130,17 @@
         </is>
       </c>
       <c r="E465" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3125</v>
       </c>
       <c r="F465" t="n">
-        <v>0.1256544502617801</v>
+        <v>0.2698412698412698</v>
       </c>
       <c r="G465" t="n">
-        <v>0.2</v>
+        <v>0.2639593908629442</v>
       </c>
       <c r="H465" t="inlineStr">
         <is>
-          <t>0.1692 (0.0388)</t>
+          <t>0.2821 (0.0265)</t>
         </is>
       </c>
     </row>
@@ -17153,7 +17157,7 @@
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
@@ -17162,13 +17166,17 @@
         </is>
       </c>
       <c r="E466" t="n">
-        <v>0.3709090909090909</v>
-      </c>
-      <c r="F466" t="inlineStr"/>
-      <c r="G466" t="inlineStr"/>
+        <v>0.1818181818181818</v>
+      </c>
+      <c r="F466" t="n">
+        <v>0.1256544502617801</v>
+      </c>
+      <c r="G466" t="n">
+        <v>0.2</v>
+      </c>
       <c r="H466" t="inlineStr">
         <is>
-          <t>0.3709 (0.0000)</t>
+          <t>0.1692 (0.0388)</t>
         </is>
       </c>
     </row>
@@ -17185,7 +17193,7 @@
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
@@ -17194,13 +17202,49 @@
         </is>
       </c>
       <c r="E467" t="n">
-        <v>0.3135593220338983</v>
-      </c>
-      <c r="F467" t="inlineStr"/>
+        <v>0.3709090909090909</v>
+      </c>
+      <c r="F467" t="n">
+        <v>0.2521739130434782</v>
+      </c>
       <c r="G467" t="inlineStr"/>
       <c r="H467" t="inlineStr">
         <is>
-          <t>0.3136 (0.0000)</t>
+          <t>0.3115 (0.0840)</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E468" t="n">
+        <v>0.3135593220338983</v>
+      </c>
+      <c r="F468" t="n">
+        <v>0.2155688622754491</v>
+      </c>
+      <c r="G468" t="inlineStr"/>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>0.2646 (0.0693)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 20:36:19)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H468"/>
+  <dimension ref="A1:H471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17101,10 +17101,12 @@
       <c r="F464" t="n">
         <v>0.2022471910112359</v>
       </c>
-      <c r="G464" t="inlineStr"/>
+      <c r="G464" t="n">
+        <v>0.2666666666666667</v>
+      </c>
       <c r="H464" t="inlineStr">
         <is>
-          <t>0.2526 (0.0713)</t>
+          <t>0.2573 (0.0510)</t>
         </is>
       </c>
     </row>
@@ -17207,10 +17209,12 @@
       <c r="F467" t="n">
         <v>0.2521739130434782</v>
       </c>
-      <c r="G467" t="inlineStr"/>
+      <c r="G467" t="n">
+        <v>0.29</v>
+      </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>0.3115 (0.0840)</t>
+          <t>0.3044 (0.0607)</t>
         </is>
       </c>
     </row>
@@ -17241,10 +17245,116 @@
       <c r="F468" t="n">
         <v>0.2155688622754491</v>
       </c>
-      <c r="G468" t="inlineStr"/>
+      <c r="G468" t="n">
+        <v>0.1780821917808219</v>
+      </c>
       <c r="H468" t="inlineStr">
         <is>
-          <t>0.2646 (0.0693)</t>
+          <t>0.2357 (0.0700)</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E469" t="n">
+        <v>0.2322097378277154</v>
+      </c>
+      <c r="F469" t="n">
+        <v>0.2212389380530974</v>
+      </c>
+      <c r="G469" t="n">
+        <v>0.2288135593220339</v>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>0.2274 (0.0056)</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E470" t="n">
+        <v>0.2135922330097087</v>
+      </c>
+      <c r="F470" t="n">
+        <v>0.2307692307692308</v>
+      </c>
+      <c r="G470" t="n">
+        <v>0.1616161616161616</v>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>0.2020 (0.0360)</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E471" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F471" t="inlineStr"/>
+      <c r="G471" t="inlineStr"/>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>0.2667 (0.0000)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 21:36:37)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H471"/>
+  <dimension ref="A1:H477"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16851,10 +16851,12 @@
       <c r="F457" t="n">
         <v>0.296875</v>
       </c>
-      <c r="G457" t="inlineStr"/>
+      <c r="G457" t="n">
+        <v>0.2547169811320755</v>
+      </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t>0.2994 (0.0036)</t>
+          <t>0.2845 (0.0260)</t>
         </is>
       </c>
     </row>
@@ -16866,31 +16868,27 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E458" t="n">
-        <v>0.3294573643410852</v>
-      </c>
-      <c r="F458" t="n">
-        <v>0.3059360730593607</v>
-      </c>
-      <c r="G458" t="n">
-        <v>0.2222222222222222</v>
-      </c>
+        <v>0.1621621621621622</v>
+      </c>
+      <c r="F458" t="inlineStr"/>
+      <c r="G458" t="inlineStr"/>
       <c r="H458" t="inlineStr">
         <is>
-          <t>0.2859 (0.0564)</t>
+          <t>0.1622 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -16902,31 +16900,31 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E459" t="n">
-        <v>0.3007518796992481</v>
+        <v>0.3294573643410852</v>
       </c>
       <c r="F459" t="n">
-        <v>0.1627906976744186</v>
+        <v>0.3059360730593607</v>
       </c>
       <c r="G459" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>0.2151 (0.0748)</t>
+          <t>0.2859 (0.0564)</t>
         </is>
       </c>
     </row>
@@ -16938,31 +16936,27 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E460" t="n">
-        <v>0.3321033210332103</v>
-      </c>
-      <c r="F460" t="n">
-        <v>0.2543859649122807</v>
-      </c>
-      <c r="G460" t="n">
-        <v>0.2901554404145077</v>
-      </c>
+        <v>0.2285714285714286</v>
+      </c>
+      <c r="F460" t="inlineStr"/>
+      <c r="G460" t="inlineStr"/>
       <c r="H460" t="inlineStr">
         <is>
-          <t>0.2922 (0.0389)</t>
+          <t>0.2286 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -16979,7 +16973,7 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
@@ -16988,17 +16982,17 @@
         </is>
       </c>
       <c r="E461" t="n">
-        <v>0.1209302325581395</v>
+        <v>0.3007518796992481</v>
       </c>
       <c r="F461" t="n">
-        <v>0.1182795698924731</v>
+        <v>0.1627906976744186</v>
       </c>
       <c r="G461" t="n">
-        <v>0.1548387096774194</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H461" t="inlineStr">
         <is>
-          <t>0.1313 (0.0204)</t>
+          <t>0.2151 (0.0748)</t>
         </is>
       </c>
     </row>
@@ -17015,7 +17009,7 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
@@ -17024,17 +17018,17 @@
         </is>
       </c>
       <c r="E462" t="n">
-        <v>0.391304347826087</v>
+        <v>0.3321033210332103</v>
       </c>
       <c r="F462" t="n">
-        <v>0.3221476510067114</v>
+        <v>0.2543859649122807</v>
       </c>
       <c r="G462" t="n">
-        <v>0.3011583011583012</v>
+        <v>0.2901554404145077</v>
       </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t>0.3382 (0.0472)</t>
+          <t>0.2922 (0.0389)</t>
         </is>
       </c>
     </row>
@@ -17051,7 +17045,7 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
@@ -17060,17 +17054,17 @@
         </is>
       </c>
       <c r="E463" t="n">
-        <v>0.2068965517241379</v>
+        <v>0.1209302325581395</v>
       </c>
       <c r="F463" t="n">
-        <v>0.1837837837837838</v>
+        <v>0.1182795698924731</v>
       </c>
       <c r="G463" t="n">
-        <v>0.2054794520547945</v>
+        <v>0.1548387096774194</v>
       </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t>0.1987 (0.0130)</t>
+          <t>0.1313 (0.0204)</t>
         </is>
       </c>
     </row>
@@ -17082,31 +17076,31 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E464" t="n">
-        <v>0.303030303030303</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="F464" t="n">
-        <v>0.2022471910112359</v>
+        <v>0.3221476510067114</v>
       </c>
       <c r="G464" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.3011583011583012</v>
       </c>
       <c r="H464" t="inlineStr">
         <is>
-          <t>0.2573 (0.0510)</t>
+          <t>0.3382 (0.0472)</t>
         </is>
       </c>
     </row>
@@ -17118,31 +17112,31 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E465" t="n">
-        <v>0.3125</v>
+        <v>0.2068965517241379</v>
       </c>
       <c r="F465" t="n">
-        <v>0.2698412698412698</v>
+        <v>0.1837837837837838</v>
       </c>
       <c r="G465" t="n">
-        <v>0.2639593908629442</v>
+        <v>0.2054794520547945</v>
       </c>
       <c r="H465" t="inlineStr">
         <is>
-          <t>0.2821 (0.0265)</t>
+          <t>0.1987 (0.0130)</t>
         </is>
       </c>
     </row>
@@ -17159,7 +17153,7 @@
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
@@ -17168,17 +17162,17 @@
         </is>
       </c>
       <c r="E466" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="F466" t="n">
-        <v>0.1256544502617801</v>
+        <v>0.2022471910112359</v>
       </c>
       <c r="G466" t="n">
-        <v>0.2</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="H466" t="inlineStr">
         <is>
-          <t>0.1692 (0.0388)</t>
+          <t>0.2573 (0.0510)</t>
         </is>
       </c>
     </row>
@@ -17195,7 +17189,7 @@
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
@@ -17204,17 +17198,17 @@
         </is>
       </c>
       <c r="E467" t="n">
-        <v>0.3709090909090909</v>
+        <v>0.3125</v>
       </c>
       <c r="F467" t="n">
-        <v>0.2521739130434782</v>
+        <v>0.2698412698412698</v>
       </c>
       <c r="G467" t="n">
-        <v>0.29</v>
+        <v>0.2639593908629442</v>
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>0.3044 (0.0607)</t>
+          <t>0.2821 (0.0265)</t>
         </is>
       </c>
     </row>
@@ -17231,7 +17225,7 @@
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
@@ -17240,89 +17234,89 @@
         </is>
       </c>
       <c r="E468" t="n">
-        <v>0.3135593220338983</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F468" t="n">
-        <v>0.2155688622754491</v>
+        <v>0.1256544502617801</v>
       </c>
       <c r="G468" t="n">
-        <v>0.1780821917808219</v>
+        <v>0.2</v>
       </c>
       <c r="H468" t="inlineStr">
         <is>
-          <t>0.2357 (0.0700)</t>
+          <t>0.1692 (0.0388)</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E469" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.3709090909090909</v>
       </c>
       <c r="F469" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2521739130434782</v>
       </c>
       <c r="G469" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.29</v>
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.3044 (0.0607)</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E470" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.3135593220338983</v>
       </c>
       <c r="F470" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2155688622754491</v>
       </c>
       <c r="G470" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.1780821917808219</v>
       </c>
       <c r="H470" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2357 (0.0700)</t>
         </is>
       </c>
     </row>
@@ -17339,22 +17333,240 @@
       </c>
       <c r="C471" t="inlineStr">
         <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E471" t="n">
+        <v>0.2595419847328244</v>
+      </c>
+      <c r="F471" t="n">
+        <v>0.2164948453608248</v>
+      </c>
+      <c r="G471" t="n">
+        <v>0.228310502283105</v>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>0.2348 (0.0222)</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E472" t="n">
+        <v>0.2322097378277154</v>
+      </c>
+      <c r="F472" t="n">
+        <v>0.2212389380530974</v>
+      </c>
+      <c r="G472" t="n">
+        <v>0.2288135593220339</v>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>0.2274 (0.0056)</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E473" t="n">
+        <v>0.2135922330097087</v>
+      </c>
+      <c r="F473" t="n">
+        <v>0.2307692307692308</v>
+      </c>
+      <c r="G473" t="n">
+        <v>0.1616161616161616</v>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>0.2020 (0.0360)</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>DecisionTree</t>
+        </is>
+      </c>
+      <c r="E474" t="n">
+        <v>0.2683982683982684</v>
+      </c>
+      <c r="F474" t="n">
+        <v>0.2333333333333333</v>
+      </c>
+      <c r="G474" t="n">
+        <v>0.2046511627906977</v>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>0.2355 (0.0319)</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>dt</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D471" t="inlineStr">
+      <c r="D475" t="inlineStr">
         <is>
           <t>DecisionTree</t>
         </is>
       </c>
-      <c r="E471" t="n">
+      <c r="E475" t="n">
         <v>0.2666666666666667</v>
       </c>
-      <c r="F471" t="inlineStr"/>
-      <c r="G471" t="inlineStr"/>
-      <c r="H471" t="inlineStr">
-        <is>
-          <t>0.2667 (0.0000)</t>
+      <c r="F475" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G475" t="n">
+        <v>0.1940928270042194</v>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>0.2330 (0.0366)</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E476" t="n">
+        <v>0.2358974358974359</v>
+      </c>
+      <c r="F476" t="n">
+        <v>0.2840909090909091</v>
+      </c>
+      <c r="G476" t="n">
+        <v>0.2153846153846154</v>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>0.2451 (0.0353)</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E477" t="n">
+        <v>0.1714285714285714</v>
+      </c>
+      <c r="F477" t="n">
+        <v>0.1746031746031746</v>
+      </c>
+      <c r="G477" t="inlineStr"/>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>0.1730 (0.0022)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 22:36:55)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H477"/>
+  <dimension ref="A1:H481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17513,7 +17513,7 @@
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D476" t="inlineStr">
@@ -17522,17 +17522,17 @@
         </is>
       </c>
       <c r="E476" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F476" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G476" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -17549,24 +17549,170 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E477" t="n">
+        <v>0.2358974358974359</v>
+      </c>
+      <c r="F477" t="n">
+        <v>0.2840909090909091</v>
+      </c>
+      <c r="G477" t="n">
+        <v>0.2153846153846154</v>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>0.2451 (0.0353)</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
           <t>Morgan</t>
         </is>
       </c>
-      <c r="D477" t="inlineStr">
+      <c r="D478" t="inlineStr">
         <is>
           <t>RandomForest</t>
         </is>
       </c>
-      <c r="E477" t="n">
+      <c r="E478" t="n">
         <v>0.1714285714285714</v>
       </c>
-      <c r="F477" t="n">
+      <c r="F478" t="n">
         <v>0.1746031746031746</v>
       </c>
-      <c r="G477" t="inlineStr"/>
-      <c r="H477" t="inlineStr">
-        <is>
-          <t>0.1730 (0.0022)</t>
+      <c r="G478" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>0.1570 (0.0278)</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E479" t="n">
+        <v>0.3370786516853932</v>
+      </c>
+      <c r="F479" t="n">
+        <v>0.3091787439613526</v>
+      </c>
+      <c r="G479" t="n">
+        <v>0.1438848920863309</v>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>0.2634 (0.1044)</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E480" t="n">
+        <v>0.1940298507462687</v>
+      </c>
+      <c r="F480" t="n">
+        <v>0.1481481481481481</v>
+      </c>
+      <c r="G480" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>0.1585 (0.0316)</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E481" t="n">
+        <v>0.2087912087912088</v>
+      </c>
+      <c r="F481" t="n">
+        <v>0.2738095238095238</v>
+      </c>
+      <c r="G481" t="n">
+        <v>0.2705882352941176</v>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-04 23:37:14)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H481"/>
+  <dimension ref="A1:H483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16952,11 +16952,13 @@
       <c r="E460" t="n">
         <v>0.2285714285714286</v>
       </c>
-      <c r="F460" t="inlineStr"/>
+      <c r="F460" t="n">
+        <v>0.2239382239382239</v>
+      </c>
       <c r="G460" t="inlineStr"/>
       <c r="H460" t="inlineStr">
         <is>
-          <t>0.2286 (0.0000)</t>
+          <t>0.2263 (0.0033)</t>
         </is>
       </c>
     </row>
@@ -17713,6 +17715,72 @@
       <c r="H481" t="inlineStr">
         <is>
           <t>0.2511 (0.0366)</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E482" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F482" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G482" t="inlineStr"/>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>0.1918 (0.0537)</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E483" t="n">
+        <v>0.2469135802469136</v>
+      </c>
+      <c r="F483" t="inlineStr"/>
+      <c r="G483" t="inlineStr"/>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>0.2469 (0.0000)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 00:37:32)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -17745,10 +17745,12 @@
       <c r="F482" t="n">
         <v>0.2297297297297297</v>
       </c>
-      <c r="G482" t="inlineStr"/>
+      <c r="G482" t="n">
+        <v>0.1654135338345865</v>
+      </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.1918 (0.0537)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -17776,11 +17778,13 @@
       <c r="E483" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F483" t="inlineStr"/>
+      <c r="F483" t="n">
+        <v>0.1651376146788991</v>
+      </c>
       <c r="G483" t="inlineStr"/>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.2469 (0.0000)</t>
+          <t>0.2060 (0.0578)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 01:37:50)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H483"/>
+  <dimension ref="A1:H484"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16955,10 +16955,12 @@
       <c r="F460" t="n">
         <v>0.2239382239382239</v>
       </c>
-      <c r="G460" t="inlineStr"/>
+      <c r="G460" t="n">
+        <v>0.1831501831501831</v>
+      </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>0.2263 (0.0033)</t>
+          <t>0.2119 (0.0250)</t>
         </is>
       </c>
     </row>
@@ -17767,7 +17769,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
@@ -17776,15 +17778,49 @@
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.2469135802469136</v>
-      </c>
-      <c r="F483" t="n">
-        <v>0.1651376146788991</v>
-      </c>
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F483" t="inlineStr"/>
       <c r="G483" t="inlineStr"/>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.2060 (0.0578)</t>
+          <t>0.2260 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E484" t="n">
+        <v>0.2469135802469136</v>
+      </c>
+      <c r="F484" t="n">
+        <v>0.1651376146788991</v>
+      </c>
+      <c r="G484" t="n">
+        <v>0.1238938053097345</v>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>0.1786 (0.0626)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 02:38:08)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H484"/>
+  <dimension ref="A1:H488"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16884,11 +16884,13 @@
       <c r="E458" t="n">
         <v>0.1621621621621622</v>
       </c>
-      <c r="F458" t="inlineStr"/>
+      <c r="F458" t="n">
+        <v>0.2200956937799043</v>
+      </c>
       <c r="G458" t="inlineStr"/>
       <c r="H458" t="inlineStr">
         <is>
-          <t>0.1622 (0.0000)</t>
+          <t>0.1911 (0.0410)</t>
         </is>
       </c>
     </row>
@@ -16972,31 +16974,27 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E461" t="n">
-        <v>0.3007518796992481</v>
-      </c>
-      <c r="F461" t="n">
-        <v>0.1627906976744186</v>
-      </c>
-      <c r="G461" t="n">
-        <v>0.1818181818181818</v>
-      </c>
+        <v>0.3294797687861272</v>
+      </c>
+      <c r="F461" t="inlineStr"/>
+      <c r="G461" t="inlineStr"/>
       <c r="H461" t="inlineStr">
         <is>
-          <t>0.2151 (0.0748)</t>
+          <t>0.3295 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17008,31 +17006,27 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E462" t="n">
-        <v>0.3321033210332103</v>
-      </c>
-      <c r="F462" t="n">
-        <v>0.2543859649122807</v>
-      </c>
-      <c r="G462" t="n">
-        <v>0.2901554404145077</v>
-      </c>
+        <v>0.3111111111111111</v>
+      </c>
+      <c r="F462" t="inlineStr"/>
+      <c r="G462" t="inlineStr"/>
       <c r="H462" t="inlineStr">
         <is>
-          <t>0.2922 (0.0389)</t>
+          <t>0.3111 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17049,7 +17043,7 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
@@ -17058,17 +17052,17 @@
         </is>
       </c>
       <c r="E463" t="n">
-        <v>0.1209302325581395</v>
+        <v>0.3007518796992481</v>
       </c>
       <c r="F463" t="n">
-        <v>0.1182795698924731</v>
+        <v>0.1627906976744186</v>
       </c>
       <c r="G463" t="n">
-        <v>0.1548387096774194</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t>0.1313 (0.0204)</t>
+          <t>0.2151 (0.0748)</t>
         </is>
       </c>
     </row>
@@ -17085,7 +17079,7 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
@@ -17094,17 +17088,17 @@
         </is>
       </c>
       <c r="E464" t="n">
-        <v>0.391304347826087</v>
+        <v>0.3321033210332103</v>
       </c>
       <c r="F464" t="n">
-        <v>0.3221476510067114</v>
+        <v>0.2543859649122807</v>
       </c>
       <c r="G464" t="n">
-        <v>0.3011583011583012</v>
+        <v>0.2901554404145077</v>
       </c>
       <c r="H464" t="inlineStr">
         <is>
-          <t>0.3382 (0.0472)</t>
+          <t>0.2922 (0.0389)</t>
         </is>
       </c>
     </row>
@@ -17121,7 +17115,7 @@
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
@@ -17130,17 +17124,17 @@
         </is>
       </c>
       <c r="E465" t="n">
-        <v>0.2068965517241379</v>
+        <v>0.1209302325581395</v>
       </c>
       <c r="F465" t="n">
-        <v>0.1837837837837838</v>
+        <v>0.1182795698924731</v>
       </c>
       <c r="G465" t="n">
-        <v>0.2054794520547945</v>
+        <v>0.1548387096774194</v>
       </c>
       <c r="H465" t="inlineStr">
         <is>
-          <t>0.1987 (0.0130)</t>
+          <t>0.1313 (0.0204)</t>
         </is>
       </c>
     </row>
@@ -17152,31 +17146,31 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E466" t="n">
-        <v>0.303030303030303</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="F466" t="n">
-        <v>0.2022471910112359</v>
+        <v>0.3221476510067114</v>
       </c>
       <c r="G466" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.3011583011583012</v>
       </c>
       <c r="H466" t="inlineStr">
         <is>
-          <t>0.2573 (0.0510)</t>
+          <t>0.3382 (0.0472)</t>
         </is>
       </c>
     </row>
@@ -17188,31 +17182,31 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E467" t="n">
-        <v>0.3125</v>
+        <v>0.2068965517241379</v>
       </c>
       <c r="F467" t="n">
-        <v>0.2698412698412698</v>
+        <v>0.1837837837837838</v>
       </c>
       <c r="G467" t="n">
-        <v>0.2639593908629442</v>
+        <v>0.2054794520547945</v>
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>0.2821 (0.0265)</t>
+          <t>0.1987 (0.0130)</t>
         </is>
       </c>
     </row>
@@ -17229,7 +17223,7 @@
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
@@ -17238,17 +17232,17 @@
         </is>
       </c>
       <c r="E468" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="F468" t="n">
-        <v>0.1256544502617801</v>
+        <v>0.2022471910112359</v>
       </c>
       <c r="G468" t="n">
-        <v>0.2</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="H468" t="inlineStr">
         <is>
-          <t>0.1692 (0.0388)</t>
+          <t>0.2573 (0.0510)</t>
         </is>
       </c>
     </row>
@@ -17265,7 +17259,7 @@
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
@@ -17274,17 +17268,17 @@
         </is>
       </c>
       <c r="E469" t="n">
-        <v>0.3709090909090909</v>
+        <v>0.3125</v>
       </c>
       <c r="F469" t="n">
-        <v>0.2521739130434782</v>
+        <v>0.2698412698412698</v>
       </c>
       <c r="G469" t="n">
-        <v>0.29</v>
+        <v>0.2639593908629442</v>
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>0.3044 (0.0607)</t>
+          <t>0.2821 (0.0265)</t>
         </is>
       </c>
     </row>
@@ -17301,7 +17295,7 @@
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
@@ -17310,89 +17304,89 @@
         </is>
       </c>
       <c r="E470" t="n">
-        <v>0.3135593220338983</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F470" t="n">
-        <v>0.2155688622754491</v>
+        <v>0.1256544502617801</v>
       </c>
       <c r="G470" t="n">
-        <v>0.1780821917808219</v>
+        <v>0.2</v>
       </c>
       <c r="H470" t="inlineStr">
         <is>
-          <t>0.2357 (0.0700)</t>
+          <t>0.1692 (0.0388)</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D471" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E471" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.3709090909090909</v>
       </c>
       <c r="F471" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2521739130434782</v>
       </c>
       <c r="G471" t="n">
-        <v>0.228310502283105</v>
+        <v>0.29</v>
       </c>
       <c r="H471" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.3044 (0.0607)</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D472" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E472" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.3135593220338983</v>
       </c>
       <c r="F472" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2155688622754491</v>
       </c>
       <c r="G472" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.1780821917808219</v>
       </c>
       <c r="H472" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2357 (0.0700)</t>
         </is>
       </c>
     </row>
@@ -17409,7 +17403,7 @@
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D473" t="inlineStr">
@@ -17418,17 +17412,17 @@
         </is>
       </c>
       <c r="E473" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F473" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G473" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -17445,7 +17439,7 @@
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D474" t="inlineStr">
@@ -17454,17 +17448,17 @@
         </is>
       </c>
       <c r="E474" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F474" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G474" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -17481,7 +17475,7 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
@@ -17490,17 +17484,17 @@
         </is>
       </c>
       <c r="E475" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F475" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G475" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H475" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -17512,31 +17506,31 @@
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D476" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E476" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F476" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G476" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -17548,31 +17542,31 @@
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E477" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F477" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2383419689119171</v>
       </c>
       <c r="G477" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1940928270042194</v>
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -17584,31 +17578,27 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E478" t="n">
-        <v>0.1714285714285714</v>
-      </c>
-      <c r="F478" t="n">
-        <v>0.1746031746031746</v>
-      </c>
-      <c r="G478" t="n">
-        <v>0.125</v>
-      </c>
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="F478" t="inlineStr"/>
+      <c r="G478" t="inlineStr"/>
       <c r="H478" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2632 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17625,7 +17615,7 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
@@ -17634,17 +17624,17 @@
         </is>
       </c>
       <c r="E479" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F479" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G479" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H479" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -17661,7 +17651,7 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
@@ -17670,17 +17660,17 @@
         </is>
       </c>
       <c r="E480" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F480" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G480" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -17692,31 +17682,31 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E481" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F481" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G481" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.125</v>
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -17728,31 +17718,31 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F482" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G482" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -17764,27 +17754,31 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.2259887005649718</v>
-      </c>
-      <c r="F483" t="inlineStr"/>
-      <c r="G483" t="inlineStr"/>
+        <v>0.1940298507462687</v>
+      </c>
+      <c r="F483" t="n">
+        <v>0.1481481481481481</v>
+      </c>
+      <c r="G483" t="n">
+        <v>0.1333333333333333</v>
+      </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.2260 (0.0000)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -17801,24 +17795,164 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E484" t="n">
+        <v>0.232258064516129</v>
+      </c>
+      <c r="F484" t="inlineStr"/>
+      <c r="G484" t="inlineStr"/>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>0.2323 (0.0000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E485" t="n">
+        <v>0.2087912087912088</v>
+      </c>
+      <c r="F485" t="n">
+        <v>0.2738095238095238</v>
+      </c>
+      <c r="G485" t="n">
+        <v>0.2705882352941176</v>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>0.2511 (0.0366)</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E486" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F486" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G486" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E487" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F487" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G487" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D484" t="inlineStr">
+      <c r="D488" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E484" t="n">
+      <c r="E488" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F484" t="n">
+      <c r="F488" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G484" t="n">
+      <c r="G488" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H484" t="inlineStr">
+      <c r="H488" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 03:38:26)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H488"/>
+  <dimension ref="A1:H489"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16907,7 +16907,7 @@
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
@@ -16916,17 +16916,13 @@
         </is>
       </c>
       <c r="E459" t="n">
-        <v>0.3294573643410852</v>
-      </c>
-      <c r="F459" t="n">
-        <v>0.3059360730593607</v>
-      </c>
-      <c r="G459" t="n">
-        <v>0.2222222222222222</v>
-      </c>
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F459" t="inlineStr"/>
+      <c r="G459" t="inlineStr"/>
       <c r="H459" t="inlineStr">
         <is>
-          <t>0.2859 (0.0564)</t>
+          <t>0.3333 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -16943,7 +16939,7 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
@@ -16952,17 +16948,17 @@
         </is>
       </c>
       <c r="E460" t="n">
-        <v>0.2285714285714286</v>
+        <v>0.3294573643410852</v>
       </c>
       <c r="F460" t="n">
-        <v>0.2239382239382239</v>
+        <v>0.3059360730593607</v>
       </c>
       <c r="G460" t="n">
-        <v>0.1831501831501831</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>0.2119 (0.0250)</t>
+          <t>0.2859 (0.0564)</t>
         </is>
       </c>
     </row>
@@ -16979,7 +16975,7 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
@@ -16988,13 +16984,17 @@
         </is>
       </c>
       <c r="E461" t="n">
-        <v>0.3294797687861272</v>
-      </c>
-      <c r="F461" t="inlineStr"/>
-      <c r="G461" t="inlineStr"/>
+        <v>0.2285714285714286</v>
+      </c>
+      <c r="F461" t="n">
+        <v>0.2239382239382239</v>
+      </c>
+      <c r="G461" t="n">
+        <v>0.1831501831501831</v>
+      </c>
       <c r="H461" t="inlineStr">
         <is>
-          <t>0.3295 (0.0000)</t>
+          <t>0.2119 (0.0250)</t>
         </is>
       </c>
     </row>
@@ -17011,7 +17011,7 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
@@ -17020,13 +17020,13 @@
         </is>
       </c>
       <c r="E462" t="n">
-        <v>0.3111111111111111</v>
+        <v>0.3294797687861272</v>
       </c>
       <c r="F462" t="inlineStr"/>
       <c r="G462" t="inlineStr"/>
       <c r="H462" t="inlineStr">
         <is>
-          <t>0.3111 (0.0000)</t>
+          <t>0.3295 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17038,31 +17038,27 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E463" t="n">
-        <v>0.3007518796992481</v>
-      </c>
-      <c r="F463" t="n">
-        <v>0.1627906976744186</v>
-      </c>
-      <c r="G463" t="n">
-        <v>0.1818181818181818</v>
-      </c>
+        <v>0.3111111111111111</v>
+      </c>
+      <c r="F463" t="inlineStr"/>
+      <c r="G463" t="inlineStr"/>
       <c r="H463" t="inlineStr">
         <is>
-          <t>0.2151 (0.0748)</t>
+          <t>0.3111 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17079,7 +17075,7 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
@@ -17088,17 +17084,17 @@
         </is>
       </c>
       <c r="E464" t="n">
-        <v>0.3321033210332103</v>
+        <v>0.3007518796992481</v>
       </c>
       <c r="F464" t="n">
-        <v>0.2543859649122807</v>
+        <v>0.1627906976744186</v>
       </c>
       <c r="G464" t="n">
-        <v>0.2901554404145077</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H464" t="inlineStr">
         <is>
-          <t>0.2922 (0.0389)</t>
+          <t>0.2151 (0.0748)</t>
         </is>
       </c>
     </row>
@@ -17115,7 +17111,7 @@
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
@@ -17124,17 +17120,17 @@
         </is>
       </c>
       <c r="E465" t="n">
-        <v>0.1209302325581395</v>
+        <v>0.3321033210332103</v>
       </c>
       <c r="F465" t="n">
-        <v>0.1182795698924731</v>
+        <v>0.2543859649122807</v>
       </c>
       <c r="G465" t="n">
-        <v>0.1548387096774194</v>
+        <v>0.2901554404145077</v>
       </c>
       <c r="H465" t="inlineStr">
         <is>
-          <t>0.1313 (0.0204)</t>
+          <t>0.2922 (0.0389)</t>
         </is>
       </c>
     </row>
@@ -17151,7 +17147,7 @@
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
@@ -17160,17 +17156,17 @@
         </is>
       </c>
       <c r="E466" t="n">
-        <v>0.391304347826087</v>
+        <v>0.1209302325581395</v>
       </c>
       <c r="F466" t="n">
-        <v>0.3221476510067114</v>
+        <v>0.1182795698924731</v>
       </c>
       <c r="G466" t="n">
-        <v>0.3011583011583012</v>
+        <v>0.1548387096774194</v>
       </c>
       <c r="H466" t="inlineStr">
         <is>
-          <t>0.3382 (0.0472)</t>
+          <t>0.1313 (0.0204)</t>
         </is>
       </c>
     </row>
@@ -17187,7 +17183,7 @@
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
@@ -17196,17 +17192,17 @@
         </is>
       </c>
       <c r="E467" t="n">
-        <v>0.2068965517241379</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="F467" t="n">
-        <v>0.1837837837837838</v>
+        <v>0.3221476510067114</v>
       </c>
       <c r="G467" t="n">
-        <v>0.2054794520547945</v>
+        <v>0.3011583011583012</v>
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>0.1987 (0.0130)</t>
+          <t>0.3382 (0.0472)</t>
         </is>
       </c>
     </row>
@@ -17218,31 +17214,31 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E468" t="n">
-        <v>0.303030303030303</v>
+        <v>0.2068965517241379</v>
       </c>
       <c r="F468" t="n">
-        <v>0.2022471910112359</v>
+        <v>0.1837837837837838</v>
       </c>
       <c r="G468" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2054794520547945</v>
       </c>
       <c r="H468" t="inlineStr">
         <is>
-          <t>0.2573 (0.0510)</t>
+          <t>0.1987 (0.0130)</t>
         </is>
       </c>
     </row>
@@ -17259,7 +17255,7 @@
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
@@ -17268,17 +17264,17 @@
         </is>
       </c>
       <c r="E469" t="n">
-        <v>0.3125</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="F469" t="n">
-        <v>0.2698412698412698</v>
+        <v>0.2022471910112359</v>
       </c>
       <c r="G469" t="n">
-        <v>0.2639593908629442</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>0.2821 (0.0265)</t>
+          <t>0.2573 (0.0510)</t>
         </is>
       </c>
     </row>
@@ -17295,7 +17291,7 @@
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
@@ -17304,17 +17300,17 @@
         </is>
       </c>
       <c r="E470" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3125</v>
       </c>
       <c r="F470" t="n">
-        <v>0.1256544502617801</v>
+        <v>0.2698412698412698</v>
       </c>
       <c r="G470" t="n">
-        <v>0.2</v>
+        <v>0.2639593908629442</v>
       </c>
       <c r="H470" t="inlineStr">
         <is>
-          <t>0.1692 (0.0388)</t>
+          <t>0.2821 (0.0265)</t>
         </is>
       </c>
     </row>
@@ -17331,7 +17327,7 @@
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D471" t="inlineStr">
@@ -17340,17 +17336,17 @@
         </is>
       </c>
       <c r="E471" t="n">
-        <v>0.3709090909090909</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F471" t="n">
-        <v>0.2521739130434782</v>
+        <v>0.1256544502617801</v>
       </c>
       <c r="G471" t="n">
-        <v>0.29</v>
+        <v>0.2</v>
       </c>
       <c r="H471" t="inlineStr">
         <is>
-          <t>0.3044 (0.0607)</t>
+          <t>0.1692 (0.0388)</t>
         </is>
       </c>
     </row>
@@ -17367,7 +17363,7 @@
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D472" t="inlineStr">
@@ -17376,53 +17372,53 @@
         </is>
       </c>
       <c r="E472" t="n">
-        <v>0.3135593220338983</v>
+        <v>0.3709090909090909</v>
       </c>
       <c r="F472" t="n">
-        <v>0.2155688622754491</v>
+        <v>0.2521739130434782</v>
       </c>
       <c r="G472" t="n">
-        <v>0.1780821917808219</v>
+        <v>0.29</v>
       </c>
       <c r="H472" t="inlineStr">
         <is>
-          <t>0.2357 (0.0700)</t>
+          <t>0.3044 (0.0607)</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D473" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E473" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.3135593220338983</v>
       </c>
       <c r="F473" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2155688622754491</v>
       </c>
       <c r="G473" t="n">
-        <v>0.228310502283105</v>
+        <v>0.1780821917808219</v>
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2357 (0.0700)</t>
         </is>
       </c>
     </row>
@@ -17439,7 +17435,7 @@
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D474" t="inlineStr">
@@ -17448,17 +17444,17 @@
         </is>
       </c>
       <c r="E474" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F474" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G474" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -17475,7 +17471,7 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
@@ -17484,17 +17480,17 @@
         </is>
       </c>
       <c r="E475" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F475" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G475" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H475" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -17511,7 +17507,7 @@
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D476" t="inlineStr">
@@ -17520,17 +17516,17 @@
         </is>
       </c>
       <c r="E476" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F476" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G476" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -17547,7 +17543,7 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
@@ -17556,17 +17552,17 @@
         </is>
       </c>
       <c r="E477" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F477" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G477" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -17578,27 +17574,31 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E478" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F478" t="inlineStr"/>
-      <c r="G478" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F478" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G478" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>0.2632 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -17610,31 +17610,27 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E479" t="n">
-        <v>0.196078431372549</v>
-      </c>
-      <c r="F479" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G479" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="F479" t="inlineStr"/>
+      <c r="G479" t="inlineStr"/>
       <c r="H479" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2632 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17651,7 +17647,7 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
@@ -17660,17 +17656,17 @@
         </is>
       </c>
       <c r="E480" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F480" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G480" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -17687,7 +17683,7 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
@@ -17696,17 +17692,17 @@
         </is>
       </c>
       <c r="E481" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F481" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G481" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -17723,7 +17719,7 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
@@ -17732,17 +17728,17 @@
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F482" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G482" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -17759,7 +17755,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
@@ -17768,17 +17764,17 @@
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F483" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G483" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -17790,27 +17786,31 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.232258064516129</v>
-      </c>
-      <c r="F484" t="inlineStr"/>
-      <c r="G484" t="inlineStr"/>
+        <v>0.1940298507462687</v>
+      </c>
+      <c r="F484" t="n">
+        <v>0.1481481481481481</v>
+      </c>
+      <c r="G484" t="n">
+        <v>0.1333333333333333</v>
+      </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.2323 (0.0000)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -17827,7 +17827,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17836,17 +17836,15 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F485" t="n">
-        <v>0.2738095238095238</v>
-      </c>
-      <c r="G485" t="n">
-        <v>0.2705882352941176</v>
-      </c>
+        <v>0.2385321100917431</v>
+      </c>
+      <c r="G485" t="inlineStr"/>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2354 (0.0044)</t>
         </is>
       </c>
     </row>
@@ -17863,7 +17861,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17872,17 +17870,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F486" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G486" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -17899,7 +17897,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17908,17 +17906,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F487" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G487" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -17935,24 +17933,60 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E488" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F488" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G488" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D488" t="inlineStr">
+      <c r="D489" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E488" t="n">
+      <c r="E489" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F488" t="n">
+      <c r="F489" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G488" t="n">
+      <c r="G489" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H488" t="inlineStr">
+      <c r="H489" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 04:38:44)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -17626,11 +17626,13 @@
       <c r="E479" t="n">
         <v>0.2631578947368421</v>
       </c>
-      <c r="F479" t="inlineStr"/>
+      <c r="F479" t="n">
+        <v>0.2592592592592592</v>
+      </c>
       <c r="G479" t="inlineStr"/>
       <c r="H479" t="inlineStr">
         <is>
-          <t>0.2632 (0.0000)</t>
+          <t>0.2612 (0.0028)</t>
         </is>
       </c>
     </row>
@@ -17841,10 +17843,12 @@
       <c r="F485" t="n">
         <v>0.2385321100917431</v>
       </c>
-      <c r="G485" t="inlineStr"/>
+      <c r="G485" t="n">
+        <v>0.2131147540983606</v>
+      </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.2354 (0.0044)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 05:39:02)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H489"/>
+  <dimension ref="A1:H490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16902,27 +16902,27 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E459" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.3445945945945946</v>
       </c>
       <c r="F459" t="inlineStr"/>
       <c r="G459" t="inlineStr"/>
       <c r="H459" t="inlineStr">
         <is>
-          <t>0.3333 (0.0000)</t>
+          <t>0.3446 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -16939,7 +16939,7 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
@@ -16948,17 +16948,13 @@
         </is>
       </c>
       <c r="E460" t="n">
-        <v>0.3294573643410852</v>
-      </c>
-      <c r="F460" t="n">
-        <v>0.3059360730593607</v>
-      </c>
-      <c r="G460" t="n">
-        <v>0.2222222222222222</v>
-      </c>
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F460" t="inlineStr"/>
+      <c r="G460" t="inlineStr"/>
       <c r="H460" t="inlineStr">
         <is>
-          <t>0.2859 (0.0564)</t>
+          <t>0.3333 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -16975,7 +16971,7 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
@@ -16984,17 +16980,17 @@
         </is>
       </c>
       <c r="E461" t="n">
-        <v>0.2285714285714286</v>
+        <v>0.3294573643410852</v>
       </c>
       <c r="F461" t="n">
-        <v>0.2239382239382239</v>
+        <v>0.3059360730593607</v>
       </c>
       <c r="G461" t="n">
-        <v>0.1831501831501831</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="H461" t="inlineStr">
         <is>
-          <t>0.2119 (0.0250)</t>
+          <t>0.2859 (0.0564)</t>
         </is>
       </c>
     </row>
@@ -17011,7 +17007,7 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
@@ -17020,13 +17016,17 @@
         </is>
       </c>
       <c r="E462" t="n">
-        <v>0.3294797687861272</v>
-      </c>
-      <c r="F462" t="inlineStr"/>
-      <c r="G462" t="inlineStr"/>
+        <v>0.2285714285714286</v>
+      </c>
+      <c r="F462" t="n">
+        <v>0.2239382239382239</v>
+      </c>
+      <c r="G462" t="n">
+        <v>0.1831501831501831</v>
+      </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t>0.3295 (0.0000)</t>
+          <t>0.2119 (0.0250)</t>
         </is>
       </c>
     </row>
@@ -17043,7 +17043,7 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
@@ -17052,13 +17052,13 @@
         </is>
       </c>
       <c r="E463" t="n">
-        <v>0.3111111111111111</v>
+        <v>0.3294797687861272</v>
       </c>
       <c r="F463" t="inlineStr"/>
       <c r="G463" t="inlineStr"/>
       <c r="H463" t="inlineStr">
         <is>
-          <t>0.3111 (0.0000)</t>
+          <t>0.3295 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17070,31 +17070,27 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E464" t="n">
-        <v>0.3007518796992481</v>
-      </c>
-      <c r="F464" t="n">
-        <v>0.1627906976744186</v>
-      </c>
-      <c r="G464" t="n">
-        <v>0.1818181818181818</v>
-      </c>
+        <v>0.3111111111111111</v>
+      </c>
+      <c r="F464" t="inlineStr"/>
+      <c r="G464" t="inlineStr"/>
       <c r="H464" t="inlineStr">
         <is>
-          <t>0.2151 (0.0748)</t>
+          <t>0.3111 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17111,7 +17107,7 @@
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
@@ -17120,17 +17116,17 @@
         </is>
       </c>
       <c r="E465" t="n">
-        <v>0.3321033210332103</v>
+        <v>0.3007518796992481</v>
       </c>
       <c r="F465" t="n">
-        <v>0.2543859649122807</v>
+        <v>0.1627906976744186</v>
       </c>
       <c r="G465" t="n">
-        <v>0.2901554404145077</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H465" t="inlineStr">
         <is>
-          <t>0.2922 (0.0389)</t>
+          <t>0.2151 (0.0748)</t>
         </is>
       </c>
     </row>
@@ -17147,7 +17143,7 @@
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
@@ -17156,17 +17152,17 @@
         </is>
       </c>
       <c r="E466" t="n">
-        <v>0.1209302325581395</v>
+        <v>0.3321033210332103</v>
       </c>
       <c r="F466" t="n">
-        <v>0.1182795698924731</v>
+        <v>0.2543859649122807</v>
       </c>
       <c r="G466" t="n">
-        <v>0.1548387096774194</v>
+        <v>0.2901554404145077</v>
       </c>
       <c r="H466" t="inlineStr">
         <is>
-          <t>0.1313 (0.0204)</t>
+          <t>0.2922 (0.0389)</t>
         </is>
       </c>
     </row>
@@ -17183,7 +17179,7 @@
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
@@ -17192,17 +17188,17 @@
         </is>
       </c>
       <c r="E467" t="n">
-        <v>0.391304347826087</v>
+        <v>0.1209302325581395</v>
       </c>
       <c r="F467" t="n">
-        <v>0.3221476510067114</v>
+        <v>0.1182795698924731</v>
       </c>
       <c r="G467" t="n">
-        <v>0.3011583011583012</v>
+        <v>0.1548387096774194</v>
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>0.3382 (0.0472)</t>
+          <t>0.1313 (0.0204)</t>
         </is>
       </c>
     </row>
@@ -17219,7 +17215,7 @@
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
@@ -17228,17 +17224,17 @@
         </is>
       </c>
       <c r="E468" t="n">
-        <v>0.2068965517241379</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="F468" t="n">
-        <v>0.1837837837837838</v>
+        <v>0.3221476510067114</v>
       </c>
       <c r="G468" t="n">
-        <v>0.2054794520547945</v>
+        <v>0.3011583011583012</v>
       </c>
       <c r="H468" t="inlineStr">
         <is>
-          <t>0.1987 (0.0130)</t>
+          <t>0.3382 (0.0472)</t>
         </is>
       </c>
     </row>
@@ -17250,31 +17246,31 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E469" t="n">
-        <v>0.303030303030303</v>
+        <v>0.2068965517241379</v>
       </c>
       <c r="F469" t="n">
-        <v>0.2022471910112359</v>
+        <v>0.1837837837837838</v>
       </c>
       <c r="G469" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2054794520547945</v>
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>0.2573 (0.0510)</t>
+          <t>0.1987 (0.0130)</t>
         </is>
       </c>
     </row>
@@ -17291,7 +17287,7 @@
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
@@ -17300,17 +17296,17 @@
         </is>
       </c>
       <c r="E470" t="n">
-        <v>0.3125</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="F470" t="n">
-        <v>0.2698412698412698</v>
+        <v>0.2022471910112359</v>
       </c>
       <c r="G470" t="n">
-        <v>0.2639593908629442</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="H470" t="inlineStr">
         <is>
-          <t>0.2821 (0.0265)</t>
+          <t>0.2573 (0.0510)</t>
         </is>
       </c>
     </row>
@@ -17327,7 +17323,7 @@
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D471" t="inlineStr">
@@ -17336,17 +17332,17 @@
         </is>
       </c>
       <c r="E471" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3125</v>
       </c>
       <c r="F471" t="n">
-        <v>0.1256544502617801</v>
+        <v>0.2698412698412698</v>
       </c>
       <c r="G471" t="n">
-        <v>0.2</v>
+        <v>0.2639593908629442</v>
       </c>
       <c r="H471" t="inlineStr">
         <is>
-          <t>0.1692 (0.0388)</t>
+          <t>0.2821 (0.0265)</t>
         </is>
       </c>
     </row>
@@ -17363,7 +17359,7 @@
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D472" t="inlineStr">
@@ -17372,17 +17368,17 @@
         </is>
       </c>
       <c r="E472" t="n">
-        <v>0.3709090909090909</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F472" t="n">
-        <v>0.2521739130434782</v>
+        <v>0.1256544502617801</v>
       </c>
       <c r="G472" t="n">
-        <v>0.29</v>
+        <v>0.2</v>
       </c>
       <c r="H472" t="inlineStr">
         <is>
-          <t>0.3044 (0.0607)</t>
+          <t>0.1692 (0.0388)</t>
         </is>
       </c>
     </row>
@@ -17399,7 +17395,7 @@
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D473" t="inlineStr">
@@ -17408,53 +17404,53 @@
         </is>
       </c>
       <c r="E473" t="n">
-        <v>0.3135593220338983</v>
+        <v>0.3709090909090909</v>
       </c>
       <c r="F473" t="n">
-        <v>0.2155688622754491</v>
+        <v>0.2521739130434782</v>
       </c>
       <c r="G473" t="n">
-        <v>0.1780821917808219</v>
+        <v>0.29</v>
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>0.2357 (0.0700)</t>
+          <t>0.3044 (0.0607)</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D474" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E474" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.3135593220338983</v>
       </c>
       <c r="F474" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2155688622754491</v>
       </c>
       <c r="G474" t="n">
-        <v>0.228310502283105</v>
+        <v>0.1780821917808219</v>
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2357 (0.0700)</t>
         </is>
       </c>
     </row>
@@ -17471,7 +17467,7 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
@@ -17480,17 +17476,17 @@
         </is>
       </c>
       <c r="E475" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F475" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G475" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H475" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -17507,7 +17503,7 @@
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D476" t="inlineStr">
@@ -17516,17 +17512,17 @@
         </is>
       </c>
       <c r="E476" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F476" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G476" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -17543,7 +17539,7 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
@@ -17552,17 +17548,17 @@
         </is>
       </c>
       <c r="E477" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F477" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G477" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -17579,7 +17575,7 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
@@ -17588,17 +17584,17 @@
         </is>
       </c>
       <c r="E478" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F478" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G478" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -17610,29 +17606,31 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E479" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F479" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G479" t="inlineStr"/>
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G479" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H479" t="inlineStr">
         <is>
-          <t>0.2612 (0.0028)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -17644,31 +17642,31 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E480" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F480" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G480" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -17685,7 +17683,7 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
@@ -17694,17 +17692,17 @@
         </is>
       </c>
       <c r="E481" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F481" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G481" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -17721,7 +17719,7 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
@@ -17730,17 +17728,17 @@
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F482" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G482" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -17757,7 +17755,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
@@ -17766,17 +17764,17 @@
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F483" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G483" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -17793,7 +17791,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -17802,17 +17800,17 @@
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F484" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G484" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -17824,31 +17822,31 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F485" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G485" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -17865,7 +17863,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17874,17 +17872,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F486" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G486" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -17901,7 +17899,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17910,17 +17908,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F487" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G487" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -17937,7 +17935,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17946,17 +17944,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F488" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G488" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -17973,24 +17971,60 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E489" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F489" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G489" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D489" t="inlineStr">
+      <c r="D490" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E489" t="n">
+      <c r="E490" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F489" t="n">
+      <c r="F490" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G489" t="n">
+      <c r="G490" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H489" t="inlineStr">
+      <c r="H490" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 06:39:20)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -16887,10 +16887,12 @@
       <c r="F458" t="n">
         <v>0.2200956937799043</v>
       </c>
-      <c r="G458" t="inlineStr"/>
+      <c r="G458" t="n">
+        <v>0.223463687150838</v>
+      </c>
       <c r="H458" t="inlineStr">
         <is>
-          <t>0.1911 (0.0410)</t>
+          <t>0.2019 (0.0345)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 07:39:38)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H490"/>
+  <dimension ref="A1:H491"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17680,31 +17680,27 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E481" t="n">
-        <v>0.196078431372549</v>
-      </c>
-      <c r="F481" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G481" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.163265306122449</v>
+      </c>
+      <c r="F481" t="inlineStr"/>
+      <c r="G481" t="inlineStr"/>
       <c r="H481" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.1633 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17721,7 +17717,7 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
@@ -17730,17 +17726,17 @@
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F482" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G482" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -17757,7 +17753,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
@@ -17766,17 +17762,17 @@
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F483" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G483" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -17793,7 +17789,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -17802,17 +17798,17 @@
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F484" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G484" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -17829,7 +17825,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17838,17 +17834,17 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F485" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G485" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -17860,31 +17856,31 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F486" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G486" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -17901,7 +17897,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17910,17 +17906,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F487" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G487" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -17937,7 +17933,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17946,17 +17942,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F488" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G488" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -17973,7 +17969,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17982,17 +17978,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G489" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -18009,24 +18005,60 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E490" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F490" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G490" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D490" t="inlineStr">
+      <c r="D491" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E490" t="n">
+      <c r="E491" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F490" t="n">
+      <c r="F491" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G490" t="n">
+      <c r="G491" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H490" t="inlineStr">
+      <c r="H491" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 08:39:55)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H491"/>
+  <dimension ref="A1:H492"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16837,7 +16837,7 @@
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D457" t="inlineStr">
@@ -16846,17 +16846,13 @@
         </is>
       </c>
       <c r="E457" t="n">
-        <v>0.302013422818792</v>
-      </c>
-      <c r="F457" t="n">
-        <v>0.296875</v>
-      </c>
-      <c r="G457" t="n">
-        <v>0.2547169811320755</v>
-      </c>
+        <v>0.2965779467680608</v>
+      </c>
+      <c r="F457" t="inlineStr"/>
+      <c r="G457" t="inlineStr"/>
       <c r="H457" t="inlineStr">
         <is>
-          <t>0.2845 (0.0260)</t>
+          <t>0.2966 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -16873,7 +16869,7 @@
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
@@ -16882,17 +16878,17 @@
         </is>
       </c>
       <c r="E458" t="n">
-        <v>0.1621621621621622</v>
+        <v>0.302013422818792</v>
       </c>
       <c r="F458" t="n">
-        <v>0.2200956937799043</v>
+        <v>0.296875</v>
       </c>
       <c r="G458" t="n">
-        <v>0.223463687150838</v>
+        <v>0.2547169811320755</v>
       </c>
       <c r="H458" t="inlineStr">
         <is>
-          <t>0.2019 (0.0345)</t>
+          <t>0.2845 (0.0260)</t>
         </is>
       </c>
     </row>
@@ -16909,7 +16905,7 @@
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
@@ -16918,13 +16914,17 @@
         </is>
       </c>
       <c r="E459" t="n">
-        <v>0.3445945945945946</v>
-      </c>
-      <c r="F459" t="inlineStr"/>
-      <c r="G459" t="inlineStr"/>
+        <v>0.1621621621621622</v>
+      </c>
+      <c r="F459" t="n">
+        <v>0.2200956937799043</v>
+      </c>
+      <c r="G459" t="n">
+        <v>0.223463687150838</v>
+      </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>0.3446 (0.0000)</t>
+          <t>0.2019 (0.0345)</t>
         </is>
       </c>
     </row>
@@ -16936,27 +16936,27 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E460" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.3445945945945946</v>
       </c>
       <c r="F460" t="inlineStr"/>
       <c r="G460" t="inlineStr"/>
       <c r="H460" t="inlineStr">
         <is>
-          <t>0.3333 (0.0000)</t>
+          <t>0.3446 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -16973,7 +16973,7 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
@@ -16982,17 +16982,13 @@
         </is>
       </c>
       <c r="E461" t="n">
-        <v>0.3294573643410852</v>
-      </c>
-      <c r="F461" t="n">
-        <v>0.3059360730593607</v>
-      </c>
-      <c r="G461" t="n">
-        <v>0.2222222222222222</v>
-      </c>
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F461" t="inlineStr"/>
+      <c r="G461" t="inlineStr"/>
       <c r="H461" t="inlineStr">
         <is>
-          <t>0.2859 (0.0564)</t>
+          <t>0.3333 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17009,7 +17005,7 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
@@ -17018,17 +17014,17 @@
         </is>
       </c>
       <c r="E462" t="n">
-        <v>0.2285714285714286</v>
+        <v>0.3294573643410852</v>
       </c>
       <c r="F462" t="n">
-        <v>0.2239382239382239</v>
+        <v>0.3059360730593607</v>
       </c>
       <c r="G462" t="n">
-        <v>0.1831501831501831</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t>0.2119 (0.0250)</t>
+          <t>0.2859 (0.0564)</t>
         </is>
       </c>
     </row>
@@ -17045,7 +17041,7 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
@@ -17054,13 +17050,17 @@
         </is>
       </c>
       <c r="E463" t="n">
-        <v>0.3294797687861272</v>
-      </c>
-      <c r="F463" t="inlineStr"/>
-      <c r="G463" t="inlineStr"/>
+        <v>0.2285714285714286</v>
+      </c>
+      <c r="F463" t="n">
+        <v>0.2239382239382239</v>
+      </c>
+      <c r="G463" t="n">
+        <v>0.1831501831501831</v>
+      </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t>0.3295 (0.0000)</t>
+          <t>0.2119 (0.0250)</t>
         </is>
       </c>
     </row>
@@ -17077,7 +17077,7 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
@@ -17086,13 +17086,13 @@
         </is>
       </c>
       <c r="E464" t="n">
-        <v>0.3111111111111111</v>
+        <v>0.3294797687861272</v>
       </c>
       <c r="F464" t="inlineStr"/>
       <c r="G464" t="inlineStr"/>
       <c r="H464" t="inlineStr">
         <is>
-          <t>0.3111 (0.0000)</t>
+          <t>0.3295 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17104,31 +17104,29 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E465" t="n">
-        <v>0.3007518796992481</v>
+        <v>0.3111111111111111</v>
       </c>
       <c r="F465" t="n">
-        <v>0.1627906976744186</v>
-      </c>
-      <c r="G465" t="n">
-        <v>0.1818181818181818</v>
-      </c>
+        <v>0.2696629213483146</v>
+      </c>
+      <c r="G465" t="inlineStr"/>
       <c r="H465" t="inlineStr">
         <is>
-          <t>0.2151 (0.0748)</t>
+          <t>0.2904 (0.0293)</t>
         </is>
       </c>
     </row>
@@ -17145,7 +17143,7 @@
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
@@ -17154,17 +17152,17 @@
         </is>
       </c>
       <c r="E466" t="n">
-        <v>0.3321033210332103</v>
+        <v>0.3007518796992481</v>
       </c>
       <c r="F466" t="n">
-        <v>0.2543859649122807</v>
+        <v>0.1627906976744186</v>
       </c>
       <c r="G466" t="n">
-        <v>0.2901554404145077</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H466" t="inlineStr">
         <is>
-          <t>0.2922 (0.0389)</t>
+          <t>0.2151 (0.0748)</t>
         </is>
       </c>
     </row>
@@ -17181,7 +17179,7 @@
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
@@ -17190,17 +17188,17 @@
         </is>
       </c>
       <c r="E467" t="n">
-        <v>0.1209302325581395</v>
+        <v>0.3321033210332103</v>
       </c>
       <c r="F467" t="n">
-        <v>0.1182795698924731</v>
+        <v>0.2543859649122807</v>
       </c>
       <c r="G467" t="n">
-        <v>0.1548387096774194</v>
+        <v>0.2901554404145077</v>
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>0.1313 (0.0204)</t>
+          <t>0.2922 (0.0389)</t>
         </is>
       </c>
     </row>
@@ -17217,7 +17215,7 @@
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
@@ -17226,17 +17224,17 @@
         </is>
       </c>
       <c r="E468" t="n">
-        <v>0.391304347826087</v>
+        <v>0.1209302325581395</v>
       </c>
       <c r="F468" t="n">
-        <v>0.3221476510067114</v>
+        <v>0.1182795698924731</v>
       </c>
       <c r="G468" t="n">
-        <v>0.3011583011583012</v>
+        <v>0.1548387096774194</v>
       </c>
       <c r="H468" t="inlineStr">
         <is>
-          <t>0.3382 (0.0472)</t>
+          <t>0.1313 (0.0204)</t>
         </is>
       </c>
     </row>
@@ -17253,7 +17251,7 @@
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
@@ -17262,17 +17260,17 @@
         </is>
       </c>
       <c r="E469" t="n">
-        <v>0.2068965517241379</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="F469" t="n">
-        <v>0.1837837837837838</v>
+        <v>0.3221476510067114</v>
       </c>
       <c r="G469" t="n">
-        <v>0.2054794520547945</v>
+        <v>0.3011583011583012</v>
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>0.1987 (0.0130)</t>
+          <t>0.3382 (0.0472)</t>
         </is>
       </c>
     </row>
@@ -17284,31 +17282,31 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E470" t="n">
-        <v>0.303030303030303</v>
+        <v>0.2068965517241379</v>
       </c>
       <c r="F470" t="n">
-        <v>0.2022471910112359</v>
+        <v>0.1837837837837838</v>
       </c>
       <c r="G470" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2054794520547945</v>
       </c>
       <c r="H470" t="inlineStr">
         <is>
-          <t>0.2573 (0.0510)</t>
+          <t>0.1987 (0.0130)</t>
         </is>
       </c>
     </row>
@@ -17325,7 +17323,7 @@
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D471" t="inlineStr">
@@ -17334,17 +17332,17 @@
         </is>
       </c>
       <c r="E471" t="n">
-        <v>0.3125</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="F471" t="n">
-        <v>0.2698412698412698</v>
+        <v>0.2022471910112359</v>
       </c>
       <c r="G471" t="n">
-        <v>0.2639593908629442</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="H471" t="inlineStr">
         <is>
-          <t>0.2821 (0.0265)</t>
+          <t>0.2573 (0.0510)</t>
         </is>
       </c>
     </row>
@@ -17361,7 +17359,7 @@
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D472" t="inlineStr">
@@ -17370,17 +17368,17 @@
         </is>
       </c>
       <c r="E472" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3125</v>
       </c>
       <c r="F472" t="n">
-        <v>0.1256544502617801</v>
+        <v>0.2698412698412698</v>
       </c>
       <c r="G472" t="n">
-        <v>0.2</v>
+        <v>0.2639593908629442</v>
       </c>
       <c r="H472" t="inlineStr">
         <is>
-          <t>0.1692 (0.0388)</t>
+          <t>0.2821 (0.0265)</t>
         </is>
       </c>
     </row>
@@ -17397,7 +17395,7 @@
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D473" t="inlineStr">
@@ -17406,17 +17404,17 @@
         </is>
       </c>
       <c r="E473" t="n">
-        <v>0.3709090909090909</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F473" t="n">
-        <v>0.2521739130434782</v>
+        <v>0.1256544502617801</v>
       </c>
       <c r="G473" t="n">
-        <v>0.29</v>
+        <v>0.2</v>
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>0.3044 (0.0607)</t>
+          <t>0.1692 (0.0388)</t>
         </is>
       </c>
     </row>
@@ -17433,7 +17431,7 @@
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D474" t="inlineStr">
@@ -17442,53 +17440,53 @@
         </is>
       </c>
       <c r="E474" t="n">
-        <v>0.3135593220338983</v>
+        <v>0.3709090909090909</v>
       </c>
       <c r="F474" t="n">
-        <v>0.2155688622754491</v>
+        <v>0.2521739130434782</v>
       </c>
       <c r="G474" t="n">
-        <v>0.1780821917808219</v>
+        <v>0.29</v>
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t>0.2357 (0.0700)</t>
+          <t>0.3044 (0.0607)</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E475" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.3135593220338983</v>
       </c>
       <c r="F475" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2155688622754491</v>
       </c>
       <c r="G475" t="n">
-        <v>0.228310502283105</v>
+        <v>0.1780821917808219</v>
       </c>
       <c r="H475" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2357 (0.0700)</t>
         </is>
       </c>
     </row>
@@ -17505,7 +17503,7 @@
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D476" t="inlineStr">
@@ -17514,17 +17512,17 @@
         </is>
       </c>
       <c r="E476" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F476" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G476" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -17541,7 +17539,7 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
@@ -17550,17 +17548,17 @@
         </is>
       </c>
       <c r="E477" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F477" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G477" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -17577,7 +17575,7 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
@@ -17586,17 +17584,17 @@
         </is>
       </c>
       <c r="E478" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F478" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G478" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -17613,7 +17611,7 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
@@ -17622,17 +17620,17 @@
         </is>
       </c>
       <c r="E479" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F479" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G479" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H479" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -17644,31 +17642,31 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E480" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F480" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2383419689119171</v>
       </c>
       <c r="G480" t="n">
-        <v>0.2377622377622378</v>
+        <v>0.1940928270042194</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -17685,7 +17683,7 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
@@ -17694,13 +17692,17 @@
         </is>
       </c>
       <c r="E481" t="n">
-        <v>0.163265306122449</v>
-      </c>
-      <c r="F481" t="inlineStr"/>
-      <c r="G481" t="inlineStr"/>
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="F481" t="n">
+        <v>0.2592592592592592</v>
+      </c>
+      <c r="G481" t="n">
+        <v>0.2377622377622378</v>
+      </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>0.1633 (0.0000)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -17712,31 +17714,27 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.196078431372549</v>
-      </c>
-      <c r="F482" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G482" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.163265306122449</v>
+      </c>
+      <c r="F482" t="inlineStr"/>
+      <c r="G482" t="inlineStr"/>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.1633 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17753,7 +17751,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
@@ -17762,17 +17760,17 @@
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F483" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G483" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -17789,7 +17787,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -17798,17 +17796,17 @@
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F484" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G484" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -17825,7 +17823,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17834,17 +17832,17 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F485" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G485" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -17861,7 +17859,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17870,17 +17868,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F486" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G486" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -17892,31 +17890,31 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F487" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G487" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -17933,7 +17931,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17942,17 +17940,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F488" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G488" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -17969,7 +17967,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17978,17 +17976,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G489" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18005,7 +18003,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18014,17 +18012,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F490" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G490" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -18041,24 +18039,60 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E491" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F491" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G491" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D491" t="inlineStr">
+      <c r="D492" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E491" t="n">
+      <c r="E492" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F491" t="n">
+      <c r="F492" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G491" t="n">
+      <c r="G492" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H491" t="inlineStr">
+      <c r="H492" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 09:40:15)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -17088,11 +17088,13 @@
       <c r="E464" t="n">
         <v>0.3294797687861272</v>
       </c>
-      <c r="F464" t="inlineStr"/>
+      <c r="F464" t="n">
+        <v>0.2527075812274368</v>
+      </c>
       <c r="G464" t="inlineStr"/>
       <c r="H464" t="inlineStr">
         <is>
-          <t>0.3295 (0.0000)</t>
+          <t>0.2911 (0.0543)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 10:40:33)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -16984,11 +16984,13 @@
       <c r="E461" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="F461" t="inlineStr"/>
+      <c r="F461" t="n">
+        <v>0.2748091603053435</v>
+      </c>
       <c r="G461" t="inlineStr"/>
       <c r="H461" t="inlineStr">
         <is>
-          <t>0.3333 (0.0000)</t>
+          <t>0.3041 (0.0414)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 11:40:51)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H492"/>
+  <dimension ref="A1:H493"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16968,29 +16968,27 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E461" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="F461" t="n">
-        <v>0.2748091603053435</v>
-      </c>
+        <v>0.2648401826484018</v>
+      </c>
+      <c r="F461" t="inlineStr"/>
       <c r="G461" t="inlineStr"/>
       <c r="H461" t="inlineStr">
         <is>
-          <t>0.3041 (0.0414)</t>
+          <t>0.2648 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17007,7 +17005,7 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
@@ -17016,17 +17014,15 @@
         </is>
       </c>
       <c r="E462" t="n">
-        <v>0.3294573643410852</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F462" t="n">
-        <v>0.3059360730593607</v>
-      </c>
-      <c r="G462" t="n">
-        <v>0.2222222222222222</v>
-      </c>
+        <v>0.2748091603053435</v>
+      </c>
+      <c r="G462" t="inlineStr"/>
       <c r="H462" t="inlineStr">
         <is>
-          <t>0.2859 (0.0564)</t>
+          <t>0.3041 (0.0414)</t>
         </is>
       </c>
     </row>
@@ -17043,7 +17039,7 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
@@ -17052,17 +17048,17 @@
         </is>
       </c>
       <c r="E463" t="n">
-        <v>0.2285714285714286</v>
+        <v>0.3294573643410852</v>
       </c>
       <c r="F463" t="n">
-        <v>0.2239382239382239</v>
+        <v>0.3059360730593607</v>
       </c>
       <c r="G463" t="n">
-        <v>0.1831501831501831</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t>0.2119 (0.0250)</t>
+          <t>0.2859 (0.0564)</t>
         </is>
       </c>
     </row>
@@ -17079,7 +17075,7 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
@@ -17088,15 +17084,17 @@
         </is>
       </c>
       <c r="E464" t="n">
-        <v>0.3294797687861272</v>
+        <v>0.2285714285714286</v>
       </c>
       <c r="F464" t="n">
-        <v>0.2527075812274368</v>
-      </c>
-      <c r="G464" t="inlineStr"/>
+        <v>0.2239382239382239</v>
+      </c>
+      <c r="G464" t="n">
+        <v>0.1831501831501831</v>
+      </c>
       <c r="H464" t="inlineStr">
         <is>
-          <t>0.2911 (0.0543)</t>
+          <t>0.2119 (0.0250)</t>
         </is>
       </c>
     </row>
@@ -17113,7 +17111,7 @@
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
@@ -17122,15 +17120,15 @@
         </is>
       </c>
       <c r="E465" t="n">
-        <v>0.3111111111111111</v>
+        <v>0.3294797687861272</v>
       </c>
       <c r="F465" t="n">
-        <v>0.2696629213483146</v>
+        <v>0.2527075812274368</v>
       </c>
       <c r="G465" t="inlineStr"/>
       <c r="H465" t="inlineStr">
         <is>
-          <t>0.2904 (0.0293)</t>
+          <t>0.2911 (0.0543)</t>
         </is>
       </c>
     </row>
@@ -17142,31 +17140,29 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E466" t="n">
-        <v>0.3007518796992481</v>
+        <v>0.3111111111111111</v>
       </c>
       <c r="F466" t="n">
-        <v>0.1627906976744186</v>
-      </c>
-      <c r="G466" t="n">
-        <v>0.1818181818181818</v>
-      </c>
+        <v>0.2696629213483146</v>
+      </c>
+      <c r="G466" t="inlineStr"/>
       <c r="H466" t="inlineStr">
         <is>
-          <t>0.2151 (0.0748)</t>
+          <t>0.2904 (0.0293)</t>
         </is>
       </c>
     </row>
@@ -17183,7 +17179,7 @@
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
@@ -17192,17 +17188,17 @@
         </is>
       </c>
       <c r="E467" t="n">
-        <v>0.3321033210332103</v>
+        <v>0.3007518796992481</v>
       </c>
       <c r="F467" t="n">
-        <v>0.2543859649122807</v>
+        <v>0.1627906976744186</v>
       </c>
       <c r="G467" t="n">
-        <v>0.2901554404145077</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>0.2922 (0.0389)</t>
+          <t>0.2151 (0.0748)</t>
         </is>
       </c>
     </row>
@@ -17219,7 +17215,7 @@
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
@@ -17228,17 +17224,17 @@
         </is>
       </c>
       <c r="E468" t="n">
-        <v>0.1209302325581395</v>
+        <v>0.3321033210332103</v>
       </c>
       <c r="F468" t="n">
-        <v>0.1182795698924731</v>
+        <v>0.2543859649122807</v>
       </c>
       <c r="G468" t="n">
-        <v>0.1548387096774194</v>
+        <v>0.2901554404145077</v>
       </c>
       <c r="H468" t="inlineStr">
         <is>
-          <t>0.1313 (0.0204)</t>
+          <t>0.2922 (0.0389)</t>
         </is>
       </c>
     </row>
@@ -17255,7 +17251,7 @@
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
@@ -17264,17 +17260,17 @@
         </is>
       </c>
       <c r="E469" t="n">
-        <v>0.391304347826087</v>
+        <v>0.1209302325581395</v>
       </c>
       <c r="F469" t="n">
-        <v>0.3221476510067114</v>
+        <v>0.1182795698924731</v>
       </c>
       <c r="G469" t="n">
-        <v>0.3011583011583012</v>
+        <v>0.1548387096774194</v>
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>0.3382 (0.0472)</t>
+          <t>0.1313 (0.0204)</t>
         </is>
       </c>
     </row>
@@ -17291,7 +17287,7 @@
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
@@ -17300,17 +17296,17 @@
         </is>
       </c>
       <c r="E470" t="n">
-        <v>0.2068965517241379</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="F470" t="n">
-        <v>0.1837837837837838</v>
+        <v>0.3221476510067114</v>
       </c>
       <c r="G470" t="n">
-        <v>0.2054794520547945</v>
+        <v>0.3011583011583012</v>
       </c>
       <c r="H470" t="inlineStr">
         <is>
-          <t>0.1987 (0.0130)</t>
+          <t>0.3382 (0.0472)</t>
         </is>
       </c>
     </row>
@@ -17322,31 +17318,31 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D471" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E471" t="n">
-        <v>0.303030303030303</v>
+        <v>0.2068965517241379</v>
       </c>
       <c r="F471" t="n">
-        <v>0.2022471910112359</v>
+        <v>0.1837837837837838</v>
       </c>
       <c r="G471" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2054794520547945</v>
       </c>
       <c r="H471" t="inlineStr">
         <is>
-          <t>0.2573 (0.0510)</t>
+          <t>0.1987 (0.0130)</t>
         </is>
       </c>
     </row>
@@ -17363,7 +17359,7 @@
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D472" t="inlineStr">
@@ -17372,17 +17368,17 @@
         </is>
       </c>
       <c r="E472" t="n">
-        <v>0.3125</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="F472" t="n">
-        <v>0.2698412698412698</v>
+        <v>0.2022471910112359</v>
       </c>
       <c r="G472" t="n">
-        <v>0.2639593908629442</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="H472" t="inlineStr">
         <is>
-          <t>0.2821 (0.0265)</t>
+          <t>0.2573 (0.0510)</t>
         </is>
       </c>
     </row>
@@ -17399,7 +17395,7 @@
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D473" t="inlineStr">
@@ -17408,17 +17404,17 @@
         </is>
       </c>
       <c r="E473" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3125</v>
       </c>
       <c r="F473" t="n">
-        <v>0.1256544502617801</v>
+        <v>0.2698412698412698</v>
       </c>
       <c r="G473" t="n">
-        <v>0.2</v>
+        <v>0.2639593908629442</v>
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>0.1692 (0.0388)</t>
+          <t>0.2821 (0.0265)</t>
         </is>
       </c>
     </row>
@@ -17435,7 +17431,7 @@
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D474" t="inlineStr">
@@ -17444,17 +17440,17 @@
         </is>
       </c>
       <c r="E474" t="n">
-        <v>0.3709090909090909</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F474" t="n">
-        <v>0.2521739130434782</v>
+        <v>0.1256544502617801</v>
       </c>
       <c r="G474" t="n">
-        <v>0.29</v>
+        <v>0.2</v>
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t>0.3044 (0.0607)</t>
+          <t>0.1692 (0.0388)</t>
         </is>
       </c>
     </row>
@@ -17471,7 +17467,7 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
@@ -17480,53 +17476,53 @@
         </is>
       </c>
       <c r="E475" t="n">
-        <v>0.3135593220338983</v>
+        <v>0.3709090909090909</v>
       </c>
       <c r="F475" t="n">
-        <v>0.2155688622754491</v>
+        <v>0.2521739130434782</v>
       </c>
       <c r="G475" t="n">
-        <v>0.1780821917808219</v>
+        <v>0.29</v>
       </c>
       <c r="H475" t="inlineStr">
         <is>
-          <t>0.2357 (0.0700)</t>
+          <t>0.3044 (0.0607)</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_ERa_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D476" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E476" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.3135593220338983</v>
       </c>
       <c r="F476" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2155688622754491</v>
       </c>
       <c r="G476" t="n">
-        <v>0.228310502283105</v>
+        <v>0.1780821917808219</v>
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2357 (0.0700)</t>
         </is>
       </c>
     </row>
@@ -17543,7 +17539,7 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
@@ -17552,17 +17548,17 @@
         </is>
       </c>
       <c r="E477" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F477" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G477" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -17579,7 +17575,7 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
@@ -17588,17 +17584,17 @@
         </is>
       </c>
       <c r="E478" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F478" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G478" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -17615,7 +17611,7 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
@@ -17624,17 +17620,17 @@
         </is>
       </c>
       <c r="E479" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F479" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G479" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H479" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -17651,7 +17647,7 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
@@ -17660,17 +17656,17 @@
         </is>
       </c>
       <c r="E480" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F480" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G480" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -17682,31 +17678,31 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E481" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F481" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2383419689119171</v>
       </c>
       <c r="G481" t="n">
-        <v>0.2377622377622378</v>
+        <v>0.1940928270042194</v>
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -17723,7 +17719,7 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
@@ -17732,13 +17728,17 @@
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.163265306122449</v>
-      </c>
-      <c r="F482" t="inlineStr"/>
-      <c r="G482" t="inlineStr"/>
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="F482" t="n">
+        <v>0.2592592592592592</v>
+      </c>
+      <c r="G482" t="n">
+        <v>0.2377622377622378</v>
+      </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.1633 (0.0000)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -17750,31 +17750,29 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.196078431372549</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F483" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G483" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G483" t="inlineStr"/>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.1830 (0.0279)</t>
         </is>
       </c>
     </row>
@@ -17791,7 +17789,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -17800,17 +17798,17 @@
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F484" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G484" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -17827,7 +17825,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17836,17 +17834,17 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F485" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G485" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -17863,7 +17861,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17872,17 +17870,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F486" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G486" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -17899,7 +17897,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17908,17 +17906,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F487" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G487" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -17930,31 +17928,31 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F488" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G488" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -17971,7 +17969,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17980,17 +17978,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G489" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -18007,7 +18005,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18016,17 +18014,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F490" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G490" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18043,7 +18041,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18052,17 +18050,17 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G491" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -18079,24 +18077,60 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E492" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F492" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G492" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D492" t="inlineStr">
+      <c r="D493" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E492" t="n">
+      <c r="E493" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F492" t="n">
+      <c r="F493" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G492" t="n">
+      <c r="G493" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H492" t="inlineStr">
+      <c r="H493" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 15:42:04)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H493"/>
+  <dimension ref="A1:H494"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17159,10 +17159,12 @@
       <c r="F466" t="n">
         <v>0.2696629213483146</v>
       </c>
-      <c r="G466" t="inlineStr"/>
+      <c r="G466" t="n">
+        <v>0.3053435114503817</v>
+      </c>
       <c r="H466" t="inlineStr">
         <is>
-          <t>0.2904 (0.0293)</t>
+          <t>0.2954 (0.0225)</t>
         </is>
       </c>
     </row>
@@ -17769,10 +17771,12 @@
       <c r="F483" t="n">
         <v>0.2027027027027027</v>
       </c>
-      <c r="G483" t="inlineStr"/>
+      <c r="G483" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.1830 (0.0279)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -17784,31 +17788,27 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.196078431372549</v>
-      </c>
-      <c r="F484" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G484" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.2747252747252747</v>
+      </c>
+      <c r="F484" t="inlineStr"/>
+      <c r="G484" t="inlineStr"/>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2747 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17825,7 +17825,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17834,17 +17834,17 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F485" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G485" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -17861,7 +17861,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17870,17 +17870,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F486" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G486" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -17897,7 +17897,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17906,17 +17906,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F487" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G487" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -17933,7 +17933,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17942,17 +17942,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F488" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G488" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -17964,31 +17964,31 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G489" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -18005,7 +18005,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18014,17 +18014,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F490" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G490" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -18041,7 +18041,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18050,17 +18050,17 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G491" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18086,17 +18086,17 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G492" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -18113,24 +18113,60 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E493" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F493" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G493" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D493" t="inlineStr">
+      <c r="D494" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E493" t="n">
+      <c r="E494" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F493" t="n">
+      <c r="F494" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G493" t="n">
+      <c r="G494" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H493" t="inlineStr">
+      <c r="H494" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 16:42:20)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H494"/>
+  <dimension ref="A1:H495"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16952,11 +16952,13 @@
       <c r="E460" t="n">
         <v>0.3445945945945946</v>
       </c>
-      <c r="F460" t="inlineStr"/>
+      <c r="F460" t="n">
+        <v>0.2242990654205607</v>
+      </c>
       <c r="G460" t="inlineStr"/>
       <c r="H460" t="inlineStr">
         <is>
-          <t>0.3446 (0.0000)</t>
+          <t>0.2844 (0.0851)</t>
         </is>
       </c>
     </row>
@@ -17019,10 +17021,12 @@
       <c r="F462" t="n">
         <v>0.2748091603053435</v>
       </c>
-      <c r="G462" t="inlineStr"/>
+      <c r="G462" t="n">
+        <v>0.3255813953488372</v>
+      </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t>0.3041 (0.0414)</t>
+          <t>0.3112 (0.0318)</t>
         </is>
       </c>
     </row>
@@ -17125,10 +17129,12 @@
       <c r="F465" t="n">
         <v>0.2527075812274368</v>
       </c>
-      <c r="G465" t="inlineStr"/>
+      <c r="G465" t="n">
+        <v>0.2681159420289855</v>
+      </c>
       <c r="H465" t="inlineStr">
         <is>
-          <t>0.2911 (0.0543)</t>
+          <t>0.2834 (0.0406)</t>
         </is>
       </c>
     </row>
@@ -17788,27 +17794,27 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.3054187192118227</v>
       </c>
       <c r="F484" t="inlineStr"/>
       <c r="G484" t="inlineStr"/>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.2747 (0.0000)</t>
+          <t>0.3054 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17820,31 +17826,31 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F485" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G485" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -17861,7 +17867,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17870,17 +17876,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F486" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G486" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -17897,7 +17903,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17906,17 +17912,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F487" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G487" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -17933,7 +17939,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17942,17 +17948,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F488" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G488" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -17969,7 +17975,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17978,17 +17984,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F489" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G489" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -18000,31 +18006,31 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F490" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G490" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -18041,7 +18047,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18050,17 +18056,17 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G491" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18083,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18086,17 +18092,17 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G492" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18113,7 +18119,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18122,17 +18128,17 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F493" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G493" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -18149,24 +18155,60 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E494" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F494" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G494" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D494" t="inlineStr">
+      <c r="D495" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E494" t="n">
+      <c r="E495" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F494" t="n">
+      <c r="F495" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G494" t="n">
+      <c r="G495" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H494" t="inlineStr">
+      <c r="H495" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 17:42:36)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H495"/>
+  <dimension ref="A1:H499"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17537,7 +17537,7 @@
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
@@ -17547,7 +17547,7 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
@@ -17556,24 +17556,24 @@
         </is>
       </c>
       <c r="E477" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F477" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.3161764705882353</v>
       </c>
       <c r="G477" t="n">
-        <v>0.228310502283105</v>
+        <v>0.316205533596838</v>
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.3169 (0.0011)</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B478" t="inlineStr">
@@ -17583,7 +17583,7 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
@@ -17592,24 +17592,24 @@
         </is>
       </c>
       <c r="E478" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2290748898678414</v>
       </c>
       <c r="F478" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.256198347107438</v>
       </c>
       <c r="G478" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.2629107981220657</v>
       </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2494 (0.0179)</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B479" t="inlineStr">
@@ -17619,7 +17619,7 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
@@ -17628,17 +17628,13 @@
         </is>
       </c>
       <c r="E479" t="n">
-        <v>0.2135922330097087</v>
-      </c>
-      <c r="F479" t="n">
-        <v>0.2307692307692308</v>
-      </c>
-      <c r="G479" t="n">
-        <v>0.1616161616161616</v>
-      </c>
+        <v>0.2807017543859649</v>
+      </c>
+      <c r="F479" t="inlineStr"/>
+      <c r="G479" t="inlineStr"/>
       <c r="H479" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2807 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17655,7 +17651,7 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
@@ -17664,17 +17660,17 @@
         </is>
       </c>
       <c r="E480" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F480" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G480" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -17691,7 +17687,7 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
@@ -17700,17 +17696,17 @@
         </is>
       </c>
       <c r="E481" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F481" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G481" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -17722,31 +17718,31 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F482" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G482" t="n">
-        <v>0.2377622377622378</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -17758,31 +17754,31 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F483" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G483" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -17794,27 +17790,31 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.3054187192118227</v>
-      </c>
-      <c r="F484" t="inlineStr"/>
-      <c r="G484" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F484" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G484" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.3054 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -17826,7 +17826,7 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
@@ -17836,21 +17836,21 @@
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F485" t="n">
-        <v>0.258575197889182</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G485" t="n">
-        <v>0.1852861035422343</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -17862,31 +17862,31 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.196078431372549</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F486" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2027027027027027</v>
       </c>
       <c r="G486" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.2138364779874214</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -17898,31 +17898,27 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.2358974358974359</v>
-      </c>
-      <c r="F487" t="n">
-        <v>0.2840909090909091</v>
-      </c>
-      <c r="G487" t="n">
-        <v>0.2153846153846154</v>
-      </c>
+        <v>0.3054187192118227</v>
+      </c>
+      <c r="F487" t="inlineStr"/>
+      <c r="G487" t="inlineStr"/>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.3054 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17934,31 +17930,31 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F488" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G488" t="n">
-        <v>0.125</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -17970,31 +17966,27 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.3370786516853932</v>
-      </c>
-      <c r="F489" t="n">
-        <v>0.3091787439613526</v>
-      </c>
-      <c r="G489" t="n">
-        <v>0.1438848920863309</v>
-      </c>
+        <v>0.16</v>
+      </c>
+      <c r="F489" t="inlineStr"/>
+      <c r="G489" t="inlineStr"/>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1600 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18011,7 +18003,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18020,17 +18012,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F490" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G490" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18042,31 +18034,31 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.232258064516129</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G491" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -18078,31 +18070,31 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G492" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.125</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -18114,31 +18106,31 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F493" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G493" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -18150,31 +18142,31 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F494" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G494" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -18191,24 +18183,168 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E495" t="n">
+        <v>0.232258064516129</v>
+      </c>
+      <c r="F495" t="n">
+        <v>0.2385321100917431</v>
+      </c>
+      <c r="G495" t="n">
+        <v>0.2131147540983606</v>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>0.2280 (0.0132)</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E496" t="n">
+        <v>0.2087912087912088</v>
+      </c>
+      <c r="F496" t="n">
+        <v>0.2738095238095238</v>
+      </c>
+      <c r="G496" t="n">
+        <v>0.2705882352941176</v>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>0.2511 (0.0366)</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E497" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F497" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G497" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E498" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F498" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G498" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D495" t="inlineStr">
+      <c r="D499" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E495" t="n">
+      <c r="E499" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F495" t="n">
+      <c r="F499" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G495" t="n">
+      <c r="G499" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H495" t="inlineStr">
+      <c r="H499" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 18:42:55)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H499"/>
+  <dimension ref="A1:H506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17547,7 +17547,7 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
@@ -17556,17 +17556,17 @@
         </is>
       </c>
       <c r="E477" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.2534246575342466</v>
       </c>
       <c r="F477" t="n">
-        <v>0.3161764705882353</v>
+        <v>0.302788844621514</v>
       </c>
       <c r="G477" t="n">
-        <v>0.316205533596838</v>
+        <v>0.2775510204081633</v>
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>0.3169 (0.0011)</t>
+          <t>0.2779 (0.0247)</t>
         </is>
       </c>
     </row>
@@ -17583,7 +17583,7 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
@@ -17592,17 +17592,17 @@
         </is>
       </c>
       <c r="E478" t="n">
-        <v>0.2290748898678414</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F478" t="n">
-        <v>0.256198347107438</v>
+        <v>0.3161764705882353</v>
       </c>
       <c r="G478" t="n">
-        <v>0.2629107981220657</v>
+        <v>0.316205533596838</v>
       </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>0.2494 (0.0179)</t>
+          <t>0.3169 (0.0011)</t>
         </is>
       </c>
     </row>
@@ -17619,7 +17619,7 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
@@ -17628,20 +17628,24 @@
         </is>
       </c>
       <c r="E479" t="n">
-        <v>0.2807017543859649</v>
-      </c>
-      <c r="F479" t="inlineStr"/>
-      <c r="G479" t="inlineStr"/>
+        <v>0.2290748898678414</v>
+      </c>
+      <c r="F479" t="n">
+        <v>0.256198347107438</v>
+      </c>
+      <c r="G479" t="n">
+        <v>0.2629107981220657</v>
+      </c>
       <c r="H479" t="inlineStr">
         <is>
-          <t>0.2807 (0.0000)</t>
+          <t>0.2494 (0.0179)</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B480" t="inlineStr">
@@ -17651,7 +17655,7 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
@@ -17660,24 +17664,24 @@
         </is>
       </c>
       <c r="E480" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.319327731092437</v>
       </c>
       <c r="F480" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2845849802371542</v>
       </c>
       <c r="G480" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2331838565022422</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2790 (0.0433)</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B481" t="inlineStr">
@@ -17687,7 +17691,7 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
@@ -17696,197 +17700,187 @@
         </is>
       </c>
       <c r="E481" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="F481" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2786885245901639</v>
       </c>
       <c r="G481" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.3665338645418327</v>
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.3086 (0.0501)</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.2135922330097087</v>
-      </c>
-      <c r="F482" t="n">
-        <v>0.2307692307692308</v>
-      </c>
-      <c r="G482" t="n">
-        <v>0.1616161616161616</v>
-      </c>
+        <v>0.2923076923076923</v>
+      </c>
+      <c r="F482" t="inlineStr"/>
+      <c r="G482" t="inlineStr"/>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2923 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F483" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G483" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F484" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G484" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F485" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G485" t="n">
-        <v>0.2377622377622378</v>
-      </c>
+        <v>0.4054054054054054</v>
+      </c>
+      <c r="F485" t="inlineStr"/>
+      <c r="G485" t="inlineStr"/>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.4054 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F486" t="n">
-        <v>0.2027027027027027</v>
-      </c>
-      <c r="G486" t="n">
-        <v>0.2138364779874214</v>
-      </c>
+        <v>0.1940298507462687</v>
+      </c>
+      <c r="G486" t="inlineStr"/>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2103 (0.0231)</t>
         </is>
       </c>
     </row>
@@ -17898,27 +17892,31 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.3054187192118227</v>
-      </c>
-      <c r="F487" t="inlineStr"/>
-      <c r="G487" t="inlineStr"/>
+        <v>0.2595419847328244</v>
+      </c>
+      <c r="F487" t="n">
+        <v>0.2164948453608248</v>
+      </c>
+      <c r="G487" t="n">
+        <v>0.228310502283105</v>
+      </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.3054 (0.0000)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -17930,7 +17928,7 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
@@ -17940,21 +17938,21 @@
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F488" t="n">
-        <v>0.258575197889182</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G488" t="n">
-        <v>0.1852861035422343</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -17966,7 +17964,7 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
@@ -17976,17 +17974,21 @@
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="F489" t="inlineStr"/>
-      <c r="G489" t="inlineStr"/>
+        <v>0.2135922330097087</v>
+      </c>
+      <c r="F489" t="n">
+        <v>0.2307692307692308</v>
+      </c>
+      <c r="G489" t="n">
+        <v>0.1616161616161616</v>
+      </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.1600 (0.0000)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -17998,31 +18000,31 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F490" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G490" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18034,31 +18036,31 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2383419689119171</v>
       </c>
       <c r="G491" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1940928270042194</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18070,31 +18072,31 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F492" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G492" t="n">
-        <v>0.125</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18106,31 +18108,31 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F493" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.2027027027027027</v>
       </c>
       <c r="G493" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.2138364779874214</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -18142,31 +18144,27 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.1940298507462687</v>
-      </c>
-      <c r="F494" t="n">
-        <v>0.1481481481481481</v>
-      </c>
-      <c r="G494" t="n">
-        <v>0.1333333333333333</v>
-      </c>
+        <v>0.3054187192118227</v>
+      </c>
+      <c r="F494" t="inlineStr"/>
+      <c r="G494" t="inlineStr"/>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.3054 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18178,31 +18176,31 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.232258064516129</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F495" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G495" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -18214,31 +18212,27 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.2087912087912088</v>
-      </c>
-      <c r="F496" t="n">
-        <v>0.2738095238095238</v>
-      </c>
-      <c r="G496" t="n">
-        <v>0.2705882352941176</v>
-      </c>
+        <v>0.16</v>
+      </c>
+      <c r="F496" t="inlineStr"/>
+      <c r="G496" t="inlineStr"/>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.1600 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18250,31 +18244,31 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F497" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G497" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18286,31 +18280,31 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G498" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -18322,29 +18316,281 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E499" t="n">
+        <v>0.1714285714285714</v>
+      </c>
+      <c r="F499" t="n">
+        <v>0.1746031746031746</v>
+      </c>
+      <c r="G499" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>0.1570 (0.0278)</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E500" t="n">
+        <v>0.3370786516853932</v>
+      </c>
+      <c r="F500" t="n">
+        <v>0.3091787439613526</v>
+      </c>
+      <c r="G500" t="n">
+        <v>0.1438848920863309</v>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>0.2634 (0.1044)</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E501" t="n">
+        <v>0.1940298507462687</v>
+      </c>
+      <c r="F501" t="n">
+        <v>0.1481481481481481</v>
+      </c>
+      <c r="G501" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>0.1585 (0.0316)</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
           <t>xgb</t>
         </is>
       </c>
-      <c r="C499" t="inlineStr">
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E502" t="n">
+        <v>0.232258064516129</v>
+      </c>
+      <c r="F502" t="n">
+        <v>0.2385321100917431</v>
+      </c>
+      <c r="G502" t="n">
+        <v>0.2131147540983606</v>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>0.2280 (0.0132)</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E503" t="n">
+        <v>0.2087912087912088</v>
+      </c>
+      <c r="F503" t="n">
+        <v>0.2738095238095238</v>
+      </c>
+      <c r="G503" t="n">
+        <v>0.2705882352941176</v>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>0.2511 (0.0366)</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E504" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F504" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G504" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E505" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F505" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G505" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
         <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D499" t="inlineStr">
+      <c r="D506" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E499" t="n">
+      <c r="E506" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F499" t="n">
+      <c r="F506" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G499" t="n">
+      <c r="G506" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H499" t="inlineStr">
+      <c r="H506" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 19:43:13)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H506"/>
+  <dimension ref="A1:H508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17738,11 +17738,15 @@
       <c r="E482" t="n">
         <v>0.2923076923076923</v>
       </c>
-      <c r="F482" t="inlineStr"/>
-      <c r="G482" t="inlineStr"/>
+      <c r="F482" t="n">
+        <v>0.2844444444444444</v>
+      </c>
+      <c r="G482" t="n">
+        <v>0.2627737226277372</v>
+      </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.2923 (0.0000)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -17842,11 +17846,15 @@
       <c r="E485" t="n">
         <v>0.4054054054054054</v>
       </c>
-      <c r="F485" t="inlineStr"/>
-      <c r="G485" t="inlineStr"/>
+      <c r="F485" t="n">
+        <v>0.362962962962963</v>
+      </c>
+      <c r="G485" t="n">
+        <v>0.3852459016393442</v>
+      </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.4054 (0.0000)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -17877,82 +17885,80 @@
       <c r="F486" t="n">
         <v>0.1940298507462687</v>
       </c>
-      <c r="G486" t="inlineStr"/>
+      <c r="G486" t="n">
+        <v>0.1774193548387097</v>
+      </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.2103 (0.0231)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F487" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G487" t="n">
-        <v>0.228310502283105</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.2322097378277154</v>
-      </c>
-      <c r="F488" t="n">
-        <v>0.2212389380530974</v>
-      </c>
-      <c r="G488" t="n">
-        <v>0.2288135593220339</v>
-      </c>
+        <v>0.1818181818181818</v>
+      </c>
+      <c r="F488" t="inlineStr"/>
+      <c r="G488" t="inlineStr"/>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.1818 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17969,7 +17975,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17978,17 +17984,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G489" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18005,7 +18011,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18014,17 +18020,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F490" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G490" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -18041,7 +18047,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18050,17 +18056,17 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G491" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -18072,31 +18078,31 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G492" t="n">
-        <v>0.2377622377622378</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18108,31 +18114,31 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F493" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2383419689119171</v>
       </c>
       <c r="G493" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.1940928270042194</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18149,7 +18155,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -18158,13 +18164,17 @@
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.3054187192118227</v>
-      </c>
-      <c r="F494" t="inlineStr"/>
-      <c r="G494" t="inlineStr"/>
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="F494" t="n">
+        <v>0.2592592592592592</v>
+      </c>
+      <c r="G494" t="n">
+        <v>0.2377622377622378</v>
+      </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.3054 (0.0000)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18176,31 +18186,31 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F495" t="n">
-        <v>0.258575197889182</v>
+        <v>0.2027027027027027</v>
       </c>
       <c r="G495" t="n">
-        <v>0.1852861035422343</v>
+        <v>0.2138364779874214</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -18212,27 +18222,27 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.16</v>
+        <v>0.3054187192118227</v>
       </c>
       <c r="F496" t="inlineStr"/>
       <c r="G496" t="inlineStr"/>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.1600 (0.0000)</t>
+          <t>0.3054 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18244,31 +18254,31 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F497" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G497" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -18280,31 +18290,29 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.16</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2840909090909091</v>
-      </c>
-      <c r="G498" t="n">
-        <v>0.2153846153846154</v>
-      </c>
+        <v>0.2094240837696335</v>
+      </c>
+      <c r="G498" t="inlineStr"/>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1847 (0.0349)</t>
         </is>
       </c>
     </row>
@@ -18321,7 +18329,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
@@ -18330,17 +18338,17 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F499" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G499" t="n">
-        <v>0.125</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18357,7 +18365,7 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
@@ -18366,17 +18374,17 @@
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F500" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G500" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -18393,7 +18401,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
@@ -18402,17 +18410,17 @@
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F501" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G501" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.125</v>
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -18424,31 +18432,31 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.232258064516129</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F502" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G502" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -18460,31 +18468,31 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F503" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G503" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -18501,7 +18509,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
@@ -18510,17 +18518,17 @@
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F504" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G504" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -18537,7 +18545,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -18546,17 +18554,17 @@
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F505" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G505" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18573,24 +18581,96 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E506" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F506" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G506" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E507" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F507" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G507" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D506" t="inlineStr">
+      <c r="D508" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E506" t="n">
+      <c r="E508" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F506" t="n">
+      <c r="F508" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G506" t="n">
+      <c r="G508" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H506" t="inlineStr">
+      <c r="H508" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 20:43:31)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H508"/>
+  <dimension ref="A1:H511"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17954,83 +17954,79 @@
       <c r="E488" t="n">
         <v>0.1818181818181818</v>
       </c>
-      <c r="F488" t="inlineStr"/>
-      <c r="G488" t="inlineStr"/>
+      <c r="F488" t="n">
+        <v>0.2159090909090909</v>
+      </c>
+      <c r="G488" t="n">
+        <v>0.2413793103448276</v>
+      </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.1818 (0.0000)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.2595419847328244</v>
-      </c>
-      <c r="F489" t="n">
-        <v>0.2164948453608248</v>
-      </c>
-      <c r="G489" t="n">
-        <v>0.228310502283105</v>
-      </c>
+        <v>0.3444976076555024</v>
+      </c>
+      <c r="F489" t="inlineStr"/>
+      <c r="G489" t="inlineStr"/>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.3445 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.2322097378277154</v>
-      </c>
-      <c r="F490" t="n">
-        <v>0.2212389380530974</v>
-      </c>
-      <c r="G490" t="n">
-        <v>0.2288135593220339</v>
-      </c>
+        <v>0.225</v>
+      </c>
+      <c r="F490" t="inlineStr"/>
+      <c r="G490" t="inlineStr"/>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2250 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18047,7 +18043,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18056,17 +18052,17 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G491" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18083,7 +18079,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18092,17 +18088,17 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G492" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -18119,7 +18115,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18128,17 +18124,17 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F493" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G493" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -18150,31 +18146,31 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F494" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G494" t="n">
-        <v>0.2377622377622378</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18186,31 +18182,31 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F495" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2383419689119171</v>
       </c>
       <c r="G495" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.1940928270042194</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18223,7 @@
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
@@ -18236,13 +18232,13 @@
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.3054187192118227</v>
+        <v>0.2487046632124352</v>
       </c>
       <c r="F496" t="inlineStr"/>
       <c r="G496" t="inlineStr"/>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.3054 (0.0000)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18254,7 +18250,7 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
@@ -18264,21 +18260,21 @@
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F497" t="n">
-        <v>0.258575197889182</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G497" t="n">
-        <v>0.1852861035422343</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18290,7 +18286,7 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
@@ -18300,19 +18296,21 @@
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.16</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2094240837696335</v>
-      </c>
-      <c r="G498" t="inlineStr"/>
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G498" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.1847 (0.0349)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -18324,31 +18322,27 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.196078431372549</v>
-      </c>
-      <c r="F499" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G499" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.3054187192118227</v>
+      </c>
+      <c r="F499" t="inlineStr"/>
+      <c r="G499" t="inlineStr"/>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.3054 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18360,7 +18354,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
@@ -18370,21 +18364,21 @@
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F500" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G500" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -18396,7 +18390,7 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
@@ -18406,21 +18400,19 @@
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.16</v>
       </c>
       <c r="F501" t="n">
-        <v>0.1746031746031746</v>
-      </c>
-      <c r="G501" t="n">
-        <v>0.125</v>
-      </c>
+        <v>0.2094240837696335</v>
+      </c>
+      <c r="G501" t="inlineStr"/>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.1847 (0.0349)</t>
         </is>
       </c>
     </row>
@@ -18437,7 +18429,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -18446,17 +18438,17 @@
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F502" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G502" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18473,7 +18465,7 @@
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -18482,17 +18474,17 @@
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F503" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G503" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -18504,31 +18496,31 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F504" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G504" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.125</v>
       </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -18540,31 +18532,31 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F505" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G505" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -18576,31 +18568,31 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F506" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G506" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -18617,7 +18609,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18626,17 +18618,17 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F507" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G507" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -18653,24 +18645,132 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E508" t="n">
+        <v>0.2087912087912088</v>
+      </c>
+      <c r="F508" t="n">
+        <v>0.2738095238095238</v>
+      </c>
+      <c r="G508" t="n">
+        <v>0.2705882352941176</v>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>0.2511 (0.0366)</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E509" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F509" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G509" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E510" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F510" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G510" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D508" t="inlineStr">
+      <c r="D511" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E508" t="n">
+      <c r="E511" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F508" t="n">
+      <c r="F511" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G508" t="n">
+      <c r="G511" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H508" t="inlineStr">
+      <c r="H511" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 21:43:49)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H511"/>
+  <dimension ref="A1:H513"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17916,17 +17916,13 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.3317535545023697</v>
-      </c>
-      <c r="F487" t="n">
-        <v>0.2831050228310502</v>
-      </c>
-      <c r="G487" t="n">
-        <v>0.3723404255319149</v>
-      </c>
+        <v>0.3047619047619048</v>
+      </c>
+      <c r="F487" t="inlineStr"/>
+      <c r="G487" t="inlineStr"/>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.3048 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17943,7 +17939,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17952,17 +17948,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F488" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G488" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
@@ -17979,7 +17975,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17988,13 +17984,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.3444976076555024</v>
-      </c>
-      <c r="F489" t="inlineStr"/>
-      <c r="G489" t="inlineStr"/>
+        <v>0.1818181818181818</v>
+      </c>
+      <c r="F489" t="n">
+        <v>0.2159090909090909</v>
+      </c>
+      <c r="G489" t="n">
+        <v>0.2413793103448276</v>
+      </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.3445 (0.0000)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
@@ -18011,7 +18011,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18020,49 +18020,49 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.225</v>
-      </c>
-      <c r="F490" t="inlineStr"/>
+        <v>0.3444976076555024</v>
+      </c>
+      <c r="F490" t="n">
+        <v>0.3265306122448979</v>
+      </c>
       <c r="G490" t="inlineStr"/>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.2250 (0.0000)</t>
+          <t>0.3355 (0.0127)</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.225</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2164948453608248</v>
-      </c>
-      <c r="G491" t="n">
-        <v>0.228310502283105</v>
-      </c>
+        <v>0.2281879194630873</v>
+      </c>
+      <c r="G491" t="inlineStr"/>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2266 (0.0023)</t>
         </is>
       </c>
     </row>
@@ -18079,7 +18079,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18088,17 +18088,17 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G492" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18115,7 +18115,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18124,17 +18124,17 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F493" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G493" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -18151,7 +18151,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -18160,17 +18160,17 @@
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F494" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G494" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -18187,7 +18187,7 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
@@ -18196,17 +18196,17 @@
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F495" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G495" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18218,27 +18218,31 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F496" t="inlineStr"/>
-      <c r="G496" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F496" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G496" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18255,7 +18259,7 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
@@ -18264,17 +18268,13 @@
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F497" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G497" t="n">
-        <v>0.2377622377622378</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F497" t="inlineStr"/>
+      <c r="G497" t="inlineStr"/>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18291,7 +18291,7 @@
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
@@ -18300,17 +18300,17 @@
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G498" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18327,7 +18327,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
@@ -18336,13 +18336,17 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.3054187192118227</v>
-      </c>
-      <c r="F499" t="inlineStr"/>
-      <c r="G499" t="inlineStr"/>
+        <v>0.163265306122449</v>
+      </c>
+      <c r="F499" t="n">
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G499" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.3054 (0.0000)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -18354,31 +18358,27 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.2747252747252747</v>
-      </c>
-      <c r="F500" t="n">
-        <v>0.258575197889182</v>
-      </c>
-      <c r="G500" t="n">
-        <v>0.1852861035422343</v>
-      </c>
+        <v>0.3054187192118227</v>
+      </c>
+      <c r="F500" t="inlineStr"/>
+      <c r="G500" t="inlineStr"/>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.3054 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18390,29 +18390,27 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="F501" t="n">
-        <v>0.2094240837696335</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F501" t="inlineStr"/>
       <c r="G501" t="inlineStr"/>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.1847 (0.0349)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18424,31 +18422,31 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F502" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G502" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -18460,31 +18458,29 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.16</v>
       </c>
       <c r="F503" t="n">
-        <v>0.2840909090909091</v>
-      </c>
-      <c r="G503" t="n">
-        <v>0.2153846153846154</v>
-      </c>
+        <v>0.2094240837696335</v>
+      </c>
+      <c r="G503" t="inlineStr"/>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1847 (0.0349)</t>
         </is>
       </c>
     </row>
@@ -18501,7 +18497,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
@@ -18510,17 +18506,17 @@
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F504" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G504" t="n">
-        <v>0.125</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18537,7 +18533,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -18546,17 +18542,17 @@
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F505" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G505" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -18573,7 +18569,7 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
@@ -18582,17 +18578,17 @@
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F506" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G506" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.125</v>
       </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -18604,31 +18600,31 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.232258064516129</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F507" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G507" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -18640,31 +18636,31 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F508" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G508" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -18681,7 +18677,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
@@ -18690,17 +18686,17 @@
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F509" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G509" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -18717,7 +18713,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -18726,17 +18722,17 @@
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G510" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18753,24 +18749,96 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E511" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F511" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G511" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E512" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F512" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G512" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D511" t="inlineStr">
+      <c r="D513" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E511" t="n">
+      <c r="E513" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F511" t="n">
+      <c r="F513" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G511" t="n">
+      <c r="G513" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H511" t="inlineStr">
+      <c r="H513" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 22:44:08)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H513"/>
+  <dimension ref="A1:H514"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17918,11 +17918,13 @@
       <c r="E487" t="n">
         <v>0.3047619047619048</v>
       </c>
-      <c r="F487" t="inlineStr"/>
+      <c r="F487" t="n">
+        <v>0.2727272727272727</v>
+      </c>
       <c r="G487" t="inlineStr"/>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.3048 (0.0000)</t>
+          <t>0.2887 (0.0227)</t>
         </is>
       </c>
     </row>
@@ -18025,10 +18027,12 @@
       <c r="F490" t="n">
         <v>0.3265306122448979</v>
       </c>
-      <c r="G490" t="inlineStr"/>
+      <c r="G490" t="n">
+        <v>0.3636363636363636</v>
+      </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.3355 (0.0127)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
@@ -18059,10 +18063,12 @@
       <c r="F491" t="n">
         <v>0.2281879194630873</v>
       </c>
-      <c r="G491" t="inlineStr"/>
+      <c r="G491" t="n">
+        <v>0.2676056338028169</v>
+      </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2266 (0.0023)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18477,10 +18483,12 @@
       <c r="F503" t="n">
         <v>0.2094240837696335</v>
       </c>
-      <c r="G503" t="inlineStr"/>
+      <c r="G503" t="n">
+        <v>0.1619047619047619</v>
+      </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.1847 (0.0349)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -18492,31 +18500,27 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.196078431372549</v>
-      </c>
-      <c r="F504" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G504" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.2641509433962264</v>
+      </c>
+      <c r="F504" t="inlineStr"/>
+      <c r="G504" t="inlineStr"/>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2642 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18533,7 +18537,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -18542,17 +18546,17 @@
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F505" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G505" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18569,7 +18573,7 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
@@ -18578,17 +18582,17 @@
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F506" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G506" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -18605,7 +18609,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18614,17 +18618,17 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F507" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G507" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -18641,7 +18645,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
@@ -18650,17 +18654,17 @@
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F508" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G508" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -18672,31 +18676,31 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F509" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G509" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -18713,7 +18717,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -18722,17 +18726,17 @@
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G510" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -18749,7 +18753,7 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
@@ -18758,17 +18762,17 @@
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F511" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G511" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18785,7 +18789,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -18794,17 +18798,17 @@
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F512" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G512" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -18821,24 +18825,60 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E513" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F513" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G513" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D513" t="inlineStr">
+      <c r="D514" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E513" t="n">
+      <c r="E514" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F513" t="n">
+      <c r="F514" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G513" t="n">
+      <c r="G514" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H513" t="inlineStr">
+      <c r="H514" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-05 23:44:28)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H514"/>
+  <dimension ref="A1:H517"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17722,31 +17722,27 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.2923076923076923</v>
-      </c>
-      <c r="F482" t="n">
-        <v>0.2844444444444444</v>
-      </c>
-      <c r="G482" t="n">
-        <v>0.2627737226277372</v>
-      </c>
+        <v>0.3497757847533632</v>
+      </c>
+      <c r="F482" t="inlineStr"/>
+      <c r="G482" t="inlineStr"/>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.3498 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17763,7 +17759,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
@@ -17772,17 +17768,17 @@
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F483" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G483" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -17799,7 +17795,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -17808,17 +17804,17 @@
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F484" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G484" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -17835,7 +17831,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17844,17 +17840,17 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F485" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G485" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -17871,7 +17867,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17880,17 +17876,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F486" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G486" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -17902,29 +17898,31 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F487" t="n">
-        <v>0.2727272727272727</v>
-      </c>
-      <c r="G487" t="inlineStr"/>
+        <v>0.1940298507462687</v>
+      </c>
+      <c r="G487" t="n">
+        <v>0.1774193548387097</v>
+      </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.2887 (0.0227)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -17941,7 +17939,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17950,17 +17948,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F488" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G488" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -17977,7 +17975,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17986,17 +17984,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G489" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
@@ -18013,7 +18011,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18022,17 +18020,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F490" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G490" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
@@ -18049,7 +18047,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18058,53 +18056,53 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.225</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G491" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.225</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G492" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18121,7 +18119,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18130,17 +18128,17 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F493" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G493" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18157,7 +18155,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -18166,17 +18164,17 @@
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F494" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G494" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -18193,7 +18191,7 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
@@ -18202,17 +18200,17 @@
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F495" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G495" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -18229,7 +18227,7 @@
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
@@ -18238,17 +18236,17 @@
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F496" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G496" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18260,27 +18258,31 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F497" t="inlineStr"/>
-      <c r="G497" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F497" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G497" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18297,7 +18299,7 @@
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
@@ -18306,17 +18308,13 @@
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F498" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G498" t="n">
-        <v>0.2377622377622378</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F498" t="inlineStr"/>
+      <c r="G498" t="inlineStr"/>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18333,7 +18331,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
@@ -18342,17 +18340,17 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F499" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G499" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18369,7 +18367,7 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
@@ -18378,13 +18376,17 @@
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.3054187192118227</v>
-      </c>
-      <c r="F500" t="inlineStr"/>
-      <c r="G500" t="inlineStr"/>
+        <v>0.163265306122449</v>
+      </c>
+      <c r="F500" t="n">
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G500" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.3054 (0.0000)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -18401,7 +18403,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
@@ -18410,13 +18412,13 @@
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.198581560283688</v>
+        <v>0.3054187192118227</v>
       </c>
       <c r="F501" t="inlineStr"/>
       <c r="G501" t="inlineStr"/>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.3054 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18428,31 +18430,27 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.2747252747252747</v>
-      </c>
-      <c r="F502" t="n">
-        <v>0.258575197889182</v>
-      </c>
-      <c r="G502" t="n">
-        <v>0.1852861035422343</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F502" t="inlineStr"/>
+      <c r="G502" t="inlineStr"/>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18469,7 +18467,7 @@
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -18478,17 +18476,13 @@
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="F503" t="n">
-        <v>0.2094240837696335</v>
-      </c>
-      <c r="G503" t="n">
-        <v>0.1619047619047619</v>
-      </c>
+        <v>0.2583025830258303</v>
+      </c>
+      <c r="F503" t="inlineStr"/>
+      <c r="G503" t="inlineStr"/>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.2583 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18505,7 +18499,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
@@ -18514,13 +18508,17 @@
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.2641509433962264</v>
-      </c>
-      <c r="F504" t="inlineStr"/>
-      <c r="G504" t="inlineStr"/>
+        <v>0.2747252747252747</v>
+      </c>
+      <c r="F504" t="n">
+        <v>0.258575197889182</v>
+      </c>
+      <c r="G504" t="n">
+        <v>0.1852861035422343</v>
+      </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.2642 (0.0000)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -18532,31 +18530,31 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.196078431372549</v>
+        <v>0.16</v>
       </c>
       <c r="F505" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2094240837696335</v>
       </c>
       <c r="G505" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.1619047619047619</v>
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -18568,31 +18566,27 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.2358974358974359</v>
-      </c>
-      <c r="F506" t="n">
-        <v>0.2840909090909091</v>
-      </c>
-      <c r="G506" t="n">
-        <v>0.2153846153846154</v>
-      </c>
+        <v>0.2575107296137339</v>
+      </c>
+      <c r="F506" t="inlineStr"/>
+      <c r="G506" t="inlineStr"/>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.2575 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18604,31 +18598,27 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.1714285714285714</v>
-      </c>
-      <c r="F507" t="n">
-        <v>0.1746031746031746</v>
-      </c>
-      <c r="G507" t="n">
-        <v>0.125</v>
-      </c>
+        <v>0.2641509433962264</v>
+      </c>
+      <c r="F507" t="inlineStr"/>
+      <c r="G507" t="inlineStr"/>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2642 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18645,7 +18635,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
@@ -18654,17 +18644,17 @@
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F508" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G508" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18681,7 +18671,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
@@ -18690,17 +18680,17 @@
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F509" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G509" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -18712,31 +18702,31 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G510" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.125</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -18748,31 +18738,31 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F511" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G511" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -18784,31 +18774,31 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F512" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G512" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -18825,7 +18815,7 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
@@ -18834,17 +18824,17 @@
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F513" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G513" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -18861,24 +18851,132 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E514" t="n">
+        <v>0.2087912087912088</v>
+      </c>
+      <c r="F514" t="n">
+        <v>0.2738095238095238</v>
+      </c>
+      <c r="G514" t="n">
+        <v>0.2705882352941176</v>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>0.2511 (0.0366)</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E515" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F515" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G515" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E516" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F516" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G516" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D514" t="inlineStr">
+      <c r="D517" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E514" t="n">
+      <c r="E517" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F514" t="n">
+      <c r="F517" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G514" t="n">
+      <c r="G517" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H514" t="inlineStr">
+      <c r="H517" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 00:44:45)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -17738,11 +17738,13 @@
       <c r="E482" t="n">
         <v>0.3497757847533632</v>
       </c>
-      <c r="F482" t="inlineStr"/>
+      <c r="F482" t="n">
+        <v>0.2918454935622318</v>
+      </c>
       <c r="G482" t="inlineStr"/>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.3498 (0.0000)</t>
+          <t>0.3208 (0.0410)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 01:45:01)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -17741,10 +17741,12 @@
       <c r="F482" t="n">
         <v>0.2918454935622318</v>
       </c>
-      <c r="G482" t="inlineStr"/>
+      <c r="G482" t="n">
+        <v>0.3255813953488372</v>
+      </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.3208 (0.0410)</t>
+          <t>0.3224 (0.0291)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 02:45:19)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H517"/>
+  <dimension ref="A1:H518"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17758,31 +17758,27 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.2923076923076923</v>
-      </c>
-      <c r="F483" t="n">
-        <v>0.2844444444444444</v>
-      </c>
-      <c r="G483" t="n">
-        <v>0.2627737226277372</v>
-      </c>
+        <v>0.2054054054054054</v>
+      </c>
+      <c r="F483" t="inlineStr"/>
+      <c r="G483" t="inlineStr"/>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.2054 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17799,7 +17795,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -17808,17 +17804,17 @@
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F484" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G484" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -17835,7 +17831,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17844,17 +17840,17 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F485" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G485" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -17871,7 +17867,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17880,17 +17876,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F486" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G486" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -17907,7 +17903,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17916,17 +17912,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F487" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G487" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -17938,31 +17934,31 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F488" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G488" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -17979,7 +17975,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17988,17 +17984,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G489" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -18015,7 +18011,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18024,17 +18020,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F490" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G490" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
@@ -18051,7 +18047,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18060,17 +18056,17 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F491" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G491" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
@@ -18087,7 +18083,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18096,53 +18092,53 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.225</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G492" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.225</v>
       </c>
       <c r="F493" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G493" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18159,7 +18155,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -18168,17 +18164,17 @@
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F494" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G494" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18195,7 +18191,7 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
@@ -18204,17 +18200,17 @@
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F495" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G495" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -18231,7 +18227,7 @@
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
@@ -18240,17 +18236,17 @@
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F496" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G496" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -18267,7 +18263,7 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
@@ -18276,17 +18272,17 @@
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F497" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G497" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18298,27 +18294,31 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F498" t="inlineStr"/>
-      <c r="G498" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F498" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G498" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18335,7 +18335,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
@@ -18344,17 +18344,13 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F499" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G499" t="n">
-        <v>0.2377622377622378</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F499" t="inlineStr"/>
+      <c r="G499" t="inlineStr"/>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18371,7 +18367,7 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
@@ -18380,17 +18376,17 @@
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F500" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G500" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18407,7 +18403,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
@@ -18416,13 +18412,17 @@
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.3054187192118227</v>
-      </c>
-      <c r="F501" t="inlineStr"/>
-      <c r="G501" t="inlineStr"/>
+        <v>0.163265306122449</v>
+      </c>
+      <c r="F501" t="n">
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G501" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.3054 (0.0000)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -18439,7 +18439,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -18448,13 +18448,13 @@
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.198581560283688</v>
+        <v>0.3054187192118227</v>
       </c>
       <c r="F502" t="inlineStr"/>
       <c r="G502" t="inlineStr"/>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.3054 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18466,27 +18466,27 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.2583025830258303</v>
+        <v>0.198581560283688</v>
       </c>
       <c r="F503" t="inlineStr"/>
       <c r="G503" t="inlineStr"/>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.2583 (0.0000)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18503,7 +18503,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
@@ -18512,17 +18512,13 @@
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.2747252747252747</v>
-      </c>
-      <c r="F504" t="n">
-        <v>0.258575197889182</v>
-      </c>
-      <c r="G504" t="n">
-        <v>0.1852861035422343</v>
-      </c>
+        <v>0.2583025830258303</v>
+      </c>
+      <c r="F504" t="inlineStr"/>
+      <c r="G504" t="inlineStr"/>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2583 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18539,7 +18535,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -18548,17 +18544,17 @@
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.16</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F505" t="n">
-        <v>0.2094240837696335</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G505" t="n">
-        <v>0.1619047619047619</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -18575,7 +18571,7 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
@@ -18584,13 +18580,17 @@
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.2575107296137339</v>
-      </c>
-      <c r="F506" t="inlineStr"/>
-      <c r="G506" t="inlineStr"/>
+        <v>0.16</v>
+      </c>
+      <c r="F506" t="n">
+        <v>0.2094240837696335</v>
+      </c>
+      <c r="G506" t="n">
+        <v>0.1619047619047619</v>
+      </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.2575 (0.0000)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -18607,7 +18607,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18616,13 +18616,13 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F507" t="inlineStr"/>
       <c r="G507" t="inlineStr"/>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2642 (0.0000)</t>
+          <t>0.2575 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18634,31 +18634,27 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.196078431372549</v>
-      </c>
-      <c r="F508" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G508" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.2641509433962264</v>
+      </c>
+      <c r="F508" t="inlineStr"/>
+      <c r="G508" t="inlineStr"/>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2642 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18675,7 +18671,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
@@ -18684,17 +18680,17 @@
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F509" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G509" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18711,7 +18707,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -18720,17 +18716,17 @@
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F510" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G510" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -18747,7 +18743,7 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
@@ -18756,17 +18752,17 @@
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F511" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G511" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -18783,7 +18779,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -18792,17 +18788,17 @@
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F512" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G512" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -18814,31 +18810,31 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F513" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G513" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -18855,7 +18851,7 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
@@ -18864,17 +18860,17 @@
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F514" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G514" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -18891,7 +18887,7 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
@@ -18900,17 +18896,17 @@
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F515" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G515" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18927,7 +18923,7 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
@@ -18936,17 +18932,17 @@
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F516" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G516" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -18963,24 +18959,60 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E517" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F517" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G517" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D517" t="inlineStr">
+      <c r="D518" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E517" t="n">
+      <c r="E518" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F517" t="n">
+      <c r="F518" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G517" t="n">
+      <c r="G518" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H517" t="inlineStr">
+      <c r="H518" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 04:45:55)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H518"/>
+  <dimension ref="A1:H519"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17790,31 +17790,31 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.2923076923076923</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="F484" t="n">
-        <v>0.2844444444444444</v>
+        <v>0.2972292191435768</v>
       </c>
       <c r="G484" t="n">
-        <v>0.2627737226277372</v>
+        <v>0.3169398907103825</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -17831,7 +17831,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17840,17 +17840,17 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F485" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G485" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -17867,7 +17867,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17876,17 +17876,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F486" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G486" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -17903,7 +17903,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17912,17 +17912,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F487" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G487" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -17939,7 +17939,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17948,17 +17948,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F488" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G488" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -17970,31 +17970,31 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G489" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -18011,7 +18011,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18020,17 +18020,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F490" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G490" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -18047,7 +18047,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18056,17 +18056,17 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G491" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
@@ -18083,7 +18083,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18092,17 +18092,17 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F492" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G492" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
@@ -18119,7 +18119,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18128,53 +18128,53 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.225</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F493" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G493" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.225</v>
       </c>
       <c r="F494" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G494" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18191,7 +18191,7 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
@@ -18200,17 +18200,17 @@
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F495" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G495" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
@@ -18236,17 +18236,17 @@
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F496" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G496" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -18263,7 +18263,7 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
@@ -18272,17 +18272,17 @@
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F497" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G497" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -18299,7 +18299,7 @@
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
@@ -18308,17 +18308,17 @@
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G498" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18330,27 +18330,31 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F499" t="inlineStr"/>
-      <c r="G499" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F499" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G499" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18367,7 +18371,7 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
@@ -18376,17 +18380,13 @@
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F500" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G500" t="n">
-        <v>0.2377622377622378</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F500" t="inlineStr"/>
+      <c r="G500" t="inlineStr"/>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18403,7 +18403,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
@@ -18412,17 +18412,17 @@
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F501" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G501" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18439,7 +18439,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -18448,13 +18448,17 @@
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.3054187192118227</v>
-      </c>
-      <c r="F502" t="inlineStr"/>
-      <c r="G502" t="inlineStr"/>
+        <v>0.163265306122449</v>
+      </c>
+      <c r="F502" t="n">
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G502" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.3054 (0.0000)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -18471,7 +18475,7 @@
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -18480,13 +18484,15 @@
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F503" t="inlineStr"/>
+        <v>0.3054187192118227</v>
+      </c>
+      <c r="F503" t="n">
+        <v>0.2517482517482518</v>
+      </c>
       <c r="G503" t="inlineStr"/>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -18498,27 +18504,27 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.2583025830258303</v>
+        <v>0.198581560283688</v>
       </c>
       <c r="F504" t="inlineStr"/>
       <c r="G504" t="inlineStr"/>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.2583 (0.0000)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18535,7 +18541,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -18544,17 +18550,13 @@
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2747252747252747</v>
-      </c>
-      <c r="F505" t="n">
-        <v>0.258575197889182</v>
-      </c>
-      <c r="G505" t="n">
-        <v>0.1852861035422343</v>
-      </c>
+        <v>0.2583025830258303</v>
+      </c>
+      <c r="F505" t="inlineStr"/>
+      <c r="G505" t="inlineStr"/>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2583 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18571,7 +18573,7 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
@@ -18580,17 +18582,17 @@
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.16</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F506" t="n">
-        <v>0.2094240837696335</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G506" t="n">
-        <v>0.1619047619047619</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -18607,7 +18609,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18616,13 +18618,17 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.2575107296137339</v>
-      </c>
-      <c r="F507" t="inlineStr"/>
-      <c r="G507" t="inlineStr"/>
+        <v>0.16</v>
+      </c>
+      <c r="F507" t="n">
+        <v>0.2094240837696335</v>
+      </c>
+      <c r="G507" t="n">
+        <v>0.1619047619047619</v>
+      </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2575 (0.0000)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -18639,7 +18645,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
@@ -18648,13 +18654,13 @@
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F508" t="inlineStr"/>
       <c r="G508" t="inlineStr"/>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.2642 (0.0000)</t>
+          <t>0.2575 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18666,31 +18672,27 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.196078431372549</v>
-      </c>
-      <c r="F509" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G509" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.2641509433962264</v>
+      </c>
+      <c r="F509" t="inlineStr"/>
+      <c r="G509" t="inlineStr"/>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2642 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18707,7 +18709,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -18716,17 +18718,17 @@
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G510" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18743,7 +18745,7 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
@@ -18752,17 +18754,17 @@
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F511" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G511" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -18779,7 +18781,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -18788,17 +18790,17 @@
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F512" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G512" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -18815,7 +18817,7 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
@@ -18824,17 +18826,17 @@
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F513" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G513" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -18846,31 +18848,31 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F514" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G514" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18889,7 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
@@ -18896,17 +18898,17 @@
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F515" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G515" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -18923,7 +18925,7 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
@@ -18932,17 +18934,17 @@
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F516" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G516" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18959,7 +18961,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
@@ -18968,17 +18970,17 @@
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F517" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G517" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -18995,24 +18997,60 @@
       </c>
       <c r="C518" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E518" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F518" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G518" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D518" t="inlineStr">
+      <c r="D519" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E518" t="n">
+      <c r="E519" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F518" t="n">
+      <c r="F519" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G518" t="n">
+      <c r="G519" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H518" t="inlineStr">
+      <c r="H519" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 05:46:15)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -18688,11 +18688,13 @@
       <c r="E509" t="n">
         <v>0.2641509433962264</v>
       </c>
-      <c r="F509" t="inlineStr"/>
+      <c r="F509" t="n">
+        <v>0.2566371681415929</v>
+      </c>
       <c r="G509" t="inlineStr"/>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.2642 (0.0000)</t>
+          <t>0.2604 (0.0053)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 06:46:34)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H519"/>
+  <dimension ref="A1:H520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17774,11 +17774,13 @@
       <c r="E483" t="n">
         <v>0.2054054054054054</v>
       </c>
-      <c r="F483" t="inlineStr"/>
+      <c r="F483" t="n">
+        <v>0.2408376963350785</v>
+      </c>
       <c r="G483" t="inlineStr"/>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.2054 (0.0000)</t>
+          <t>0.2231 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -17826,31 +17828,27 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.2923076923076923</v>
-      </c>
-      <c r="F485" t="n">
-        <v>0.2844444444444444</v>
-      </c>
-      <c r="G485" t="n">
-        <v>0.2627737226277372</v>
-      </c>
+        <v>0.2288135593220339</v>
+      </c>
+      <c r="F485" t="inlineStr"/>
+      <c r="G485" t="inlineStr"/>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.2288 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17867,7 +17865,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17876,17 +17874,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F486" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G486" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -17903,7 +17901,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17912,17 +17910,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F487" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G487" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -17939,7 +17937,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17948,17 +17946,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F488" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G488" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -17975,7 +17973,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17984,17 +17982,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F489" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G489" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18006,31 +18004,31 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F490" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G490" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -18047,7 +18045,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18056,17 +18054,17 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G491" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -18083,7 +18081,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18092,17 +18090,17 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G492" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
@@ -18119,7 +18117,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18128,17 +18126,17 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F493" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G493" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
@@ -18155,7 +18153,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -18164,53 +18162,53 @@
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.225</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F494" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G494" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.225</v>
       </c>
       <c r="F495" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G495" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18225,7 @@
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
@@ -18236,17 +18234,17 @@
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F496" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G496" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18263,7 +18261,7 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
@@ -18272,17 +18270,17 @@
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F497" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G497" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -18299,7 +18297,7 @@
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
@@ -18308,17 +18306,17 @@
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G498" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -18335,7 +18333,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
@@ -18344,17 +18342,17 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F499" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G499" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18366,27 +18364,31 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F500" t="inlineStr"/>
-      <c r="G500" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F500" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G500" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18403,7 +18405,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
@@ -18412,17 +18414,13 @@
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F501" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G501" t="n">
-        <v>0.2377622377622378</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F501" t="inlineStr"/>
+      <c r="G501" t="inlineStr"/>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18439,7 +18437,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -18448,17 +18446,17 @@
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F502" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G502" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18475,7 +18473,7 @@
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -18484,15 +18482,17 @@
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.3054187192118227</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F503" t="n">
-        <v>0.2517482517482518</v>
-      </c>
-      <c r="G503" t="inlineStr"/>
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G503" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -18509,7 +18509,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
@@ -18518,13 +18518,15 @@
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F504" t="inlineStr"/>
+        <v>0.3054187192118227</v>
+      </c>
+      <c r="F504" t="n">
+        <v>0.2517482517482518</v>
+      </c>
       <c r="G504" t="inlineStr"/>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -18536,27 +18538,27 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2583025830258303</v>
+        <v>0.198581560283688</v>
       </c>
       <c r="F505" t="inlineStr"/>
       <c r="G505" t="inlineStr"/>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2583 (0.0000)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18573,7 +18575,7 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
@@ -18582,17 +18584,15 @@
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F506" t="n">
-        <v>0.258575197889182</v>
-      </c>
-      <c r="G506" t="n">
-        <v>0.1852861035422343</v>
-      </c>
+        <v>0.2443438914027149</v>
+      </c>
+      <c r="G506" t="inlineStr"/>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2513 (0.0099)</t>
         </is>
       </c>
     </row>
@@ -18609,7 +18609,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18618,17 +18618,17 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.16</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F507" t="n">
-        <v>0.2094240837696335</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G507" t="n">
-        <v>0.1619047619047619</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -18645,7 +18645,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
@@ -18654,13 +18654,17 @@
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.2575107296137339</v>
-      </c>
-      <c r="F508" t="inlineStr"/>
-      <c r="G508" t="inlineStr"/>
+        <v>0.16</v>
+      </c>
+      <c r="F508" t="n">
+        <v>0.2094240837696335</v>
+      </c>
+      <c r="G508" t="n">
+        <v>0.1619047619047619</v>
+      </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.2575 (0.0000)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -18677,7 +18681,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
@@ -18686,15 +18690,15 @@
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F509" t="n">
-        <v>0.2566371681415929</v>
+        <v>0.2989690721649484</v>
       </c>
       <c r="G509" t="inlineStr"/>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.2604 (0.0053)</t>
+          <t>0.2782 (0.0293)</t>
         </is>
       </c>
     </row>
@@ -18706,31 +18710,29 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G510" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.2566371681415929</v>
+      </c>
+      <c r="G510" t="inlineStr"/>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2604 (0.0053)</t>
         </is>
       </c>
     </row>
@@ -18747,7 +18749,7 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
@@ -18756,17 +18758,17 @@
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F511" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G511" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18783,7 +18785,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -18792,17 +18794,17 @@
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F512" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G512" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -18819,7 +18821,7 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
@@ -18828,17 +18830,17 @@
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F513" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G513" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -18855,7 +18857,7 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
@@ -18864,17 +18866,17 @@
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F514" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G514" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -18886,31 +18888,31 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F515" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G515" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -18927,7 +18929,7 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
@@ -18936,17 +18938,17 @@
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F516" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G516" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -18963,7 +18965,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
@@ -18972,17 +18974,17 @@
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F517" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G517" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18999,7 +19001,7 @@
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
@@ -19008,17 +19010,17 @@
         </is>
       </c>
       <c r="E518" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F518" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G518" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -19035,24 +19037,60 @@
       </c>
       <c r="C519" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E519" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F519" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G519" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D519" t="inlineStr">
+      <c r="D520" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E519" t="n">
+      <c r="E520" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F519" t="n">
+      <c r="F520" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G519" t="n">
+      <c r="G520" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H519" t="inlineStr">
+      <c r="H520" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 08:47:09)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -17844,11 +17844,13 @@
       <c r="E485" t="n">
         <v>0.2288135593220339</v>
       </c>
-      <c r="F485" t="inlineStr"/>
+      <c r="F485" t="n">
+        <v>0.2433460076045627</v>
+      </c>
       <c r="G485" t="inlineStr"/>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.2288 (0.0000)</t>
+          <t>0.2361 (0.0103)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 09:47:27)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H520"/>
+  <dimension ref="A1:H521"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17792,31 +17792,27 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.2929292929292929</v>
-      </c>
-      <c r="F484" t="n">
-        <v>0.2972292191435768</v>
-      </c>
-      <c r="G484" t="n">
-        <v>0.3169398907103825</v>
-      </c>
+        <v>0.3643122676579926</v>
+      </c>
+      <c r="F484" t="inlineStr"/>
+      <c r="G484" t="inlineStr"/>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.3024 (0.0128)</t>
+          <t>0.3643 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17833,7 +17829,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17842,15 +17838,17 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="F485" t="n">
-        <v>0.2433460076045627</v>
-      </c>
-      <c r="G485" t="inlineStr"/>
+        <v>0.2972292191435768</v>
+      </c>
+      <c r="G485" t="n">
+        <v>0.3169398907103825</v>
+      </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.2361 (0.0103)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -17862,31 +17860,29 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.2923076923076923</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="F486" t="n">
-        <v>0.2844444444444444</v>
-      </c>
-      <c r="G486" t="n">
-        <v>0.2627737226277372</v>
-      </c>
+        <v>0.2433460076045627</v>
+      </c>
+      <c r="G486" t="inlineStr"/>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.2361 (0.0103)</t>
         </is>
       </c>
     </row>
@@ -17903,7 +17899,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17912,17 +17908,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F487" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G487" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -17939,7 +17935,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17948,17 +17944,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F488" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G488" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -17975,7 +17971,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17984,17 +17980,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F489" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G489" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -18011,7 +18007,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18020,17 +18016,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F490" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G490" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18042,31 +18038,31 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G491" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -18083,7 +18079,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18092,17 +18088,17 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G492" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -18119,7 +18115,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18128,17 +18124,17 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F493" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G493" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
@@ -18155,7 +18151,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -18164,17 +18160,17 @@
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F494" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G494" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
@@ -18191,7 +18187,7 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
@@ -18200,53 +18196,53 @@
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.225</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F495" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G495" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.225</v>
       </c>
       <c r="F496" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G496" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18263,7 +18259,7 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
@@ -18272,17 +18268,17 @@
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F497" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G497" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18299,7 +18295,7 @@
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
@@ -18308,17 +18304,17 @@
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G498" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -18335,7 +18331,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
@@ -18344,17 +18340,17 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F499" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G499" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -18371,7 +18367,7 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
@@ -18380,17 +18376,17 @@
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F500" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G500" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18402,27 +18398,31 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F501" t="inlineStr"/>
-      <c r="G501" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F501" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G501" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18439,7 +18439,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -18448,17 +18448,13 @@
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F502" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G502" t="n">
-        <v>0.2377622377622378</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F502" t="inlineStr"/>
+      <c r="G502" t="inlineStr"/>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18475,7 +18471,7 @@
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -18484,17 +18480,17 @@
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F503" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G503" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18511,7 +18507,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
@@ -18520,15 +18516,17 @@
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.3054187192118227</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F504" t="n">
-        <v>0.2517482517482518</v>
-      </c>
-      <c r="G504" t="inlineStr"/>
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G504" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -18545,7 +18543,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -18554,13 +18552,15 @@
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F505" t="inlineStr"/>
+        <v>0.3054187192118227</v>
+      </c>
+      <c r="F505" t="n">
+        <v>0.2517482517482518</v>
+      </c>
       <c r="G505" t="inlineStr"/>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -18572,29 +18572,27 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.2583025830258303</v>
-      </c>
-      <c r="F506" t="n">
-        <v>0.2443438914027149</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F506" t="inlineStr"/>
       <c r="G506" t="inlineStr"/>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.2513 (0.0099)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18611,7 +18609,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18620,17 +18618,15 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F507" t="n">
-        <v>0.258575197889182</v>
-      </c>
-      <c r="G507" t="n">
-        <v>0.1852861035422343</v>
-      </c>
+        <v>0.2443438914027149</v>
+      </c>
+      <c r="G507" t="inlineStr"/>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2513 (0.0099)</t>
         </is>
       </c>
     </row>
@@ -18647,7 +18643,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
@@ -18656,17 +18652,17 @@
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.16</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F508" t="n">
-        <v>0.2094240837696335</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G508" t="n">
-        <v>0.1619047619047619</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -18683,7 +18679,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
@@ -18692,15 +18688,17 @@
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.2575107296137339</v>
+        <v>0.16</v>
       </c>
       <c r="F509" t="n">
-        <v>0.2989690721649484</v>
-      </c>
-      <c r="G509" t="inlineStr"/>
+        <v>0.2094240837696335</v>
+      </c>
+      <c r="G509" t="n">
+        <v>0.1619047619047619</v>
+      </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.2782 (0.0293)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -18717,7 +18715,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -18726,15 +18724,15 @@
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2566371681415929</v>
+        <v>0.2989690721649484</v>
       </c>
       <c r="G510" t="inlineStr"/>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.2604 (0.0053)</t>
+          <t>0.2782 (0.0293)</t>
         </is>
       </c>
     </row>
@@ -18746,31 +18744,29 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F511" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G511" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.2566371681415929</v>
+      </c>
+      <c r="G511" t="inlineStr"/>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2604 (0.0053)</t>
         </is>
       </c>
     </row>
@@ -18787,7 +18783,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -18796,17 +18792,17 @@
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F512" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G512" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18823,7 +18819,7 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
@@ -18832,17 +18828,17 @@
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F513" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G513" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -18859,7 +18855,7 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
@@ -18868,17 +18864,17 @@
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F514" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G514" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -18895,7 +18891,7 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
@@ -18904,17 +18900,17 @@
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F515" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G515" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -18926,31 +18922,31 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F516" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G516" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -18967,7 +18963,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
@@ -18976,17 +18972,17 @@
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F517" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G517" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -19003,7 +18999,7 @@
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
@@ -19012,17 +19008,17 @@
         </is>
       </c>
       <c r="E518" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F518" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G518" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19039,7 +19035,7 @@
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
@@ -19048,17 +19044,17 @@
         </is>
       </c>
       <c r="E519" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F519" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G519" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -19075,24 +19071,60 @@
       </c>
       <c r="C520" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E520" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F520" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G520" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D520" t="inlineStr">
+      <c r="D521" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E520" t="n">
+      <c r="E521" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F520" t="n">
+      <c r="F521" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G520" t="n">
+      <c r="G521" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H520" t="inlineStr">
+      <c r="H521" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 10:47:47)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H521"/>
+  <dimension ref="A1:H523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17537,7 +17537,7 @@
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
@@ -17547,7 +17547,7 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
@@ -17556,24 +17556,24 @@
         </is>
       </c>
       <c r="E477" t="n">
-        <v>0.2534246575342466</v>
+        <v>0.4751131221719457</v>
       </c>
       <c r="F477" t="n">
-        <v>0.302788844621514</v>
+        <v>0.4267990074441687</v>
       </c>
       <c r="G477" t="n">
-        <v>0.2775510204081633</v>
+        <v>0.3903903903903904</v>
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>0.2779 (0.0247)</t>
+          <t>0.4308 (0.0425)</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B478" t="inlineStr">
@@ -17583,7 +17583,7 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
@@ -17592,17 +17592,13 @@
         </is>
       </c>
       <c r="E478" t="n">
-        <v>0.3181818181818182</v>
-      </c>
-      <c r="F478" t="n">
-        <v>0.3161764705882353</v>
-      </c>
-      <c r="G478" t="n">
-        <v>0.316205533596838</v>
-      </c>
+        <v>0.3535620052770448</v>
+      </c>
+      <c r="F478" t="inlineStr"/>
+      <c r="G478" t="inlineStr"/>
       <c r="H478" t="inlineStr">
         <is>
-          <t>0.3169 (0.0011)</t>
+          <t>0.3536 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17619,7 +17615,7 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
@@ -17628,17 +17624,17 @@
         </is>
       </c>
       <c r="E479" t="n">
-        <v>0.2290748898678414</v>
+        <v>0.2534246575342466</v>
       </c>
       <c r="F479" t="n">
-        <v>0.256198347107438</v>
+        <v>0.302788844621514</v>
       </c>
       <c r="G479" t="n">
-        <v>0.2629107981220657</v>
+        <v>0.2775510204081633</v>
       </c>
       <c r="H479" t="inlineStr">
         <is>
-          <t>0.2494 (0.0179)</t>
+          <t>0.2779 (0.0247)</t>
         </is>
       </c>
     </row>
@@ -17655,7 +17651,7 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
@@ -17664,17 +17660,17 @@
         </is>
       </c>
       <c r="E480" t="n">
-        <v>0.319327731092437</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F480" t="n">
-        <v>0.2845849802371542</v>
+        <v>0.3161764705882353</v>
       </c>
       <c r="G480" t="n">
-        <v>0.2331838565022422</v>
+        <v>0.316205533596838</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>0.2790 (0.0433)</t>
+          <t>0.3169 (0.0011)</t>
         </is>
       </c>
     </row>
@@ -17691,7 +17687,7 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
@@ -17700,17 +17696,17 @@
         </is>
       </c>
       <c r="E481" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.2290748898678414</v>
       </c>
       <c r="F481" t="n">
-        <v>0.2786885245901639</v>
+        <v>0.256198347107438</v>
       </c>
       <c r="G481" t="n">
-        <v>0.3665338645418327</v>
+        <v>0.2629107981220657</v>
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>0.3086 (0.0501)</t>
+          <t>0.2494 (0.0179)</t>
         </is>
       </c>
     </row>
@@ -17722,31 +17718,31 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.3497757847533632</v>
+        <v>0.319327731092437</v>
       </c>
       <c r="F482" t="n">
-        <v>0.2918454935622318</v>
+        <v>0.2845849802371542</v>
       </c>
       <c r="G482" t="n">
-        <v>0.3255813953488372</v>
+        <v>0.2331838565022422</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.3224 (0.0291)</t>
+          <t>0.2790 (0.0433)</t>
         </is>
       </c>
     </row>
@@ -17758,29 +17754,31 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.2054054054054054</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="F483" t="n">
-        <v>0.2408376963350785</v>
-      </c>
-      <c r="G483" t="inlineStr"/>
+        <v>0.2786885245901639</v>
+      </c>
+      <c r="G483" t="n">
+        <v>0.3665338645418327</v>
+      </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.2231 (0.0251)</t>
+          <t>0.3086 (0.0501)</t>
         </is>
       </c>
     </row>
@@ -17797,7 +17795,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -17806,13 +17804,17 @@
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.3643122676579926</v>
-      </c>
-      <c r="F484" t="inlineStr"/>
-      <c r="G484" t="inlineStr"/>
+        <v>0.3497757847533632</v>
+      </c>
+      <c r="F484" t="n">
+        <v>0.2918454935622318</v>
+      </c>
+      <c r="G484" t="n">
+        <v>0.3255813953488372</v>
+      </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.3643 (0.0000)</t>
+          <t>0.3224 (0.0291)</t>
         </is>
       </c>
     </row>
@@ -17824,31 +17826,31 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.2929292929292929</v>
+        <v>0.2054054054054054</v>
       </c>
       <c r="F485" t="n">
-        <v>0.2972292191435768</v>
+        <v>0.2408376963350785</v>
       </c>
       <c r="G485" t="n">
-        <v>0.3169398907103825</v>
+        <v>0.2346368715083799</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.3024 (0.0128)</t>
+          <t>0.2270 (0.0189)</t>
         </is>
       </c>
     </row>
@@ -17860,29 +17862,27 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.2288135593220339</v>
-      </c>
-      <c r="F486" t="n">
-        <v>0.2433460076045627</v>
-      </c>
+        <v>0.3643122676579926</v>
+      </c>
+      <c r="F486" t="inlineStr"/>
       <c r="G486" t="inlineStr"/>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.2361 (0.0103)</t>
+          <t>0.3643 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17894,31 +17894,31 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.2923076923076923</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="F487" t="n">
-        <v>0.2844444444444444</v>
+        <v>0.2972292191435768</v>
       </c>
       <c r="G487" t="n">
-        <v>0.2627737226277372</v>
+        <v>0.3169398907103825</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -17930,31 +17930,31 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="F488" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2433460076045627</v>
       </c>
       <c r="G488" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2704918032786885</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2476 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -17971,7 +17971,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17980,17 +17980,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G489" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -18007,7 +18007,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18016,17 +18016,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F490" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G490" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -18043,7 +18043,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18052,17 +18052,17 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F491" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G491" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -18074,31 +18074,31 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G492" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18110,31 +18110,31 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F493" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G493" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -18151,7 +18151,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -18160,17 +18160,17 @@
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F494" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G494" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -18187,7 +18187,7 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
@@ -18196,17 +18196,17 @@
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F495" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G495" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
@@ -18223,7 +18223,7 @@
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
@@ -18232,89 +18232,89 @@
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.225</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F496" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G496" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F497" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G497" t="n">
-        <v>0.228310502283105</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.225</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G498" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18331,7 +18331,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
@@ -18340,17 +18340,17 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F499" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G499" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18367,7 +18367,7 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
@@ -18376,17 +18376,17 @@
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F500" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G500" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -18403,7 +18403,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
@@ -18412,17 +18412,17 @@
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F501" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G501" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -18434,27 +18434,31 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F502" t="inlineStr"/>
-      <c r="G502" t="inlineStr"/>
+        <v>0.2683982683982684</v>
+      </c>
+      <c r="F502" t="n">
+        <v>0.2333333333333333</v>
+      </c>
+      <c r="G502" t="n">
+        <v>0.2046511627906977</v>
+      </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18466,31 +18470,31 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F503" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2383419689119171</v>
       </c>
       <c r="G503" t="n">
-        <v>0.2377622377622378</v>
+        <v>0.1940928270042194</v>
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18507,7 +18511,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
@@ -18516,17 +18520,13 @@
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.163265306122449</v>
-      </c>
-      <c r="F504" t="n">
-        <v>0.2027027027027027</v>
-      </c>
-      <c r="G504" t="n">
-        <v>0.2138364779874214</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F504" t="inlineStr"/>
+      <c r="G504" t="inlineStr"/>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18543,7 +18543,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -18552,15 +18552,17 @@
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.3054187192118227</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F505" t="n">
-        <v>0.2517482517482518</v>
-      </c>
-      <c r="G505" t="inlineStr"/>
+        <v>0.2592592592592592</v>
+      </c>
+      <c r="G505" t="n">
+        <v>0.2377622377622378</v>
+      </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18577,7 +18579,7 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
@@ -18586,13 +18588,17 @@
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F506" t="inlineStr"/>
-      <c r="G506" t="inlineStr"/>
+        <v>0.163265306122449</v>
+      </c>
+      <c r="F506" t="n">
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G506" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -18604,29 +18610,29 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.2583025830258303</v>
+        <v>0.3054187192118227</v>
       </c>
       <c r="F507" t="n">
-        <v>0.2443438914027149</v>
+        <v>0.2517482517482518</v>
       </c>
       <c r="G507" t="inlineStr"/>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2513 (0.0099)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -18638,31 +18644,27 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.2747252747252747</v>
-      </c>
-      <c r="F508" t="n">
-        <v>0.258575197889182</v>
-      </c>
-      <c r="G508" t="n">
-        <v>0.1852861035422343</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F508" t="inlineStr"/>
+      <c r="G508" t="inlineStr"/>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18679,7 +18681,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
@@ -18688,17 +18690,15 @@
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.16</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F509" t="n">
-        <v>0.2094240837696335</v>
-      </c>
-      <c r="G509" t="n">
-        <v>0.1619047619047619</v>
-      </c>
+        <v>0.2443438914027149</v>
+      </c>
+      <c r="G509" t="inlineStr"/>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.2513 (0.0099)</t>
         </is>
       </c>
     </row>
@@ -18715,7 +18715,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -18724,15 +18724,17 @@
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.2575107296137339</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2989690721649484</v>
-      </c>
-      <c r="G510" t="inlineStr"/>
+        <v>0.258575197889182</v>
+      </c>
+      <c r="G510" t="n">
+        <v>0.1852861035422343</v>
+      </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.2782 (0.0293)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -18749,7 +18751,7 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
@@ -18758,15 +18760,17 @@
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.16</v>
       </c>
       <c r="F511" t="n">
-        <v>0.2566371681415929</v>
-      </c>
-      <c r="G511" t="inlineStr"/>
+        <v>0.2094240837696335</v>
+      </c>
+      <c r="G511" t="n">
+        <v>0.1619047619047619</v>
+      </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.2604 (0.0053)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -18778,31 +18782,29 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F512" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G512" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.2989690721649484</v>
+      </c>
+      <c r="G512" t="inlineStr"/>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2782 (0.0293)</t>
         </is>
       </c>
     </row>
@@ -18814,31 +18816,29 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F513" t="n">
-        <v>0.2840909090909091</v>
-      </c>
-      <c r="G513" t="n">
-        <v>0.2153846153846154</v>
-      </c>
+        <v>0.2566371681415929</v>
+      </c>
+      <c r="G513" t="inlineStr"/>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.2604 (0.0053)</t>
         </is>
       </c>
     </row>
@@ -18855,7 +18855,7 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
@@ -18864,17 +18864,17 @@
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F514" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G514" t="n">
-        <v>0.125</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18891,7 +18891,7 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
@@ -18900,17 +18900,17 @@
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F515" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G515" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -18927,7 +18927,7 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
@@ -18936,17 +18936,17 @@
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F516" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G516" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.125</v>
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -18958,31 +18958,31 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.232258064516129</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F517" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G517" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -18994,31 +18994,31 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E518" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F518" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G518" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -19035,7 +19035,7 @@
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
@@ -19044,17 +19044,17 @@
         </is>
       </c>
       <c r="E519" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F519" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G519" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -19071,7 +19071,7 @@
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
@@ -19080,17 +19080,17 @@
         </is>
       </c>
       <c r="E520" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F520" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G520" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19107,24 +19107,96 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E521" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F521" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G521" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E522" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F522" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G522" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D521" t="inlineStr">
+      <c r="D523" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E521" t="n">
+      <c r="E523" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F521" t="n">
+      <c r="F523" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G521" t="n">
+      <c r="G523" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H521" t="inlineStr">
+      <c r="H523" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 11:48:07)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H523"/>
+  <dimension ref="A1:H526"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17594,18 +17594,22 @@
       <c r="E478" t="n">
         <v>0.3535620052770448</v>
       </c>
-      <c r="F478" t="inlineStr"/>
-      <c r="G478" t="inlineStr"/>
+      <c r="F478" t="n">
+        <v>0.3032069970845481</v>
+      </c>
+      <c r="G478" t="n">
+        <v>0.3243243243243243</v>
+      </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>0.3536 (0.0000)</t>
+          <t>0.3270 (0.0253)</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B479" t="inlineStr">
@@ -17615,7 +17619,7 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
@@ -17624,24 +17628,22 @@
         </is>
       </c>
       <c r="E479" t="n">
-        <v>0.2534246575342466</v>
+        <v>0.4926829268292683</v>
       </c>
       <c r="F479" t="n">
-        <v>0.302788844621514</v>
-      </c>
-      <c r="G479" t="n">
-        <v>0.2775510204081633</v>
-      </c>
+        <v>0.4011299435028249</v>
+      </c>
+      <c r="G479" t="inlineStr"/>
       <c r="H479" t="inlineStr">
         <is>
-          <t>0.2779 (0.0247)</t>
+          <t>0.4469 (0.0647)</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B480" t="inlineStr">
@@ -17651,7 +17653,7 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
@@ -17660,17 +17662,17 @@
         </is>
       </c>
       <c r="E480" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.4240963855421687</v>
       </c>
       <c r="F480" t="n">
-        <v>0.3161764705882353</v>
+        <v>0.3255813953488372</v>
       </c>
       <c r="G480" t="n">
-        <v>0.316205533596838</v>
+        <v>0.3312883435582822</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>0.3169 (0.0011)</t>
+          <t>0.3603 (0.0553)</t>
         </is>
       </c>
     </row>
@@ -17687,7 +17689,7 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
@@ -17696,17 +17698,17 @@
         </is>
       </c>
       <c r="E481" t="n">
-        <v>0.2290748898678414</v>
+        <v>0.2534246575342466</v>
       </c>
       <c r="F481" t="n">
-        <v>0.256198347107438</v>
+        <v>0.302788844621514</v>
       </c>
       <c r="G481" t="n">
-        <v>0.2629107981220657</v>
+        <v>0.2775510204081633</v>
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>0.2494 (0.0179)</t>
+          <t>0.2779 (0.0247)</t>
         </is>
       </c>
     </row>
@@ -17723,7 +17725,7 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
@@ -17732,17 +17734,17 @@
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.319327731092437</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F482" t="n">
-        <v>0.2845849802371542</v>
+        <v>0.3161764705882353</v>
       </c>
       <c r="G482" t="n">
-        <v>0.2331838565022422</v>
+        <v>0.316205533596838</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.2790 (0.0433)</t>
+          <t>0.3169 (0.0011)</t>
         </is>
       </c>
     </row>
@@ -17759,7 +17761,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
@@ -17768,17 +17770,17 @@
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.2290748898678414</v>
       </c>
       <c r="F483" t="n">
-        <v>0.2786885245901639</v>
+        <v>0.256198347107438</v>
       </c>
       <c r="G483" t="n">
-        <v>0.3665338645418327</v>
+        <v>0.2629107981220657</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.3086 (0.0501)</t>
+          <t>0.2494 (0.0179)</t>
         </is>
       </c>
     </row>
@@ -17790,31 +17792,31 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.3497757847533632</v>
+        <v>0.319327731092437</v>
       </c>
       <c r="F484" t="n">
-        <v>0.2918454935622318</v>
+        <v>0.2845849802371542</v>
       </c>
       <c r="G484" t="n">
-        <v>0.3255813953488372</v>
+        <v>0.2331838565022422</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.3224 (0.0291)</t>
+          <t>0.2790 (0.0433)</t>
         </is>
       </c>
     </row>
@@ -17826,31 +17828,31 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.2054054054054054</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="F485" t="n">
-        <v>0.2408376963350785</v>
+        <v>0.2786885245901639</v>
       </c>
       <c r="G485" t="n">
-        <v>0.2346368715083799</v>
+        <v>0.3665338645418327</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.2270 (0.0189)</t>
+          <t>0.3086 (0.0501)</t>
         </is>
       </c>
     </row>
@@ -17867,7 +17869,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17876,13 +17878,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.3643122676579926</v>
-      </c>
-      <c r="F486" t="inlineStr"/>
-      <c r="G486" t="inlineStr"/>
+        <v>0.3497757847533632</v>
+      </c>
+      <c r="F486" t="n">
+        <v>0.2918454935622318</v>
+      </c>
+      <c r="G486" t="n">
+        <v>0.3255813953488372</v>
+      </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.3643 (0.0000)</t>
+          <t>0.3224 (0.0291)</t>
         </is>
       </c>
     </row>
@@ -17894,31 +17900,31 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.2929292929292929</v>
+        <v>0.2054054054054054</v>
       </c>
       <c r="F487" t="n">
-        <v>0.2972292191435768</v>
+        <v>0.2408376963350785</v>
       </c>
       <c r="G487" t="n">
-        <v>0.3169398907103825</v>
+        <v>0.2346368715083799</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.3024 (0.0128)</t>
+          <t>0.2270 (0.0189)</t>
         </is>
       </c>
     </row>
@@ -17930,31 +17936,27 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.2288135593220339</v>
-      </c>
-      <c r="F488" t="n">
-        <v>0.2433460076045627</v>
-      </c>
-      <c r="G488" t="n">
-        <v>0.2704918032786885</v>
-      </c>
+        <v>0.3643122676579926</v>
+      </c>
+      <c r="F488" t="inlineStr"/>
+      <c r="G488" t="inlineStr"/>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.2476 (0.0212)</t>
+          <t>0.3643 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17966,31 +17968,31 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.2923076923076923</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2844444444444444</v>
+        <v>0.2972292191435768</v>
       </c>
       <c r="G489" t="n">
-        <v>0.2627737226277372</v>
+        <v>0.3169398907103825</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -18002,31 +18004,31 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="F490" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2433460076045627</v>
       </c>
       <c r="G490" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2704918032786885</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2476 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18038,31 +18040,27 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.1323529411764706</v>
-      </c>
-      <c r="F491" t="n">
-        <v>0.2051282051282051</v>
-      </c>
-      <c r="G491" t="n">
-        <v>0.2097902097902098</v>
-      </c>
+        <v>0.2222222222222222</v>
+      </c>
+      <c r="F491" t="inlineStr"/>
+      <c r="G491" t="inlineStr"/>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.2222 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18079,7 +18077,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18088,17 +18086,17 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F492" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G492" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -18115,7 +18113,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18124,17 +18122,17 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F493" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G493" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -18146,31 +18144,31 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F494" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G494" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -18182,31 +18180,31 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F495" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G495" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18218,31 +18216,31 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F496" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G496" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -18259,7 +18257,7 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
@@ -18268,17 +18266,17 @@
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F497" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G497" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -18295,7 +18293,7 @@
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
@@ -18304,125 +18302,125 @@
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.225</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G498" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F499" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G499" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F500" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G500" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.225</v>
       </c>
       <c r="F501" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G501" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18439,7 +18437,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -18448,17 +18446,17 @@
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F502" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G502" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18475,7 +18473,7 @@
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -18484,17 +18482,17 @@
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F503" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G503" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -18506,27 +18504,31 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F504" t="inlineStr"/>
-      <c r="G504" t="inlineStr"/>
+        <v>0.2135922330097087</v>
+      </c>
+      <c r="F504" t="n">
+        <v>0.2307692307692308</v>
+      </c>
+      <c r="G504" t="n">
+        <v>0.1616161616161616</v>
+      </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -18538,31 +18540,31 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F505" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G505" t="n">
-        <v>0.2377622377622378</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18574,31 +18576,31 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F506" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2383419689119171</v>
       </c>
       <c r="G506" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.1940928270042194</v>
       </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18615,7 +18617,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18624,15 +18626,13 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.3054187192118227</v>
-      </c>
-      <c r="F507" t="n">
-        <v>0.2517482517482518</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F507" t="inlineStr"/>
       <c r="G507" t="inlineStr"/>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18649,7 +18649,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
@@ -18658,13 +18658,17 @@
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F508" t="inlineStr"/>
-      <c r="G508" t="inlineStr"/>
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="F508" t="n">
+        <v>0.2592592592592592</v>
+      </c>
+      <c r="G508" t="n">
+        <v>0.2377622377622378</v>
+      </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18676,29 +18680,31 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.2583025830258303</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F509" t="n">
-        <v>0.2443438914027149</v>
-      </c>
-      <c r="G509" t="inlineStr"/>
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G509" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.2513 (0.0099)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -18710,31 +18716,29 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.3054187192118227</v>
       </c>
       <c r="F510" t="n">
-        <v>0.258575197889182</v>
-      </c>
-      <c r="G510" t="n">
-        <v>0.1852861035422343</v>
-      </c>
+        <v>0.2517482517482518</v>
+      </c>
+      <c r="G510" t="inlineStr"/>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -18746,31 +18750,27 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="F511" t="n">
-        <v>0.2094240837696335</v>
-      </c>
-      <c r="G511" t="n">
-        <v>0.1619047619047619</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F511" t="inlineStr"/>
+      <c r="G511" t="inlineStr"/>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18787,7 +18787,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -18796,15 +18796,15 @@
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.2575107296137339</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F512" t="n">
-        <v>0.2989690721649484</v>
+        <v>0.2443438914027149</v>
       </c>
       <c r="G512" t="inlineStr"/>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.2782 (0.0293)</t>
+          <t>0.2513 (0.0099)</t>
         </is>
       </c>
     </row>
@@ -18821,7 +18821,7 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
@@ -18830,15 +18830,17 @@
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F513" t="n">
-        <v>0.2566371681415929</v>
-      </c>
-      <c r="G513" t="inlineStr"/>
+        <v>0.258575197889182</v>
+      </c>
+      <c r="G513" t="n">
+        <v>0.1852861035422343</v>
+      </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.2604 (0.0053)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -18850,31 +18852,31 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.196078431372549</v>
+        <v>0.16</v>
       </c>
       <c r="F514" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2094240837696335</v>
       </c>
       <c r="G514" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.1619047619047619</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -18886,31 +18888,29 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F515" t="n">
-        <v>0.2840909090909091</v>
-      </c>
-      <c r="G515" t="n">
-        <v>0.2153846153846154</v>
-      </c>
+        <v>0.2989690721649484</v>
+      </c>
+      <c r="G515" t="inlineStr"/>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.2782 (0.0293)</t>
         </is>
       </c>
     </row>
@@ -18922,31 +18922,29 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F516" t="n">
-        <v>0.1746031746031746</v>
-      </c>
-      <c r="G516" t="n">
-        <v>0.125</v>
-      </c>
+        <v>0.2566371681415929</v>
+      </c>
+      <c r="G516" t="inlineStr"/>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2604 (0.0053)</t>
         </is>
       </c>
     </row>
@@ -18963,7 +18961,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
@@ -18972,17 +18970,17 @@
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F517" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G517" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -18999,7 +18997,7 @@
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
@@ -19008,17 +19006,17 @@
         </is>
       </c>
       <c r="E518" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F518" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G518" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -19030,31 +19028,31 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E519" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F519" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G519" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.125</v>
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -19066,31 +19064,31 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E520" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F520" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G520" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -19102,31 +19100,31 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E521" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F521" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G521" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -19143,7 +19141,7 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
@@ -19152,17 +19150,17 @@
         </is>
       </c>
       <c r="E522" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F522" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G522" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H522" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -19179,24 +19177,132 @@
       </c>
       <c r="C523" t="inlineStr">
         <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E523" t="n">
+        <v>0.2087912087912088</v>
+      </c>
+      <c r="F523" t="n">
+        <v>0.2738095238095238</v>
+      </c>
+      <c r="G523" t="n">
+        <v>0.2705882352941176</v>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>0.2511 (0.0366)</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E524" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F524" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G524" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E525" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F525" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G525" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D523" t="inlineStr">
+      <c r="D526" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E523" t="n">
+      <c r="E526" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F523" t="n">
+      <c r="F526" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G523" t="n">
+      <c r="G526" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H523" t="inlineStr">
+      <c r="H526" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 12:48:26)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H526"/>
+  <dimension ref="A1:H532"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17547,7 +17547,7 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
@@ -17556,17 +17556,17 @@
         </is>
       </c>
       <c r="E477" t="n">
-        <v>0.4751131221719457</v>
+        <v>0.462882096069869</v>
       </c>
       <c r="F477" t="n">
-        <v>0.4267990074441687</v>
+        <v>0.3654822335025381</v>
       </c>
       <c r="G477" t="n">
-        <v>0.3903903903903904</v>
+        <v>0.3314285714285714</v>
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>0.4308 (0.0425)</t>
+          <t>0.3866 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -17583,7 +17583,7 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
@@ -17592,17 +17592,17 @@
         </is>
       </c>
       <c r="E478" t="n">
-        <v>0.3535620052770448</v>
+        <v>0.4751131221719457</v>
       </c>
       <c r="F478" t="n">
-        <v>0.3032069970845481</v>
+        <v>0.4267990074441687</v>
       </c>
       <c r="G478" t="n">
-        <v>0.3243243243243243</v>
+        <v>0.3903903903903904</v>
       </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>0.3270 (0.0253)</t>
+          <t>0.4308 (0.0425)</t>
         </is>
       </c>
     </row>
@@ -17619,7 +17619,7 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
@@ -17628,15 +17628,17 @@
         </is>
       </c>
       <c r="E479" t="n">
-        <v>0.4926829268292683</v>
+        <v>0.3535620052770448</v>
       </c>
       <c r="F479" t="n">
-        <v>0.4011299435028249</v>
-      </c>
-      <c r="G479" t="inlineStr"/>
+        <v>0.3032069970845481</v>
+      </c>
+      <c r="G479" t="n">
+        <v>0.3243243243243243</v>
+      </c>
       <c r="H479" t="inlineStr">
         <is>
-          <t>0.4469 (0.0647)</t>
+          <t>0.3270 (0.0253)</t>
         </is>
       </c>
     </row>
@@ -17653,7 +17655,7 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
@@ -17662,24 +17664,24 @@
         </is>
       </c>
       <c r="E480" t="n">
-        <v>0.4240963855421687</v>
+        <v>0.4926829268292683</v>
       </c>
       <c r="F480" t="n">
-        <v>0.3255813953488372</v>
+        <v>0.4011299435028249</v>
       </c>
       <c r="G480" t="n">
-        <v>0.3312883435582822</v>
+        <v>0.3544303797468354</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>0.3603 (0.0553)</t>
+          <t>0.4161 (0.0703)</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B481" t="inlineStr">
@@ -17689,7 +17691,7 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
@@ -17698,29 +17700,29 @@
         </is>
       </c>
       <c r="E481" t="n">
-        <v>0.2534246575342466</v>
+        <v>0.4240963855421687</v>
       </c>
       <c r="F481" t="n">
-        <v>0.302788844621514</v>
+        <v>0.3255813953488372</v>
       </c>
       <c r="G481" t="n">
-        <v>0.2775510204081633</v>
+        <v>0.3312883435582822</v>
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>0.2779 (0.0247)</t>
+          <t>0.3603 (0.0553)</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
@@ -17730,33 +17732,33 @@
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.4822695035460993</v>
       </c>
       <c r="F482" t="n">
-        <v>0.3161764705882353</v>
+        <v>0.4904632152588556</v>
       </c>
       <c r="G482" t="n">
-        <v>0.316205533596838</v>
+        <v>0.4634920634920635</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.3169 (0.0011)</t>
+          <t>0.4787 (0.0138)</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
@@ -17766,33 +17768,33 @@
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.2290748898678414</v>
+        <v>0.4</v>
       </c>
       <c r="F483" t="n">
-        <v>0.256198347107438</v>
+        <v>0.3867069486404834</v>
       </c>
       <c r="G483" t="n">
-        <v>0.2629107981220657</v>
+        <v>0.3094339622641509</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.2494 (0.0179)</t>
+          <t>0.3654 (0.0489)</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
@@ -17802,33 +17804,31 @@
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.319327731092437</v>
+        <v>0.5801217038539553</v>
       </c>
       <c r="F484" t="n">
-        <v>0.2845849802371542</v>
-      </c>
-      <c r="G484" t="n">
-        <v>0.2331838565022422</v>
-      </c>
+        <v>0.5185185185185185</v>
+      </c>
+      <c r="G484" t="inlineStr"/>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.2790 (0.0433)</t>
+          <t>0.5493 (0.0436)</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
@@ -17838,21 +17838,19 @@
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.4698795180722892</v>
       </c>
       <c r="F485" t="n">
-        <v>0.2786885245901639</v>
-      </c>
-      <c r="G485" t="n">
-        <v>0.3665338645418327</v>
-      </c>
+        <v>0.303030303030303</v>
+      </c>
+      <c r="G485" t="inlineStr"/>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.3086 (0.0501)</t>
+          <t>0.3865 (0.1180)</t>
         </is>
       </c>
     </row>
@@ -17864,31 +17862,31 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.3497757847533632</v>
+        <v>0.2534246575342466</v>
       </c>
       <c r="F486" t="n">
-        <v>0.2918454935622318</v>
+        <v>0.302788844621514</v>
       </c>
       <c r="G486" t="n">
-        <v>0.3255813953488372</v>
+        <v>0.2775510204081633</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.3224 (0.0291)</t>
+          <t>0.2779 (0.0247)</t>
         </is>
       </c>
     </row>
@@ -17900,31 +17898,31 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.2054054054054054</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F487" t="n">
-        <v>0.2408376963350785</v>
+        <v>0.3161764705882353</v>
       </c>
       <c r="G487" t="n">
-        <v>0.2346368715083799</v>
+        <v>0.316205533596838</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.2270 (0.0189)</t>
+          <t>0.3169 (0.0011)</t>
         </is>
       </c>
     </row>
@@ -17936,27 +17934,31 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.3643122676579926</v>
-      </c>
-      <c r="F488" t="inlineStr"/>
-      <c r="G488" t="inlineStr"/>
+        <v>0.2290748898678414</v>
+      </c>
+      <c r="F488" t="n">
+        <v>0.256198347107438</v>
+      </c>
+      <c r="G488" t="n">
+        <v>0.2629107981220657</v>
+      </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.3643 (0.0000)</t>
+          <t>0.2494 (0.0179)</t>
         </is>
       </c>
     </row>
@@ -17968,31 +17970,31 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.2929292929292929</v>
+        <v>0.319327731092437</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2972292191435768</v>
+        <v>0.2845849802371542</v>
       </c>
       <c r="G489" t="n">
-        <v>0.3169398907103825</v>
+        <v>0.2331838565022422</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.3024 (0.0128)</t>
+          <t>0.2790 (0.0433)</t>
         </is>
       </c>
     </row>
@@ -18004,31 +18006,31 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.2807017543859649</v>
       </c>
       <c r="F490" t="n">
-        <v>0.2433460076045627</v>
+        <v>0.2786885245901639</v>
       </c>
       <c r="G490" t="n">
-        <v>0.2704918032786885</v>
+        <v>0.3665338645418327</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.2476 (0.0212)</t>
+          <t>0.3086 (0.0501)</t>
         </is>
       </c>
     </row>
@@ -18040,27 +18042,31 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.2222222222222222</v>
-      </c>
-      <c r="F491" t="inlineStr"/>
-      <c r="G491" t="inlineStr"/>
+        <v>0.3497757847533632</v>
+      </c>
+      <c r="F491" t="n">
+        <v>0.2918454935622318</v>
+      </c>
+      <c r="G491" t="n">
+        <v>0.3255813953488372</v>
+      </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2222 (0.0000)</t>
+          <t>0.3224 (0.0291)</t>
         </is>
       </c>
     </row>
@@ -18072,31 +18078,31 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.2923076923076923</v>
+        <v>0.2054054054054054</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2844444444444444</v>
+        <v>0.2408376963350785</v>
       </c>
       <c r="G492" t="n">
-        <v>0.2627737226277372</v>
+        <v>0.2346368715083799</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.2270 (0.0189)</t>
         </is>
       </c>
     </row>
@@ -18108,31 +18114,27 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.3396226415094339</v>
-      </c>
-      <c r="F493" t="n">
-        <v>0.2450980392156863</v>
-      </c>
-      <c r="G493" t="n">
-        <v>0.3775510204081632</v>
-      </c>
+        <v>0.3643122676579926</v>
+      </c>
+      <c r="F493" t="inlineStr"/>
+      <c r="G493" t="inlineStr"/>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.3643 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18144,31 +18146,31 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="F494" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2972292191435768</v>
       </c>
       <c r="G494" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.3169398907103825</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -18180,31 +18182,31 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="F495" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2433460076045627</v>
       </c>
       <c r="G495" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2704918032786885</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.2476 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18216,31 +18218,27 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.2266666666666667</v>
-      </c>
-      <c r="F496" t="n">
-        <v>0.1940298507462687</v>
-      </c>
-      <c r="G496" t="n">
-        <v>0.1774193548387097</v>
-      </c>
+        <v>0.3179916317991632</v>
+      </c>
+      <c r="F496" t="inlineStr"/>
+      <c r="G496" t="inlineStr"/>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3180 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18252,31 +18250,27 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.3047619047619048</v>
-      </c>
-      <c r="F497" t="n">
-        <v>0.2727272727272727</v>
-      </c>
-      <c r="G497" t="n">
-        <v>0.2482758620689655</v>
-      </c>
+        <v>0.2222222222222222</v>
+      </c>
+      <c r="F497" t="inlineStr"/>
+      <c r="G497" t="inlineStr"/>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.2222 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18288,31 +18282,31 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G498" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -18324,31 +18318,31 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F499" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G499" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -18360,31 +18354,31 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F500" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G500" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -18396,243 +18390,247 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.225</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F501" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G501" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F502" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G502" t="n">
-        <v>0.228310502283105</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F503" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G503" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F504" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G504" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F505" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G505" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F506" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G506" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F507" t="inlineStr"/>
-      <c r="G507" t="inlineStr"/>
+        <v>0.225</v>
+      </c>
+      <c r="F507" t="n">
+        <v>0.2281879194630873</v>
+      </c>
+      <c r="G507" t="n">
+        <v>0.2676056338028169</v>
+      </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18644,31 +18642,31 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F508" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G508" t="n">
-        <v>0.2377622377622378</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18680,31 +18678,31 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F509" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G509" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -18716,29 +18714,31 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.3054187192118227</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2517482517482518</v>
-      </c>
-      <c r="G510" t="inlineStr"/>
+        <v>0.2307692307692308</v>
+      </c>
+      <c r="G510" t="n">
+        <v>0.1616161616161616</v>
+      </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -18750,27 +18750,31 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F511" t="inlineStr"/>
-      <c r="G511" t="inlineStr"/>
+        <v>0.2683982683982684</v>
+      </c>
+      <c r="F511" t="n">
+        <v>0.2333333333333333</v>
+      </c>
+      <c r="G511" t="n">
+        <v>0.2046511627906977</v>
+      </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18782,29 +18786,31 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.2583025830258303</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F512" t="n">
-        <v>0.2443438914027149</v>
-      </c>
-      <c r="G512" t="inlineStr"/>
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G512" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.2513 (0.0099)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18816,31 +18822,27 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.2747252747252747</v>
-      </c>
-      <c r="F513" t="n">
-        <v>0.258575197889182</v>
-      </c>
-      <c r="G513" t="n">
-        <v>0.1852861035422343</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F513" t="inlineStr"/>
+      <c r="G513" t="inlineStr"/>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18852,31 +18854,31 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.16</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F514" t="n">
-        <v>0.2094240837696335</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G514" t="n">
-        <v>0.1619047619047619</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18888,29 +18890,31 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.2575107296137339</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F515" t="n">
-        <v>0.2989690721649484</v>
-      </c>
-      <c r="G515" t="inlineStr"/>
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G515" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.2782 (0.0293)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -18922,29 +18926,29 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.3054187192118227</v>
       </c>
       <c r="F516" t="n">
-        <v>0.2566371681415929</v>
+        <v>0.2517482517482518</v>
       </c>
       <c r="G516" t="inlineStr"/>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.2604 (0.0053)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -18956,31 +18960,27 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.196078431372549</v>
-      </c>
-      <c r="F517" t="n">
-        <v>0.2166666666666667</v>
-      </c>
-      <c r="G517" t="n">
-        <v>0.1379310344827586</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F517" t="inlineStr"/>
+      <c r="G517" t="inlineStr"/>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18992,31 +18992,29 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E518" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F518" t="n">
-        <v>0.2840909090909091</v>
-      </c>
-      <c r="G518" t="n">
-        <v>0.2153846153846154</v>
-      </c>
+        <v>0.2443438914027149</v>
+      </c>
+      <c r="G518" t="inlineStr"/>
       <c r="H518" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.2513 (0.0099)</t>
         </is>
       </c>
     </row>
@@ -19028,31 +19026,31 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E519" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F519" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G519" t="n">
-        <v>0.125</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -19064,31 +19062,31 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E520" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.16</v>
       </c>
       <c r="F520" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.2094240837696335</v>
       </c>
       <c r="G520" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.1619047619047619</v>
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -19100,31 +19098,31 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E521" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F521" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.2989690721649484</v>
       </c>
       <c r="G521" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2825 (0.0220)</t>
         </is>
       </c>
     </row>
@@ -19136,31 +19134,31 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E522" t="n">
-        <v>0.232258064516129</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F522" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.2566371681415929</v>
       </c>
       <c r="G522" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.2551020408163265</v>
       </c>
       <c r="H522" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.2586 (0.0048)</t>
         </is>
       </c>
     </row>
@@ -19172,31 +19170,31 @@
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E523" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F523" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G523" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H523" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -19208,31 +19206,31 @@
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E524" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F524" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G524" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H524" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -19244,31 +19242,31 @@
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E525" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F525" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G525" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.125</v>
       </c>
       <c r="H525" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -19280,29 +19278,245 @@
       </c>
       <c r="B526" t="inlineStr">
         <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E526" t="n">
+        <v>0.3370786516853932</v>
+      </c>
+      <c r="F526" t="n">
+        <v>0.3091787439613526</v>
+      </c>
+      <c r="G526" t="n">
+        <v>0.1438848920863309</v>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>0.2634 (0.1044)</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E527" t="n">
+        <v>0.1940298507462687</v>
+      </c>
+      <c r="F527" t="n">
+        <v>0.1481481481481481</v>
+      </c>
+      <c r="G527" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>0.1585 (0.0316)</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
           <t>xgb</t>
         </is>
       </c>
-      <c r="C526" t="inlineStr">
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E528" t="n">
+        <v>0.232258064516129</v>
+      </c>
+      <c r="F528" t="n">
+        <v>0.2385321100917431</v>
+      </c>
+      <c r="G528" t="n">
+        <v>0.2131147540983606</v>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>0.2280 (0.0132)</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E529" t="n">
+        <v>0.2087912087912088</v>
+      </c>
+      <c r="F529" t="n">
+        <v>0.2738095238095238</v>
+      </c>
+      <c r="G529" t="n">
+        <v>0.2705882352941176</v>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>0.2511 (0.0366)</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E530" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F530" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G530" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E531" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F531" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G531" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
         <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D526" t="inlineStr">
+      <c r="D532" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E526" t="n">
+      <c r="E532" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F526" t="n">
+      <c r="F532" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G526" t="n">
+      <c r="G532" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H526" t="inlineStr">
+      <c r="H532" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 13:48:45)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H532"/>
+  <dimension ref="A1:H535"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17727,7 +17727,7 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
@@ -17736,17 +17736,17 @@
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.4822695035460993</v>
+        <v>0.5080831408775982</v>
       </c>
       <c r="F482" t="n">
-        <v>0.4904632152588556</v>
+        <v>0.4013605442176871</v>
       </c>
       <c r="G482" t="n">
-        <v>0.4634920634920635</v>
+        <v>0.4327176781002638</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.4787 (0.0138)</t>
+          <t>0.4474 (0.0549)</t>
         </is>
       </c>
     </row>
@@ -17763,7 +17763,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
@@ -17772,17 +17772,17 @@
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.4</v>
+        <v>0.4822695035460993</v>
       </c>
       <c r="F483" t="n">
-        <v>0.3867069486404834</v>
+        <v>0.4904632152588556</v>
       </c>
       <c r="G483" t="n">
-        <v>0.3094339622641509</v>
+        <v>0.4634920634920635</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.3654 (0.0489)</t>
+          <t>0.4787 (0.0138)</t>
         </is>
       </c>
     </row>
@@ -17799,7 +17799,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -17808,15 +17808,17 @@
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.5801217038539553</v>
+        <v>0.4</v>
       </c>
       <c r="F484" t="n">
-        <v>0.5185185185185185</v>
-      </c>
-      <c r="G484" t="inlineStr"/>
+        <v>0.3867069486404834</v>
+      </c>
+      <c r="G484" t="n">
+        <v>0.3094339622641509</v>
+      </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.5493 (0.0436)</t>
+          <t>0.3654 (0.0489)</t>
         </is>
       </c>
     </row>
@@ -17833,7 +17835,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17842,63 +17844,65 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.4698795180722892</v>
+        <v>0.5801217038539553</v>
       </c>
       <c r="F485" t="n">
-        <v>0.303030303030303</v>
-      </c>
-      <c r="G485" t="inlineStr"/>
+        <v>0.5185185185185185</v>
+      </c>
+      <c r="G485" t="n">
+        <v>0.5128205128205128</v>
+      </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.3865 (0.1180)</t>
+          <t>0.5372 (0.0373)</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.2534246575342466</v>
+        <v>0.4698795180722892</v>
       </c>
       <c r="F486" t="n">
-        <v>0.302788844621514</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G486" t="n">
-        <v>0.2775510204081633</v>
+        <v>0.3675213675213675</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.2779 (0.0247)</t>
+          <t>0.3801 (0.0841)</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
@@ -17908,33 +17912,33 @@
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.4839506172839506</v>
       </c>
       <c r="F487" t="n">
-        <v>0.3161764705882353</v>
+        <v>0.4502923976608187</v>
       </c>
       <c r="G487" t="n">
-        <v>0.316205533596838</v>
+        <v>0.4224422442244224</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.3169 (0.0011)</t>
+          <t>0.4522 (0.0308)</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
@@ -17944,21 +17948,19 @@
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.2290748898678414</v>
+        <v>0.3735632183908046</v>
       </c>
       <c r="F488" t="n">
-        <v>0.256198347107438</v>
-      </c>
-      <c r="G488" t="n">
-        <v>0.2629107981220657</v>
-      </c>
+        <v>0.397212543554007</v>
+      </c>
+      <c r="G488" t="inlineStr"/>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.2494 (0.0179)</t>
+          <t>0.3854 (0.0167)</t>
         </is>
       </c>
     </row>
@@ -17975,7 +17977,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17984,17 +17986,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.319327731092437</v>
+        <v>0.2534246575342466</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2845849802371542</v>
+        <v>0.302788844621514</v>
       </c>
       <c r="G489" t="n">
-        <v>0.2331838565022422</v>
+        <v>0.2775510204081633</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.2790 (0.0433)</t>
+          <t>0.2779 (0.0247)</t>
         </is>
       </c>
     </row>
@@ -18011,7 +18013,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18020,17 +18022,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F490" t="n">
-        <v>0.2786885245901639</v>
+        <v>0.3161764705882353</v>
       </c>
       <c r="G490" t="n">
-        <v>0.3665338645418327</v>
+        <v>0.316205533596838</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.3086 (0.0501)</t>
+          <t>0.3169 (0.0011)</t>
         </is>
       </c>
     </row>
@@ -18042,31 +18044,31 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.3497757847533632</v>
+        <v>0.2290748898678414</v>
       </c>
       <c r="F491" t="n">
-        <v>0.2918454935622318</v>
+        <v>0.256198347107438</v>
       </c>
       <c r="G491" t="n">
-        <v>0.3255813953488372</v>
+        <v>0.2629107981220657</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.3224 (0.0291)</t>
+          <t>0.2494 (0.0179)</t>
         </is>
       </c>
     </row>
@@ -18078,31 +18080,31 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.2054054054054054</v>
+        <v>0.319327731092437</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2408376963350785</v>
+        <v>0.2845849802371542</v>
       </c>
       <c r="G492" t="n">
-        <v>0.2346368715083799</v>
+        <v>0.2331838565022422</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2270 (0.0189)</t>
+          <t>0.2790 (0.0433)</t>
         </is>
       </c>
     </row>
@@ -18114,27 +18116,31 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.3643122676579926</v>
-      </c>
-      <c r="F493" t="inlineStr"/>
-      <c r="G493" t="inlineStr"/>
+        <v>0.2807017543859649</v>
+      </c>
+      <c r="F493" t="n">
+        <v>0.2786885245901639</v>
+      </c>
+      <c r="G493" t="n">
+        <v>0.3665338645418327</v>
+      </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.3643 (0.0000)</t>
+          <t>0.3086 (0.0501)</t>
         </is>
       </c>
     </row>
@@ -18146,7 +18152,7 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
@@ -18156,21 +18162,21 @@
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.2929292929292929</v>
+        <v>0.3497757847533632</v>
       </c>
       <c r="F494" t="n">
-        <v>0.2972292191435768</v>
+        <v>0.2918454935622318</v>
       </c>
       <c r="G494" t="n">
-        <v>0.3169398907103825</v>
+        <v>0.3255813953488372</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.3024 (0.0128)</t>
+          <t>0.3224 (0.0291)</t>
         </is>
       </c>
     </row>
@@ -18182,7 +18188,7 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
@@ -18192,21 +18198,21 @@
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.2054054054054054</v>
       </c>
       <c r="F495" t="n">
-        <v>0.2433460076045627</v>
+        <v>0.2408376963350785</v>
       </c>
       <c r="G495" t="n">
-        <v>0.2704918032786885</v>
+        <v>0.2346368715083799</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2476 (0.0212)</t>
+          <t>0.2270 (0.0189)</t>
         </is>
       </c>
     </row>
@@ -18218,7 +18224,7 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
@@ -18228,17 +18234,17 @@
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.3179916317991632</v>
+        <v>0.3643122676579926</v>
       </c>
       <c r="F496" t="inlineStr"/>
       <c r="G496" t="inlineStr"/>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.3180 (0.0000)</t>
+          <t>0.3643 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18255,7 +18261,7 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
@@ -18264,13 +18270,17 @@
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2222222222222222</v>
-      </c>
-      <c r="F497" t="inlineStr"/>
-      <c r="G497" t="inlineStr"/>
+        <v>0.2929292929292929</v>
+      </c>
+      <c r="F497" t="n">
+        <v>0.2972292191435768</v>
+      </c>
+      <c r="G497" t="n">
+        <v>0.3169398907103825</v>
+      </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2222 (0.0000)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -18282,31 +18292,31 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2923076923076923</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2844444444444444</v>
+        <v>0.2433460076045627</v>
       </c>
       <c r="G498" t="n">
-        <v>0.2627737226277372</v>
+        <v>0.2704918032786885</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.2476 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18318,31 +18328,27 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.3396226415094339</v>
-      </c>
-      <c r="F499" t="n">
-        <v>0.2450980392156863</v>
-      </c>
-      <c r="G499" t="n">
-        <v>0.3775510204081632</v>
-      </c>
+        <v>0.3179916317991632</v>
+      </c>
+      <c r="F499" t="inlineStr"/>
+      <c r="G499" t="inlineStr"/>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.3180 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18354,31 +18360,27 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.1323529411764706</v>
-      </c>
-      <c r="F500" t="n">
-        <v>0.2051282051282051</v>
-      </c>
-      <c r="G500" t="n">
-        <v>0.2097902097902098</v>
-      </c>
+        <v>0.2222222222222222</v>
+      </c>
+      <c r="F500" t="inlineStr"/>
+      <c r="G500" t="inlineStr"/>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.2222 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18395,7 +18397,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
@@ -18404,17 +18406,17 @@
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F501" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G501" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -18431,7 +18433,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -18440,17 +18442,17 @@
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F502" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G502" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -18462,31 +18464,31 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F503" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G503" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -18498,31 +18500,31 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F504" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G504" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18534,31 +18536,31 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F505" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G505" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -18575,7 +18577,7 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
@@ -18584,17 +18586,17 @@
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F506" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G506" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -18611,7 +18613,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18620,125 +18622,125 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.225</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F507" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G507" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F508" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G508" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F509" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G509" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.225</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G510" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18755,7 +18757,7 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
@@ -18764,17 +18766,17 @@
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F511" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G511" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18791,7 +18793,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -18800,17 +18802,17 @@
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F512" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G512" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -18822,27 +18824,31 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F513" t="inlineStr"/>
-      <c r="G513" t="inlineStr"/>
+        <v>0.2135922330097087</v>
+      </c>
+      <c r="F513" t="n">
+        <v>0.2307692307692308</v>
+      </c>
+      <c r="G513" t="n">
+        <v>0.1616161616161616</v>
+      </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -18854,31 +18860,31 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F514" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G514" t="n">
-        <v>0.2377622377622378</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -18890,31 +18896,31 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F515" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2383419689119171</v>
       </c>
       <c r="G515" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.1940928270042194</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -18931,7 +18937,7 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
@@ -18940,15 +18946,13 @@
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.3054187192118227</v>
-      </c>
-      <c r="F516" t="n">
-        <v>0.2517482517482518</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F516" t="inlineStr"/>
       <c r="G516" t="inlineStr"/>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18965,7 +18969,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
@@ -18974,13 +18978,17 @@
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F517" t="inlineStr"/>
-      <c r="G517" t="inlineStr"/>
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="F517" t="n">
+        <v>0.2592592592592592</v>
+      </c>
+      <c r="G517" t="n">
+        <v>0.2377622377622378</v>
+      </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -18992,29 +19000,31 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E518" t="n">
-        <v>0.2583025830258303</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F518" t="n">
-        <v>0.2443438914027149</v>
-      </c>
-      <c r="G518" t="inlineStr"/>
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G518" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>0.2513 (0.0099)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -19026,31 +19036,29 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E519" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.3054187192118227</v>
       </c>
       <c r="F519" t="n">
-        <v>0.258575197889182</v>
-      </c>
-      <c r="G519" t="n">
-        <v>0.1852861035422343</v>
-      </c>
+        <v>0.2517482517482518</v>
+      </c>
+      <c r="G519" t="inlineStr"/>
       <c r="H519" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -19062,31 +19070,27 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E520" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="F520" t="n">
-        <v>0.2094240837696335</v>
-      </c>
-      <c r="G520" t="n">
-        <v>0.1619047619047619</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F520" t="inlineStr"/>
+      <c r="G520" t="inlineStr"/>
       <c r="H520" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19103,7 +19107,7 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
@@ -19112,17 +19116,17 @@
         </is>
       </c>
       <c r="E521" t="n">
-        <v>0.2575107296137339</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F521" t="n">
-        <v>0.2989690721649484</v>
+        <v>0.2443438914027149</v>
       </c>
       <c r="G521" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.2191780821917808</v>
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>0.2825 (0.0220)</t>
+          <t>0.2406 (0.0198)</t>
         </is>
       </c>
     </row>
@@ -19139,7 +19143,7 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
@@ -19148,17 +19152,17 @@
         </is>
       </c>
       <c r="E522" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F522" t="n">
-        <v>0.2566371681415929</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G522" t="n">
-        <v>0.2551020408163265</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H522" t="inlineStr">
         <is>
-          <t>0.2586 (0.0048)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -19170,31 +19174,31 @@
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E523" t="n">
-        <v>0.196078431372549</v>
+        <v>0.16</v>
       </c>
       <c r="F523" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2094240837696335</v>
       </c>
       <c r="G523" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.1619047619047619</v>
       </c>
       <c r="H523" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -19206,31 +19210,31 @@
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E524" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F524" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2989690721649484</v>
       </c>
       <c r="G524" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H524" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.2825 (0.0220)</t>
         </is>
       </c>
     </row>
@@ -19242,31 +19246,31 @@
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E525" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F525" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2566371681415929</v>
       </c>
       <c r="G525" t="n">
-        <v>0.125</v>
+        <v>0.2551020408163265</v>
       </c>
       <c r="H525" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2586 (0.0048)</t>
         </is>
       </c>
     </row>
@@ -19283,7 +19287,7 @@
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
@@ -19292,17 +19296,17 @@
         </is>
       </c>
       <c r="E526" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F526" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G526" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H526" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -19319,7 +19323,7 @@
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
@@ -19328,17 +19332,17 @@
         </is>
       </c>
       <c r="E527" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F527" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G527" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H527" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -19350,31 +19354,31 @@
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E528" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F528" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G528" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.125</v>
       </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -19386,31 +19390,31 @@
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E529" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F529" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G529" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H529" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -19422,31 +19426,31 @@
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E530" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F530" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G530" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -19463,7 +19467,7 @@
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D531" t="inlineStr">
@@ -19472,17 +19476,17 @@
         </is>
       </c>
       <c r="E531" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F531" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G531" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H531" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -19499,24 +19503,132 @@
       </c>
       <c r="C532" t="inlineStr">
         <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E532" t="n">
+        <v>0.2087912087912088</v>
+      </c>
+      <c r="F532" t="n">
+        <v>0.2738095238095238</v>
+      </c>
+      <c r="G532" t="n">
+        <v>0.2705882352941176</v>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>0.2511 (0.0366)</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E533" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F533" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G533" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E534" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F534" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G534" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D532" t="inlineStr">
+      <c r="D535" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E532" t="n">
+      <c r="E535" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F532" t="n">
+      <c r="F535" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G532" t="n">
+      <c r="G535" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H532" t="inlineStr">
+      <c r="H535" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 14:49:04)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H535"/>
+  <dimension ref="A1:H540"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17916,17 +17916,13 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.4839506172839506</v>
-      </c>
-      <c r="F487" t="n">
-        <v>0.4502923976608187</v>
-      </c>
-      <c r="G487" t="n">
-        <v>0.4224422442244224</v>
-      </c>
+        <v>0.4855769230769231</v>
+      </c>
+      <c r="F487" t="inlineStr"/>
+      <c r="G487" t="inlineStr"/>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.4522 (0.0308)</t>
+          <t>0.4856 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17943,7 +17939,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17952,123 +17948,117 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.3735632183908046</v>
+        <v>0.4839506172839506</v>
       </c>
       <c r="F488" t="n">
-        <v>0.397212543554007</v>
-      </c>
-      <c r="G488" t="inlineStr"/>
+        <v>0.4502923976608187</v>
+      </c>
+      <c r="G488" t="n">
+        <v>0.4224422442244224</v>
+      </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.3854 (0.0167)</t>
+          <t>0.4522 (0.0308)</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.2534246575342466</v>
+        <v>0.3735632183908046</v>
       </c>
       <c r="F489" t="n">
-        <v>0.302788844621514</v>
+        <v>0.397212543554007</v>
       </c>
       <c r="G489" t="n">
-        <v>0.2775510204081633</v>
+        <v>0.3764705882352941</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.2779 (0.0247)</t>
+          <t>0.3824 (0.0129)</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.3181818181818182</v>
-      </c>
-      <c r="F490" t="n">
-        <v>0.3161764705882353</v>
-      </c>
-      <c r="G490" t="n">
-        <v>0.316205533596838</v>
-      </c>
+        <v>0.5320197044334976</v>
+      </c>
+      <c r="F490" t="inlineStr"/>
+      <c r="G490" t="inlineStr"/>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.3169 (0.0011)</t>
+          <t>0.5320 (0.0000)</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.2290748898678414</v>
-      </c>
-      <c r="F491" t="n">
-        <v>0.256198347107438</v>
-      </c>
-      <c r="G491" t="n">
-        <v>0.2629107981220657</v>
-      </c>
+        <v>0.417989417989418</v>
+      </c>
+      <c r="F491" t="inlineStr"/>
+      <c r="G491" t="inlineStr"/>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.2494 (0.0179)</t>
+          <t>0.4180 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18085,7 +18075,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18094,17 +18084,17 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.319327731092437</v>
+        <v>0.2534246575342466</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2845849802371542</v>
+        <v>0.302788844621514</v>
       </c>
       <c r="G492" t="n">
-        <v>0.2331838565022422</v>
+        <v>0.2775510204081633</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2790 (0.0433)</t>
+          <t>0.2779 (0.0247)</t>
         </is>
       </c>
     </row>
@@ -18121,7 +18111,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18130,17 +18120,17 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F493" t="n">
-        <v>0.2786885245901639</v>
+        <v>0.3161764705882353</v>
       </c>
       <c r="G493" t="n">
-        <v>0.3665338645418327</v>
+        <v>0.316205533596838</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.3086 (0.0501)</t>
+          <t>0.3169 (0.0011)</t>
         </is>
       </c>
     </row>
@@ -18152,31 +18142,31 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.3497757847533632</v>
+        <v>0.2290748898678414</v>
       </c>
       <c r="F494" t="n">
-        <v>0.2918454935622318</v>
+        <v>0.256198347107438</v>
       </c>
       <c r="G494" t="n">
-        <v>0.3255813953488372</v>
+        <v>0.2629107981220657</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.3224 (0.0291)</t>
+          <t>0.2494 (0.0179)</t>
         </is>
       </c>
     </row>
@@ -18188,31 +18178,31 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.2054054054054054</v>
+        <v>0.319327731092437</v>
       </c>
       <c r="F495" t="n">
-        <v>0.2408376963350785</v>
+        <v>0.2845849802371542</v>
       </c>
       <c r="G495" t="n">
-        <v>0.2346368715083799</v>
+        <v>0.2331838565022422</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2270 (0.0189)</t>
+          <t>0.2790 (0.0433)</t>
         </is>
       </c>
     </row>
@@ -18224,27 +18214,31 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.3643122676579926</v>
-      </c>
-      <c r="F496" t="inlineStr"/>
-      <c r="G496" t="inlineStr"/>
+        <v>0.2807017543859649</v>
+      </c>
+      <c r="F496" t="n">
+        <v>0.2786885245901639</v>
+      </c>
+      <c r="G496" t="n">
+        <v>0.3665338645418327</v>
+      </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.3643 (0.0000)</t>
+          <t>0.3086 (0.0501)</t>
         </is>
       </c>
     </row>
@@ -18256,31 +18250,27 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2929292929292929</v>
-      </c>
-      <c r="F497" t="n">
-        <v>0.2972292191435768</v>
-      </c>
-      <c r="G497" t="n">
-        <v>0.3169398907103825</v>
-      </c>
+        <v>0.2788461538461539</v>
+      </c>
+      <c r="F497" t="inlineStr"/>
+      <c r="G497" t="inlineStr"/>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.3024 (0.0128)</t>
+          <t>0.2788 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18292,31 +18282,31 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.3497757847533632</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2433460076045627</v>
+        <v>0.2918454935622318</v>
       </c>
       <c r="G498" t="n">
-        <v>0.2704918032786885</v>
+        <v>0.3255813953488372</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2476 (0.0212)</t>
+          <t>0.3224 (0.0291)</t>
         </is>
       </c>
     </row>
@@ -18328,27 +18318,31 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.3179916317991632</v>
-      </c>
-      <c r="F499" t="inlineStr"/>
-      <c r="G499" t="inlineStr"/>
+        <v>0.2054054054054054</v>
+      </c>
+      <c r="F499" t="n">
+        <v>0.2408376963350785</v>
+      </c>
+      <c r="G499" t="n">
+        <v>0.2346368715083799</v>
+      </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.3180 (0.0000)</t>
+          <t>0.2270 (0.0189)</t>
         </is>
       </c>
     </row>
@@ -18360,27 +18354,27 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.3643122676579926</v>
       </c>
       <c r="F500" t="inlineStr"/>
       <c r="G500" t="inlineStr"/>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.2222 (0.0000)</t>
+          <t>0.3643 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18392,31 +18386,27 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.2923076923076923</v>
-      </c>
-      <c r="F501" t="n">
-        <v>0.2844444444444444</v>
-      </c>
-      <c r="G501" t="n">
-        <v>0.2627737226277372</v>
-      </c>
+        <v>0.2650602409638554</v>
+      </c>
+      <c r="F501" t="inlineStr"/>
+      <c r="G501" t="inlineStr"/>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.2651 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18428,7 +18418,7 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
@@ -18438,21 +18428,21 @@
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="F502" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2972292191435768</v>
       </c>
       <c r="G502" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.3169398907103825</v>
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -18464,7 +18454,7 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
@@ -18474,21 +18464,21 @@
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="F503" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2433460076045627</v>
       </c>
       <c r="G503" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.2704918032786885</v>
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.2476 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18500,7 +18490,7 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
@@ -18510,21 +18500,17 @@
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.4054054054054054</v>
-      </c>
-      <c r="F504" t="n">
-        <v>0.362962962962963</v>
-      </c>
-      <c r="G504" t="n">
-        <v>0.3852459016393442</v>
-      </c>
+        <v>0.3179916317991632</v>
+      </c>
+      <c r="F504" t="inlineStr"/>
+      <c r="G504" t="inlineStr"/>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.3180 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18536,7 +18522,7 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
@@ -18546,21 +18532,17 @@
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2266666666666667</v>
-      </c>
-      <c r="F505" t="n">
-        <v>0.1940298507462687</v>
-      </c>
-      <c r="G505" t="n">
-        <v>0.1774193548387097</v>
-      </c>
+        <v>0.2222222222222222</v>
+      </c>
+      <c r="F505" t="inlineStr"/>
+      <c r="G505" t="inlineStr"/>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.2222 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18572,7 +18554,7 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
@@ -18582,21 +18564,21 @@
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F506" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G506" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18590,7 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
@@ -18618,21 +18600,21 @@
       </c>
       <c r="D507" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F507" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G507" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -18644,7 +18626,7 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
@@ -18654,21 +18636,21 @@
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F508" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G508" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -18680,7 +18662,7 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
@@ -18690,21 +18672,21 @@
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F509" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G509" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18716,7 +18698,7 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
@@ -18726,33 +18708,33 @@
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.225</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G510" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
@@ -18762,33 +18744,33 @@
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F511" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G511" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
@@ -18798,33 +18780,33 @@
       </c>
       <c r="D512" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F512" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G512" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
@@ -18834,33 +18816,33 @@
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F513" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G513" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
@@ -18870,33 +18852,33 @@
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F514" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G514" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
@@ -18906,21 +18888,21 @@
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.225</v>
       </c>
       <c r="F515" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G515" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18932,7 +18914,7 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
@@ -18942,17 +18924,21 @@
       </c>
       <c r="D516" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F516" t="inlineStr"/>
-      <c r="G516" t="inlineStr"/>
+        <v>0.2595419847328244</v>
+      </c>
+      <c r="F516" t="n">
+        <v>0.2164948453608248</v>
+      </c>
+      <c r="G516" t="n">
+        <v>0.228310502283105</v>
+      </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18964,7 +18950,7 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
@@ -18974,21 +18960,21 @@
       </c>
       <c r="D517" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F517" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G517" t="n">
-        <v>0.2377622377622378</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -19000,7 +18986,7 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
@@ -19010,21 +18996,21 @@
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E518" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F518" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G518" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -19036,7 +19022,7 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
@@ -19046,19 +19032,21 @@
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E519" t="n">
-        <v>0.3054187192118227</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F519" t="n">
-        <v>0.2517482517482518</v>
-      </c>
-      <c r="G519" t="inlineStr"/>
+        <v>0.2333333333333333</v>
+      </c>
+      <c r="G519" t="n">
+        <v>0.2046511627906977</v>
+      </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -19070,7 +19058,7 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
@@ -19080,17 +19068,21 @@
       </c>
       <c r="D520" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E520" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F520" t="inlineStr"/>
-      <c r="G520" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F520" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G520" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19102,7 +19094,7 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
@@ -19112,21 +19104,17 @@
       </c>
       <c r="D521" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E521" t="n">
-        <v>0.2583025830258303</v>
-      </c>
-      <c r="F521" t="n">
-        <v>0.2443438914027149</v>
-      </c>
-      <c r="G521" t="n">
-        <v>0.2191780821917808</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F521" t="inlineStr"/>
+      <c r="G521" t="inlineStr"/>
       <c r="H521" t="inlineStr">
         <is>
-          <t>0.2406 (0.0198)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19138,7 +19126,7 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
@@ -19148,21 +19136,21 @@
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E522" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F522" t="n">
-        <v>0.258575197889182</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G522" t="n">
-        <v>0.1852861035422343</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H522" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -19174,7 +19162,7 @@
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
@@ -19184,21 +19172,21 @@
       </c>
       <c r="D523" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E523" t="n">
-        <v>0.16</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F523" t="n">
-        <v>0.2094240837696335</v>
+        <v>0.2027027027027027</v>
       </c>
       <c r="G523" t="n">
-        <v>0.1619047619047619</v>
+        <v>0.2138364779874214</v>
       </c>
       <c r="H523" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -19210,7 +19198,7 @@
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
@@ -19220,21 +19208,19 @@
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E524" t="n">
-        <v>0.2575107296137339</v>
+        <v>0.3054187192118227</v>
       </c>
       <c r="F524" t="n">
-        <v>0.2989690721649484</v>
-      </c>
-      <c r="G524" t="n">
-        <v>0.2909090909090909</v>
-      </c>
+        <v>0.2517482517482518</v>
+      </c>
+      <c r="G524" t="inlineStr"/>
       <c r="H524" t="inlineStr">
         <is>
-          <t>0.2825 (0.0220)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -19246,7 +19232,7 @@
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
@@ -19256,21 +19242,17 @@
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E525" t="n">
-        <v>0.2641509433962264</v>
-      </c>
-      <c r="F525" t="n">
-        <v>0.2566371681415929</v>
-      </c>
-      <c r="G525" t="n">
-        <v>0.2551020408163265</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F525" t="inlineStr"/>
+      <c r="G525" t="inlineStr"/>
       <c r="H525" t="inlineStr">
         <is>
-          <t>0.2586 (0.0048)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19282,7 +19264,7 @@
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
@@ -19292,21 +19274,21 @@
       </c>
       <c r="D526" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E526" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F526" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2443438914027149</v>
       </c>
       <c r="G526" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.2191780821917808</v>
       </c>
       <c r="H526" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2406 (0.0198)</t>
         </is>
       </c>
     </row>
@@ -19318,7 +19300,7 @@
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
@@ -19328,21 +19310,21 @@
       </c>
       <c r="D527" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E527" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F527" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G527" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H527" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -19354,7 +19336,7 @@
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
@@ -19364,21 +19346,21 @@
       </c>
       <c r="D528" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E528" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.16</v>
       </c>
       <c r="F528" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2094240837696335</v>
       </c>
       <c r="G528" t="n">
-        <v>0.125</v>
+        <v>0.1619047619047619</v>
       </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -19390,7 +19372,7 @@
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C529" t="inlineStr">
@@ -19400,21 +19382,21 @@
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E529" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F529" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.2989690721649484</v>
       </c>
       <c r="G529" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H529" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.2825 (0.0220)</t>
         </is>
       </c>
     </row>
@@ -19426,7 +19408,7 @@
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C530" t="inlineStr">
@@ -19436,21 +19418,21 @@
       </c>
       <c r="D530" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E530" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F530" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.2566371681415929</v>
       </c>
       <c r="G530" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.2551020408163265</v>
       </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2586 (0.0048)</t>
         </is>
       </c>
     </row>
@@ -19462,7 +19444,7 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
@@ -19472,21 +19454,21 @@
       </c>
       <c r="D531" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E531" t="n">
-        <v>0.232258064516129</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F531" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G531" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H531" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19480,7 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C532" t="inlineStr">
@@ -19508,21 +19490,21 @@
       </c>
       <c r="D532" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E532" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F532" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G532" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -19534,7 +19516,7 @@
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C533" t="inlineStr">
@@ -19544,21 +19526,21 @@
       </c>
       <c r="D533" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E533" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F533" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G533" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.125</v>
       </c>
       <c r="H533" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -19570,7 +19552,7 @@
       </c>
       <c r="B534" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C534" t="inlineStr">
@@ -19580,21 +19562,21 @@
       </c>
       <c r="D534" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E534" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F534" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G534" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H534" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -19606,29 +19588,209 @@
       </c>
       <c r="B535" t="inlineStr">
         <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>RDKit</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="E535" t="n">
+        <v>0.1940298507462687</v>
+      </c>
+      <c r="F535" t="n">
+        <v>0.1481481481481481</v>
+      </c>
+      <c r="G535" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>0.1585 (0.0316)</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
           <t>xgb</t>
         </is>
       </c>
-      <c r="C535" t="inlineStr">
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Layered</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E536" t="n">
+        <v>0.232258064516129</v>
+      </c>
+      <c r="F536" t="n">
+        <v>0.2385321100917431</v>
+      </c>
+      <c r="G536" t="n">
+        <v>0.2131147540983606</v>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>0.2280 (0.0132)</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E537" t="n">
+        <v>0.2087912087912088</v>
+      </c>
+      <c r="F537" t="n">
+        <v>0.2738095238095238</v>
+      </c>
+      <c r="G537" t="n">
+        <v>0.2705882352941176</v>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>0.2511 (0.0366)</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E538" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F538" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G538" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E539" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F539" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G539" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
         <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D535" t="inlineStr">
+      <c r="D540" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E535" t="n">
+      <c r="E540" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F535" t="n">
+      <c r="F540" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G535" t="n">
+      <c r="G540" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H535" t="inlineStr">
+      <c r="H540" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 15:49:23)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H540"/>
+  <dimension ref="A1:H541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17722,31 +17722,27 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E482" t="n">
-        <v>0.5080831408775982</v>
-      </c>
-      <c r="F482" t="n">
-        <v>0.4013605442176871</v>
-      </c>
-      <c r="G482" t="n">
-        <v>0.4327176781002638</v>
-      </c>
+        <v>0.4901960784313725</v>
+      </c>
+      <c r="F482" t="inlineStr"/>
+      <c r="G482" t="inlineStr"/>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.4474 (0.0549)</t>
+          <t>0.4902 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17763,7 +17759,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
@@ -17772,17 +17768,17 @@
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.4822695035460993</v>
+        <v>0.5080831408775982</v>
       </c>
       <c r="F483" t="n">
-        <v>0.4904632152588556</v>
+        <v>0.4013605442176871</v>
       </c>
       <c r="G483" t="n">
-        <v>0.4634920634920635</v>
+        <v>0.4327176781002638</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.4787 (0.0138)</t>
+          <t>0.4474 (0.0549)</t>
         </is>
       </c>
     </row>
@@ -17799,7 +17795,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -17808,17 +17804,17 @@
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.4</v>
+        <v>0.4822695035460993</v>
       </c>
       <c r="F484" t="n">
-        <v>0.3867069486404834</v>
+        <v>0.4904632152588556</v>
       </c>
       <c r="G484" t="n">
-        <v>0.3094339622641509</v>
+        <v>0.4634920634920635</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.3654 (0.0489)</t>
+          <t>0.4787 (0.0138)</t>
         </is>
       </c>
     </row>
@@ -17835,7 +17831,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17844,17 +17840,17 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.5801217038539553</v>
+        <v>0.4</v>
       </c>
       <c r="F485" t="n">
-        <v>0.5185185185185185</v>
+        <v>0.3867069486404834</v>
       </c>
       <c r="G485" t="n">
-        <v>0.5128205128205128</v>
+        <v>0.3094339622641509</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.5372 (0.0373)</t>
+          <t>0.3654 (0.0489)</t>
         </is>
       </c>
     </row>
@@ -17871,7 +17867,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17880,17 +17876,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.4698795180722892</v>
+        <v>0.5801217038539553</v>
       </c>
       <c r="F486" t="n">
-        <v>0.303030303030303</v>
+        <v>0.5185185185185185</v>
       </c>
       <c r="G486" t="n">
-        <v>0.3675213675213675</v>
+        <v>0.5128205128205128</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.3801 (0.0841)</t>
+          <t>0.5372 (0.0373)</t>
         </is>
       </c>
     </row>
@@ -17902,27 +17898,31 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.4855769230769231</v>
-      </c>
-      <c r="F487" t="inlineStr"/>
-      <c r="G487" t="inlineStr"/>
+        <v>0.4698795180722892</v>
+      </c>
+      <c r="F487" t="n">
+        <v>0.303030303030303</v>
+      </c>
+      <c r="G487" t="n">
+        <v>0.3675213675213675</v>
+      </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.4856 (0.0000)</t>
+          <t>0.3801 (0.0841)</t>
         </is>
       </c>
     </row>
@@ -17939,7 +17939,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17948,17 +17948,15 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.4839506172839506</v>
+        <v>0.4855769230769231</v>
       </c>
       <c r="F488" t="n">
-        <v>0.4502923976608187</v>
-      </c>
-      <c r="G488" t="n">
-        <v>0.4224422442244224</v>
-      </c>
+        <v>0.4187725631768953</v>
+      </c>
+      <c r="G488" t="inlineStr"/>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.4522 (0.0308)</t>
+          <t>0.4522 (0.0472)</t>
         </is>
       </c>
     </row>
@@ -17975,7 +17973,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17984,17 +17982,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.3735632183908046</v>
+        <v>0.4839506172839506</v>
       </c>
       <c r="F489" t="n">
-        <v>0.397212543554007</v>
+        <v>0.4502923976608187</v>
       </c>
       <c r="G489" t="n">
-        <v>0.3764705882352941</v>
+        <v>0.4224422442244224</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.3824 (0.0129)</t>
+          <t>0.4522 (0.0308)</t>
         </is>
       </c>
     </row>
@@ -18011,7 +18009,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18020,13 +18018,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.5320197044334976</v>
-      </c>
-      <c r="F490" t="inlineStr"/>
-      <c r="G490" t="inlineStr"/>
+        <v>0.3735632183908046</v>
+      </c>
+      <c r="F490" t="n">
+        <v>0.397212543554007</v>
+      </c>
+      <c r="G490" t="n">
+        <v>0.3764705882352941</v>
+      </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.5320 (0.0000)</t>
+          <t>0.3824 (0.0129)</t>
         </is>
       </c>
     </row>
@@ -18043,7 +18045,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18052,49 +18054,51 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.417989417989418</v>
-      </c>
-      <c r="F491" t="inlineStr"/>
-      <c r="G491" t="inlineStr"/>
+        <v>0.5320197044334976</v>
+      </c>
+      <c r="F491" t="n">
+        <v>0.4809384164222874</v>
+      </c>
+      <c r="G491" t="n">
+        <v>0.5342465753424658</v>
+      </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.4180 (0.0000)</t>
+          <t>0.5157 (0.0302)</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.2534246575342466</v>
+        <v>0.417989417989418</v>
       </c>
       <c r="F492" t="n">
-        <v>0.302788844621514</v>
-      </c>
-      <c r="G492" t="n">
-        <v>0.2775510204081633</v>
-      </c>
+        <v>0.3711340206185567</v>
+      </c>
+      <c r="G492" t="inlineStr"/>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.2779 (0.0247)</t>
+          <t>0.3946 (0.0331)</t>
         </is>
       </c>
     </row>
@@ -18111,7 +18115,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18120,17 +18124,17 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.2534246575342466</v>
       </c>
       <c r="F493" t="n">
-        <v>0.3161764705882353</v>
+        <v>0.302788844621514</v>
       </c>
       <c r="G493" t="n">
-        <v>0.316205533596838</v>
+        <v>0.2775510204081633</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.3169 (0.0011)</t>
+          <t>0.2779 (0.0247)</t>
         </is>
       </c>
     </row>
@@ -18147,7 +18151,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -18156,17 +18160,17 @@
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.2290748898678414</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F494" t="n">
-        <v>0.256198347107438</v>
+        <v>0.3161764705882353</v>
       </c>
       <c r="G494" t="n">
-        <v>0.2629107981220657</v>
+        <v>0.316205533596838</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.2494 (0.0179)</t>
+          <t>0.3169 (0.0011)</t>
         </is>
       </c>
     </row>
@@ -18183,7 +18187,7 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
@@ -18192,17 +18196,17 @@
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.319327731092437</v>
+        <v>0.2290748898678414</v>
       </c>
       <c r="F495" t="n">
-        <v>0.2845849802371542</v>
+        <v>0.256198347107438</v>
       </c>
       <c r="G495" t="n">
-        <v>0.2331838565022422</v>
+        <v>0.2629107981220657</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2790 (0.0433)</t>
+          <t>0.2494 (0.0179)</t>
         </is>
       </c>
     </row>
@@ -18219,7 +18223,7 @@
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
@@ -18228,17 +18232,17 @@
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.319327731092437</v>
       </c>
       <c r="F496" t="n">
-        <v>0.2786885245901639</v>
+        <v>0.2845849802371542</v>
       </c>
       <c r="G496" t="n">
-        <v>0.3665338645418327</v>
+        <v>0.2331838565022422</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.3086 (0.0501)</t>
+          <t>0.2790 (0.0433)</t>
         </is>
       </c>
     </row>
@@ -18250,27 +18254,31 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2788461538461539</v>
-      </c>
-      <c r="F497" t="inlineStr"/>
-      <c r="G497" t="inlineStr"/>
+        <v>0.2807017543859649</v>
+      </c>
+      <c r="F497" t="n">
+        <v>0.2786885245901639</v>
+      </c>
+      <c r="G497" t="n">
+        <v>0.3665338645418327</v>
+      </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2788 (0.0000)</t>
+          <t>0.3086 (0.0501)</t>
         </is>
       </c>
     </row>
@@ -18287,7 +18295,7 @@
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
@@ -18296,17 +18304,13 @@
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.3497757847533632</v>
-      </c>
-      <c r="F498" t="n">
-        <v>0.2918454935622318</v>
-      </c>
-      <c r="G498" t="n">
-        <v>0.3255813953488372</v>
-      </c>
+        <v>0.2788461538461539</v>
+      </c>
+      <c r="F498" t="inlineStr"/>
+      <c r="G498" t="inlineStr"/>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.3224 (0.0291)</t>
+          <t>0.2788 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18323,7 +18327,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
@@ -18332,17 +18336,17 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.2054054054054054</v>
+        <v>0.3497757847533632</v>
       </c>
       <c r="F499" t="n">
-        <v>0.2408376963350785</v>
+        <v>0.2918454935622318</v>
       </c>
       <c r="G499" t="n">
-        <v>0.2346368715083799</v>
+        <v>0.3255813953488372</v>
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.2270 (0.0189)</t>
+          <t>0.3224 (0.0291)</t>
         </is>
       </c>
     </row>
@@ -18359,7 +18363,7 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
@@ -18368,13 +18372,17 @@
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.3643122676579926</v>
-      </c>
-      <c r="F500" t="inlineStr"/>
-      <c r="G500" t="inlineStr"/>
+        <v>0.2054054054054054</v>
+      </c>
+      <c r="F500" t="n">
+        <v>0.2408376963350785</v>
+      </c>
+      <c r="G500" t="n">
+        <v>0.2346368715083799</v>
+      </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.3643 (0.0000)</t>
+          <t>0.2270 (0.0189)</t>
         </is>
       </c>
     </row>
@@ -18391,7 +18399,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
@@ -18400,13 +18408,13 @@
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.2650602409638554</v>
+        <v>0.3643122676579926</v>
       </c>
       <c r="F501" t="inlineStr"/>
       <c r="G501" t="inlineStr"/>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.2651 (0.0000)</t>
+          <t>0.3643 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18418,31 +18426,27 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.2929292929292929</v>
-      </c>
-      <c r="F502" t="n">
-        <v>0.2972292191435768</v>
-      </c>
-      <c r="G502" t="n">
-        <v>0.3169398907103825</v>
-      </c>
+        <v>0.2650602409638554</v>
+      </c>
+      <c r="F502" t="inlineStr"/>
+      <c r="G502" t="inlineStr"/>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.3024 (0.0128)</t>
+          <t>0.2651 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18459,7 +18463,7 @@
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -18468,17 +18472,17 @@
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="F503" t="n">
-        <v>0.2433460076045627</v>
+        <v>0.2972292191435768</v>
       </c>
       <c r="G503" t="n">
-        <v>0.2704918032786885</v>
+        <v>0.3169398907103825</v>
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.2476 (0.0212)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -18495,7 +18499,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
@@ -18504,13 +18508,17 @@
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.3179916317991632</v>
-      </c>
-      <c r="F504" t="inlineStr"/>
-      <c r="G504" t="inlineStr"/>
+        <v>0.2288135593220339</v>
+      </c>
+      <c r="F504" t="n">
+        <v>0.2433460076045627</v>
+      </c>
+      <c r="G504" t="n">
+        <v>0.2704918032786885</v>
+      </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.3180 (0.0000)</t>
+          <t>0.2476 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18527,7 +18535,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -18536,13 +18544,13 @@
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.3179916317991632</v>
       </c>
       <c r="F505" t="inlineStr"/>
       <c r="G505" t="inlineStr"/>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2222 (0.0000)</t>
+          <t>0.3180 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18554,31 +18562,27 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.2923076923076923</v>
-      </c>
-      <c r="F506" t="n">
-        <v>0.2844444444444444</v>
-      </c>
-      <c r="G506" t="n">
-        <v>0.2627737226277372</v>
-      </c>
+        <v>0.2222222222222222</v>
+      </c>
+      <c r="F506" t="inlineStr"/>
+      <c r="G506" t="inlineStr"/>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.2222 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18595,7 +18599,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18604,17 +18608,17 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F507" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G507" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18635,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
@@ -18640,17 +18644,17 @@
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F508" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G508" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -18667,7 +18671,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
@@ -18676,17 +18680,17 @@
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F509" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G509" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -18703,7 +18707,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -18712,17 +18716,17 @@
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F510" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G510" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18734,31 +18738,31 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F511" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G511" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -18775,7 +18779,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -18784,17 +18788,17 @@
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F512" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G512" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -18811,7 +18815,7 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
@@ -18820,17 +18824,17 @@
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F513" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G513" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
@@ -18847,7 +18851,7 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
@@ -18856,17 +18860,17 @@
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F514" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G514" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
@@ -18883,7 +18887,7 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
@@ -18892,53 +18896,53 @@
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.225</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F515" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G515" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.225</v>
       </c>
       <c r="F516" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G516" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18955,7 +18959,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
@@ -18964,17 +18968,17 @@
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F517" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G517" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -18991,7 +18995,7 @@
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
@@ -19000,17 +19004,17 @@
         </is>
       </c>
       <c r="E518" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F518" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G518" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -19027,7 +19031,7 @@
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
@@ -19036,17 +19040,17 @@
         </is>
       </c>
       <c r="E519" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F519" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G519" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -19063,7 +19067,7 @@
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
@@ -19072,17 +19076,17 @@
         </is>
       </c>
       <c r="E520" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F520" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G520" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -19094,27 +19098,31 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E521" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F521" t="inlineStr"/>
-      <c r="G521" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F521" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G521" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19131,7 +19139,7 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
@@ -19140,17 +19148,13 @@
         </is>
       </c>
       <c r="E522" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F522" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G522" t="n">
-        <v>0.2377622377622378</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F522" t="inlineStr"/>
+      <c r="G522" t="inlineStr"/>
       <c r="H522" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19167,7 +19171,7 @@
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
@@ -19176,17 +19180,17 @@
         </is>
       </c>
       <c r="E523" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F523" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G523" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H523" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -19203,7 +19207,7 @@
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
@@ -19212,15 +19216,17 @@
         </is>
       </c>
       <c r="E524" t="n">
-        <v>0.3054187192118227</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F524" t="n">
-        <v>0.2517482517482518</v>
-      </c>
-      <c r="G524" t="inlineStr"/>
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G524" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H524" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -19237,7 +19243,7 @@
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
@@ -19246,13 +19252,15 @@
         </is>
       </c>
       <c r="E525" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F525" t="inlineStr"/>
+        <v>0.3054187192118227</v>
+      </c>
+      <c r="F525" t="n">
+        <v>0.2517482517482518</v>
+      </c>
       <c r="G525" t="inlineStr"/>
       <c r="H525" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -19264,31 +19272,27 @@
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E526" t="n">
-        <v>0.2583025830258303</v>
-      </c>
-      <c r="F526" t="n">
-        <v>0.2443438914027149</v>
-      </c>
-      <c r="G526" t="n">
-        <v>0.2191780821917808</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F526" t="inlineStr"/>
+      <c r="G526" t="inlineStr"/>
       <c r="H526" t="inlineStr">
         <is>
-          <t>0.2406 (0.0198)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19305,7 +19309,7 @@
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
@@ -19314,17 +19318,17 @@
         </is>
       </c>
       <c r="E527" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F527" t="n">
-        <v>0.258575197889182</v>
+        <v>0.2443438914027149</v>
       </c>
       <c r="G527" t="n">
-        <v>0.1852861035422343</v>
+        <v>0.2191780821917808</v>
       </c>
       <c r="H527" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2406 (0.0198)</t>
         </is>
       </c>
     </row>
@@ -19341,7 +19345,7 @@
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
@@ -19350,17 +19354,17 @@
         </is>
       </c>
       <c r="E528" t="n">
-        <v>0.16</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F528" t="n">
-        <v>0.2094240837696335</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G528" t="n">
-        <v>0.1619047619047619</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -19377,7 +19381,7 @@
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
@@ -19386,17 +19390,17 @@
         </is>
       </c>
       <c r="E529" t="n">
-        <v>0.2575107296137339</v>
+        <v>0.16</v>
       </c>
       <c r="F529" t="n">
-        <v>0.2989690721649484</v>
+        <v>0.2094240837696335</v>
       </c>
       <c r="G529" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.1619047619047619</v>
       </c>
       <c r="H529" t="inlineStr">
         <is>
-          <t>0.2825 (0.0220)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -19413,7 +19417,7 @@
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
@@ -19422,17 +19426,17 @@
         </is>
       </c>
       <c r="E530" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F530" t="n">
-        <v>0.2566371681415929</v>
+        <v>0.2989690721649484</v>
       </c>
       <c r="G530" t="n">
-        <v>0.2551020408163265</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>0.2586 (0.0048)</t>
+          <t>0.2825 (0.0220)</t>
         </is>
       </c>
     </row>
@@ -19444,31 +19448,31 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D531" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E531" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F531" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2566371681415929</v>
       </c>
       <c r="G531" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.2551020408163265</v>
       </c>
       <c r="H531" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2586 (0.0048)</t>
         </is>
       </c>
     </row>
@@ -19485,7 +19489,7 @@
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D532" t="inlineStr">
@@ -19494,17 +19498,17 @@
         </is>
       </c>
       <c r="E532" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F532" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G532" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -19521,7 +19525,7 @@
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
@@ -19530,17 +19534,17 @@
         </is>
       </c>
       <c r="E533" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F533" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G533" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H533" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -19557,7 +19561,7 @@
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D534" t="inlineStr">
@@ -19566,17 +19570,17 @@
         </is>
       </c>
       <c r="E534" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F534" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G534" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H534" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -19593,7 +19597,7 @@
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
@@ -19602,17 +19606,17 @@
         </is>
       </c>
       <c r="E535" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F535" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G535" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -19624,31 +19628,31 @@
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E536" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F536" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G536" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H536" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -19665,7 +19669,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
@@ -19674,17 +19678,17 @@
         </is>
       </c>
       <c r="E537" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F537" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G537" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -19701,7 +19705,7 @@
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
@@ -19710,17 +19714,17 @@
         </is>
       </c>
       <c r="E538" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F538" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G538" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H538" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19737,7 +19741,7 @@
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
@@ -19746,17 +19750,17 @@
         </is>
       </c>
       <c r="E539" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F539" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G539" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H539" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -19773,24 +19777,60 @@
       </c>
       <c r="C540" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E540" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F540" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G540" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D540" t="inlineStr">
+      <c r="D541" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E540" t="n">
+      <c r="E541" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F540" t="n">
+      <c r="F541" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G540" t="n">
+      <c r="G541" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H540" t="inlineStr">
+      <c r="H541" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 16:49:41)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H541"/>
+  <dimension ref="A1:H542"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17738,11 +17738,13 @@
       <c r="E482" t="n">
         <v>0.4901960784313725</v>
       </c>
-      <c r="F482" t="inlineStr"/>
+      <c r="F482" t="n">
+        <v>0.4632768361581921</v>
+      </c>
       <c r="G482" t="inlineStr"/>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.4902 (0.0000)</t>
+          <t>0.4767 (0.0190)</t>
         </is>
       </c>
     </row>
@@ -17953,10 +17955,12 @@
       <c r="F488" t="n">
         <v>0.4187725631768953</v>
       </c>
-      <c r="G488" t="inlineStr"/>
+      <c r="G488" t="n">
+        <v>0.3955223880597015</v>
+      </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.4522 (0.0472)</t>
+          <t>0.4333 (0.0467)</t>
         </is>
       </c>
     </row>
@@ -18095,10 +18099,12 @@
       <c r="F492" t="n">
         <v>0.3711340206185567</v>
       </c>
-      <c r="G492" t="inlineStr"/>
+      <c r="G492" t="n">
+        <v>0.4564315352697095</v>
+      </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.3946 (0.0331)</t>
+          <t>0.4152 (0.0427)</t>
         </is>
       </c>
     </row>
@@ -18463,7 +18469,7 @@
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -18472,17 +18478,13 @@
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.2929292929292929</v>
-      </c>
-      <c r="F503" t="n">
-        <v>0.2972292191435768</v>
-      </c>
-      <c r="G503" t="n">
-        <v>0.3169398907103825</v>
-      </c>
+        <v>0.2727272727272727</v>
+      </c>
+      <c r="F503" t="inlineStr"/>
+      <c r="G503" t="inlineStr"/>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.3024 (0.0128)</t>
+          <t>0.2727 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18499,7 +18501,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
@@ -18508,17 +18510,17 @@
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="F504" t="n">
-        <v>0.2433460076045627</v>
+        <v>0.2972292191435768</v>
       </c>
       <c r="G504" t="n">
-        <v>0.2704918032786885</v>
+        <v>0.3169398907103825</v>
       </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.2476 (0.0212)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -18535,7 +18537,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -18544,13 +18546,17 @@
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.3179916317991632</v>
-      </c>
-      <c r="F505" t="inlineStr"/>
-      <c r="G505" t="inlineStr"/>
+        <v>0.2288135593220339</v>
+      </c>
+      <c r="F505" t="n">
+        <v>0.2433460076045627</v>
+      </c>
+      <c r="G505" t="n">
+        <v>0.2704918032786885</v>
+      </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.3180 (0.0000)</t>
+          <t>0.2476 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18567,7 +18573,7 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
@@ -18576,13 +18582,13 @@
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.3179916317991632</v>
       </c>
       <c r="F506" t="inlineStr"/>
       <c r="G506" t="inlineStr"/>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.2222 (0.0000)</t>
+          <t>0.3180 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18594,31 +18600,27 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.2923076923076923</v>
-      </c>
-      <c r="F507" t="n">
-        <v>0.2844444444444444</v>
-      </c>
-      <c r="G507" t="n">
-        <v>0.2627737226277372</v>
-      </c>
+        <v>0.2222222222222222</v>
+      </c>
+      <c r="F507" t="inlineStr"/>
+      <c r="G507" t="inlineStr"/>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.2222 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18635,7 +18637,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
@@ -18644,17 +18646,17 @@
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F508" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G508" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -18671,7 +18673,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
@@ -18680,17 +18682,17 @@
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F509" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G509" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -18707,7 +18709,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -18716,17 +18718,17 @@
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F510" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G510" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -18743,7 +18745,7 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
@@ -18752,17 +18754,17 @@
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F511" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G511" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18774,31 +18776,31 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F512" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G512" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -18815,7 +18817,7 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
@@ -18824,17 +18826,17 @@
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F513" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G513" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -18851,7 +18853,7 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
@@ -18860,17 +18862,17 @@
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F514" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G514" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18889,7 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
@@ -18896,17 +18898,17 @@
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F515" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G515" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
@@ -18923,7 +18925,7 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
@@ -18932,53 +18934,53 @@
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.225</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F516" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G516" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.225</v>
       </c>
       <c r="F517" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G517" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -18995,7 +18997,7 @@
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
@@ -19004,17 +19006,17 @@
         </is>
       </c>
       <c r="E518" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F518" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G518" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -19031,7 +19033,7 @@
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
@@ -19040,17 +19042,17 @@
         </is>
       </c>
       <c r="E519" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F519" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G519" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -19067,7 +19069,7 @@
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
@@ -19076,17 +19078,17 @@
         </is>
       </c>
       <c r="E520" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F520" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G520" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -19103,7 +19105,7 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
@@ -19112,17 +19114,17 @@
         </is>
       </c>
       <c r="E521" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F521" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G521" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -19134,27 +19136,31 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E522" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F522" t="inlineStr"/>
-      <c r="G522" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F522" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G522" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H522" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19171,7 +19177,7 @@
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
@@ -19180,17 +19186,13 @@
         </is>
       </c>
       <c r="E523" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F523" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G523" t="n">
-        <v>0.2377622377622378</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F523" t="inlineStr"/>
+      <c r="G523" t="inlineStr"/>
       <c r="H523" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19207,7 +19209,7 @@
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
@@ -19216,17 +19218,17 @@
         </is>
       </c>
       <c r="E524" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F524" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G524" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H524" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -19243,7 +19245,7 @@
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
@@ -19252,15 +19254,17 @@
         </is>
       </c>
       <c r="E525" t="n">
-        <v>0.3054187192118227</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F525" t="n">
-        <v>0.2517482517482518</v>
-      </c>
-      <c r="G525" t="inlineStr"/>
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G525" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H525" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -19277,7 +19281,7 @@
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
@@ -19286,13 +19290,15 @@
         </is>
       </c>
       <c r="E526" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F526" t="inlineStr"/>
+        <v>0.3054187192118227</v>
+      </c>
+      <c r="F526" t="n">
+        <v>0.2517482517482518</v>
+      </c>
       <c r="G526" t="inlineStr"/>
       <c r="H526" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -19304,31 +19310,27 @@
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E527" t="n">
-        <v>0.2583025830258303</v>
-      </c>
-      <c r="F527" t="n">
-        <v>0.2443438914027149</v>
-      </c>
-      <c r="G527" t="n">
-        <v>0.2191780821917808</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F527" t="inlineStr"/>
+      <c r="G527" t="inlineStr"/>
       <c r="H527" t="inlineStr">
         <is>
-          <t>0.2406 (0.0198)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19345,7 +19347,7 @@
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
@@ -19354,17 +19356,17 @@
         </is>
       </c>
       <c r="E528" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F528" t="n">
-        <v>0.258575197889182</v>
+        <v>0.2443438914027149</v>
       </c>
       <c r="G528" t="n">
-        <v>0.1852861035422343</v>
+        <v>0.2191780821917808</v>
       </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2406 (0.0198)</t>
         </is>
       </c>
     </row>
@@ -19381,7 +19383,7 @@
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
@@ -19390,17 +19392,17 @@
         </is>
       </c>
       <c r="E529" t="n">
-        <v>0.16</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F529" t="n">
-        <v>0.2094240837696335</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G529" t="n">
-        <v>0.1619047619047619</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H529" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -19417,7 +19419,7 @@
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
@@ -19426,17 +19428,17 @@
         </is>
       </c>
       <c r="E530" t="n">
-        <v>0.2575107296137339</v>
+        <v>0.16</v>
       </c>
       <c r="F530" t="n">
-        <v>0.2989690721649484</v>
+        <v>0.2094240837696335</v>
       </c>
       <c r="G530" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.1619047619047619</v>
       </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>0.2825 (0.0220)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -19453,7 +19455,7 @@
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D531" t="inlineStr">
@@ -19462,17 +19464,17 @@
         </is>
       </c>
       <c r="E531" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F531" t="n">
-        <v>0.2566371681415929</v>
+        <v>0.2989690721649484</v>
       </c>
       <c r="G531" t="n">
-        <v>0.2551020408163265</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H531" t="inlineStr">
         <is>
-          <t>0.2586 (0.0048)</t>
+          <t>0.2825 (0.0220)</t>
         </is>
       </c>
     </row>
@@ -19484,31 +19486,31 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D532" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E532" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F532" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2566371681415929</v>
       </c>
       <c r="G532" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.2551020408163265</v>
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2586 (0.0048)</t>
         </is>
       </c>
     </row>
@@ -19525,7 +19527,7 @@
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
@@ -19534,17 +19536,17 @@
         </is>
       </c>
       <c r="E533" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F533" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G533" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H533" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -19561,7 +19563,7 @@
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D534" t="inlineStr">
@@ -19570,17 +19572,17 @@
         </is>
       </c>
       <c r="E534" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F534" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G534" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H534" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -19597,7 +19599,7 @@
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
@@ -19606,17 +19608,17 @@
         </is>
       </c>
       <c r="E535" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F535" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G535" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -19633,7 +19635,7 @@
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
@@ -19642,17 +19644,17 @@
         </is>
       </c>
       <c r="E536" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F536" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G536" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H536" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -19664,31 +19666,31 @@
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E537" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F537" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G537" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -19705,7 +19707,7 @@
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
@@ -19714,17 +19716,17 @@
         </is>
       </c>
       <c r="E538" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F538" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G538" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H538" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -19741,7 +19743,7 @@
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
@@ -19750,17 +19752,17 @@
         </is>
       </c>
       <c r="E539" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F539" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G539" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H539" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19777,7 +19779,7 @@
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
@@ -19786,17 +19788,17 @@
         </is>
       </c>
       <c r="E540" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F540" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G540" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H540" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -19813,24 +19815,60 @@
       </c>
       <c r="C541" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E541" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F541" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G541" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D541" t="inlineStr">
+      <c r="D542" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E541" t="n">
+      <c r="E542" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F541" t="n">
+      <c r="F542" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G541" t="n">
+      <c r="G542" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H541" t="inlineStr">
+      <c r="H542" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 17:50:01)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -17741,10 +17741,12 @@
       <c r="F482" t="n">
         <v>0.4632768361581921</v>
       </c>
-      <c r="G482" t="inlineStr"/>
+      <c r="G482" t="n">
+        <v>0.4501424501424501</v>
+      </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>0.4767 (0.0190)</t>
+          <t>0.4679 (0.0204)</t>
         </is>
       </c>
     </row>
@@ -18616,11 +18618,13 @@
       <c r="E507" t="n">
         <v>0.2222222222222222</v>
       </c>
-      <c r="F507" t="inlineStr"/>
+      <c r="F507" t="n">
+        <v>0.247787610619469</v>
+      </c>
       <c r="G507" t="inlineStr"/>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2222 (0.0000)</t>
+          <t>0.2350 (0.0181)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 19:50:41)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H542"/>
+  <dimension ref="A1:H543"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17758,31 +17758,27 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E483" t="n">
-        <v>0.5080831408775982</v>
-      </c>
-      <c r="F483" t="n">
-        <v>0.4013605442176871</v>
-      </c>
-      <c r="G483" t="n">
-        <v>0.4327176781002638</v>
-      </c>
+        <v>0.3988603988603989</v>
+      </c>
+      <c r="F483" t="inlineStr"/>
+      <c r="G483" t="inlineStr"/>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.4474 (0.0549)</t>
+          <t>0.3989 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17799,7 +17795,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -17808,17 +17804,17 @@
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.4822695035460993</v>
+        <v>0.5080831408775982</v>
       </c>
       <c r="F484" t="n">
-        <v>0.4904632152588556</v>
+        <v>0.4013605442176871</v>
       </c>
       <c r="G484" t="n">
-        <v>0.4634920634920635</v>
+        <v>0.4327176781002638</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.4787 (0.0138)</t>
+          <t>0.4474 (0.0549)</t>
         </is>
       </c>
     </row>
@@ -17835,7 +17831,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17844,17 +17840,17 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.4</v>
+        <v>0.4822695035460993</v>
       </c>
       <c r="F485" t="n">
-        <v>0.3867069486404834</v>
+        <v>0.4904632152588556</v>
       </c>
       <c r="G485" t="n">
-        <v>0.3094339622641509</v>
+        <v>0.4634920634920635</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.3654 (0.0489)</t>
+          <t>0.4787 (0.0138)</t>
         </is>
       </c>
     </row>
@@ -17871,7 +17867,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17880,17 +17876,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.5801217038539553</v>
+        <v>0.4</v>
       </c>
       <c r="F486" t="n">
-        <v>0.5185185185185185</v>
+        <v>0.3867069486404834</v>
       </c>
       <c r="G486" t="n">
-        <v>0.5128205128205128</v>
+        <v>0.3094339622641509</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.5372 (0.0373)</t>
+          <t>0.3654 (0.0489)</t>
         </is>
       </c>
     </row>
@@ -17907,7 +17903,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17916,17 +17912,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.4698795180722892</v>
+        <v>0.5801217038539553</v>
       </c>
       <c r="F487" t="n">
-        <v>0.303030303030303</v>
+        <v>0.5185185185185185</v>
       </c>
       <c r="G487" t="n">
-        <v>0.3675213675213675</v>
+        <v>0.5128205128205128</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.3801 (0.0841)</t>
+          <t>0.5372 (0.0373)</t>
         </is>
       </c>
     </row>
@@ -17938,31 +17934,31 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.4855769230769231</v>
+        <v>0.4698795180722892</v>
       </c>
       <c r="F488" t="n">
-        <v>0.4187725631768953</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G488" t="n">
-        <v>0.3955223880597015</v>
+        <v>0.3675213675213675</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.4333 (0.0467)</t>
+          <t>0.3801 (0.0841)</t>
         </is>
       </c>
     </row>
@@ -17979,7 +17975,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17988,17 +17984,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.4839506172839506</v>
+        <v>0.4855769230769231</v>
       </c>
       <c r="F489" t="n">
-        <v>0.4502923976608187</v>
+        <v>0.4187725631768953</v>
       </c>
       <c r="G489" t="n">
-        <v>0.4224422442244224</v>
+        <v>0.3955223880597015</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.4522 (0.0308)</t>
+          <t>0.4333 (0.0467)</t>
         </is>
       </c>
     </row>
@@ -18015,7 +18011,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18024,17 +18020,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.3735632183908046</v>
+        <v>0.4839506172839506</v>
       </c>
       <c r="F490" t="n">
-        <v>0.397212543554007</v>
+        <v>0.4502923976608187</v>
       </c>
       <c r="G490" t="n">
-        <v>0.3764705882352941</v>
+        <v>0.4224422442244224</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.3824 (0.0129)</t>
+          <t>0.4522 (0.0308)</t>
         </is>
       </c>
     </row>
@@ -18051,7 +18047,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18060,17 +18056,17 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.5320197044334976</v>
+        <v>0.3735632183908046</v>
       </c>
       <c r="F491" t="n">
-        <v>0.4809384164222874</v>
+        <v>0.397212543554007</v>
       </c>
       <c r="G491" t="n">
-        <v>0.5342465753424658</v>
+        <v>0.3764705882352941</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.5157 (0.0302)</t>
+          <t>0.3824 (0.0129)</t>
         </is>
       </c>
     </row>
@@ -18087,7 +18083,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18096,53 +18092,53 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.417989417989418</v>
+        <v>0.5320197044334976</v>
       </c>
       <c r="F492" t="n">
-        <v>0.3711340206185567</v>
+        <v>0.4809384164222874</v>
       </c>
       <c r="G492" t="n">
-        <v>0.4564315352697095</v>
+        <v>0.5342465753424658</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.4152 (0.0427)</t>
+          <t>0.5157 (0.0302)</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.2534246575342466</v>
+        <v>0.417989417989418</v>
       </c>
       <c r="F493" t="n">
-        <v>0.302788844621514</v>
+        <v>0.3711340206185567</v>
       </c>
       <c r="G493" t="n">
-        <v>0.2775510204081633</v>
+        <v>0.4564315352697095</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.2779 (0.0247)</t>
+          <t>0.4152 (0.0427)</t>
         </is>
       </c>
     </row>
@@ -18159,7 +18155,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -18168,17 +18164,17 @@
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.2534246575342466</v>
       </c>
       <c r="F494" t="n">
-        <v>0.3161764705882353</v>
+        <v>0.302788844621514</v>
       </c>
       <c r="G494" t="n">
-        <v>0.316205533596838</v>
+        <v>0.2775510204081633</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.3169 (0.0011)</t>
+          <t>0.2779 (0.0247)</t>
         </is>
       </c>
     </row>
@@ -18195,7 +18191,7 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
@@ -18204,17 +18200,17 @@
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.2290748898678414</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F495" t="n">
-        <v>0.256198347107438</v>
+        <v>0.3161764705882353</v>
       </c>
       <c r="G495" t="n">
-        <v>0.2629107981220657</v>
+        <v>0.316205533596838</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2494 (0.0179)</t>
+          <t>0.3169 (0.0011)</t>
         </is>
       </c>
     </row>
@@ -18231,7 +18227,7 @@
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
@@ -18240,17 +18236,17 @@
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.319327731092437</v>
+        <v>0.2290748898678414</v>
       </c>
       <c r="F496" t="n">
-        <v>0.2845849802371542</v>
+        <v>0.256198347107438</v>
       </c>
       <c r="G496" t="n">
-        <v>0.2331838565022422</v>
+        <v>0.2629107981220657</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.2790 (0.0433)</t>
+          <t>0.2494 (0.0179)</t>
         </is>
       </c>
     </row>
@@ -18267,7 +18263,7 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
@@ -18276,17 +18272,17 @@
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.319327731092437</v>
       </c>
       <c r="F497" t="n">
-        <v>0.2786885245901639</v>
+        <v>0.2845849802371542</v>
       </c>
       <c r="G497" t="n">
-        <v>0.3665338645418327</v>
+        <v>0.2331838565022422</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.3086 (0.0501)</t>
+          <t>0.2790 (0.0433)</t>
         </is>
       </c>
     </row>
@@ -18298,27 +18294,31 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2788461538461539</v>
-      </c>
-      <c r="F498" t="inlineStr"/>
-      <c r="G498" t="inlineStr"/>
+        <v>0.2807017543859649</v>
+      </c>
+      <c r="F498" t="n">
+        <v>0.2786885245901639</v>
+      </c>
+      <c r="G498" t="n">
+        <v>0.3665338645418327</v>
+      </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2788 (0.0000)</t>
+          <t>0.3086 (0.0501)</t>
         </is>
       </c>
     </row>
@@ -18335,7 +18335,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
@@ -18344,17 +18344,13 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.3497757847533632</v>
-      </c>
-      <c r="F499" t="n">
-        <v>0.2918454935622318</v>
-      </c>
-      <c r="G499" t="n">
-        <v>0.3255813953488372</v>
-      </c>
+        <v>0.2788461538461539</v>
+      </c>
+      <c r="F499" t="inlineStr"/>
+      <c r="G499" t="inlineStr"/>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.3224 (0.0291)</t>
+          <t>0.2788 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18371,7 +18367,7 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
@@ -18380,17 +18376,17 @@
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.2054054054054054</v>
+        <v>0.3497757847533632</v>
       </c>
       <c r="F500" t="n">
-        <v>0.2408376963350785</v>
+        <v>0.2918454935622318</v>
       </c>
       <c r="G500" t="n">
-        <v>0.2346368715083799</v>
+        <v>0.3255813953488372</v>
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.2270 (0.0189)</t>
+          <t>0.3224 (0.0291)</t>
         </is>
       </c>
     </row>
@@ -18407,7 +18403,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
@@ -18416,13 +18412,17 @@
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.3643122676579926</v>
-      </c>
-      <c r="F501" t="inlineStr"/>
-      <c r="G501" t="inlineStr"/>
+        <v>0.2054054054054054</v>
+      </c>
+      <c r="F501" t="n">
+        <v>0.2408376963350785</v>
+      </c>
+      <c r="G501" t="n">
+        <v>0.2346368715083799</v>
+      </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.3643 (0.0000)</t>
+          <t>0.2270 (0.0189)</t>
         </is>
       </c>
     </row>
@@ -18439,7 +18439,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -18448,13 +18448,13 @@
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.2650602409638554</v>
+        <v>0.3643122676579926</v>
       </c>
       <c r="F502" t="inlineStr"/>
       <c r="G502" t="inlineStr"/>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.2651 (0.0000)</t>
+          <t>0.3643 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18466,27 +18466,27 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.2650602409638554</v>
       </c>
       <c r="F503" t="inlineStr"/>
       <c r="G503" t="inlineStr"/>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.2727 (0.0000)</t>
+          <t>0.2651 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18503,7 +18503,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
@@ -18512,17 +18512,13 @@
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.2929292929292929</v>
-      </c>
-      <c r="F504" t="n">
-        <v>0.2972292191435768</v>
-      </c>
-      <c r="G504" t="n">
-        <v>0.3169398907103825</v>
-      </c>
+        <v>0.2727272727272727</v>
+      </c>
+      <c r="F504" t="inlineStr"/>
+      <c r="G504" t="inlineStr"/>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.3024 (0.0128)</t>
+          <t>0.2727 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18539,7 +18535,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -18548,17 +18544,17 @@
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="F505" t="n">
-        <v>0.2433460076045627</v>
+        <v>0.2972292191435768</v>
       </c>
       <c r="G505" t="n">
-        <v>0.2704918032786885</v>
+        <v>0.3169398907103825</v>
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2476 (0.0212)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -18575,7 +18571,7 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
@@ -18584,13 +18580,17 @@
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.3179916317991632</v>
-      </c>
-      <c r="F506" t="inlineStr"/>
-      <c r="G506" t="inlineStr"/>
+        <v>0.2288135593220339</v>
+      </c>
+      <c r="F506" t="n">
+        <v>0.2433460076045627</v>
+      </c>
+      <c r="G506" t="n">
+        <v>0.2704918032786885</v>
+      </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.3180 (0.0000)</t>
+          <t>0.2476 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18607,7 +18607,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18616,15 +18616,15 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.3179916317991632</v>
       </c>
       <c r="F507" t="n">
-        <v>0.247787610619469</v>
+        <v>0.3206106870229007</v>
       </c>
       <c r="G507" t="inlineStr"/>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2350 (0.0181)</t>
+          <t>0.3193 (0.0019)</t>
         </is>
       </c>
     </row>
@@ -18636,31 +18636,29 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.2923076923076923</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="F508" t="n">
-        <v>0.2844444444444444</v>
-      </c>
-      <c r="G508" t="n">
-        <v>0.2627737226277372</v>
-      </c>
+        <v>0.247787610619469</v>
+      </c>
+      <c r="G508" t="inlineStr"/>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.2350 (0.0181)</t>
         </is>
       </c>
     </row>
@@ -18677,7 +18675,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
@@ -18686,17 +18684,17 @@
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F509" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G509" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -18713,7 +18711,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -18722,17 +18720,17 @@
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G510" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -18749,7 +18747,7 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
@@ -18758,17 +18756,17 @@
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F511" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G511" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -18785,7 +18783,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -18794,17 +18792,17 @@
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F512" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G512" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18816,31 +18814,31 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F513" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G513" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -18857,7 +18855,7 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
@@ -18866,17 +18864,17 @@
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F514" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G514" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -18893,7 +18891,7 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
@@ -18902,17 +18900,17 @@
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F515" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G515" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
@@ -18929,7 +18927,7 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
@@ -18938,17 +18936,17 @@
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F516" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G516" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
@@ -18965,7 +18963,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
@@ -18974,53 +18972,53 @@
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.225</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F517" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G517" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E518" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.225</v>
       </c>
       <c r="F518" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G518" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -19037,7 +19035,7 @@
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
@@ -19046,17 +19044,17 @@
         </is>
       </c>
       <c r="E519" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F519" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G519" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -19073,7 +19071,7 @@
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
@@ -19082,17 +19080,17 @@
         </is>
       </c>
       <c r="E520" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F520" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G520" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -19109,7 +19107,7 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
@@ -19118,17 +19116,17 @@
         </is>
       </c>
       <c r="E521" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F521" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G521" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -19145,7 +19143,7 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
@@ -19154,17 +19152,17 @@
         </is>
       </c>
       <c r="E522" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F522" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G522" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H522" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -19176,27 +19174,31 @@
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E523" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F523" t="inlineStr"/>
-      <c r="G523" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F523" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G523" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H523" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19213,7 +19215,7 @@
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
@@ -19222,17 +19224,13 @@
         </is>
       </c>
       <c r="E524" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F524" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G524" t="n">
-        <v>0.2377622377622378</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F524" t="inlineStr"/>
+      <c r="G524" t="inlineStr"/>
       <c r="H524" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19249,7 +19247,7 @@
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
@@ -19258,17 +19256,17 @@
         </is>
       </c>
       <c r="E525" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F525" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G525" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H525" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -19285,7 +19283,7 @@
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
@@ -19294,15 +19292,17 @@
         </is>
       </c>
       <c r="E526" t="n">
-        <v>0.3054187192118227</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F526" t="n">
-        <v>0.2517482517482518</v>
-      </c>
-      <c r="G526" t="inlineStr"/>
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G526" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H526" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -19319,7 +19319,7 @@
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
@@ -19328,13 +19328,15 @@
         </is>
       </c>
       <c r="E527" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F527" t="inlineStr"/>
+        <v>0.3054187192118227</v>
+      </c>
+      <c r="F527" t="n">
+        <v>0.2517482517482518</v>
+      </c>
       <c r="G527" t="inlineStr"/>
       <c r="H527" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -19346,31 +19348,27 @@
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E528" t="n">
-        <v>0.2583025830258303</v>
-      </c>
-      <c r="F528" t="n">
-        <v>0.2443438914027149</v>
-      </c>
-      <c r="G528" t="n">
-        <v>0.2191780821917808</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F528" t="inlineStr"/>
+      <c r="G528" t="inlineStr"/>
       <c r="H528" t="inlineStr">
         <is>
-          <t>0.2406 (0.0198)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19387,7 +19385,7 @@
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
@@ -19396,17 +19394,17 @@
         </is>
       </c>
       <c r="E529" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F529" t="n">
-        <v>0.258575197889182</v>
+        <v>0.2443438914027149</v>
       </c>
       <c r="G529" t="n">
-        <v>0.1852861035422343</v>
+        <v>0.2191780821917808</v>
       </c>
       <c r="H529" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2406 (0.0198)</t>
         </is>
       </c>
     </row>
@@ -19423,7 +19421,7 @@
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
@@ -19432,17 +19430,17 @@
         </is>
       </c>
       <c r="E530" t="n">
-        <v>0.16</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F530" t="n">
-        <v>0.2094240837696335</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G530" t="n">
-        <v>0.1619047619047619</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -19459,7 +19457,7 @@
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D531" t="inlineStr">
@@ -19468,17 +19466,17 @@
         </is>
       </c>
       <c r="E531" t="n">
-        <v>0.2575107296137339</v>
+        <v>0.16</v>
       </c>
       <c r="F531" t="n">
-        <v>0.2989690721649484</v>
+        <v>0.2094240837696335</v>
       </c>
       <c r="G531" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.1619047619047619</v>
       </c>
       <c r="H531" t="inlineStr">
         <is>
-          <t>0.2825 (0.0220)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -19495,7 +19493,7 @@
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D532" t="inlineStr">
@@ -19504,17 +19502,17 @@
         </is>
       </c>
       <c r="E532" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F532" t="n">
-        <v>0.2566371681415929</v>
+        <v>0.2989690721649484</v>
       </c>
       <c r="G532" t="n">
-        <v>0.2551020408163265</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>0.2586 (0.0048)</t>
+          <t>0.2825 (0.0220)</t>
         </is>
       </c>
     </row>
@@ -19526,31 +19524,31 @@
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E533" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F533" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2566371681415929</v>
       </c>
       <c r="G533" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.2551020408163265</v>
       </c>
       <c r="H533" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2586 (0.0048)</t>
         </is>
       </c>
     </row>
@@ -19567,7 +19565,7 @@
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D534" t="inlineStr">
@@ -19576,17 +19574,17 @@
         </is>
       </c>
       <c r="E534" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F534" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G534" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H534" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -19603,7 +19601,7 @@
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
@@ -19612,17 +19610,17 @@
         </is>
       </c>
       <c r="E535" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F535" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G535" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -19639,7 +19637,7 @@
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
@@ -19648,17 +19646,17 @@
         </is>
       </c>
       <c r="E536" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F536" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G536" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H536" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -19675,7 +19673,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
@@ -19684,17 +19682,17 @@
         </is>
       </c>
       <c r="E537" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F537" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G537" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -19706,31 +19704,31 @@
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E538" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F538" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G538" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H538" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -19747,7 +19745,7 @@
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
@@ -19756,17 +19754,17 @@
         </is>
       </c>
       <c r="E539" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F539" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G539" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H539" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -19783,7 +19781,7 @@
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
@@ -19792,17 +19790,17 @@
         </is>
       </c>
       <c r="E540" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F540" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G540" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H540" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19819,7 +19817,7 @@
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">
@@ -19828,17 +19826,17 @@
         </is>
       </c>
       <c r="E541" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F541" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G541" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H541" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -19855,24 +19853,60 @@
       </c>
       <c r="C542" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E542" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F542" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G542" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D542" t="inlineStr">
+      <c r="D543" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E542" t="n">
+      <c r="E543" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F542" t="n">
+      <c r="F543" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G542" t="n">
+      <c r="G543" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H542" t="inlineStr">
+      <c r="H543" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 20:51:12)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -18450,11 +18450,13 @@
       <c r="E502" t="n">
         <v>0.3643122676579926</v>
       </c>
-      <c r="F502" t="inlineStr"/>
+      <c r="F502" t="n">
+        <v>0.3203883495145631</v>
+      </c>
       <c r="G502" t="inlineStr"/>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.3643 (0.0000)</t>
+          <t>0.3424 (0.0311)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 22:51:51)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H543"/>
+  <dimension ref="A1:H544"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17790,31 +17790,31 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.5080831408775982</v>
+        <v>0.5163636363636364</v>
       </c>
       <c r="F484" t="n">
-        <v>0.4013605442176871</v>
+        <v>0.465587044534413</v>
       </c>
       <c r="G484" t="n">
-        <v>0.4327176781002638</v>
+        <v>0.4183006535947713</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.4474 (0.0549)</t>
+          <t>0.4668 (0.0490)</t>
         </is>
       </c>
     </row>
@@ -17831,7 +17831,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17840,17 +17840,17 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.4822695035460993</v>
+        <v>0.5080831408775982</v>
       </c>
       <c r="F485" t="n">
-        <v>0.4904632152588556</v>
+        <v>0.4013605442176871</v>
       </c>
       <c r="G485" t="n">
-        <v>0.4634920634920635</v>
+        <v>0.4327176781002638</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.4787 (0.0138)</t>
+          <t>0.4474 (0.0549)</t>
         </is>
       </c>
     </row>
@@ -17867,7 +17867,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17876,17 +17876,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.4</v>
+        <v>0.4822695035460993</v>
       </c>
       <c r="F486" t="n">
-        <v>0.3867069486404834</v>
+        <v>0.4904632152588556</v>
       </c>
       <c r="G486" t="n">
-        <v>0.3094339622641509</v>
+        <v>0.4634920634920635</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.3654 (0.0489)</t>
+          <t>0.4787 (0.0138)</t>
         </is>
       </c>
     </row>
@@ -17903,7 +17903,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17912,17 +17912,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.5801217038539553</v>
+        <v>0.4</v>
       </c>
       <c r="F487" t="n">
-        <v>0.5185185185185185</v>
+        <v>0.3867069486404834</v>
       </c>
       <c r="G487" t="n">
-        <v>0.5128205128205128</v>
+        <v>0.3094339622641509</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.5372 (0.0373)</t>
+          <t>0.3654 (0.0489)</t>
         </is>
       </c>
     </row>
@@ -17939,7 +17939,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17948,17 +17948,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.4698795180722892</v>
+        <v>0.5801217038539553</v>
       </c>
       <c r="F488" t="n">
-        <v>0.303030303030303</v>
+        <v>0.5185185185185185</v>
       </c>
       <c r="G488" t="n">
-        <v>0.3675213675213675</v>
+        <v>0.5128205128205128</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.3801 (0.0841)</t>
+          <t>0.5372 (0.0373)</t>
         </is>
       </c>
     </row>
@@ -17970,31 +17970,31 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.4855769230769231</v>
+        <v>0.4698795180722892</v>
       </c>
       <c r="F489" t="n">
-        <v>0.4187725631768953</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G489" t="n">
-        <v>0.3955223880597015</v>
+        <v>0.3675213675213675</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.4333 (0.0467)</t>
+          <t>0.3801 (0.0841)</t>
         </is>
       </c>
     </row>
@@ -18011,7 +18011,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18020,17 +18020,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.4839506172839506</v>
+        <v>0.4855769230769231</v>
       </c>
       <c r="F490" t="n">
-        <v>0.4502923976608187</v>
+        <v>0.4187725631768953</v>
       </c>
       <c r="G490" t="n">
-        <v>0.4224422442244224</v>
+        <v>0.3955223880597015</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.4522 (0.0308)</t>
+          <t>0.4333 (0.0467)</t>
         </is>
       </c>
     </row>
@@ -18047,7 +18047,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18056,17 +18056,17 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.3735632183908046</v>
+        <v>0.4839506172839506</v>
       </c>
       <c r="F491" t="n">
-        <v>0.397212543554007</v>
+        <v>0.4502923976608187</v>
       </c>
       <c r="G491" t="n">
-        <v>0.3764705882352941</v>
+        <v>0.4224422442244224</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.3824 (0.0129)</t>
+          <t>0.4522 (0.0308)</t>
         </is>
       </c>
     </row>
@@ -18083,7 +18083,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18092,17 +18092,17 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.5320197044334976</v>
+        <v>0.3735632183908046</v>
       </c>
       <c r="F492" t="n">
-        <v>0.4809384164222874</v>
+        <v>0.397212543554007</v>
       </c>
       <c r="G492" t="n">
-        <v>0.5342465753424658</v>
+        <v>0.3764705882352941</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.5157 (0.0302)</t>
+          <t>0.3824 (0.0129)</t>
         </is>
       </c>
     </row>
@@ -18119,7 +18119,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18128,53 +18128,53 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.417989417989418</v>
+        <v>0.5320197044334976</v>
       </c>
       <c r="F493" t="n">
-        <v>0.3711340206185567</v>
+        <v>0.4809384164222874</v>
       </c>
       <c r="G493" t="n">
-        <v>0.4564315352697095</v>
+        <v>0.5342465753424658</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.4152 (0.0427)</t>
+          <t>0.5157 (0.0302)</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.2534246575342466</v>
+        <v>0.417989417989418</v>
       </c>
       <c r="F494" t="n">
-        <v>0.302788844621514</v>
+        <v>0.3711340206185567</v>
       </c>
       <c r="G494" t="n">
-        <v>0.2775510204081633</v>
+        <v>0.4564315352697095</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.2779 (0.0247)</t>
+          <t>0.4152 (0.0427)</t>
         </is>
       </c>
     </row>
@@ -18191,7 +18191,7 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
@@ -18200,17 +18200,17 @@
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.2534246575342466</v>
       </c>
       <c r="F495" t="n">
-        <v>0.3161764705882353</v>
+        <v>0.302788844621514</v>
       </c>
       <c r="G495" t="n">
-        <v>0.316205533596838</v>
+        <v>0.2775510204081633</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.3169 (0.0011)</t>
+          <t>0.2779 (0.0247)</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
@@ -18236,17 +18236,17 @@
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.2290748898678414</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F496" t="n">
-        <v>0.256198347107438</v>
+        <v>0.3161764705882353</v>
       </c>
       <c r="G496" t="n">
-        <v>0.2629107981220657</v>
+        <v>0.316205533596838</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.2494 (0.0179)</t>
+          <t>0.3169 (0.0011)</t>
         </is>
       </c>
     </row>
@@ -18263,7 +18263,7 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
@@ -18272,17 +18272,17 @@
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.319327731092437</v>
+        <v>0.2290748898678414</v>
       </c>
       <c r="F497" t="n">
-        <v>0.2845849802371542</v>
+        <v>0.256198347107438</v>
       </c>
       <c r="G497" t="n">
-        <v>0.2331838565022422</v>
+        <v>0.2629107981220657</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2790 (0.0433)</t>
+          <t>0.2494 (0.0179)</t>
         </is>
       </c>
     </row>
@@ -18299,7 +18299,7 @@
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
@@ -18308,17 +18308,17 @@
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.319327731092437</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2786885245901639</v>
+        <v>0.2845849802371542</v>
       </c>
       <c r="G498" t="n">
-        <v>0.3665338645418327</v>
+        <v>0.2331838565022422</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.3086 (0.0501)</t>
+          <t>0.2790 (0.0433)</t>
         </is>
       </c>
     </row>
@@ -18330,27 +18330,31 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.2788461538461539</v>
-      </c>
-      <c r="F499" t="inlineStr"/>
-      <c r="G499" t="inlineStr"/>
+        <v>0.2807017543859649</v>
+      </c>
+      <c r="F499" t="n">
+        <v>0.2786885245901639</v>
+      </c>
+      <c r="G499" t="n">
+        <v>0.3665338645418327</v>
+      </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.2788 (0.0000)</t>
+          <t>0.3086 (0.0501)</t>
         </is>
       </c>
     </row>
@@ -18367,7 +18371,7 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
@@ -18376,17 +18380,13 @@
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.3497757847533632</v>
-      </c>
-      <c r="F500" t="n">
-        <v>0.2918454935622318</v>
-      </c>
-      <c r="G500" t="n">
-        <v>0.3255813953488372</v>
-      </c>
+        <v>0.2788461538461539</v>
+      </c>
+      <c r="F500" t="inlineStr"/>
+      <c r="G500" t="inlineStr"/>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.3224 (0.0291)</t>
+          <t>0.2788 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18403,7 +18403,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
@@ -18412,17 +18412,17 @@
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.2054054054054054</v>
+        <v>0.3497757847533632</v>
       </c>
       <c r="F501" t="n">
-        <v>0.2408376963350785</v>
+        <v>0.2918454935622318</v>
       </c>
       <c r="G501" t="n">
-        <v>0.2346368715083799</v>
+        <v>0.3255813953488372</v>
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.2270 (0.0189)</t>
+          <t>0.3224 (0.0291)</t>
         </is>
       </c>
     </row>
@@ -18439,7 +18439,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -18448,15 +18448,17 @@
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.3643122676579926</v>
+        <v>0.2054054054054054</v>
       </c>
       <c r="F502" t="n">
-        <v>0.3203883495145631</v>
-      </c>
-      <c r="G502" t="inlineStr"/>
+        <v>0.2408376963350785</v>
+      </c>
+      <c r="G502" t="n">
+        <v>0.2346368715083799</v>
+      </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.3424 (0.0311)</t>
+          <t>0.2270 (0.0189)</t>
         </is>
       </c>
     </row>
@@ -18473,7 +18475,7 @@
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -18482,13 +18484,15 @@
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.2650602409638554</v>
-      </c>
-      <c r="F503" t="inlineStr"/>
+        <v>0.3643122676579926</v>
+      </c>
+      <c r="F503" t="n">
+        <v>0.3203883495145631</v>
+      </c>
       <c r="G503" t="inlineStr"/>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.2651 (0.0000)</t>
+          <t>0.3424 (0.0311)</t>
         </is>
       </c>
     </row>
@@ -18500,27 +18504,27 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.2650602409638554</v>
       </c>
       <c r="F504" t="inlineStr"/>
       <c r="G504" t="inlineStr"/>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.2727 (0.0000)</t>
+          <t>0.2651 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18537,7 +18541,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -18546,17 +18550,13 @@
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2929292929292929</v>
-      </c>
-      <c r="F505" t="n">
-        <v>0.2972292191435768</v>
-      </c>
-      <c r="G505" t="n">
-        <v>0.3169398907103825</v>
-      </c>
+        <v>0.2727272727272727</v>
+      </c>
+      <c r="F505" t="inlineStr"/>
+      <c r="G505" t="inlineStr"/>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.3024 (0.0128)</t>
+          <t>0.2727 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18573,7 +18573,7 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
@@ -18582,17 +18582,17 @@
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="F506" t="n">
-        <v>0.2433460076045627</v>
+        <v>0.2972292191435768</v>
       </c>
       <c r="G506" t="n">
-        <v>0.2704918032786885</v>
+        <v>0.3169398907103825</v>
       </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.2476 (0.0212)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -18609,7 +18609,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18618,15 +18618,17 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.3179916317991632</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="F507" t="n">
-        <v>0.3206106870229007</v>
-      </c>
-      <c r="G507" t="inlineStr"/>
+        <v>0.2433460076045627</v>
+      </c>
+      <c r="G507" t="n">
+        <v>0.2704918032786885</v>
+      </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.3193 (0.0019)</t>
+          <t>0.2476 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18643,7 +18645,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
@@ -18652,15 +18654,15 @@
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.3179916317991632</v>
       </c>
       <c r="F508" t="n">
-        <v>0.247787610619469</v>
+        <v>0.3206106870229007</v>
       </c>
       <c r="G508" t="inlineStr"/>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.2350 (0.0181)</t>
+          <t>0.3193 (0.0019)</t>
         </is>
       </c>
     </row>
@@ -18672,31 +18674,29 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.2923076923076923</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="F509" t="n">
-        <v>0.2844444444444444</v>
-      </c>
-      <c r="G509" t="n">
-        <v>0.2627737226277372</v>
-      </c>
+        <v>0.247787610619469</v>
+      </c>
+      <c r="G509" t="inlineStr"/>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.2350 (0.0181)</t>
         </is>
       </c>
     </row>
@@ -18713,7 +18713,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -18722,17 +18722,17 @@
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G510" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -18749,7 +18749,7 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
@@ -18758,17 +18758,17 @@
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F511" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G511" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -18785,7 +18785,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -18794,17 +18794,17 @@
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F512" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G512" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -18821,7 +18821,7 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
@@ -18830,17 +18830,17 @@
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F513" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G513" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18852,31 +18852,31 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F514" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G514" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -18893,7 +18893,7 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
@@ -18902,17 +18902,17 @@
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F515" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G515" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -18929,7 +18929,7 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
@@ -18938,17 +18938,17 @@
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F516" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G516" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
@@ -18965,7 +18965,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
@@ -18974,17 +18974,17 @@
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F517" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G517" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
@@ -19001,7 +19001,7 @@
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
@@ -19010,53 +19010,53 @@
         </is>
       </c>
       <c r="E518" t="n">
-        <v>0.225</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F518" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G518" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E519" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.225</v>
       </c>
       <c r="F519" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G519" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -19073,7 +19073,7 @@
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
@@ -19082,17 +19082,17 @@
         </is>
       </c>
       <c r="E520" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F520" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G520" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -19109,7 +19109,7 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
@@ -19118,17 +19118,17 @@
         </is>
       </c>
       <c r="E521" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F521" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G521" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -19145,7 +19145,7 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
@@ -19154,17 +19154,17 @@
         </is>
       </c>
       <c r="E522" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F522" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G522" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H522" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -19181,7 +19181,7 @@
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
@@ -19190,17 +19190,17 @@
         </is>
       </c>
       <c r="E523" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F523" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G523" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H523" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -19212,27 +19212,31 @@
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E524" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F524" t="inlineStr"/>
-      <c r="G524" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F524" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G524" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H524" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19249,7 +19253,7 @@
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
@@ -19258,17 +19262,13 @@
         </is>
       </c>
       <c r="E525" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F525" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G525" t="n">
-        <v>0.2377622377622378</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F525" t="inlineStr"/>
+      <c r="G525" t="inlineStr"/>
       <c r="H525" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19285,7 +19285,7 @@
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
@@ -19294,17 +19294,17 @@
         </is>
       </c>
       <c r="E526" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F526" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G526" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H526" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -19321,7 +19321,7 @@
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
@@ -19330,15 +19330,17 @@
         </is>
       </c>
       <c r="E527" t="n">
-        <v>0.3054187192118227</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F527" t="n">
-        <v>0.2517482517482518</v>
-      </c>
-      <c r="G527" t="inlineStr"/>
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G527" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H527" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -19355,7 +19357,7 @@
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
@@ -19364,13 +19366,15 @@
         </is>
       </c>
       <c r="E528" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F528" t="inlineStr"/>
+        <v>0.3054187192118227</v>
+      </c>
+      <c r="F528" t="n">
+        <v>0.2517482517482518</v>
+      </c>
       <c r="G528" t="inlineStr"/>
       <c r="H528" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -19382,31 +19386,27 @@
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E529" t="n">
-        <v>0.2583025830258303</v>
-      </c>
-      <c r="F529" t="n">
-        <v>0.2443438914027149</v>
-      </c>
-      <c r="G529" t="n">
-        <v>0.2191780821917808</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F529" t="inlineStr"/>
+      <c r="G529" t="inlineStr"/>
       <c r="H529" t="inlineStr">
         <is>
-          <t>0.2406 (0.0198)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19423,7 +19423,7 @@
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
@@ -19432,17 +19432,17 @@
         </is>
       </c>
       <c r="E530" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F530" t="n">
-        <v>0.258575197889182</v>
+        <v>0.2443438914027149</v>
       </c>
       <c r="G530" t="n">
-        <v>0.1852861035422343</v>
+        <v>0.2191780821917808</v>
       </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2406 (0.0198)</t>
         </is>
       </c>
     </row>
@@ -19459,7 +19459,7 @@
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D531" t="inlineStr">
@@ -19468,17 +19468,17 @@
         </is>
       </c>
       <c r="E531" t="n">
-        <v>0.16</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F531" t="n">
-        <v>0.2094240837696335</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G531" t="n">
-        <v>0.1619047619047619</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H531" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -19495,7 +19495,7 @@
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D532" t="inlineStr">
@@ -19504,17 +19504,17 @@
         </is>
       </c>
       <c r="E532" t="n">
-        <v>0.2575107296137339</v>
+        <v>0.16</v>
       </c>
       <c r="F532" t="n">
-        <v>0.2989690721649484</v>
+        <v>0.2094240837696335</v>
       </c>
       <c r="G532" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.1619047619047619</v>
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>0.2825 (0.0220)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -19531,7 +19531,7 @@
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
@@ -19540,17 +19540,17 @@
         </is>
       </c>
       <c r="E533" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F533" t="n">
-        <v>0.2566371681415929</v>
+        <v>0.2989690721649484</v>
       </c>
       <c r="G533" t="n">
-        <v>0.2551020408163265</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H533" t="inlineStr">
         <is>
-          <t>0.2586 (0.0048)</t>
+          <t>0.2825 (0.0220)</t>
         </is>
       </c>
     </row>
@@ -19562,31 +19562,31 @@
       </c>
       <c r="B534" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D534" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E534" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F534" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2566371681415929</v>
       </c>
       <c r="G534" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.2551020408163265</v>
       </c>
       <c r="H534" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2586 (0.0048)</t>
         </is>
       </c>
     </row>
@@ -19603,7 +19603,7 @@
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
@@ -19612,17 +19612,17 @@
         </is>
       </c>
       <c r="E535" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F535" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G535" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -19639,7 +19639,7 @@
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
@@ -19648,17 +19648,17 @@
         </is>
       </c>
       <c r="E536" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F536" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G536" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H536" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -19675,7 +19675,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
@@ -19684,17 +19684,17 @@
         </is>
       </c>
       <c r="E537" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F537" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G537" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -19711,7 +19711,7 @@
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
@@ -19720,17 +19720,17 @@
         </is>
       </c>
       <c r="E538" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F538" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G538" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H538" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -19742,31 +19742,31 @@
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E539" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F539" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G539" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H539" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -19783,7 +19783,7 @@
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
@@ -19792,17 +19792,17 @@
         </is>
       </c>
       <c r="E540" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F540" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G540" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H540" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -19819,7 +19819,7 @@
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">
@@ -19828,17 +19828,17 @@
         </is>
       </c>
       <c r="E541" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F541" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G541" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H541" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19855,7 +19855,7 @@
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D542" t="inlineStr">
@@ -19864,17 +19864,17 @@
         </is>
       </c>
       <c r="E542" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F542" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G542" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H542" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -19891,24 +19891,60 @@
       </c>
       <c r="C543" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E543" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F543" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G543" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D543" t="inlineStr">
+      <c r="D544" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E543" t="n">
+      <c r="E544" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F543" t="n">
+      <c r="F544" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G543" t="n">
+      <c r="G544" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H543" t="inlineStr">
+      <c r="H544" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-06 23:52:12)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -17774,11 +17774,13 @@
       <c r="E483" t="n">
         <v>0.3988603988603989</v>
       </c>
-      <c r="F483" t="inlineStr"/>
+      <c r="F483" t="n">
+        <v>0.4313725490196079</v>
+      </c>
       <c r="G483" t="inlineStr"/>
       <c r="H483" t="inlineStr">
         <is>
-          <t>0.3989 (0.0000)</t>
+          <t>0.4151 (0.0230)</t>
         </is>
       </c>
     </row>
@@ -18552,11 +18554,13 @@
       <c r="E505" t="n">
         <v>0.2727272727272727</v>
       </c>
-      <c r="F505" t="inlineStr"/>
+      <c r="F505" t="n">
+        <v>0.2421875</v>
+      </c>
       <c r="G505" t="inlineStr"/>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2727 (0.0000)</t>
+          <t>0.2575 (0.0216)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-07 00:52:31)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H544"/>
+  <dimension ref="A1:H545"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17828,31 +17828,27 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.5080831408775982</v>
-      </c>
-      <c r="F485" t="n">
-        <v>0.4013605442176871</v>
-      </c>
-      <c r="G485" t="n">
-        <v>0.4327176781002638</v>
-      </c>
+        <v>0.3816793893129771</v>
+      </c>
+      <c r="F485" t="inlineStr"/>
+      <c r="G485" t="inlineStr"/>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.4474 (0.0549)</t>
+          <t>0.3817 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17869,7 +17865,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -17878,17 +17874,17 @@
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.4822695035460993</v>
+        <v>0.5080831408775982</v>
       </c>
       <c r="F486" t="n">
-        <v>0.4904632152588556</v>
+        <v>0.4013605442176871</v>
       </c>
       <c r="G486" t="n">
-        <v>0.4634920634920635</v>
+        <v>0.4327176781002638</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.4787 (0.0138)</t>
+          <t>0.4474 (0.0549)</t>
         </is>
       </c>
     </row>
@@ -17905,7 +17901,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17914,17 +17910,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.4</v>
+        <v>0.4822695035460993</v>
       </c>
       <c r="F487" t="n">
-        <v>0.3867069486404834</v>
+        <v>0.4904632152588556</v>
       </c>
       <c r="G487" t="n">
-        <v>0.3094339622641509</v>
+        <v>0.4634920634920635</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.3654 (0.0489)</t>
+          <t>0.4787 (0.0138)</t>
         </is>
       </c>
     </row>
@@ -17941,7 +17937,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17950,17 +17946,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.5801217038539553</v>
+        <v>0.4</v>
       </c>
       <c r="F488" t="n">
-        <v>0.5185185185185185</v>
+        <v>0.3867069486404834</v>
       </c>
       <c r="G488" t="n">
-        <v>0.5128205128205128</v>
+        <v>0.3094339622641509</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.5372 (0.0373)</t>
+          <t>0.3654 (0.0489)</t>
         </is>
       </c>
     </row>
@@ -17977,7 +17973,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17986,17 +17982,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.4698795180722892</v>
+        <v>0.5801217038539553</v>
       </c>
       <c r="F489" t="n">
-        <v>0.303030303030303</v>
+        <v>0.5185185185185185</v>
       </c>
       <c r="G489" t="n">
-        <v>0.3675213675213675</v>
+        <v>0.5128205128205128</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.3801 (0.0841)</t>
+          <t>0.5372 (0.0373)</t>
         </is>
       </c>
     </row>
@@ -18008,31 +18004,31 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.4855769230769231</v>
+        <v>0.4698795180722892</v>
       </c>
       <c r="F490" t="n">
-        <v>0.4187725631768953</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G490" t="n">
-        <v>0.3955223880597015</v>
+        <v>0.3675213675213675</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.4333 (0.0467)</t>
+          <t>0.3801 (0.0841)</t>
         </is>
       </c>
     </row>
@@ -18049,7 +18045,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18058,17 +18054,17 @@
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.4839506172839506</v>
+        <v>0.4855769230769231</v>
       </c>
       <c r="F491" t="n">
-        <v>0.4502923976608187</v>
+        <v>0.4187725631768953</v>
       </c>
       <c r="G491" t="n">
-        <v>0.4224422442244224</v>
+        <v>0.3955223880597015</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.4522 (0.0308)</t>
+          <t>0.4333 (0.0467)</t>
         </is>
       </c>
     </row>
@@ -18085,7 +18081,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18094,17 +18090,17 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.3735632183908046</v>
+        <v>0.4839506172839506</v>
       </c>
       <c r="F492" t="n">
-        <v>0.397212543554007</v>
+        <v>0.4502923976608187</v>
       </c>
       <c r="G492" t="n">
-        <v>0.3764705882352941</v>
+        <v>0.4224422442244224</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.3824 (0.0129)</t>
+          <t>0.4522 (0.0308)</t>
         </is>
       </c>
     </row>
@@ -18121,7 +18117,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18130,17 +18126,17 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.5320197044334976</v>
+        <v>0.3735632183908046</v>
       </c>
       <c r="F493" t="n">
-        <v>0.4809384164222874</v>
+        <v>0.397212543554007</v>
       </c>
       <c r="G493" t="n">
-        <v>0.5342465753424658</v>
+        <v>0.3764705882352941</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.5157 (0.0302)</t>
+          <t>0.3824 (0.0129)</t>
         </is>
       </c>
     </row>
@@ -18157,7 +18153,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -18166,53 +18162,53 @@
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.417989417989418</v>
+        <v>0.5320197044334976</v>
       </c>
       <c r="F494" t="n">
-        <v>0.3711340206185567</v>
+        <v>0.4809384164222874</v>
       </c>
       <c r="G494" t="n">
-        <v>0.4564315352697095</v>
+        <v>0.5342465753424658</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.4152 (0.0427)</t>
+          <t>0.5157 (0.0302)</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.2534246575342466</v>
+        <v>0.417989417989418</v>
       </c>
       <c r="F495" t="n">
-        <v>0.302788844621514</v>
+        <v>0.3711340206185567</v>
       </c>
       <c r="G495" t="n">
-        <v>0.2775510204081633</v>
+        <v>0.4564315352697095</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.2779 (0.0247)</t>
+          <t>0.4152 (0.0427)</t>
         </is>
       </c>
     </row>
@@ -18229,7 +18225,7 @@
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
@@ -18238,17 +18234,17 @@
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.2534246575342466</v>
       </c>
       <c r="F496" t="n">
-        <v>0.3161764705882353</v>
+        <v>0.302788844621514</v>
       </c>
       <c r="G496" t="n">
-        <v>0.316205533596838</v>
+        <v>0.2775510204081633</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.3169 (0.0011)</t>
+          <t>0.2779 (0.0247)</t>
         </is>
       </c>
     </row>
@@ -18265,7 +18261,7 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
@@ -18274,17 +18270,17 @@
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.2290748898678414</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F497" t="n">
-        <v>0.256198347107438</v>
+        <v>0.3161764705882353</v>
       </c>
       <c r="G497" t="n">
-        <v>0.2629107981220657</v>
+        <v>0.316205533596838</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.2494 (0.0179)</t>
+          <t>0.3169 (0.0011)</t>
         </is>
       </c>
     </row>
@@ -18301,7 +18297,7 @@
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
@@ -18310,17 +18306,17 @@
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.319327731092437</v>
+        <v>0.2290748898678414</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2845849802371542</v>
+        <v>0.256198347107438</v>
       </c>
       <c r="G498" t="n">
-        <v>0.2331838565022422</v>
+        <v>0.2629107981220657</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2790 (0.0433)</t>
+          <t>0.2494 (0.0179)</t>
         </is>
       </c>
     </row>
@@ -18337,7 +18333,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
@@ -18346,17 +18342,17 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.319327731092437</v>
       </c>
       <c r="F499" t="n">
-        <v>0.2786885245901639</v>
+        <v>0.2845849802371542</v>
       </c>
       <c r="G499" t="n">
-        <v>0.3665338645418327</v>
+        <v>0.2331838565022422</v>
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.3086 (0.0501)</t>
+          <t>0.2790 (0.0433)</t>
         </is>
       </c>
     </row>
@@ -18368,27 +18364,31 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.2788461538461539</v>
-      </c>
-      <c r="F500" t="inlineStr"/>
-      <c r="G500" t="inlineStr"/>
+        <v>0.2807017543859649</v>
+      </c>
+      <c r="F500" t="n">
+        <v>0.2786885245901639</v>
+      </c>
+      <c r="G500" t="n">
+        <v>0.3665338645418327</v>
+      </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.2788 (0.0000)</t>
+          <t>0.3086 (0.0501)</t>
         </is>
       </c>
     </row>
@@ -18405,7 +18405,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
@@ -18414,17 +18414,13 @@
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.3497757847533632</v>
-      </c>
-      <c r="F501" t="n">
-        <v>0.2918454935622318</v>
-      </c>
-      <c r="G501" t="n">
-        <v>0.3255813953488372</v>
-      </c>
+        <v>0.2788461538461539</v>
+      </c>
+      <c r="F501" t="inlineStr"/>
+      <c r="G501" t="inlineStr"/>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.3224 (0.0291)</t>
+          <t>0.2788 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18441,7 +18437,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -18450,17 +18446,17 @@
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.2054054054054054</v>
+        <v>0.3497757847533632</v>
       </c>
       <c r="F502" t="n">
-        <v>0.2408376963350785</v>
+        <v>0.2918454935622318</v>
       </c>
       <c r="G502" t="n">
-        <v>0.2346368715083799</v>
+        <v>0.3255813953488372</v>
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.2270 (0.0189)</t>
+          <t>0.3224 (0.0291)</t>
         </is>
       </c>
     </row>
@@ -18477,7 +18473,7 @@
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -18486,15 +18482,17 @@
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.3643122676579926</v>
+        <v>0.2054054054054054</v>
       </c>
       <c r="F503" t="n">
-        <v>0.3203883495145631</v>
-      </c>
-      <c r="G503" t="inlineStr"/>
+        <v>0.2408376963350785</v>
+      </c>
+      <c r="G503" t="n">
+        <v>0.2346368715083799</v>
+      </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.3424 (0.0311)</t>
+          <t>0.2270 (0.0189)</t>
         </is>
       </c>
     </row>
@@ -18511,7 +18509,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
@@ -18520,13 +18518,15 @@
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.2650602409638554</v>
-      </c>
-      <c r="F504" t="inlineStr"/>
+        <v>0.3643122676579926</v>
+      </c>
+      <c r="F504" t="n">
+        <v>0.3203883495145631</v>
+      </c>
       <c r="G504" t="inlineStr"/>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.2651 (0.0000)</t>
+          <t>0.3424 (0.0311)</t>
         </is>
       </c>
     </row>
@@ -18538,29 +18538,27 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2727272727272727</v>
-      </c>
-      <c r="F505" t="n">
-        <v>0.2421875</v>
-      </c>
+        <v>0.2650602409638554</v>
+      </c>
+      <c r="F505" t="inlineStr"/>
       <c r="G505" t="inlineStr"/>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2575 (0.0216)</t>
+          <t>0.2651 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18577,7 +18575,7 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
@@ -18586,17 +18584,15 @@
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.2929292929292929</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="F506" t="n">
-        <v>0.2972292191435768</v>
-      </c>
-      <c r="G506" t="n">
-        <v>0.3169398907103825</v>
-      </c>
+        <v>0.2421875</v>
+      </c>
+      <c r="G506" t="inlineStr"/>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.3024 (0.0128)</t>
+          <t>0.2575 (0.0216)</t>
         </is>
       </c>
     </row>
@@ -18613,7 +18609,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18622,17 +18618,17 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="F507" t="n">
-        <v>0.2433460076045627</v>
+        <v>0.2972292191435768</v>
       </c>
       <c r="G507" t="n">
-        <v>0.2704918032786885</v>
+        <v>0.3169398907103825</v>
       </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.2476 (0.0212)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -18649,7 +18645,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
@@ -18658,15 +18654,17 @@
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.3179916317991632</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="F508" t="n">
-        <v>0.3206106870229007</v>
-      </c>
-      <c r="G508" t="inlineStr"/>
+        <v>0.2433460076045627</v>
+      </c>
+      <c r="G508" t="n">
+        <v>0.2704918032786885</v>
+      </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.3193 (0.0019)</t>
+          <t>0.2476 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18683,7 +18681,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
@@ -18692,15 +18690,15 @@
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.3179916317991632</v>
       </c>
       <c r="F509" t="n">
-        <v>0.247787610619469</v>
+        <v>0.3206106870229007</v>
       </c>
       <c r="G509" t="inlineStr"/>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.2350 (0.0181)</t>
+          <t>0.3193 (0.0019)</t>
         </is>
       </c>
     </row>
@@ -18712,31 +18710,31 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.2923076923076923</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="F510" t="n">
-        <v>0.2844444444444444</v>
+        <v>0.247787610619469</v>
       </c>
       <c r="G510" t="n">
-        <v>0.2627737226277372</v>
+        <v>0.3055555555555556</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.2585 (0.0427)</t>
         </is>
       </c>
     </row>
@@ -18753,7 +18751,7 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
@@ -18762,17 +18760,17 @@
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F511" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G511" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -18789,7 +18787,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -18798,17 +18796,17 @@
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F512" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G512" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -18825,7 +18823,7 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
@@ -18834,17 +18832,17 @@
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F513" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G513" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -18861,7 +18859,7 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
@@ -18870,17 +18868,17 @@
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F514" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G514" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18892,31 +18890,31 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F515" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G515" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -18933,7 +18931,7 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
@@ -18942,17 +18940,17 @@
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F516" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="G516" t="n">
-        <v>0.3723404255319149</v>
+        <v>0.2482758620689655</v>
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.3291 (0.0447)</t>
+          <t>0.2753 (0.0283)</t>
         </is>
       </c>
     </row>
@@ -18969,7 +18967,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
@@ -18978,17 +18976,17 @@
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.3317535545023697</v>
       </c>
       <c r="F517" t="n">
-        <v>0.2159090909090909</v>
+        <v>0.2831050228310502</v>
       </c>
       <c r="G517" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.3723404255319149</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>0.2130 (0.0299)</t>
+          <t>0.3291 (0.0447)</t>
         </is>
       </c>
     </row>
@@ -19005,7 +19003,7 @@
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
@@ -19014,17 +19012,17 @@
         </is>
       </c>
       <c r="E518" t="n">
-        <v>0.3444976076555024</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F518" t="n">
-        <v>0.3265306122448979</v>
+        <v>0.2159090909090909</v>
       </c>
       <c r="G518" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.2413793103448276</v>
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>0.3449 (0.0186)</t>
+          <t>0.2130 (0.0299)</t>
         </is>
       </c>
     </row>
@@ -19041,7 +19039,7 @@
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
@@ -19050,53 +19048,53 @@
         </is>
       </c>
       <c r="E519" t="n">
-        <v>0.225</v>
+        <v>0.3444976076555024</v>
       </c>
       <c r="F519" t="n">
-        <v>0.2281879194630873</v>
+        <v>0.3265306122448979</v>
       </c>
       <c r="G519" t="n">
-        <v>0.2676056338028169</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>0.2403 (0.0237)</t>
+          <t>0.3449 (0.0186)</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PGC_ERR_Antagonist</t>
         </is>
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E520" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.225</v>
       </c>
       <c r="F520" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.2281879194630873</v>
       </c>
       <c r="G520" t="n">
-        <v>0.228310502283105</v>
+        <v>0.2676056338028169</v>
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.2403 (0.0237)</t>
         </is>
       </c>
     </row>
@@ -19113,7 +19111,7 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
@@ -19122,17 +19120,17 @@
         </is>
       </c>
       <c r="E521" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F521" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G521" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -19149,7 +19147,7 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
@@ -19158,17 +19156,17 @@
         </is>
       </c>
       <c r="E522" t="n">
-        <v>0.2135922330097087</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F522" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G522" t="n">
-        <v>0.1616161616161616</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H522" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -19185,7 +19183,7 @@
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
@@ -19194,17 +19192,17 @@
         </is>
       </c>
       <c r="E523" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2135922330097087</v>
       </c>
       <c r="F523" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="G523" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.1616161616161616</v>
       </c>
       <c r="H523" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -19221,7 +19219,7 @@
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
@@ -19230,17 +19228,17 @@
         </is>
       </c>
       <c r="E524" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F524" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G524" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H524" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -19252,27 +19250,31 @@
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E525" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F525" t="inlineStr"/>
-      <c r="G525" t="inlineStr"/>
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F525" t="n">
+        <v>0.2383419689119171</v>
+      </c>
+      <c r="G525" t="n">
+        <v>0.1940928270042194</v>
+      </c>
       <c r="H525" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19289,7 +19291,7 @@
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
@@ -19298,17 +19300,13 @@
         </is>
       </c>
       <c r="E526" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="F526" t="n">
-        <v>0.2592592592592592</v>
-      </c>
-      <c r="G526" t="n">
-        <v>0.2377622377622378</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F526" t="inlineStr"/>
+      <c r="G526" t="inlineStr"/>
       <c r="H526" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19325,7 +19323,7 @@
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
@@ -19334,17 +19332,17 @@
         </is>
       </c>
       <c r="E527" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F527" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="G527" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.2377622377622378</v>
       </c>
       <c r="H527" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -19361,7 +19359,7 @@
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
@@ -19370,15 +19368,17 @@
         </is>
       </c>
       <c r="E528" t="n">
-        <v>0.3054187192118227</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F528" t="n">
-        <v>0.2517482517482518</v>
-      </c>
-      <c r="G528" t="inlineStr"/>
+        <v>0.2027027027027027</v>
+      </c>
+      <c r="G528" t="n">
+        <v>0.2138364779874214</v>
+      </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
@@ -19404,13 +19404,15 @@
         </is>
       </c>
       <c r="E529" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F529" t="inlineStr"/>
+        <v>0.3054187192118227</v>
+      </c>
+      <c r="F529" t="n">
+        <v>0.2517482517482518</v>
+      </c>
       <c r="G529" t="inlineStr"/>
       <c r="H529" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -19422,31 +19424,27 @@
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E530" t="n">
-        <v>0.2583025830258303</v>
-      </c>
-      <c r="F530" t="n">
-        <v>0.2443438914027149</v>
-      </c>
-      <c r="G530" t="n">
-        <v>0.2191780821917808</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F530" t="inlineStr"/>
+      <c r="G530" t="inlineStr"/>
       <c r="H530" t="inlineStr">
         <is>
-          <t>0.2406 (0.0198)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19463,7 +19461,7 @@
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D531" t="inlineStr">
@@ -19472,17 +19470,17 @@
         </is>
       </c>
       <c r="E531" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F531" t="n">
-        <v>0.258575197889182</v>
+        <v>0.2443438914027149</v>
       </c>
       <c r="G531" t="n">
-        <v>0.1852861035422343</v>
+        <v>0.2191780821917808</v>
       </c>
       <c r="H531" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2406 (0.0198)</t>
         </is>
       </c>
     </row>
@@ -19499,7 +19497,7 @@
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D532" t="inlineStr">
@@ -19508,17 +19506,17 @@
         </is>
       </c>
       <c r="E532" t="n">
-        <v>0.16</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F532" t="n">
-        <v>0.2094240837696335</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G532" t="n">
-        <v>0.1619047619047619</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -19535,7 +19533,7 @@
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
@@ -19544,17 +19542,17 @@
         </is>
       </c>
       <c r="E533" t="n">
-        <v>0.2575107296137339</v>
+        <v>0.16</v>
       </c>
       <c r="F533" t="n">
-        <v>0.2989690721649484</v>
+        <v>0.2094240837696335</v>
       </c>
       <c r="G533" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.1619047619047619</v>
       </c>
       <c r="H533" t="inlineStr">
         <is>
-          <t>0.2825 (0.0220)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -19571,7 +19569,7 @@
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D534" t="inlineStr">
@@ -19580,17 +19578,17 @@
         </is>
       </c>
       <c r="E534" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F534" t="n">
-        <v>0.2566371681415929</v>
+        <v>0.2989690721649484</v>
       </c>
       <c r="G534" t="n">
-        <v>0.2551020408163265</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H534" t="inlineStr">
         <is>
-          <t>0.2586 (0.0048)</t>
+          <t>0.2825 (0.0220)</t>
         </is>
       </c>
     </row>
@@ -19602,31 +19600,31 @@
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E535" t="n">
-        <v>0.196078431372549</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F535" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2566371681415929</v>
       </c>
       <c r="G535" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.2551020408163265</v>
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.2586 (0.0048)</t>
         </is>
       </c>
     </row>
@@ -19643,7 +19641,7 @@
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
@@ -19652,17 +19650,17 @@
         </is>
       </c>
       <c r="E536" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F536" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G536" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H536" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -19679,7 +19677,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
@@ -19688,17 +19686,17 @@
         </is>
       </c>
       <c r="E537" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F537" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G537" t="n">
-        <v>0.125</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -19715,7 +19713,7 @@
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
@@ -19724,17 +19722,17 @@
         </is>
       </c>
       <c r="E538" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F538" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G538" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.125</v>
       </c>
       <c r="H538" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -19751,7 +19749,7 @@
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
@@ -19760,17 +19758,17 @@
         </is>
       </c>
       <c r="E539" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F539" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G539" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H539" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -19782,31 +19780,31 @@
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E540" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F540" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G540" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H540" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -19823,7 +19821,7 @@
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">
@@ -19832,17 +19830,17 @@
         </is>
       </c>
       <c r="E541" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F541" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G541" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H541" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -19859,7 +19857,7 @@
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D542" t="inlineStr">
@@ -19868,17 +19866,17 @@
         </is>
       </c>
       <c r="E542" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.2087912087912088</v>
       </c>
       <c r="F542" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2738095238095238</v>
       </c>
       <c r="G542" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.2705882352941176</v>
       </c>
       <c r="H542" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.2511 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19895,7 +19893,7 @@
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D543" t="inlineStr">
@@ -19904,17 +19902,17 @@
         </is>
       </c>
       <c r="E543" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="F543" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2297297297297297</v>
       </c>
       <c r="G543" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.1654135338345865</v>
       </c>
       <c r="H543" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.1830 (0.0409)</t>
         </is>
       </c>
     </row>
@@ -19931,24 +19929,60 @@
       </c>
       <c r="C544" t="inlineStr">
         <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E544" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F544" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G544" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D544" t="inlineStr">
+      <c r="D545" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E544" t="n">
+      <c r="E545" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F544" t="n">
+      <c r="F545" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G544" t="n">
+      <c r="G545" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H544" t="inlineStr">
+      <c r="H545" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-07 01:52:49)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H545"/>
+  <dimension ref="A1:H548"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18695,10 +18695,12 @@
       <c r="F509" t="n">
         <v>0.3206106870229007</v>
       </c>
-      <c r="G509" t="inlineStr"/>
+      <c r="G509" t="n">
+        <v>0.3728813559322034</v>
+      </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.3193 (0.0019)</t>
+          <t>0.3372 (0.0310)</t>
         </is>
       </c>
     </row>
@@ -19101,7 +19103,7 @@
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PR_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B521" t="inlineStr">
@@ -19111,7 +19113,7 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
@@ -19120,24 +19122,24 @@
         </is>
       </c>
       <c r="E521" t="n">
-        <v>0.2595419847328244</v>
+        <v>0.5421903052064632</v>
       </c>
       <c r="F521" t="n">
-        <v>0.2164948453608248</v>
+        <v>0.4725738396624473</v>
       </c>
       <c r="G521" t="n">
-        <v>0.228310502283105</v>
+        <v>0.5</v>
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>0.2348 (0.0222)</t>
+          <t>0.5049 (0.0351)</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PR_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B522" t="inlineStr">
@@ -19147,7 +19149,7 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
@@ -19156,24 +19158,24 @@
         </is>
       </c>
       <c r="E522" t="n">
-        <v>0.2322097378277154</v>
+        <v>0.4712643678160919</v>
       </c>
       <c r="F522" t="n">
-        <v>0.2212389380530974</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="G522" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.4718614718614719</v>
       </c>
       <c r="H522" t="inlineStr">
         <is>
-          <t>0.2274 (0.0056)</t>
+          <t>0.4699 (0.0028)</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>TOX21_p53_BLA_p2_ratio</t>
+          <t>TOX21_PR_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B523" t="inlineStr">
@@ -19183,7 +19185,7 @@
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
@@ -19192,17 +19194,13 @@
         </is>
       </c>
       <c r="E523" t="n">
-        <v>0.2135922330097087</v>
-      </c>
-      <c r="F523" t="n">
-        <v>0.2307692307692308</v>
-      </c>
-      <c r="G523" t="n">
-        <v>0.1616161616161616</v>
-      </c>
+        <v>0.5263157894736842</v>
+      </c>
+      <c r="F523" t="inlineStr"/>
+      <c r="G523" t="inlineStr"/>
       <c r="H523" t="inlineStr">
         <is>
-          <t>0.2020 (0.0360)</t>
+          <t>0.5263 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19219,7 +19217,7 @@
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
@@ -19228,17 +19226,17 @@
         </is>
       </c>
       <c r="E524" t="n">
-        <v>0.2683982683982684</v>
+        <v>0.2595419847328244</v>
       </c>
       <c r="F524" t="n">
-        <v>0.2333333333333333</v>
+        <v>0.2164948453608248</v>
       </c>
       <c r="G524" t="n">
-        <v>0.2046511627906977</v>
+        <v>0.228310502283105</v>
       </c>
       <c r="H524" t="inlineStr">
         <is>
-          <t>0.2355 (0.0319)</t>
+          <t>0.2348 (0.0222)</t>
         </is>
       </c>
     </row>
@@ -19255,7 +19253,7 @@
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
@@ -19264,17 +19262,17 @@
         </is>
       </c>
       <c r="E525" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2322097378277154</v>
       </c>
       <c r="F525" t="n">
-        <v>0.2383419689119171</v>
+        <v>0.2212389380530974</v>
       </c>
       <c r="G525" t="n">
-        <v>0.1940928270042194</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="H525" t="inlineStr">
         <is>
-          <t>0.2330 (0.0366)</t>
+          <t>0.2274 (0.0056)</t>
         </is>
       </c>
     </row>
@@ -19286,27 +19284,31 @@
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E526" t="n">
-        <v>0.2487046632124352</v>
-      </c>
-      <c r="F526" t="inlineStr"/>
-      <c r="G526" t="inlineStr"/>
+        <v>0.2135922330097087</v>
+      </c>
+      <c r="F526" t="n">
+        <v>0.2307692307692308</v>
+      </c>
+      <c r="G526" t="n">
+        <v>0.1616161616161616</v>
+      </c>
       <c r="H526" t="inlineStr">
         <is>
-          <t>0.2487 (0.0000)</t>
+          <t>0.2020 (0.0360)</t>
         </is>
       </c>
     </row>
@@ -19318,31 +19320,31 @@
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E527" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2683982683982684</v>
       </c>
       <c r="F527" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="G527" t="n">
-        <v>0.2377622377622378</v>
+        <v>0.2046511627906977</v>
       </c>
       <c r="H527" t="inlineStr">
         <is>
-          <t>0.2534 (0.0137)</t>
+          <t>0.2355 (0.0319)</t>
         </is>
       </c>
     </row>
@@ -19354,31 +19356,31 @@
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E528" t="n">
-        <v>0.163265306122449</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="F528" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2383419689119171</v>
       </c>
       <c r="G528" t="n">
-        <v>0.2138364779874214</v>
+        <v>0.1940928270042194</v>
       </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>0.1933 (0.0266)</t>
+          <t>0.2330 (0.0366)</t>
         </is>
       </c>
     </row>
@@ -19395,7 +19397,7 @@
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
@@ -19404,15 +19406,13 @@
         </is>
       </c>
       <c r="E529" t="n">
-        <v>0.3054187192118227</v>
-      </c>
-      <c r="F529" t="n">
-        <v>0.2517482517482518</v>
-      </c>
+        <v>0.2487046632124352</v>
+      </c>
+      <c r="F529" t="inlineStr"/>
       <c r="G529" t="inlineStr"/>
       <c r="H529" t="inlineStr">
         <is>
-          <t>0.2786 (0.0380)</t>
+          <t>0.2487 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19429,7 +19429,7 @@
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
@@ -19438,13 +19438,17 @@
         </is>
       </c>
       <c r="E530" t="n">
-        <v>0.198581560283688</v>
-      </c>
-      <c r="F530" t="inlineStr"/>
-      <c r="G530" t="inlineStr"/>
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="F530" t="n">
+        <v>0.2592592592592592</v>
+      </c>
+      <c r="G530" t="n">
+        <v>0.2377622377622378</v>
+      </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>0.1986 (0.0000)</t>
+          <t>0.2534 (0.0137)</t>
         </is>
       </c>
     </row>
@@ -19456,31 +19460,31 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D531" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E531" t="n">
-        <v>0.2583025830258303</v>
+        <v>0.163265306122449</v>
       </c>
       <c r="F531" t="n">
-        <v>0.2443438914027149</v>
+        <v>0.2027027027027027</v>
       </c>
       <c r="G531" t="n">
-        <v>0.2191780821917808</v>
+        <v>0.2138364779874214</v>
       </c>
       <c r="H531" t="inlineStr">
         <is>
-          <t>0.2406 (0.0198)</t>
+          <t>0.1933 (0.0266)</t>
         </is>
       </c>
     </row>
@@ -19492,31 +19496,29 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D532" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E532" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.3054187192118227</v>
       </c>
       <c r="F532" t="n">
-        <v>0.258575197889182</v>
-      </c>
-      <c r="G532" t="n">
-        <v>0.1852861035422343</v>
-      </c>
+        <v>0.2517482517482518</v>
+      </c>
+      <c r="G532" t="inlineStr"/>
       <c r="H532" t="inlineStr">
         <is>
-          <t>0.2395 (0.0477)</t>
+          <t>0.2786 (0.0380)</t>
         </is>
       </c>
     </row>
@@ -19528,31 +19530,27 @@
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E533" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="F533" t="n">
-        <v>0.2094240837696335</v>
-      </c>
-      <c r="G533" t="n">
-        <v>0.1619047619047619</v>
-      </c>
+        <v>0.198581560283688</v>
+      </c>
+      <c r="F533" t="inlineStr"/>
+      <c r="G533" t="inlineStr"/>
       <c r="H533" t="inlineStr">
         <is>
-          <t>0.1771 (0.0280)</t>
+          <t>0.1986 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -19569,7 +19567,7 @@
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D534" t="inlineStr">
@@ -19578,17 +19576,17 @@
         </is>
       </c>
       <c r="E534" t="n">
-        <v>0.2575107296137339</v>
+        <v>0.2583025830258303</v>
       </c>
       <c r="F534" t="n">
-        <v>0.2989690721649484</v>
+        <v>0.2443438914027149</v>
       </c>
       <c r="G534" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.2191780821917808</v>
       </c>
       <c r="H534" t="inlineStr">
         <is>
-          <t>0.2825 (0.0220)</t>
+          <t>0.2406 (0.0198)</t>
         </is>
       </c>
     </row>
@@ -19605,7 +19603,7 @@
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
@@ -19614,17 +19612,17 @@
         </is>
       </c>
       <c r="E535" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2747252747252747</v>
       </c>
       <c r="F535" t="n">
-        <v>0.2566371681415929</v>
+        <v>0.258575197889182</v>
       </c>
       <c r="G535" t="n">
-        <v>0.2551020408163265</v>
+        <v>0.1852861035422343</v>
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>0.2586 (0.0048)</t>
+          <t>0.2395 (0.0477)</t>
         </is>
       </c>
     </row>
@@ -19636,31 +19634,31 @@
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E536" t="n">
-        <v>0.196078431372549</v>
+        <v>0.16</v>
       </c>
       <c r="F536" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2094240837696335</v>
       </c>
       <c r="G536" t="n">
-        <v>0.1379310344827586</v>
+        <v>0.1619047619047619</v>
       </c>
       <c r="H536" t="inlineStr">
         <is>
-          <t>0.1836 (0.0408)</t>
+          <t>0.1771 (0.0280)</t>
         </is>
       </c>
     </row>
@@ -19672,31 +19670,31 @@
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E537" t="n">
-        <v>0.2358974358974359</v>
+        <v>0.2575107296137339</v>
       </c>
       <c r="F537" t="n">
-        <v>0.2840909090909091</v>
+        <v>0.2989690721649484</v>
       </c>
       <c r="G537" t="n">
-        <v>0.2153846153846154</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>0.2451 (0.0353)</t>
+          <t>0.2825 (0.0220)</t>
         </is>
       </c>
     </row>
@@ -19708,31 +19706,31 @@
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E538" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.2641509433962264</v>
       </c>
       <c r="F538" t="n">
-        <v>0.1746031746031746</v>
+        <v>0.2566371681415929</v>
       </c>
       <c r="G538" t="n">
-        <v>0.125</v>
+        <v>0.2551020408163265</v>
       </c>
       <c r="H538" t="inlineStr">
         <is>
-          <t>0.1570 (0.0278)</t>
+          <t>0.2586 (0.0048)</t>
         </is>
       </c>
     </row>
@@ -19749,7 +19747,7 @@
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
@@ -19758,17 +19756,17 @@
         </is>
       </c>
       <c r="E539" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.196078431372549</v>
       </c>
       <c r="F539" t="n">
-        <v>0.3091787439613526</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G539" t="n">
-        <v>0.1438848920863309</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="H539" t="inlineStr">
         <is>
-          <t>0.2634 (0.1044)</t>
+          <t>0.1836 (0.0408)</t>
         </is>
       </c>
     </row>
@@ -19785,7 +19783,7 @@
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
@@ -19794,17 +19792,17 @@
         </is>
       </c>
       <c r="E540" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F540" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.2840909090909091</v>
       </c>
       <c r="G540" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="H540" t="inlineStr">
         <is>
-          <t>0.1585 (0.0316)</t>
+          <t>0.2451 (0.0353)</t>
         </is>
       </c>
     </row>
@@ -19816,31 +19814,31 @@
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E541" t="n">
-        <v>0.232258064516129</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F541" t="n">
-        <v>0.2385321100917431</v>
+        <v>0.1746031746031746</v>
       </c>
       <c r="G541" t="n">
-        <v>0.2131147540983606</v>
+        <v>0.125</v>
       </c>
       <c r="H541" t="inlineStr">
         <is>
-          <t>0.2280 (0.0132)</t>
+          <t>0.1570 (0.0278)</t>
         </is>
       </c>
     </row>
@@ -19852,31 +19850,31 @@
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D542" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E542" t="n">
-        <v>0.2087912087912088</v>
+        <v>0.3370786516853932</v>
       </c>
       <c r="F542" t="n">
-        <v>0.2738095238095238</v>
+        <v>0.3091787439613526</v>
       </c>
       <c r="G542" t="n">
-        <v>0.2705882352941176</v>
+        <v>0.1438848920863309</v>
       </c>
       <c r="H542" t="inlineStr">
         <is>
-          <t>0.2511 (0.0366)</t>
+          <t>0.2634 (0.1044)</t>
         </is>
       </c>
     </row>
@@ -19888,31 +19886,31 @@
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D543" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E543" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="F543" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="G543" t="n">
-        <v>0.1654135338345865</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="H543" t="inlineStr">
         <is>
-          <t>0.1830 (0.0409)</t>
+          <t>0.1585 (0.0316)</t>
         </is>
       </c>
     </row>
@@ -19929,7 +19927,7 @@
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D544" t="inlineStr">
@@ -19938,17 +19936,17 @@
         </is>
       </c>
       <c r="E544" t="n">
-        <v>0.2259887005649718</v>
+        <v>0.232258064516129</v>
       </c>
       <c r="F544" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2385321100917431</v>
       </c>
       <c r="G544" t="n">
-        <v>0.1728395061728395</v>
+        <v>0.2131147540983606</v>
       </c>
       <c r="H544" t="inlineStr">
         <is>
-          <t>0.2114 (0.0337)</t>
+          <t>0.2280 (0.0132)</t>
         </is>
       </c>
     </row>
@@ -19965,24 +19963,132 @@
       </c>
       <c r="C545" t="inlineStr">
         <is>
+          <t>MACCS</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E545" t="n">
+        <v>0.2087912087912088</v>
+      </c>
+      <c r="F545" t="n">
+        <v>0.2738095238095238</v>
+      </c>
+      <c r="G545" t="n">
+        <v>0.2705882352941176</v>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>0.2511 (0.0366)</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Morgan</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E546" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="F546" t="n">
+        <v>0.2297297297297297</v>
+      </c>
+      <c r="G546" t="n">
+        <v>0.1654135338345865</v>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>0.1830 (0.0409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E547" t="n">
+        <v>0.2259887005649718</v>
+      </c>
+      <c r="F547" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="G547" t="n">
+        <v>0.1728395061728395</v>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>0.2114 (0.0337)</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>TOX21_p53_BLA_p2_ratio</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>xgb</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
           <t>RDKit</t>
         </is>
       </c>
-      <c r="D545" t="inlineStr">
+      <c r="D548" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E545" t="n">
+      <c r="E548" t="n">
         <v>0.2469135802469136</v>
       </c>
-      <c r="F545" t="n">
+      <c r="F548" t="n">
         <v>0.1651376146788991</v>
       </c>
-      <c r="G545" t="n">
+      <c r="G548" t="n">
         <v>0.1238938053097345</v>
       </c>
-      <c r="H545" t="inlineStr">
+      <c r="H548" t="inlineStr">
         <is>
           <t>0.1786 (0.0626)</t>
         </is>

</xml_diff>

<commit_message>
Logs: auto summary & updates (2025-10-07 02:53:08)
</commit_message>
<xml_diff>
--- a/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
+++ b/ToxCast_model/experiments/training/DART_MTL/logs/seed_multi_best_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H548"/>
+  <dimension ref="A1:H551"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17792,31 +17792,27 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E484" t="n">
-        <v>0.5163636363636364</v>
-      </c>
-      <c r="F484" t="n">
-        <v>0.465587044534413</v>
-      </c>
-      <c r="G484" t="n">
-        <v>0.4183006535947713</v>
-      </c>
+        <v>0.5463659147869674</v>
+      </c>
+      <c r="F484" t="inlineStr"/>
+      <c r="G484" t="inlineStr"/>
       <c r="H484" t="inlineStr">
         <is>
-          <t>0.4668 (0.0490)</t>
+          <t>0.5464 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -17833,7 +17829,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17842,13 +17838,17 @@
         </is>
       </c>
       <c r="E485" t="n">
-        <v>0.3816793893129771</v>
-      </c>
-      <c r="F485" t="inlineStr"/>
-      <c r="G485" t="inlineStr"/>
+        <v>0.5163636363636364</v>
+      </c>
+      <c r="F485" t="n">
+        <v>0.465587044534413</v>
+      </c>
+      <c r="G485" t="n">
+        <v>0.4183006535947713</v>
+      </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>0.3817 (0.0000)</t>
+          <t>0.4668 (0.0490)</t>
         </is>
       </c>
     </row>
@@ -17860,31 +17860,29 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E486" t="n">
-        <v>0.5080831408775982</v>
+        <v>0.3816793893129771</v>
       </c>
       <c r="F486" t="n">
-        <v>0.4013605442176871</v>
-      </c>
-      <c r="G486" t="n">
-        <v>0.4327176781002638</v>
-      </c>
+        <v>0.3822714681440443</v>
+      </c>
+      <c r="G486" t="inlineStr"/>
       <c r="H486" t="inlineStr">
         <is>
-          <t>0.4474 (0.0549)</t>
+          <t>0.3820 (0.0004)</t>
         </is>
       </c>
     </row>
@@ -17901,7 +17899,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -17910,17 +17908,17 @@
         </is>
       </c>
       <c r="E487" t="n">
-        <v>0.4822695035460993</v>
+        <v>0.5080831408775982</v>
       </c>
       <c r="F487" t="n">
-        <v>0.4904632152588556</v>
+        <v>0.4013605442176871</v>
       </c>
       <c r="G487" t="n">
-        <v>0.4634920634920635</v>
+        <v>0.4327176781002638</v>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>0.4787 (0.0138)</t>
+          <t>0.4474 (0.0549)</t>
         </is>
       </c>
     </row>
@@ -17937,7 +17935,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -17946,17 +17944,17 @@
         </is>
       </c>
       <c r="E488" t="n">
-        <v>0.4</v>
+        <v>0.4822695035460993</v>
       </c>
       <c r="F488" t="n">
-        <v>0.3867069486404834</v>
+        <v>0.4904632152588556</v>
       </c>
       <c r="G488" t="n">
-        <v>0.3094339622641509</v>
+        <v>0.4634920634920635</v>
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>0.3654 (0.0489)</t>
+          <t>0.4787 (0.0138)</t>
         </is>
       </c>
     </row>
@@ -17973,7 +17971,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -17982,17 +17980,17 @@
         </is>
       </c>
       <c r="E489" t="n">
-        <v>0.5801217038539553</v>
+        <v>0.4</v>
       </c>
       <c r="F489" t="n">
-        <v>0.5185185185185185</v>
+        <v>0.3867069486404834</v>
       </c>
       <c r="G489" t="n">
-        <v>0.5128205128205128</v>
+        <v>0.3094339622641509</v>
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>0.5372 (0.0373)</t>
+          <t>0.3654 (0.0489)</t>
         </is>
       </c>
     </row>
@@ -18009,7 +18007,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18018,17 +18016,17 @@
         </is>
       </c>
       <c r="E490" t="n">
-        <v>0.4698795180722892</v>
+        <v>0.5801217038539553</v>
       </c>
       <c r="F490" t="n">
-        <v>0.303030303030303</v>
+        <v>0.5185185185185185</v>
       </c>
       <c r="G490" t="n">
-        <v>0.3675213675213675</v>
+        <v>0.5128205128205128</v>
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>0.3801 (0.0841)</t>
+          <t>0.5372 (0.0373)</t>
         </is>
       </c>
     </row>
@@ -18040,31 +18038,31 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E491" t="n">
-        <v>0.4855769230769231</v>
+        <v>0.4698795180722892</v>
       </c>
       <c r="F491" t="n">
-        <v>0.4187725631768953</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G491" t="n">
-        <v>0.3955223880597015</v>
+        <v>0.3675213675213675</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>0.4333 (0.0467)</t>
+          <t>0.3801 (0.0841)</t>
         </is>
       </c>
     </row>
@@ -18081,7 +18079,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18090,17 +18088,17 @@
         </is>
       </c>
       <c r="E492" t="n">
-        <v>0.4839506172839506</v>
+        <v>0.4855769230769231</v>
       </c>
       <c r="F492" t="n">
-        <v>0.4502923976608187</v>
+        <v>0.4187725631768953</v>
       </c>
       <c r="G492" t="n">
-        <v>0.4224422442244224</v>
+        <v>0.3955223880597015</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>0.4522 (0.0308)</t>
+          <t>0.4333 (0.0467)</t>
         </is>
       </c>
     </row>
@@ -18117,7 +18115,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -18126,17 +18124,17 @@
         </is>
       </c>
       <c r="E493" t="n">
-        <v>0.3735632183908046</v>
+        <v>0.4839506172839506</v>
       </c>
       <c r="F493" t="n">
-        <v>0.397212543554007</v>
+        <v>0.4502923976608187</v>
       </c>
       <c r="G493" t="n">
-        <v>0.3764705882352941</v>
+        <v>0.4224422442244224</v>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>0.3824 (0.0129)</t>
+          <t>0.4522 (0.0308)</t>
         </is>
       </c>
     </row>
@@ -18153,7 +18151,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -18162,17 +18160,17 @@
         </is>
       </c>
       <c r="E494" t="n">
-        <v>0.5320197044334976</v>
+        <v>0.3735632183908046</v>
       </c>
       <c r="F494" t="n">
-        <v>0.4809384164222874</v>
+        <v>0.397212543554007</v>
       </c>
       <c r="G494" t="n">
-        <v>0.5342465753424658</v>
+        <v>0.3764705882352941</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>0.5157 (0.0302)</t>
+          <t>0.3824 (0.0129)</t>
         </is>
       </c>
     </row>
@@ -18189,7 +18187,7 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
@@ -18198,53 +18196,53 @@
         </is>
       </c>
       <c r="E495" t="n">
-        <v>0.417989417989418</v>
+        <v>0.5320197044334976</v>
       </c>
       <c r="F495" t="n">
-        <v>0.3711340206185567</v>
+        <v>0.4809384164222874</v>
       </c>
       <c r="G495" t="n">
-        <v>0.4564315352697095</v>
+        <v>0.5342465753424658</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>0.4152 (0.0427)</t>
+          <t>0.5157 (0.0302)</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
         <is>
-          <t>TOX21_PGC_ERR_Antagonist</t>
+          <t>TOX21_ERb_BLA_Antagonist_ratio</t>
         </is>
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>dt</t>
+          <t>xgb</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E496" t="n">
-        <v>0.2534246575342466</v>
+        <v>0.417989417989418</v>
       </c>
       <c r="F496" t="n">
-        <v>0.302788844621514</v>
+        <v>0.3711340206185567</v>
       </c>
       <c r="G496" t="n">
-        <v>0.2775510204081633</v>
+        <v>0.4564315352697095</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>0.2779 (0.0247)</t>
+          <t>0.4152 (0.0427)</t>
         </is>
       </c>
     </row>
@@ -18261,7 +18259,7 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
@@ -18270,17 +18268,17 @@
         </is>
       </c>
       <c r="E497" t="n">
-        <v>0.3181818181818182</v>
+        <v>0.2534246575342466</v>
       </c>
       <c r="F497" t="n">
-        <v>0.3161764705882353</v>
+        <v>0.302788844621514</v>
       </c>
       <c r="G497" t="n">
-        <v>0.316205533596838</v>
+        <v>0.2775510204081633</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>0.3169 (0.0011)</t>
+          <t>0.2779 (0.0247)</t>
         </is>
       </c>
     </row>
@@ -18297,7 +18295,7 @@
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
@@ -18306,17 +18304,17 @@
         </is>
       </c>
       <c r="E498" t="n">
-        <v>0.2290748898678414</v>
+        <v>0.3181818181818182</v>
       </c>
       <c r="F498" t="n">
-        <v>0.256198347107438</v>
+        <v>0.3161764705882353</v>
       </c>
       <c r="G498" t="n">
-        <v>0.2629107981220657</v>
+        <v>0.316205533596838</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>0.2494 (0.0179)</t>
+          <t>0.3169 (0.0011)</t>
         </is>
       </c>
     </row>
@@ -18333,7 +18331,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
@@ -18342,17 +18340,17 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>0.319327731092437</v>
+        <v>0.2290748898678414</v>
       </c>
       <c r="F499" t="n">
-        <v>0.2845849802371542</v>
+        <v>0.256198347107438</v>
       </c>
       <c r="G499" t="n">
-        <v>0.2331838565022422</v>
+        <v>0.2629107981220657</v>
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>0.2790 (0.0433)</t>
+          <t>0.2494 (0.0179)</t>
         </is>
       </c>
     </row>
@@ -18369,7 +18367,7 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
@@ -18378,17 +18376,17 @@
         </is>
       </c>
       <c r="E500" t="n">
-        <v>0.2807017543859649</v>
+        <v>0.319327731092437</v>
       </c>
       <c r="F500" t="n">
-        <v>0.2786885245901639</v>
+        <v>0.2845849802371542</v>
       </c>
       <c r="G500" t="n">
-        <v>0.3665338645418327</v>
+        <v>0.2331838565022422</v>
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>0.3086 (0.0501)</t>
+          <t>0.2790 (0.0433)</t>
         </is>
       </c>
     </row>
@@ -18400,27 +18398,31 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>gbt</t>
+          <t>dt</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="E501" t="n">
-        <v>0.2788461538461539</v>
-      </c>
-      <c r="F501" t="inlineStr"/>
-      <c r="G501" t="inlineStr"/>
+        <v>0.2807017543859649</v>
+      </c>
+      <c r="F501" t="n">
+        <v>0.2786885245901639</v>
+      </c>
+      <c r="G501" t="n">
+        <v>0.3665338645418327</v>
+      </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>0.2788 (0.0000)</t>
+          <t>0.3086 (0.0501)</t>
         </is>
       </c>
     </row>
@@ -18437,7 +18439,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -18446,17 +18448,13 @@
         </is>
       </c>
       <c r="E502" t="n">
-        <v>0.3497757847533632</v>
-      </c>
-      <c r="F502" t="n">
-        <v>0.2918454935622318</v>
-      </c>
-      <c r="G502" t="n">
-        <v>0.3255813953488372</v>
-      </c>
+        <v>0.2788461538461539</v>
+      </c>
+      <c r="F502" t="inlineStr"/>
+      <c r="G502" t="inlineStr"/>
       <c r="H502" t="inlineStr">
         <is>
-          <t>0.3224 (0.0291)</t>
+          <t>0.2788 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18473,7 +18471,7 @@
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -18482,17 +18480,17 @@
         </is>
       </c>
       <c r="E503" t="n">
-        <v>0.2054054054054054</v>
+        <v>0.3497757847533632</v>
       </c>
       <c r="F503" t="n">
-        <v>0.2408376963350785</v>
+        <v>0.2918454935622318</v>
       </c>
       <c r="G503" t="n">
-        <v>0.2346368715083799</v>
+        <v>0.3255813953488372</v>
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>0.2270 (0.0189)</t>
+          <t>0.3224 (0.0291)</t>
         </is>
       </c>
     </row>
@@ -18509,7 +18507,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
@@ -18518,15 +18516,17 @@
         </is>
       </c>
       <c r="E504" t="n">
-        <v>0.3643122676579926</v>
+        <v>0.2054054054054054</v>
       </c>
       <c r="F504" t="n">
-        <v>0.3203883495145631</v>
-      </c>
-      <c r="G504" t="inlineStr"/>
+        <v>0.2408376963350785</v>
+      </c>
+      <c r="G504" t="n">
+        <v>0.2346368715083799</v>
+      </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>0.3424 (0.0311)</t>
+          <t>0.2270 (0.0189)</t>
         </is>
       </c>
     </row>
@@ -18543,7 +18543,7 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
@@ -18552,13 +18552,15 @@
         </is>
       </c>
       <c r="E505" t="n">
-        <v>0.2650602409638554</v>
-      </c>
-      <c r="F505" t="inlineStr"/>
+        <v>0.3643122676579926</v>
+      </c>
+      <c r="F505" t="n">
+        <v>0.3203883495145631</v>
+      </c>
       <c r="G505" t="inlineStr"/>
       <c r="H505" t="inlineStr">
         <is>
-          <t>0.2651 (0.0000)</t>
+          <t>0.3424 (0.0311)</t>
         </is>
       </c>
     </row>
@@ -18570,29 +18572,27 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>logistic</t>
+          <t>gbt</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>LogisticRegression</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="E506" t="n">
-        <v>0.2727272727272727</v>
-      </c>
-      <c r="F506" t="n">
-        <v>0.2421875</v>
-      </c>
+        <v>0.2650602409638554</v>
+      </c>
+      <c r="F506" t="inlineStr"/>
       <c r="G506" t="inlineStr"/>
       <c r="H506" t="inlineStr">
         <is>
-          <t>0.2575 (0.0216)</t>
+          <t>0.2651 (0.0000)</t>
         </is>
       </c>
     </row>
@@ -18609,7 +18609,7 @@
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -18618,17 +18618,15 @@
         </is>
       </c>
       <c r="E507" t="n">
-        <v>0.2929292929292929</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="F507" t="n">
-        <v>0.2972292191435768</v>
-      </c>
-      <c r="G507" t="n">
-        <v>0.3169398907103825</v>
-      </c>
+        <v>0.2421875</v>
+      </c>
+      <c r="G507" t="inlineStr"/>
       <c r="H507" t="inlineStr">
         <is>
-          <t>0.3024 (0.0128)</t>
+          <t>0.2575 (0.0216)</t>
         </is>
       </c>
     </row>
@@ -18645,7 +18643,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
@@ -18654,17 +18652,17 @@
         </is>
       </c>
       <c r="E508" t="n">
-        <v>0.2288135593220339</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="F508" t="n">
-        <v>0.2433460076045627</v>
+        <v>0.2972292191435768</v>
       </c>
       <c r="G508" t="n">
-        <v>0.2704918032786885</v>
+        <v>0.3169398907103825</v>
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>0.2476 (0.0212)</t>
+          <t>0.3024 (0.0128)</t>
         </is>
       </c>
     </row>
@@ -18681,7 +18679,7 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
@@ -18690,17 +18688,17 @@
         </is>
       </c>
       <c r="E509" t="n">
-        <v>0.3179916317991632</v>
+        <v>0.2288135593220339</v>
       </c>
       <c r="F509" t="n">
-        <v>0.3206106870229007</v>
+        <v>0.2433460076045627</v>
       </c>
       <c r="G509" t="n">
-        <v>0.3728813559322034</v>
+        <v>0.2704918032786885</v>
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>0.3372 (0.0310)</t>
+          <t>0.2476 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18717,7 +18715,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -18726,17 +18724,17 @@
         </is>
       </c>
       <c r="E510" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.3179916317991632</v>
       </c>
       <c r="F510" t="n">
-        <v>0.247787610619469</v>
+        <v>0.3206106870229007</v>
       </c>
       <c r="G510" t="n">
-        <v>0.3055555555555556</v>
+        <v>0.3728813559322034</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>0.2585 (0.0427)</t>
+          <t>0.3372 (0.0310)</t>
         </is>
       </c>
     </row>
@@ -18748,31 +18746,31 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>rf</t>
+          <t>logistic</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="E511" t="n">
-        <v>0.2923076923076923</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="F511" t="n">
-        <v>0.2844444444444444</v>
+        <v>0.247787610619469</v>
       </c>
       <c r="G511" t="n">
-        <v>0.2627737226277372</v>
+        <v>0.3055555555555556</v>
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>0.2798 (0.0153)</t>
+          <t>0.2585 (0.0427)</t>
         </is>
       </c>
     </row>
@@ -18789,7 +18787,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -18798,17 +18796,17 @@
         </is>
       </c>
       <c r="E512" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.2923076923076923</v>
       </c>
       <c r="F512" t="n">
-        <v>0.2450980392156863</v>
+        <v>0.2844444444444444</v>
       </c>
       <c r="G512" t="n">
-        <v>0.3775510204081632</v>
+        <v>0.2627737226277372</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>0.3208 (0.0682)</t>
+          <t>0.2798 (0.0153)</t>
         </is>
       </c>
     </row>
@@ -18825,7 +18823,7 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Morgan</t>
+          <t>MACCS</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
@@ -18834,17 +18832,17 @@
         </is>
       </c>
       <c r="E513" t="n">
-        <v>0.1323529411764706</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="F513" t="n">
-        <v>0.2051282051282051</v>
+        <v>0.2450980392156863</v>
       </c>
       <c r="G513" t="n">
-        <v>0.2097902097902098</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>0.1824 (0.0434)</t>
+          <t>0.3208 (0.0682)</t>
         </is>
       </c>
     </row>
@@ -18861,7 +18859,7 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Morgan</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
@@ -18870,17 +18868,17 @@
         </is>
       </c>
       <c r="E514" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.1323529411764706</v>
       </c>
       <c r="F514" t="n">
-        <v>0.362962962962963</v>
+        <v>0.2051282051282051</v>
       </c>
       <c r="G514" t="n">
-        <v>0.3852459016393442</v>
+        <v>0.2097902097902098</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>0.3845 (0.0212)</t>
+          <t>0.1824 (0.0434)</t>
         </is>
       </c>
     </row>
@@ -18897,7 +18895,7 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>RDKit</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
@@ -18906,17 +18904,17 @@
         </is>
       </c>
       <c r="E515" t="n">
-        <v>0.2266666666666667</v>
+        <v>0.4054054054054054</v>
       </c>
       <c r="F515" t="n">
-        <v>0.1940298507462687</v>
+        <v>0.362962962962963</v>
       </c>
       <c r="G515" t="n">
-        <v>0.1774193548387097</v>
+        <v>0.3852459016393442</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>0.1994 (0.0251)</t>
+          <t>0.3845 (0.0212)</t>
         </is>
       </c>
     </row>
@@ -18928,31 +18926,31 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>xgb</t>
+          <t>rf</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Layered</t>
+          <t>RDKit</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E516" t="n">
-        <v>0.3047619047619048</v>
+        <v>0.2266666666666667</v>
       </c>
       <c r="F516" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.1940298507462687</v>
       </c>
       <c r="G516" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.1774193548387097</v>
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>0.2753 (0.0283)</t>
+          <t>0.1994 (0.0251)</t>
         </is>
       </c>
     </row>
@@ -18969,7 +18967,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>MACCS</t>
+          <t>Layered</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
@@ -18978,17 +18976,17 @@
         </is>
       </c>
       <c r="E517" t="n">
-        <v>0.3317535545023697</v>
+        <v>0.3047619047619048</v>
       </c>
       <c r="F517" t="n">
-        <v>0.2831050228310502</v>
+        <v>0.2727272727272727</v>
       </c>